<commit_message>
feat: sort eligibility report and dashboard tables by episode count descending
</commit_message>
<xml_diff>
--- a/eligible_episodes_pool.xlsx
+++ b/eligible_episodes_pool.xlsx
@@ -13925,7 +13925,7 @@
         <v>精算媽咪的家計簿</v>
       </c>
       <c r="C516" t="str">
-        <v>#768 財富自由的公式竟是「能力減去慾望」？破解理財焦慮，用「餘裕」與無聊投資奪回人生選擇權 來賓：蔡宇哲、郝旭烈</v>
+        <v>#768 財富自由的公式竟���「能力減去慾望」？破解理財焦慮，用「餘裕」與無聊投資奪回人生選擇權 來賓：蔡宇哲、郝旭烈</v>
       </c>
       <c r="D516" t="str">
         <v>2026-04-05</v>
@@ -20733,7 +20733,7 @@
         <v>說話人聲</v>
       </c>
       <c r="C812" t="str">
-        <v>EP.45 ｜【說話人聲-會客室】你為什麼會這樣說話？（下）用聲音練出你的表達天賦</v>
+        <v>EP.45 ｜【說話人聲-會客室】你為什麼會這樣說話？（下）用聲音練出���的表達天賦</v>
       </c>
       <c r="D812" t="str">
         <v>2026-01-18</v>
@@ -20876,13 +20876,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>山姆書書</v>
+        <v>郝旭烈/郝聲音</v>
       </c>
       <c r="C2" t="str">
-        <v>山姆書書</v>
+        <v>郝聲音</v>
       </c>
       <c r="D2">
-        <v>24</v>
+        <v>175</v>
       </c>
       <c r="E2" t="str">
         <v>合格</v>
@@ -20896,13 +20896,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>主播/主持人朱楚文</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="C3" t="str">
-        <v>科技領航家</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D3">
-        <v>24</v>
+        <v>75</v>
       </c>
       <c r="E3" t="str">
         <v>合格</v>
@@ -20916,13 +20916,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>蕭邦</v>
       </c>
       <c r="C4" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D4">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="E4" t="str">
         <v>合格</v>
@@ -20936,13 +20936,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>佐依Zoey</v>
+        <v>Dr Selena</v>
       </c>
       <c r="C5" t="str">
-        <v>佐編茶水間</v>
+        <v>小資變有錢｜Dr.Selena生活理財王</v>
       </c>
       <c r="D5">
-        <v>14</v>
+        <v>50</v>
       </c>
       <c r="E5" t="str">
         <v>合格</v>
@@ -20956,13 +20956,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>別人的工作最有趣｜Fiona</v>
+        <v>林程揚｜Hank大叔</v>
       </c>
       <c r="C6" t="str">
-        <v>別人的工作最有趣</v>
+        <v>能量黑客</v>
       </c>
       <c r="D6">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="E6" t="str">
         <v>合格</v>
@@ -20996,13 +20996,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="C8" t="str">
-        <v>《姐姐不想懂事了》 | Soft Rebellion</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D8">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="E8" t="str">
         <v>合格</v>
@@ -21016,13 +21016,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>林程揚｜Hank大叔</v>
+        <v>美股夢想家</v>
       </c>
       <c r="C9" t="str">
-        <v>能量黑客</v>
+        <v>夢想家說股事</v>
       </c>
       <c r="D9">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="E9" t="str">
         <v>合格</v>
@@ -21036,13 +21036,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>美業幹什麼｜蔡佩陵</v>
       </c>
       <c r="C10" t="str">
-        <v>哇賽心理學</v>
+        <v>美業幹什麼</v>
       </c>
       <c r="D10">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="E10" t="str">
         <v>合格</v>
@@ -21076,13 +21076,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>美股夢想家</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="C12" t="str">
-        <v>夢想家說股事</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D12">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="E12" t="str">
         <v>合格</v>
@@ -21096,13 +21096,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>美業幹什麼｜蔡佩陵</v>
+        <v>聲音表達講師林依柔</v>
       </c>
       <c r="C13" t="str">
-        <v>美業幹什麼</v>
+        <v>說話人聲</v>
       </c>
       <c r="D13">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E13" t="str">
         <v>合格</v>
@@ -21116,13 +21116,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>孫子玲</v>
+        <v>莫菲穿搭</v>
       </c>
       <c r="C14" t="str">
-        <v>子玲的親子聊心屋-媽咪的自我成長&amp;親子教養</v>
+        <v>【莫轉台】-試穿新人生</v>
       </c>
       <c r="D14">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E14" t="str">
         <v>合格</v>
@@ -21136,13 +21136,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>山姆書書</v>
       </c>
       <c r="C15" t="str">
-        <v>郝聲音</v>
+        <v>山姆書書</v>
       </c>
       <c r="D15">
-        <v>175</v>
+        <v>24</v>
       </c>
       <c r="E15" t="str">
         <v>合格</v>
@@ -21156,13 +21156,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>張忘形</v>
+        <v>主播/主持人朱楚文</v>
       </c>
       <c r="C16" t="str">
-        <v>人類行為研究社</v>
+        <v>科技領航家</v>
       </c>
       <c r="D16">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E16" t="str">
         <v>合格</v>
@@ -21176,13 +21176,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>莫菲穿搭</v>
+        <v>別人的工作最有趣｜Fiona</v>
       </c>
       <c r="C17" t="str">
-        <v>【莫轉台】-試穿新人生</v>
+        <v>別人的工作最有趣</v>
       </c>
       <c r="D17">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E17" t="str">
         <v>合格</v>
@@ -21196,13 +21196,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="C18" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D18">
-        <v>75</v>
+        <v>24</v>
       </c>
       <c r="E18" t="str">
         <v>合格</v>
@@ -21216,13 +21216,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>蕭邦</v>
+        <v>張忘形</v>
       </c>
       <c r="C19" t="str">
-        <v>蕭邦相談室</v>
+        <v>人類行為研究社</v>
       </c>
       <c r="D19">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="E19" t="str">
         <v>合格</v>
@@ -21236,13 +21236,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>聲音表達講師林依柔</v>
+        <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
       </c>
       <c r="C20" t="str">
-        <v>說話人聲</v>
+        <v>《姐姐不想懂事了》 | Soft Rebellion</v>
       </c>
       <c r="D20">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E20" t="str">
         <v>合格</v>
@@ -21256,13 +21256,13 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>孫子玲</v>
       </c>
       <c r="C21" t="str">
-        <v>蘇心時光</v>
+        <v>子玲的親子聊心屋-媽咪的自我成長&amp;親子教養</v>
       </c>
       <c r="D21">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E21" t="str">
         <v>合格</v>
@@ -21276,13 +21276,13 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>Dr Selena</v>
+        <v>佐依Zoey</v>
       </c>
       <c r="C22" t="str">
-        <v>小資變有錢｜Dr.Selena生活理財王</v>
+        <v>佐編茶水間</v>
       </c>
       <c r="D22">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="E22" t="str">
         <v>合格</v>
@@ -21296,19 +21296,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>30節約男子</v>
+        <v>潘思璇ＣＰ</v>
       </c>
       <c r="C23" t="str">
-        <v>財富餐車不打烊</v>
+        <v>CP有主見</v>
       </c>
       <c r="D23">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E23" t="str">
         <v>資格不符</v>
       </c>
       <c r="F23" t="str">
-        <v>資格不符 (無 Podcast 節目)</v>
+        <v>資格不符 (發片集數不足 12 集)</v>
       </c>
     </row>
     <row r="24">
@@ -21316,19 +21316,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>丁菱娟</v>
+        <v>慢活夫妻Dewi&amp;George</v>
       </c>
       <c r="C24" t="str">
-        <v>丁菱娟邊走邊想</v>
+        <v>慢活夫妻－專業美股投資與理財</v>
       </c>
       <c r="D24">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E24" t="str">
         <v>資格不符</v>
       </c>
       <c r="F24" t="str">
-        <v>資格不符 (無 Podcast 節目)</v>
+        <v>資格不符 (發片集數不足 12 集)</v>
       </c>
     </row>
     <row r="25">
@@ -21336,19 +21336,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>人生啊！小歐</v>
+        <v>崔咪</v>
       </c>
       <c r="C25" t="str">
-        <v>人生啊｜用我的人生故事，陪你看懂自己</v>
+        <v>一不小心太漂亮</v>
       </c>
       <c r="D25">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E25" t="str">
         <v>資格不符</v>
       </c>
       <c r="F25" t="str">
-        <v>資格不符 (無 Podcast 節目)</v>
+        <v>資格不符 (發片集數不足 12 集)</v>
       </c>
     </row>
     <row r="26">
@@ -21356,19 +21356,19 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>下半場陪談師＿張嘉茹老師</v>
+        <v>樂筆</v>
       </c>
       <c r="C26" t="str">
-        <v>下半場陪談師</v>
+        <v>歡迎光臨</v>
       </c>
       <c r="D26">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E26" t="str">
         <v>資格不符</v>
       </c>
       <c r="F26" t="str">
-        <v>資格不符 (無 Podcast 節目)</v>
+        <v>資格不符 (發片集數不足 12 集)</v>
       </c>
     </row>
     <row r="27">
@@ -21376,10 +21376,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>小河馬媽媽</v>
+        <v>30節約男子</v>
       </c>
       <c r="C27" t="str">
-        <v>來晚無添加河粉吧！</v>
+        <v>財富餐車不打烊</v>
       </c>
       <c r="D27">
         <v>0</v>
@@ -21396,10 +21396,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>小思大維｜雪柔</v>
+        <v>丁菱娟</v>
       </c>
       <c r="C28" t="str">
-        <v>小思大維</v>
+        <v>丁菱娟邊走邊想</v>
       </c>
       <c r="D28">
         <v>0</v>
@@ -21416,10 +21416,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>不敗教主-陳重銘</v>
+        <v>人生啊！小歐</v>
       </c>
       <c r="C29" t="str">
-        <v>不敗教主-陳重銘</v>
+        <v>人生啊｜用我的人生故事，陪你看懂自己</v>
       </c>
       <c r="D29">
         <v>0</v>
@@ -21436,10 +21436,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>五吉郎</v>
+        <v>下半場陪談師＿張嘉茹老師</v>
       </c>
       <c r="C30" t="str">
-        <v>五</v>
+        <v>下半場陪談師</v>
       </c>
       <c r="D30">
         <v>0</v>
@@ -21456,10 +21456,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="str">
-        <v>文森說書</v>
+        <v>小河馬媽媽</v>
       </c>
       <c r="C31" t="str">
-        <v>文森說書</v>
+        <v>來晚無添加河粉吧！</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -21476,10 +21476,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="str">
-        <v>犬兒媽咪の育兒手帳</v>
+        <v>小思大維｜雪柔</v>
       </c>
       <c r="C32" t="str">
-        <v>育兒專機</v>
+        <v>小思大維</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -21496,10 +21496,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="str">
-        <v>王琄</v>
+        <v>不敗教主-陳重銘</v>
       </c>
       <c r="C33" t="str">
-        <v>琄蜜莉的異想世界</v>
+        <v>不敗教主-陳重銘</v>
       </c>
       <c r="D33">
         <v>0</v>
@@ -21516,10 +21516,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="str">
-        <v>尼可這樣說</v>
+        <v>五吉郎</v>
       </c>
       <c r="C34" t="str">
-        <v>尼</v>
+        <v>五</v>
       </c>
       <c r="D34">
         <v>0</v>
@@ -21536,10 +21536,10 @@
         <v>34</v>
       </c>
       <c r="B35" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>文森說書</v>
       </c>
       <c r="C35" t="str">
-        <v>布姐的沙發</v>
+        <v>文森說書</v>
       </c>
       <c r="D35">
         <v>0</v>
@@ -21556,10 +21556,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="str">
-        <v>布萊恩老師</v>
+        <v>犬兒媽咪の育兒手帳</v>
       </c>
       <c r="C36" t="str">
-        <v>布萊恩老師</v>
+        <v>育兒專機</v>
       </c>
       <c r="D36">
         <v>0</v>
@@ -21576,10 +21576,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="str">
-        <v>幼兒情緒教育學院-萬叔的心café</v>
+        <v>王琄</v>
       </c>
       <c r="C37" t="str">
-        <v>幼兒情緒教育學院-萬叔的心café</v>
+        <v>琄蜜莉的異想世界</v>
       </c>
       <c r="D37">
         <v>0</v>
@@ -21596,10 +21596,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="C38" t="str">
-        <v>下一本讀什麼</v>
+        <v>尼</v>
       </c>
       <c r="D38">
         <v>0</v>
@@ -21616,10 +21616,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="str">
-        <v>全遠距工作的行銷人|Coco</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="C39" t="str">
-        <v>—</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D39">
         <v>0</v>
@@ -21636,10 +21636,10 @@
         <v>39</v>
       </c>
       <c r="B40" t="str">
-        <v>即薑抵達｜薑咪</v>
+        <v>布萊恩老師</v>
       </c>
       <c r="C40" t="str">
-        <v>即薑抵達https://open.spotify.com/show/6ZUSdp6iLOWJqay7uKTBxO</v>
+        <v>布萊恩老師</v>
       </c>
       <c r="D40">
         <v>0</v>
@@ -21656,10 +21656,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="str">
-        <v>我的動齡限量版</v>
+        <v>幼兒情緒教育學院-萬叔的心café</v>
       </c>
       <c r="C41" t="str">
-        <v>我的動齡限量版</v>
+        <v>幼兒情緒教育學院-萬叔的心café</v>
       </c>
       <c r="D41">
         <v>0</v>
@@ -21676,10 +21676,10 @@
         <v>41</v>
       </c>
       <c r="B42" t="str">
-        <v>李柏鋒的擴大機</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="C42" t="str">
-        <v>聽進理投</v>
+        <v>下一本讀什麼</v>
       </c>
       <c r="D42">
         <v>0</v>
@@ -21688,7 +21688,7 @@
         <v>資格不符</v>
       </c>
       <c r="F42" t="str">
-        <v>資格不符 (發片集數不足 12 集)</v>
+        <v>資格不符 (無 Podcast 節目)</v>
       </c>
     </row>
     <row r="43">
@@ -21696,10 +21696,10 @@
         <v>42</v>
       </c>
       <c r="B43" t="str">
-        <v>林慧</v>
+        <v>全遠距工作的行銷人|Coco</v>
       </c>
       <c r="C43" t="str">
-        <v>SoWhat做自己很難嗎？</v>
+        <v>—</v>
       </c>
       <c r="D43">
         <v>0</v>
@@ -21716,10 +21716,10 @@
         <v>43</v>
       </c>
       <c r="B44" t="str">
-        <v>治療師瑪奇</v>
+        <v>即薑抵達｜薑咪</v>
       </c>
       <c r="C44" t="str">
-        <v>教出你的路</v>
+        <v>即薑抵達https://open.spotify.com/show/6ZUSdp6iLOWJqay7uKTBxO</v>
       </c>
       <c r="D44">
         <v>0</v>
@@ -21736,10 +21736,10 @@
         <v>44</v>
       </c>
       <c r="B45" t="str">
-        <v>玩命之徒｜林尚諾大師兄</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="C45" t="str">
-        <v>玩命之徒</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="D45">
         <v>0</v>
@@ -21756,10 +21756,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="str">
-        <v>育兒專機｜犬媽</v>
+        <v>李柏鋒的擴大機</v>
       </c>
       <c r="C46" t="str">
-        <v>育兒專機</v>
+        <v>聽進理投</v>
       </c>
       <c r="D46">
         <v>0</v>
@@ -21768,7 +21768,7 @@
         <v>資格不符</v>
       </c>
       <c r="F46" t="str">
-        <v>資格不符 (無 Podcast 節目)</v>
+        <v>資格不符 (發片集數不足 12 集)</v>
       </c>
     </row>
     <row r="47">
@@ -21776,10 +21776,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="str">
-        <v>阿駿日常</v>
+        <v>林慧</v>
       </c>
       <c r="C47" t="str">
-        <v>阿</v>
+        <v>SoWhat做自己很難嗎？</v>
       </c>
       <c r="D47">
         <v>0</v>
@@ -21796,10 +21796,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="str">
-        <v>品牌女子A娜</v>
+        <v>治療師瑪奇</v>
       </c>
       <c r="C48" t="str">
-        <v>你也想紅嗎</v>
+        <v>教出你的路</v>
       </c>
       <c r="D48">
         <v>0</v>
@@ -21816,10 +21816,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="str">
-        <v>胡咪老師</v>
+        <v>玩命之徒｜林尚諾大師兄</v>
       </c>
       <c r="C49" t="str">
-        <v>分手的99個理由</v>
+        <v>玩命之徒</v>
       </c>
       <c r="D49">
         <v>0</v>
@@ -21836,10 +21836,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="str">
-        <v>孫治華</v>
+        <v>育兒專機｜犬媽</v>
       </c>
       <c r="C50" t="str">
-        <v>人生挖挖WoW-企業人生策略學</v>
+        <v>育兒專機</v>
       </c>
       <c r="D50">
         <v>0</v>
@@ -21856,10 +21856,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>迷途艾比</v>
+        <v>阿駿日常</v>
       </c>
       <c r="C51" t="str">
-        <v>迷途星球</v>
+        <v>阿</v>
       </c>
       <c r="D51">
         <v>0</v>
@@ -21868,7 +21868,7 @@
         <v>資格不符</v>
       </c>
       <c r="F51" t="str">
-        <v>資格不符 (發片集數不足 12 集)</v>
+        <v>資格不符 (無 Podcast 節目)</v>
       </c>
     </row>
     <row r="52">
@@ -21876,10 +21876,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="str">
-        <v>高言值表達力教練｜竺宥璋｜小竺</v>
+        <v>品牌女子A娜</v>
       </c>
       <c r="C52" t="str">
-        <v>—</v>
+        <v>你也想紅嗎</v>
       </c>
       <c r="D52">
         <v>0</v>
@@ -21896,19 +21896,19 @@
         <v>52</v>
       </c>
       <c r="B53" t="str">
-        <v>崔咪</v>
+        <v>胡咪老師</v>
       </c>
       <c r="C53" t="str">
-        <v>一不小心太漂亮</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D53">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E53" t="str">
         <v>資格不符</v>
       </c>
       <c r="F53" t="str">
-        <v>資格不符 (發片集數不足 12 集)</v>
+        <v>資格不符 (無 Podcast 節目)</v>
       </c>
     </row>
     <row r="54">
@@ -21916,10 +21916,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="str">
-        <v>張書書</v>
+        <v>孫治華</v>
       </c>
       <c r="C54" t="str">
-        <v>張書書</v>
+        <v>人生挖挖WoW-企業人生策略學</v>
       </c>
       <c r="D54">
         <v>0</v>
@@ -21936,10 +21936,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="str">
-        <v>斜槓空姐cindy</v>
+        <v>迷途艾比</v>
       </c>
       <c r="C55" t="str">
-        <v>斜槓空姐cindy</v>
+        <v>迷途星球</v>
       </c>
       <c r="D55">
         <v>0</v>
@@ -21948,7 +21948,7 @@
         <v>資格不符</v>
       </c>
       <c r="F55" t="str">
-        <v>資格不符 (無 Podcast 節目)</v>
+        <v>資格不符 (發片集數不足 12 集)</v>
       </c>
     </row>
     <row r="56">
@@ -21956,10 +21956,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="str">
-        <v>曼蒂歐逆-轉型之路</v>
+        <v>高言值表達力教練｜竺宥璋｜小竺</v>
       </c>
       <c r="C56" t="str">
-        <v>曼蒂歐逆-轉型之路</v>
+        <v>—</v>
       </c>
       <c r="D56">
         <v>0</v>
@@ -21976,10 +21976,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="str">
-        <v>梁哲維</v>
+        <v>張書書</v>
       </c>
       <c r="C57" t="str">
-        <v>哲維說書</v>
+        <v>張書書</v>
       </c>
       <c r="D57">
         <v>0</v>
@@ -21996,10 +21996,10 @@
         <v>57</v>
       </c>
       <c r="B58" t="str">
-        <v>莊舒涵（卡姊）</v>
+        <v>斜槓空姐cindy</v>
       </c>
       <c r="C58" t="str">
-        <v>我不是病人，我是卡姊！</v>
+        <v>斜槓空姐cindy</v>
       </c>
       <c r="D58">
         <v>0</v>
@@ -22016,10 +22016,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="str">
-        <v>喬王的投資理財筆記</v>
+        <v>曼蒂歐逆-轉型之路</v>
       </c>
       <c r="C59" t="str">
-        <v>斜槓槓槓槓</v>
+        <v>曼蒂歐逆-轉型之路</v>
       </c>
       <c r="D59">
         <v>0</v>
@@ -22036,10 +22036,10 @@
         <v>59</v>
       </c>
       <c r="B60" t="str">
-        <v>無所不試無樂不作</v>
+        <v>梁哲維</v>
       </c>
       <c r="C60" t="str">
-        <v>無所不試無樂不作</v>
+        <v>哲維說書</v>
       </c>
       <c r="D60">
         <v>0</v>
@@ -22056,10 +22056,10 @@
         <v>60</v>
       </c>
       <c r="B61" t="str">
-        <v>微光中的貓| Claire Hsiao</v>
+        <v>莊舒涵（卡姊）</v>
       </c>
       <c r="C61" t="str">
-        <v>微光中的北極星</v>
+        <v>我不是病人，我是卡姊！</v>
       </c>
       <c r="D61">
         <v>0</v>
@@ -22076,10 +22076,10 @@
         <v>61</v>
       </c>
       <c r="B62" t="str">
-        <v>楊月娥（楊肉爐）</v>
+        <v>喬王的投資理財筆記</v>
       </c>
       <c r="C62" t="str">
-        <v>楊肉盧</v>
+        <v>斜槓槓槓槓</v>
       </c>
       <c r="D62">
         <v>0</v>
@@ -22096,10 +22096,10 @@
         <v>62</v>
       </c>
       <c r="B63" t="str">
-        <v>雷浩斯價值投資網</v>
+        <v>無所不試無樂不作</v>
       </c>
       <c r="C63" t="str">
-        <v>雷浩斯價值投資網</v>
+        <v>無所不試無樂不作</v>
       </c>
       <c r="D63">
         <v>0</v>
@@ -22116,19 +22116,19 @@
         <v>63</v>
       </c>
       <c r="B64" t="str">
-        <v>慢活夫妻Dewi&amp;George</v>
+        <v>微光中的貓| Claire Hsiao</v>
       </c>
       <c r="C64" t="str">
-        <v>慢活夫妻－專業美股投資與理財</v>
+        <v>微光中的北極星</v>
       </c>
       <c r="D64">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E64" t="str">
         <v>資格不符</v>
       </c>
       <c r="F64" t="str">
-        <v>資格不符 (發片集數不足 12 集)</v>
+        <v>資格不符 (無 Podcast 節目)</v>
       </c>
     </row>
     <row r="65">
@@ -22136,10 +22136,10 @@
         <v>64</v>
       </c>
       <c r="B65" t="str">
-        <v>瑪那熊諮商心理師</v>
+        <v>楊月娥（楊肉爐）</v>
       </c>
       <c r="C65" t="str">
-        <v>瑪那熊諮商心理師</v>
+        <v>楊肉盧</v>
       </c>
       <c r="D65">
         <v>0</v>
@@ -22156,10 +22156,10 @@
         <v>65</v>
       </c>
       <c r="B66" t="str">
-        <v>維琪的幸福叮嚀</v>
+        <v>雷浩斯價值投資網</v>
       </c>
       <c r="C66" t="str">
-        <v>能量黑客</v>
+        <v>雷浩斯價值投資網</v>
       </c>
       <c r="D66">
         <v>0</v>
@@ -22176,10 +22176,10 @@
         <v>66</v>
       </c>
       <c r="B67" t="str">
-        <v>趙函穎的營養健康週報</v>
+        <v>瑪那熊諮商心理師</v>
       </c>
       <c r="C67" t="str">
-        <v>趙函穎的營養健康報報</v>
+        <v>瑪那熊諮商心理師</v>
       </c>
       <c r="D67">
         <v>0</v>
@@ -22196,10 +22196,10 @@
         <v>67</v>
       </c>
       <c r="B68" t="str">
-        <v>劉亦酉</v>
+        <v>維琪的幸福叮嚀</v>
       </c>
       <c r="C68" t="str">
-        <v>劉亦酉</v>
+        <v>能量黑客</v>
       </c>
       <c r="D68">
         <v>0</v>
@@ -22216,10 +22216,10 @@
         <v>68</v>
       </c>
       <c r="B69" t="str">
-        <v>廣播主持人_楊凱涵</v>
+        <v>趙函穎的營養健康週報</v>
       </c>
       <c r="C69" t="str">
-        <v>請多包涵/ BaoHan Talk</v>
+        <v>趙函穎的營養健康報報</v>
       </c>
       <c r="D69">
         <v>0</v>
@@ -22236,19 +22236,19 @@
         <v>69</v>
       </c>
       <c r="B70" t="str">
-        <v>樂筆</v>
+        <v>劉亦酉</v>
       </c>
       <c r="C70" t="str">
-        <v>歡迎光臨</v>
+        <v>劉亦酉</v>
       </c>
       <c r="D70">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E70" t="str">
         <v>資格不符</v>
       </c>
       <c r="F70" t="str">
-        <v>資格不符 (發片集數不足 12 集)</v>
+        <v>資格不符 (無 Podcast 節目)</v>
       </c>
     </row>
     <row r="71">
@@ -22256,19 +22256,19 @@
         <v>70</v>
       </c>
       <c r="B71" t="str">
-        <v>潘思璇ＣＰ</v>
+        <v>廣播主持人_楊凱涵</v>
       </c>
       <c r="C71" t="str">
-        <v>CP有主見</v>
+        <v>請多包涵/ BaoHan Talk</v>
       </c>
       <c r="D71">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="E71" t="str">
         <v>資格不符</v>
       </c>
       <c r="F71" t="str">
-        <v>資格不符 (發片集數不足 12 集)</v>
+        <v>資格不符 (無 Podcast 節目)</v>
       </c>
     </row>
     <row r="72">

</xml_diff>

<commit_message>
feat: read KOL list directly from Excel '合作名單' sheet as source of truth
</commit_message>
<xml_diff>
--- a/eligible_episodes_pool.xlsx
+++ b/eligible_episodes_pool.xlsx
@@ -2121,7 +2121,7 @@
         <v>曼蒂歐逆-轉型之路</v>
       </c>
       <c r="C6" t="str">
-        <v>曼蒂歐逆-轉型之路</v>
+        <v/>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -2181,7 +2181,7 @@
         <v>人生啊！小歐</v>
       </c>
       <c r="C9" t="str">
-        <v>人生啊｜用我的人生故事，陪你看懂自己</v>
+        <v/>
       </c>
       <c r="D9" t="str">
         <v/>
@@ -2201,7 +2201,7 @@
         <v>下半場陪談師＿張嘉茹老師</v>
       </c>
       <c r="C10" t="str">
-        <v>下半場陪談師</v>
+        <v/>
       </c>
       <c r="D10" t="str">
         <v/>
@@ -2241,7 +2241,7 @@
         <v>斜槓空姐cindy</v>
       </c>
       <c r="C12" t="str">
-        <v>斜槓空姐cindy</v>
+        <v/>
       </c>
       <c r="D12" t="str">
         <v/>
@@ -2361,7 +2361,7 @@
         <v>瑪那熊諮商心理師</v>
       </c>
       <c r="C18" t="str">
-        <v>瑪那熊諮商心理師</v>
+        <v/>
       </c>
       <c r="D18" t="str">
         <v/>
@@ -2581,7 +2581,7 @@
         <v>布萊恩老師</v>
       </c>
       <c r="C29" t="str">
-        <v>布萊恩老師</v>
+        <v/>
       </c>
       <c r="D29" t="str">
         <v/>
@@ -2601,7 +2601,7 @@
         <v>全遠距工作的行銷人|Coco</v>
       </c>
       <c r="C30" t="str">
-        <v>全遠距工作的行銷人|Coco</v>
+        <v/>
       </c>
       <c r="D30" t="str">
         <v/>
@@ -2701,7 +2701,7 @@
         <v>高言值表達力教練｜竺宥璋｜小竺</v>
       </c>
       <c r="C35" t="str">
-        <v>高言值表達力教練｜竺宥璋｜小竺</v>
+        <v/>
       </c>
       <c r="D35" t="str">
         <v/>
@@ -2721,7 +2721,7 @@
         <v>張書書</v>
       </c>
       <c r="C36" t="str">
-        <v>張書書</v>
+        <v/>
       </c>
       <c r="D36" t="str">
         <v/>
@@ -2761,7 +2761,7 @@
         <v>劉亦酉</v>
       </c>
       <c r="C38" t="str">
-        <v>劉亦酉</v>
+        <v/>
       </c>
       <c r="D38" t="str">
         <v/>
@@ -2921,7 +2921,7 @@
         <v>Coco｜全遠距工作的行銷人</v>
       </c>
       <c r="C46" t="str">
-        <v>Coco｜全遠距工作的行銷人</v>
+        <v/>
       </c>
       <c r="D46" t="str">
         <v/>
@@ -3181,7 +3181,7 @@
         <v>雷浩斯價值投資網</v>
       </c>
       <c r="C59" t="str">
-        <v>雷浩斯價值投資網</v>
+        <v/>
       </c>
       <c r="D59" t="str">
         <v/>
@@ -3521,7 +3521,7 @@
         <v>幼兒情緒教育學院-萬叔的心café</v>
       </c>
       <c r="C76" t="str">
-        <v>幼兒情緒教育學院-萬叔的心café</v>
+        <v/>
       </c>
       <c r="D76" t="str">
         <v/>
@@ -3541,7 +3541,7 @@
         <v>阿駿日常</v>
       </c>
       <c r="C77" t="str">
-        <v>阿駿日常</v>
+        <v/>
       </c>
       <c r="D77" t="str">
         <v/>
@@ -5517,7 +5517,7 @@
         <v>宋家小館</v>
       </c>
       <c r="C66" t="str">
-        <v>EP155 | 當收藏成為一種命運：RedBar創辦人Joe的錶與人生哲學</v>
+        <v>EP155 | 當收藏成為一種命���：RedBar創辦人Joe的錶與人生哲學</v>
       </c>
       <c r="D66" t="str">
         <v>2026-01-06</v>
@@ -8446,7 +8446,7 @@
         <v>五吉郎</v>
       </c>
       <c r="C167" t="str">
-        <v>EP153｜小孩子才做選擇？想要「全拿」的背後，你必須具備這套頂級策略思維（Feat. PaGamO企業服務��業群總經理/女人進階 主理人 Eva 張怡婷）</v>
+        <v>EP153｜小孩子才做選擇？想要「全拿」的背後，你必須具備這套頂級策略思維（Feat. PaGamO企業服務事業群總經理/女人進階 主理人 Eva 張怡婷）</v>
       </c>
       <c r="D167" t="str">
         <v>2026-04-23</v>
@@ -15145,7 +15145,7 @@
         <v>文森說書</v>
       </c>
       <c r="C398" t="str">
-        <v>這些人都有工作，但為什麼只能住在街頭？｜《老窮奇幻紀事》</v>
+        <v>這些人都有工作，但為什麼只能住在���頭？｜《老窮奇幻紀事》</v>
       </c>
       <c r="D398" t="str">
         <v>2026-04-17</v>
@@ -15812,7 +15812,7 @@
         <v>下一本讀什麼？</v>
       </c>
       <c r="C421" t="str">
-        <v>EP.603 《快樂性感��百萬富翁》讀後心得：達成所有目標…之後呢？</v>
+        <v>EP.603 《快樂性感的百萬富翁》讀後心得：達成所有目標…之後呢？</v>
       </c>
       <c r="D421" t="str">
         <v>2026-05-11</v>
@@ -17233,7 +17233,7 @@
         <v>佐編茶水間</v>
       </c>
       <c r="C470" t="str">
-        <v>#340 #Natasha｜��彩的人生，究竟長什麼模樣？我們存在的意義又是什麼？</v>
+        <v>#340 #Natasha｜���彩的人生，究竟長什麼模樣？我們存在的意義又是什麼？</v>
       </c>
       <c r="D470" t="str">
         <v>2026-05-03</v>
@@ -17349,7 +17349,7 @@
         <v>佐編茶水間</v>
       </c>
       <c r="C474" t="str">
-        <v>#我，是誰？S2E5｜讓自己的內在減少敵對關係，關鍵��於「看見優點」的能力</v>
+        <v>#我，是誰？S2E5｜讓自己的內在減少敵對關係，關鍵���於「看見優點」的能力</v>
       </c>
       <c r="D474" t="str">
         <v>2026-04-01</v>
@@ -17523,7 +17523,7 @@
         <v>佐編茶水間</v>
       </c>
       <c r="C480" t="str">
-        <v>#338 #李霈瑜｜生活中扮演多個��色如何平衡？怎麼包容自己做到真正接納？❤️</v>
+        <v>#338 #李霈瑜｜生活中扮演多個���色如何平衡？怎麼包容自己做到真正接納？❤️</v>
       </c>
       <c r="D480" t="str">
         <v>2026-02-08</v>
@@ -27180,7 +27180,7 @@
         <v>閱讀聊樂KEY</v>
       </c>
       <c r="C813" t="str">
-        <v>EP213 越學越焦慮？郝旭烈���解現代人知識內耗：不教你讀書，教你鬆綁、放過自己 | 郝會讀書 | 郝哥</v>
+        <v>EP213 越學越焦慮？郝旭烈破解現代人知識內耗：不教你讀書，教你鬆綁、放過自己 | 郝會讀�� | 郝哥</v>
       </c>
       <c r="D813" t="str">
         <v>2026-05-26</v>
@@ -27325,7 +27325,7 @@
         <v>閱讀聊樂KEY</v>
       </c>
       <c r="C818" t="str">
-        <v>EP208 不帶評判，才是理解一個人的開始，用正念放下評判，改寫你的人生劇本 | 趙安安博士</v>
+        <v>EP208 不帶評判，才是理解一個人的開始，用正念放下評判，���寫你的人生劇本 | 趙安安博士</v>
       </c>
       <c r="D818" t="str">
         <v>2026-04-21</v>
@@ -27731,7 +27731,7 @@
         <v>閱讀聊樂KEY</v>
       </c>
       <c r="C832" t="str">
-        <v>EP194 為什麼你的努力沒人看見？打造 AI 搶不走的職場亮點｜獨創現場力 ���震宇</v>
+        <v>EP194 為什麼你的努力沒人看見？打造 AI 搶不走的職場亮點｜獨創現場力 洪震宇</v>
       </c>
       <c r="D832" t="str">
         <v>2026-01-13</v>
@@ -27934,7 +27934,7 @@
         <v>小資變有錢｜Dr.Selena生活理財王</v>
       </c>
       <c r="C839" t="str">
-        <v>全球房地��特輯：下一個亞洲財富熱點在哪裡？馬來西亞投資置產與退休趨勢解析!</v>
+        <v>全球房地產特輯：下一個亞洲財富熱點在哪裡？馬來西亞投資置產與退休趨勢解析!</v>
       </c>
       <c r="D839" t="str">
         <v>2026-05-30</v>
@@ -28601,7 +28601,7 @@
         <v>小資變有錢｜Dr.Selena生活理財王</v>
       </c>
       <c r="C862" t="str">
-        <v>郝哥專訪：從金錢焦慮到人��選擇權：一步步走向真正的財富自由</v>
+        <v>郝哥專訪：從金錢焦慮到人生選擇權：一步步走向真正的財富自由</v>
       </c>
       <c r="D862" t="str">
         <v>2026-03-12</v>
@@ -28630,7 +28630,7 @@
         <v>小資變有錢｜Dr.Selena生活理財王</v>
       </c>
       <c r="C863" t="str">
-        <v>小資愛樂活：你每天吃的那一碗米，真的安心嗎��從土地到餐桌，找回真正的安心!</v>
+        <v>小資愛樂活：你每天吃的那一碗米，真的安心嗎？從土地到餐桌，找回真正的安心!</v>
       </c>
       <c r="D863" t="str">
         <v>2026-03-08</v>
@@ -30718,7 +30718,7 @@
         <v>科技領航家</v>
       </c>
       <c r="C935" t="str">
-        <v>EP333 AI 走進醫療現場：智慧醫療的關鍵轉捩點到了嗎？  Ft. 華碩智慧健康產品企劃課經理 賴政宇</v>
+        <v>EP333 AI ��進醫療現場：智慧醫療的關鍵轉捩點到了嗎？  Ft. 華碩智慧健康產品企劃課經理 賴政宇</v>
       </c>
       <c r="D935" t="str">
         <v>2026-01-20</v>
@@ -34024,7 +34024,7 @@
         <v>不敗教主陳重銘</v>
       </c>
       <c r="C1049" t="str">
-        <v>EP599比特幣跌到腰斬，現���能進場投資嗎？</v>
+        <v>EP599比特幣跌到腰斬，現在能進場投資嗎？</v>
       </c>
       <c r="D1049" t="str">
         <v>2026-02-25</v>
@@ -44348,7 +44348,7 @@
         <v>郝聲音</v>
       </c>
       <c r="C1405" t="str">
-        <v>郝聲音：（上）「你在學飛，我在學放手」：從誤會到理解，從疏遠到靠近，46封修復關係的親子書信好書分享 ～ 吳緁苓, 林昀靜, 林廷旭</v>
+        <v>郝聲���：（上）「你在學飛，我在學放手」：從誤會到理解，從疏遠到靠近，46封修復關係的親子書信好書分享 ～ 吳緁苓, 林昀靜, 林廷旭</v>
       </c>
       <c r="D1405" t="str">
         <v>2026-04-23</v>
@@ -44899,7 +44899,7 @@
         <v>郝聲音</v>
       </c>
       <c r="C1424" t="str">
-        <v>郝聲音：（上）阿金的「火星計劃」：如果你「相信」你可以，最後不僅你可以，你也會帶著一群人一起可以</v>
+        <v>郝聲音：（上）阿金的「火星計劃」：如果你「相信」你可以，最後不僅你可以，你也會��著一群人一起可以</v>
       </c>
       <c r="D1424" t="str">
         <v>2026-04-04</v>
@@ -45740,7 +45740,7 @@
         <v>郝聲音</v>
       </c>
       <c r="C1453" t="str">
-        <v>郝聲音：（上）Sun自由教���的「自由選擇人生」</v>
+        <v>郝聲音：（上）Sun自由教練的「自由選擇人生」</v>
       </c>
       <c r="D1453" t="str">
         <v>2026-03-11</v>
@@ -46030,7 +46030,7 @@
         <v>郝聲音</v>
       </c>
       <c r="C1463" t="str">
-        <v>郝聲音：（上）張添皓醫師好書分享 「大人的牙齒保健室」：牙好人不老，從口腔開始打造你的健康���壽方程式</v>
+        <v>郝聲音：（上）張添皓醫師好書分享 「大人的牙齒保健室」：牙好人不老，從口腔開始打造你的健康長壽方程式</v>
       </c>
       <c r="D1463" t="str">
         <v>2026-03-01</v>
@@ -47306,7 +47306,7 @@
         <v>郝聲音</v>
       </c>
       <c r="C1507" t="str">
-        <v>郝聲音：（上）蔡思怡老師：『神展開的國文教室』最有梗的女神國學閱讀筆記，從經典名篇到當代視角，全面打開人生思辨腦</v>
+        <v>郝聲音：（上）蔡思怡老師：『神展開的國文教室』最有梗的女神國學閱讀筆記，從經典名篇到當代視角，全面��開人生思辨腦</v>
       </c>
       <c r="D1507" t="str">
         <v>2026-01-16</v>
@@ -47944,7 +47944,7 @@
         <v>小思大維</v>
       </c>
       <c r="C1529" t="str">
-        <v>第二十七關 | AI天才的對決（討論篇）有了AI當小幫手，還需要讀書嗎？AI時代真正要學的是什麼呢？</v>
+        <v>第二十七關 | AI天才的對決（討論篇）有了AI當小幫��，還需要讀書嗎？AI時代真正要學的是什麼呢？</v>
       </c>
       <c r="D1529" t="str">
         <v>2026-04-08</v>
@@ -48698,7 +48698,7 @@
         <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="C1555" t="str">
-        <v>EP219：【��典家庭CEO】育兒現場走音怎麼辦？從動物音樂會的細節看管理，教養不是起跑點的競爭，是「基本功」的複利投資ft. 薩克斯風音樂家爸爸 沈子傑</v>
+        <v>EP219：【非典家庭CEO】育兒現場走音怎麼辦？從動物音樂會的細節看管理，教養不是起跑點的競爭，是「基本功」的複利投資ft. 薩克斯風音樂家爸爸 沈子傑</v>
       </c>
       <c r="D1555" t="str">
         <v>2026-03-25</v>
@@ -50786,7 +50786,7 @@
         <v>子玲的親子聊心屋-媽咪的自我成長&amp;親子教養</v>
       </c>
       <c r="C1627" t="str">
-        <v>#103 ▍孩子講話總是很跳躍 ,如何培養說話邏輯 ? &lt;兒童自信表達專家-依柔老師&gt;</v>
+        <v>#103 ▍孩子講話總是很跳躍 ,如何培養說話邏輯 ? &lt;兒童自信���達專家-依柔老師&gt;</v>
       </c>
       <c r="D1627" t="str">
         <v>2026-04-27</v>
@@ -52497,7 +52497,7 @@
         <v>說話人聲</v>
       </c>
       <c r="C1686" t="str">
-        <v>EP.52｜【說話人聲-會客室】用達人力量翻轉職涯迷惘（上）超越達人計畫點亮國中生的未來</v>
+        <v>EP.52｜【說話人聲-會���室】用達人力量翻轉職涯迷惘（上）超越達人計畫點亮國中生的未來</v>
       </c>
       <c r="D1686" t="str">
         <v>2026-03-15</v>
@@ -54419,7 +54419,7 @@
         <v>人生啊！小歐</v>
       </c>
       <c r="C60" t="str">
-        <v>人生啊｜用我的人生故事，陪你看懂自己</v>
+        <v>無</v>
       </c>
       <c r="D60">
         <v>0</v>
@@ -54445,7 +54445,7 @@
         <v>下半場陪談師＿張嘉茹老師</v>
       </c>
       <c r="C61" t="str">
-        <v>下半場陪談師</v>
+        <v>無</v>
       </c>
       <c r="D61">
         <v>0</v>
@@ -54471,7 +54471,7 @@
         <v>布萊恩老師</v>
       </c>
       <c r="C62" t="str">
-        <v>布萊恩老師</v>
+        <v>無</v>
       </c>
       <c r="D62">
         <v>0</v>
@@ -54497,7 +54497,7 @@
         <v>幼兒情緒教育學院-萬叔的心café</v>
       </c>
       <c r="C63" t="str">
-        <v>幼兒情緒教育學院-萬叔的心café</v>
+        <v>無</v>
       </c>
       <c r="D63">
         <v>0</v>
@@ -54523,7 +54523,7 @@
         <v>全遠距工作的行銷人|Coco</v>
       </c>
       <c r="C64" t="str">
-        <v>全遠距工作的行銷人|Coco</v>
+        <v>無</v>
       </c>
       <c r="D64">
         <v>0</v>
@@ -54575,7 +54575,7 @@
         <v>阿駿日常</v>
       </c>
       <c r="C66" t="str">
-        <v>阿駿日常</v>
+        <v>無</v>
       </c>
       <c r="D66">
         <v>0</v>
@@ -54627,7 +54627,7 @@
         <v>高言值表達力教練｜竺宥璋｜小竺</v>
       </c>
       <c r="C68" t="str">
-        <v>高言值表達力教練｜竺宥璋｜小竺</v>
+        <v>無</v>
       </c>
       <c r="D68">
         <v>0</v>
@@ -54653,7 +54653,7 @@
         <v>張書書</v>
       </c>
       <c r="C69" t="str">
-        <v>張書書</v>
+        <v>無</v>
       </c>
       <c r="D69">
         <v>0</v>
@@ -54679,7 +54679,7 @@
         <v>斜槓空姐cindy</v>
       </c>
       <c r="C70" t="str">
-        <v>斜槓空姐cindy</v>
+        <v>無</v>
       </c>
       <c r="D70">
         <v>0</v>
@@ -54705,7 +54705,7 @@
         <v>曼蒂歐逆-轉型之路</v>
       </c>
       <c r="C71" t="str">
-        <v>曼蒂歐逆-轉型之路</v>
+        <v>無</v>
       </c>
       <c r="D71">
         <v>0</v>
@@ -54757,7 +54757,7 @@
         <v>雷浩斯價值投資網</v>
       </c>
       <c r="C73" t="str">
-        <v>雷浩斯價值投資網</v>
+        <v>無</v>
       </c>
       <c r="D73">
         <v>0</v>
@@ -54783,7 +54783,7 @@
         <v>瑪那熊諮商心理師</v>
       </c>
       <c r="C74" t="str">
-        <v>瑪那熊諮商心理師</v>
+        <v>無</v>
       </c>
       <c r="D74">
         <v>0</v>
@@ -54835,7 +54835,7 @@
         <v>劉亦酉</v>
       </c>
       <c r="C76" t="str">
-        <v>劉亦酉</v>
+        <v>無</v>
       </c>
       <c r="D76">
         <v>0</v>
@@ -54913,7 +54913,7 @@
         <v>Coco｜全遠距工作的行銷人</v>
       </c>
       <c r="C79" t="str">
-        <v>Coco｜全遠距工作的行銷人</v>
+        <v>無</v>
       </c>
       <c r="D79">
         <v>0</v>

</xml_diff>

<commit_message>
feat: implement Apple Podcast chart presence leaderboard and Line Chart trend
</commit_message>
<xml_diff>
--- a/eligible_episodes_pool.xlsx
+++ b/eligible_episodes_pool.xlsx
@@ -7,6 +7,7 @@
     <sheet name="KOL 節目名單" sheetId="2" r:id="rId2"/>
     <sheet name="合格單集池" sheetId="3" r:id="rId3"/>
     <sheet name="發片量統計與資格判定" sheetId="4" r:id="rId4"/>
+    <sheet name="Apple榜單歷史排行" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -9229,7 +9230,7 @@
         <v>五吉郎</v>
       </c>
       <c r="C194" t="str">
-        <v>EP146｜寫給每一個在深夜裡獨自內耗的你：我們該如何溫柔地接納自己的失去？（Feat. 作家 林思齊）</v>
+        <v>EP146｜寫給每一個在深夜裡獨自內耗的你：我們該如何溫柔地接納自己的失���？（Feat. 作家 林思齊）</v>
       </c>
       <c r="D194" t="str">
         <v>2026-04-01</v>
@@ -15145,7 +15146,7 @@
         <v>文森說書</v>
       </c>
       <c r="C398" t="str">
-        <v>這些人都有工作，但為什麼只能住在���頭？｜《老窮奇幻紀事》</v>
+        <v>這些人都有工作，但為什麼只能住在街頭？｜《老窮奇幻紀事》</v>
       </c>
       <c r="D398" t="str">
         <v>2026-04-17</v>
@@ -30718,7 +30719,7 @@
         <v>科技領航家</v>
       </c>
       <c r="C935" t="str">
-        <v>EP333 AI ��進醫療現場：智慧醫療的關鍵轉捩點到了嗎？  Ft. 華碩智慧健康產品企劃課經理 賴政宇</v>
+        <v>EP333 AI 走進醫療現場：智慧醫療的關鍵轉捩點到了嗎？  Ft. 華碩智慧健康產品企劃課經理 賴政宇</v>
       </c>
       <c r="D935" t="str">
         <v>2026-01-20</v>
@@ -31182,7 +31183,7 @@
         <v>航海王的富人學</v>
       </c>
       <c r="C951" t="str">
-        <v>富人學🔆第一百一十堂｜『終極資產』</v>
+        <v>富人學🔆第一百���十堂｜『終極資產』</v>
       </c>
       <c r="D951" t="str">
         <v>2026-03-10</v>
@@ -34024,7 +34025,7 @@
         <v>不敗教主陳重銘</v>
       </c>
       <c r="C1049" t="str">
-        <v>EP599比特幣跌到腰斬，現在能進場投資嗎？</v>
+        <v>EP599比特幣跌到腰斬，現���能進場投資嗎？</v>
       </c>
       <c r="D1049" t="str">
         <v>2026-02-25</v>
@@ -42898,7 +42899,7 @@
         <v>郝聲音</v>
       </c>
       <c r="C1355" t="str">
-        <v>郝聲音出外景：（下）哲維說書，訪問郝哥新書「郝會讀書」教你將成長、財富、邏輯與教養的經典智慧，轉化成人生可用的觀點</v>
+        <v>郝聲音出外景：（下）哲維說書，訪問郝哥新書「郝會讀書」教你將成長、財���、邏輯與教養的經典智慧，轉化成人生可用的觀點</v>
       </c>
       <c r="D1355" t="str">
         <v>2026-06-10</v>
@@ -44348,7 +44349,7 @@
         <v>郝聲音</v>
       </c>
       <c r="C1405" t="str">
-        <v>郝聲���：（上）「你在學飛，我在學放手」：從誤會到理解，從疏遠到靠近，46封修復關係的親子書信好書分享 ～ 吳緁苓, 林昀靜, 林廷旭</v>
+        <v>郝聲音：（上）「你在學飛，我在學放手」：從誤會到理解，從疏遠到靠近，46封修復關係的親子書信好書分享 ～ 吳緁苓, 林昀靜, 林廷旭</v>
       </c>
       <c r="D1405" t="str">
         <v>2026-04-23</v>
@@ -44899,7 +44900,7 @@
         <v>郝聲音</v>
       </c>
       <c r="C1424" t="str">
-        <v>郝聲音：（上）阿金的「火星計劃」：如果你「相信」你可以，最後不僅你可以，你也會��著一群人一起可以</v>
+        <v>郝聲音：（上）阿金的「火星計劃」：如果你「相信」你可以，最後不僅你可以，你也會帶著一群人一起可以</v>
       </c>
       <c r="D1424" t="str">
         <v>2026-04-04</v>
@@ -45682,7 +45683,7 @@
         <v>郝聲音</v>
       </c>
       <c r="C1451" t="str">
-        <v>郝聲音：（上）王奕淳醫師好書分享「減糖護腎211TOP蔬食健康餐盤」跟著醫生這樣吃，遠離糖尿病、腎臟病危機</v>
+        <v>郝聲音：（上）王奕淳醫��好書分享「減糖護腎211TOP蔬食健康餐盤」跟著醫生這樣吃，遠離糖尿病、腎臟病危機</v>
       </c>
       <c r="D1451" t="str">
         <v>2026-03-13</v>
@@ -45827,7 +45828,7 @@
         <v>郝聲音</v>
       </c>
       <c r="C1456" t="str">
-        <v>郝聲音：（下）沃醫學執行長Jessie，從「熱情」到「信任」的創業破框之路</v>
+        <v>郝聲音：���下）沃醫學執行長Jessie，從「熱情」到「信任」的創業破框之路</v>
       </c>
       <c r="D1456" t="str">
         <v>2026-03-08</v>
@@ -47306,7 +47307,7 @@
         <v>郝聲音</v>
       </c>
       <c r="C1507" t="str">
-        <v>郝聲音：（上）蔡思怡老師：『神展開的國文教室』最有梗的女神國學閱讀筆記，從經典名篇到當代視角，全面��開人生思辨腦</v>
+        <v>郝聲音：（上）蔡思怡老師：『神展開的國文教室』最有梗的女神國學閱讀筆記，從經典名篇到當代視角，全面打開人生思辨腦</v>
       </c>
       <c r="D1507" t="str">
         <v>2026-01-16</v>
@@ -48698,7 +48699,7 @@
         <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="C1555" t="str">
-        <v>EP219：【非典家庭CEO】育兒現場走音怎麼辦？從動物音樂會的細節看管理，教養不是起跑點的競爭，是「基本功」的複利投資ft. 薩克斯風音樂家爸爸 沈子傑</v>
+        <v>EP219：【��典家庭CEO】育兒現場走音怎麼辦？從動物音樂會的細節看管理，教養不是起跑點的競爭，是「基本功」的複利投資ft. 薩克斯風音樂家爸爸 沈子傑</v>
       </c>
       <c r="D1555" t="str">
         <v>2026-03-25</v>
@@ -50786,7 +50787,7 @@
         <v>子玲的親子聊心屋-媽咪的自我成長&amp;親子教養</v>
       </c>
       <c r="C1627" t="str">
-        <v>#103 ▍孩子講話總是很跳躍 ,如何培養說話邏輯 ? &lt;兒童自信���達專家-依柔老師&gt;</v>
+        <v>#103 ▍孩子講話總是很跳躍 ,如何培養說話邏輯 ? &lt;兒童自信表達專家-依柔老師&gt;</v>
       </c>
       <c r="D1627" t="str">
         <v>2026-04-27</v>
@@ -52497,7 +52498,7 @@
         <v>說話人聲</v>
       </c>
       <c r="C1686" t="str">
-        <v>EP.52｜【說話人聲-會���室】用達人力量翻轉職涯迷惘（上）超越達人計畫點亮國中生的未來</v>
+        <v>EP.52｜【說話人聲-會客室】用達人力量翻轉職涯迷惘（上）超越達人計畫點亮國中生的未來</v>
       </c>
       <c r="D1686" t="str">
         <v>2026-03-15</v>
@@ -54962,4 +54963,239 @@
     <ignoredError numberStoredAsText="1" sqref="A1:H80"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>名次</v>
+      </c>
+      <c r="B1" t="str">
+        <v>合作夥伴</v>
+      </c>
+      <c r="C1" t="str">
+        <v>節目名稱</v>
+      </c>
+      <c r="D1" t="str">
+        <v>在榜天數</v>
+      </c>
+      <c r="E1" t="str">
+        <v>在榜率</v>
+      </c>
+      <c r="F1" t="str">
+        <v>平均排名</v>
+      </c>
+      <c r="G1" t="str">
+        <v>最佳排名</v>
+      </c>
+      <c r="H1" t="str">
+        <v>歷史名次軌跡</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Apple Podcast 連結</v>
+      </c>
+      <c r="J1" t="str">
+        <v>RSS 連結</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>瓦基閱讀前哨站</v>
+      </c>
+      <c r="C2" t="str">
+        <v>下一本讀什麼？</v>
+      </c>
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="F2" t="str">
+        <v>#26.8</v>
+      </c>
+      <c r="G2" t="str">
+        <v>#23</v>
+      </c>
+      <c r="H2" t="str">
+        <v>06-14(#31), 06-15(#26), 06-16(#27), 06-17(#23)</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://podcasts.apple.com/tw/podcast/%E4%B8%8B%E4%B8%80%E6%9C%AC%E8%AE%80%E4%BB%80%E9%BA%BC/id1532820533?uo=4</v>
+      </c>
+      <c r="J2" t="str">
+        <v>https://feed.firstory.me/rss/user/cl39lz2ky01co01ugaba7gr9y</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>哇賽心理學_蔡宇哲</v>
+      </c>
+      <c r="C3" t="str">
+        <v>哇賽心理學</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+      <c r="E3" t="str">
+        <v>100%</v>
+      </c>
+      <c r="F3" t="str">
+        <v>#28</v>
+      </c>
+      <c r="G3" t="str">
+        <v>#24</v>
+      </c>
+      <c r="H3" t="str">
+        <v>06-14(#30), 06-15(#24), 06-16(#26), 06-17(#32)</v>
+      </c>
+      <c r="I3" t="str">
+        <v>https://podcasts.apple.com/tw/podcast/%E5%93%87%E8%B3%BD%E5%BF%83%E7%90%86%E5%AD%B8/id1500162537</v>
+      </c>
+      <c r="J3" t="str">
+        <v>https://feed.firstory.me/rss/user/ck7t2fz77qu7g0873ln5hz5cl</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="C4" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="D4">
+        <v>4</v>
+      </c>
+      <c r="E4" t="str">
+        <v>100%</v>
+      </c>
+      <c r="F4" t="str">
+        <v>#47.5</v>
+      </c>
+      <c r="G4" t="str">
+        <v>#41</v>
+      </c>
+      <c r="H4" t="str">
+        <v>06-14(#47), 06-15(#46), 06-16(#41), 06-17(#56)</v>
+      </c>
+      <c r="I4" t="str">
+        <v>https://podcasts.apple.com/tw/podcast/%E9%83%9D%E8%81%B2%E9%9F%B3/id1533782597</v>
+      </c>
+      <c r="J4" t="str">
+        <v>https://feed.firstory.me/rss/user/ckfnpunqe136d08003p6lzdmn</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>GK爸爸</v>
+      </c>
+      <c r="C5" t="str">
+        <v>GK爸爸原創故事繪本</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5" t="str">
+        <v>100%</v>
+      </c>
+      <c r="F5" t="str">
+        <v>#48.5</v>
+      </c>
+      <c r="G5" t="str">
+        <v>#37</v>
+      </c>
+      <c r="H5" t="str">
+        <v>06-14(#43), 06-15(#37), 06-16(#57), 06-17(#57)</v>
+      </c>
+      <c r="I5" t="str">
+        <v>https://podcasts.apple.com/tw/podcast/gk%E7%88%B8%E7%88%B8%E5%8E%9F%E5%89%B5%E6%95%85%E4%BA%8B%E7%B9%AA%E6%9C%AC/id1525978220?uo=4</v>
+      </c>
+      <c r="J5" t="str">
+        <v>https://feed.firstory.me/rss/user/cke9o73prwmij0839gmffmzhj</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>別人的工作最有趣｜Fiona</v>
+      </c>
+      <c r="C6" t="str">
+        <v>別人的工作最有趣</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6" t="str">
+        <v>50%</v>
+      </c>
+      <c r="F6" t="str">
+        <v>#88.5</v>
+      </c>
+      <c r="G6" t="str">
+        <v>#79</v>
+      </c>
+      <c r="H6" t="str">
+        <v>06-14(#79), 06-15(#98)</v>
+      </c>
+      <c r="I6" t="str">
+        <v>https://podcasts.apple.com/tw/podcast/%E5%88%A5%E4%BA%BA%E7%9A%84%E5%B7%A5%E4%BD%9C%E6%9C%80%E6%9C%89%E8%B6%A3/id1626274583</v>
+      </c>
+      <c r="J6" t="str">
+        <v>https://feeds.soundon.fm/podcasts/d9d66aa1-b352-43f8-8324-064d3248538e.xml</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>文森說書</v>
+      </c>
+      <c r="C7" t="str">
+        <v>文森說書</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="str">
+        <v>50%</v>
+      </c>
+      <c r="F7" t="str">
+        <v>#92</v>
+      </c>
+      <c r="G7" t="str">
+        <v>#91</v>
+      </c>
+      <c r="H7" t="str">
+        <v>06-14(#91), 06-15(#93)</v>
+      </c>
+      <c r="I7" t="str">
+        <v>https://podcasts.apple.com/tw/podcast/%E6%96%87%E6%A3%AE%E8%AA%AA%E6%9B%B8/id1513786617?uo=4</v>
+      </c>
+      <c r="J7" t="str">
+        <v>https://rss.buzzsprout.com/1096139.rss</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete POC 9-episode evaluation, update Excel sheet, and compile dashboard
</commit_message>
<xml_diff>
--- a/eligible_episodes_pool.xlsx
+++ b/eligible_episodes_pool.xlsx
@@ -8,6 +8,7 @@
     <sheet name="合格單集池" sheetId="3" r:id="rId3"/>
     <sheet name="發片量統計與資格判定" sheetId="4" r:id="rId4"/>
     <sheet name="Apple榜單歷史排行" sheetId="5" r:id="rId5"/>
+    <sheet name="POC評分結果" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -57600,4 +57601,443 @@
     <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AI4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>合作夥伴</v>
+      </c>
+      <c r="B1" t="str">
+        <v>節目名稱</v>
+      </c>
+      <c r="C1" t="str">
+        <v>抽樣單集 1</v>
+      </c>
+      <c r="D1" t="str">
+        <v>抽樣單集 2</v>
+      </c>
+      <c r="E1" t="str">
+        <v>抽樣單集 3</v>
+      </c>
+      <c r="F1" t="str">
+        <v>最佳內容架構獎_得分</v>
+      </c>
+      <c r="G1" t="str">
+        <v>最佳內容架構獎_評語</v>
+      </c>
+      <c r="H1" t="str">
+        <v>最佳內容架構獎_是否合規</v>
+      </c>
+      <c r="I1" t="str">
+        <v>最佳默契獎_得分</v>
+      </c>
+      <c r="J1" t="str">
+        <v>最佳默契獎_評語</v>
+      </c>
+      <c r="K1" t="str">
+        <v>最佳默契獎_是否合規</v>
+      </c>
+      <c r="L1" t="str">
+        <v>最神單元企劃獎_得分</v>
+      </c>
+      <c r="M1" t="str">
+        <v>最神單元企劃獎_評語</v>
+      </c>
+      <c r="N1" t="str">
+        <v>最神單元企劃獎_是否合規</v>
+      </c>
+      <c r="O1" t="str">
+        <v>最佳男播音員獎_得分</v>
+      </c>
+      <c r="P1" t="str">
+        <v>最佳男播音員獎_評語</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>最佳男播音員獎_是否合規</v>
+      </c>
+      <c r="R1" t="str">
+        <v>最佳女播音員獎_得分</v>
+      </c>
+      <c r="S1" t="str">
+        <v>最佳女播音員獎_評語</v>
+      </c>
+      <c r="T1" t="str">
+        <v>最佳女播音員獎_是否合規</v>
+      </c>
+      <c r="U1" t="str">
+        <v>聽完馬上獎（極致推坑王）_得分</v>
+      </c>
+      <c r="V1" t="str">
+        <v>聽完馬上獎（極致推坑王）_評語</v>
+      </c>
+      <c r="W1" t="str">
+        <v>聽完馬上獎（極致推坑王）_是否合規</v>
+      </c>
+      <c r="X1" t="str">
+        <v>只有你在獎（稀有藍海守護者）_得分</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>只有你在獎（稀有藍海守護者）_評語</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>只有你在獎（稀有藍海守護者）_是否合規</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>自我探索獎_得分</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>自我探索獎_評語</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>自我探索獎_是否合規</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>講不完大獎 / 泡麵沒熟獎 (時長精煉度)_得分</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>講不完大獎 / 泡麵沒熟獎 (時長精煉度)_評語</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>講不完大獎 / 泡麵沒熟獎 (時長精煉度)_是否合規</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>醒醒再獎 / 年度療癒獎 / 深夜輕輕獎 (意向)_得分</v>
+      </c>
+      <c r="AH1" t="str">
+        <v>醒醒再獎 / 年度療癒獎 / 深夜輕輕獎 (意向)_評語</v>
+      </c>
+      <c r="AI1" t="str">
+        <v>醒醒再獎 / 年度療癒獎 / 深夜輕輕獎 (意向)_是否合規</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="B2" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="C2" t="str">
+        <v>郝聲音：（上）設計師KiKi，從繪畫到設計的熱愛之路，到引領他人感受設計之美的「走讀」行旅～</v>
+      </c>
+      <c r="D2" t="str">
+        <v>郝聲音：（下）終於跟MJ林明樟老師合體！用「財務腦」打通「業務力」，讓商業與人生獲利生生不息！</v>
+      </c>
+      <c r="E2" t="str">
+        <v>郝聲音：（下） 蘇絢慧老師好書分享，『隱性內耗』：看不見的傷，如何消磨你的能量？</v>
+      </c>
+      <c r="F2">
+        <v>7.5</v>
+      </c>
+      <c r="G2" t="str">
+        <v>開場能點出主題，但段落間的邏輯轉折較為口語化，有時顯得散漫，結尾總結點到為止，深度不足。</v>
+      </c>
+      <c r="H2" t="str">
+        <v>符合</v>
+      </c>
+      <c r="I2">
+        <v>8.5</v>
+      </c>
+      <c r="J2" t="str">
+        <v>主持人與來賓（設計師、MJ老師）互動良好，接話與延伸觀點流暢，偶有幽默吐槽，整體對談氛圍佳。</v>
+      </c>
+      <c r="K2" t="str">
+        <v>符合</v>
+      </c>
+      <c r="L2">
+        <v>8</v>
+      </c>
+      <c r="M2" t="str">
+        <v>企劃（設計師生涯、財務腦力）選題具備一定興趣點，但內容深度與實操工具的提供較為有限，訪談問題較為基礎。</v>
+      </c>
+      <c r="N2" t="str">
+        <v>符合</v>
+      </c>
+      <c r="O2">
+        <v>8.5</v>
+      </c>
+      <c r="P2" t="str">
+        <v>口條尚可，偶有贅字，語速穩定，音量平穩，但情感渲染力與共鳴感較為平淡。</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>符合</v>
+      </c>
+      <c r="R2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="S2" t="str">
+        <v>節目無女主持人</v>
+      </c>
+      <c r="T2" t="str">
+        <v>不適用</v>
+      </c>
+      <c r="U2">
+        <v>6.5</v>
+      </c>
+      <c r="V2" t="str">
+        <v>單集結尾僅有預告下一集內容，缺少明確的行動呼籲（訂閱、社群互動、購買等），推坑力不足。</v>
+      </c>
+      <c r="W2" t="str">
+        <v>不符合(原因：單集結尾均缺少呼籲訂閱與��群互動行動)</v>
+      </c>
+      <c r="X2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Z2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="AA2">
+        <v>8</v>
+      </c>
+      <c r="AB2" t="str">
+        <v>節目內容觸及「設計生涯」、「財務腦力」、「人生選擇」等，能啟發聽眾思考個人成長與職涯發展，但深度與心靈啟發力較前兩者稍弱。</v>
+      </c>
+      <c r="AC2" t="str">
+        <v>符合</v>
+      </c>
+      <c r="AD2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="AE2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="AF2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="AG2">
+        <v>8.5</v>
+      </c>
+      <c r="AH2" t="str">
+        <v>節目氛圍輕鬆、幽默，主持人與來賓對談自然，偶有笑聲，聽感具備一定的陪伴與放鬆感，偏向「年度療癒獎」的意向。</v>
+      </c>
+      <c r="AI2" t="str">
+        <v>符合</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="B3" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="C3" t="str">
+        <v>GD229｜明明不想去卻說「好」？揭開你不敢拒絕的心理盲點與精神內耗！</v>
+      </c>
+      <c r="D3" t="str">
+        <v>GD221｜別再被情緒牽著鼻子走！開口前停頓 3 秒鐘，瞬間改寫你的人生劇本</v>
+      </c>
+      <c r="E3" t="str">
+        <v>EP169｜蝦皮內捲太絕望？夜校打雜工逆襲：我如何在亞馬遜高門檻戰場穩賺美金！（Feat. AZ-Helper 創辦人 Jonathan 里長伯）</v>
+      </c>
+      <c r="F3">
+        <v>8.5</v>
+      </c>
+      <c r="G3" t="str">
+        <v>節目結構清晰，開場迅速點出主題與聽眾痛點（不敢拒絕的心理盲點），段落轉折邏輯分明，結尾有總結與行動呼籲。</v>
+      </c>
+      <c r="H3" t="str">
+        <v>符合</v>
+      </c>
+      <c r="I3">
+        <v>8</v>
+      </c>
+      <c r="J3" t="str">
+        <v>節目為單人主持，故此獎項不適用。</v>
+      </c>
+      <c r="K3" t="str">
+        <v>不適用</v>
+      </c>
+      <c r="L3">
+        <v>9.5</v>
+      </c>
+      <c r="M3" t="str">
+        <v>選題（不敢拒絕的心理���點）具備市場差異化與新穎包裝，內容提供實操方法與清晰的心理學觀點，實用價值高。</v>
+      </c>
+      <c r="N3" t="str">
+        <v>符合</v>
+      </c>
+      <c r="O3">
+        <v>9</v>
+      </c>
+      <c r="P3" t="str">
+        <v>口條流暢，贅字率低，語速適中（約 180-220 字/分），音量平穩，具備親和力與引導能力。</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>符合</v>
+      </c>
+      <c r="R3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="S3" t="str">
+        <v>節目無女主持人</v>
+      </c>
+      <c r="T3" t="str">
+        <v>不適用</v>
+      </c>
+      <c r="U3">
+        <v>9.5</v>
+      </c>
+      <c r="V3" t="str">
+        <v>節目結尾有明確的行動挑戰（練習對自己誠實、心裡默數一二三），呼籲加入社群，具備極強的推坑力與實踐引導。</v>
+      </c>
+      <c r="W3" t="str">
+        <v>符合</v>
+      </c>
+      <c r="X3">
+        <v>7.5</v>
+      </c>
+      <c r="Y3" t="str">
+        <v>節目主題聚焦於「不敢拒絕」、「情緒管理」、「跨境電商」等，雖有市場區隔，但非極度冷門的藍海議題。</v>
+      </c>
+      <c r="Z3" t="str">
+        <v>符合</v>
+      </c>
+      <c r="AA3">
+        <v>9.5</v>
+      </c>
+      <c r="AB3" t="str">
+        <v>節目深入探討「不敢拒絕」、「情緒管理」、「自我價值」等議題，引導聽眾反思內在狀態，鼓勵獨立思考與拿回主導權。</v>
+      </c>
+      <c r="AC3" t="str">
+        <v>符合</v>
+      </c>
+      <c r="AD3">
+        <v>4</v>
+      </c>
+      <c r="AE3" t="str">
+        <v>單集時長約 7-10 分鐘，未達「講不完大獎」的 60 分鐘門檻，但接近「泡麵沒熟獎」的 10-15 分鐘門檻，時長精煉度僅部分符合。</v>
+      </c>
+      <c r="AF3" t="str">
+        <v>不符合(原因：時長未達 60 分鐘門檻，僅接近 10-15 分鐘門檻)</v>
+      </c>
+      <c r="AG3">
+        <v>9.5</v>
+      </c>
+      <c r="AH3" t="str">
+        <v>節目氛圍積極、正向，主持人語調明快有朝氣，聽感能帶來精神振奮感，符合「醒醒再獎」的意向。</v>
+      </c>
+      <c r="AI3" t="str">
+        <v>符合</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>哇賽心理學_蔡宇哲</v>
+      </c>
+      <c r="B4" t="str">
+        <v>哇賽心理學</v>
+      </c>
+      <c r="C4" t="str">
+        <v>掌握你的金錢性格，打造幸福家庭理財ft.精算媽咪珊迪兔｜哇賽心觀點ep194</v>
+      </c>
+      <c r="D4" t="str">
+        <v>多巴胺陷阱！戒不掉的不是癮，是深層的焦慮ft.蘇琮祺心理師｜哇賽心觀點ep193</v>
+      </c>
+      <c r="E4" t="str">
+        <v>療癒創傷，溫柔擁抱完整的自己ft.留佩萱博士｜哇賽療心室ep148</v>
+      </c>
+      <c r="F4">
+        <v>8</v>
+      </c>
+      <c r="G4" t="str">
+        <v>內容架構尚可，但開場���導較為平淡，結尾總結不夠精闢，部分單集轉折略顯鬆散。</v>
+      </c>
+      <c r="H4" t="str">
+        <v>符合</v>
+      </c>
+      <c r="I4">
+        <v>9.5</v>
+      </c>
+      <c r="J4" t="str">
+        <v>主持人與來賓（心理師）互動流暢自然，接話頻率高且能延伸話題，有共鳴笑聲，展現專業的對談默契。</v>
+      </c>
+      <c r="K4" t="str">
+        <v>符合</v>
+      </c>
+      <c r="L4">
+        <v>9</v>
+      </c>
+      <c r="M4" t="str">
+        <v>企劃（金錢性格、創傷療癒）切入角度具備深度與實用性，能啟發聽眾思考，訪談引導性強。</v>
+      </c>
+      <c r="N4" t="str">
+        <v>符合</v>
+      </c>
+      <c r="O4">
+        <v>8</v>
+      </c>
+      <c r="P4" t="str">
+        <v>口條清晰，贅字率低，語速穩定，音量平穩，但作為主持人，在引導與情感表達上較為內斂。</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>符合</v>
+      </c>
+      <c r="R4">
+        <v>9</v>
+      </c>
+      <c r="S4" t="str">
+        <v>主持人（娜娜）口條清晰，語速適中，音量平穩，具備溫暖的語調與親和力，能有效引導來賓。</v>
+      </c>
+      <c r="T4" t="str">
+        <v>符合</v>
+      </c>
+      <c r="U4">
+        <v>8</v>
+      </c>
+      <c r="V4" t="str">
+        <v>節目中提及新書練習與 app 研發，有引導聽眾自我覺察與行動的意圖，但呼籲訂閱或互動的直接性較弱。</v>
+      </c>
+      <c r="W4" t="str">
+        <v>符合</v>
+      </c>
+      <c r="X4">
+        <v>9.5</v>
+      </c>
+      <c r="Y4" t="str">
+        <v>節目探討「金錢性格」、「創傷療癒」、「多巴胺陷阱」等議題，具備心理學的深度與稀有性，論述完整。</v>
+      </c>
+      <c r="Z4" t="str">
+        <v>符合</v>
+      </c>
+      <c r="AA4">
+        <v>9</v>
+      </c>
+      <c r="AB4" t="str">
+        <v>節目內容觸及「金錢性格」、「創傷療癒」、「內耗」等，引導聽眾自我覺察與理解，具有心靈啟發力。</v>
+      </c>
+      <c r="AC4" t="str">
+        <v>符合</v>
+      </c>
+      <c r="AD4">
+        <v>4</v>
+      </c>
+      <c r="AE4" t="str">
+        <v>單集時長約 30-40 分鐘，未達「講不完大獎」的 60 分鐘門檻，也未達「泡麵沒熟獎」的 10-15 分鐘門檻，時長精煉度不符合兩獎項定義。</v>
+      </c>
+      <c r="AF4" t="str">
+        <v>不符合(原因：時長不符合該時長獎項之門檻)</v>
+      </c>
+      <c r="AG4">
+        <v>7</v>
+      </c>
+      <c r="AH4" t="str">
+        <v>節目氛圍偏向知識性與探��性，主持人語調溫和，但較少展現積極的晨間活力或深夜的療癒陪伴感，意向較不明確。</v>
+      </c>
+      <c r="AI4" t="str">
+        <v>符合</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:AI4"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: restore 10-point scale and enforce correct duo/female host exclusion rules
</commit_message>
<xml_diff>
--- a/eligible_episodes_pool.xlsx
+++ b/eligible_episodes_pool.xlsx
@@ -57739,14 +57739,14 @@
       <c r="H2" t="str">
         <v>符合</v>
       </c>
-      <c r="I2">
-        <v>8.5</v>
+      <c r="I2" t="str">
+        <v>N/A</v>
       </c>
       <c r="J2" t="str">
-        <v>主持人與來賓（設計師、MJ老師）互動良好，接話與延伸觀點流暢，偶有幽默吐槽，整體對談氛圍佳。</v>
+        <v>單人主持節目，不適用此獎項。</v>
       </c>
       <c r="K2" t="str">
-        <v>符合</v>
+        <v>不適用</v>
       </c>
       <c r="L2">
         <v>8</v>
@@ -57770,7 +57770,7 @@
         <v>N/A</v>
       </c>
       <c r="S2" t="str">
-        <v>節目無女主持人</v>
+        <v>節目無女主持人，不適用此獎項。</v>
       </c>
       <c r="T2" t="str">
         <v>不適用</v>
@@ -57846,11 +57846,11 @@
       <c r="H3" t="str">
         <v>符合</v>
       </c>
-      <c r="I3">
-        <v>8</v>
+      <c r="I3" t="str">
+        <v>N/A</v>
       </c>
       <c r="J3" t="str">
-        <v>節目為單人主持，故此獎項不適用。</v>
+        <v>單人主持節目，不適用此獎項。</v>
       </c>
       <c r="K3" t="str">
         <v>不適用</v>
@@ -57877,7 +57877,7 @@
         <v>N/A</v>
       </c>
       <c r="S3" t="str">
-        <v>節目無女主持人</v>
+        <v>節目無女主持人，不適用此獎項。</v>
       </c>
       <c r="T3" t="str">
         <v>不適用</v>

</xml_diff>

<commit_message>
feat: split long-form and short-form awards, update excel, and rebuild dashboard
</commit_message>
<xml_diff>
--- a/eligible_episodes_pool.xlsx
+++ b/eligible_episodes_pool.xlsx
@@ -57605,7 +57605,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI4"/>
+  <dimension ref="A1:AL4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -57696,21 +57696,30 @@
         <v>自我探索獎_是否合規</v>
       </c>
       <c r="AD1" t="str">
-        <v>講不完大獎 / 泡麵沒熟獎 (時長精煉度)_得分</v>
+        <v>講不完大獎_得分</v>
       </c>
       <c r="AE1" t="str">
-        <v>講不完大獎 / 泡麵沒熟獎 (時長精煉度)_評語</v>
+        <v>講不完大獎_評語</v>
       </c>
       <c r="AF1" t="str">
-        <v>講不完大獎 / 泡麵沒熟獎 (時長精煉度)_是否合規</v>
+        <v>講不完大獎_是否合規</v>
       </c>
       <c r="AG1" t="str">
+        <v>泡麵沒熟獎_得分</v>
+      </c>
+      <c r="AH1" t="str">
+        <v>泡麵沒熟獎_評語</v>
+      </c>
+      <c r="AI1" t="str">
+        <v>泡麵沒熟獎_是否合規</v>
+      </c>
+      <c r="AJ1" t="str">
         <v>醒醒再獎 / 年度療癒獎 / 深夜輕輕獎 (意向)_得分</v>
       </c>
-      <c r="AH1" t="str">
+      <c r="AK1" t="str">
         <v>醒醒再獎 / 年度療癒獎 / 深夜輕輕獎 (意向)_評語</v>
       </c>
-      <c r="AI1" t="str">
+      <c r="AL1" t="str">
         <v>醒醒再獎 / 年度療癒獎 / 深夜輕輕獎 (意向)_是否合規</v>
       </c>
     </row>
@@ -57734,7 +57743,7 @@
         <v>7.5</v>
       </c>
       <c r="G2" t="str">
-        <v>開場能點出主題，但段落間的邏輯轉折較為口語化，有時顯得散漫，結尾總結點到為止，深度不足。</v>
+        <v>單集 1 開頭有明確的節目介紹與本集主題預告，但內容較為鬆散，聊天性質較重，段落轉折不夠清晰。單集 2 與 3 亦有類似情況，結尾總結力道較弱。</v>
       </c>
       <c r="H2" t="str">
         <v>符合</v>
@@ -57749,10 +57758,10 @@
         <v>不適用</v>
       </c>
       <c r="L2">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="M2" t="str">
-        <v>企劃（設計師生涯、財務腦力）選題具備一定興趣點，但內容深度與實操工具的提供較為有限，訪談問題較為基礎。</v>
+        <v>企劃主題（設計師生涯、財務腦與業務力、隱性內耗）具備一定的深度，但選題切入角度較為傳統，實用價值與��度有提升空間，訪談深度較為表面。</v>
       </c>
       <c r="N2" t="str">
         <v>符合</v>
@@ -57761,7 +57770,7 @@
         <v>8.5</v>
       </c>
       <c r="P2" t="str">
-        <v>口條尚可，偶有贅字，語速穩定，音量平穩，但情感渲染力與共鳴感較為平淡。</v>
+        <v>主持人郝哥口條尚稱流暢，但偶有贅字（如「那個」、「就是」），語速穩定，音量平穩，具備一定的親和力與情感表達。</v>
       </c>
       <c r="Q2" t="str">
         <v>符合</v>
@@ -57779,45 +57788,54 @@
         <v>6.5</v>
       </c>
       <c r="V2" t="str">
-        <v>單集結尾僅有預告下一集內容，缺少明確的行動呼籲（訂閱、社群互動、購買等），推坑力不足。</v>
+        <v>單集結尾均缺少明確的行動呼籲（如訂閱、追蹤、社群互動），僅有節目結束的道別，推坑力道較弱。</v>
       </c>
       <c r="W2" t="str">
-        <v>不符合(原因：單集結尾均缺少呼籲訂閱與��群互動行動)</v>
-      </c>
-      <c r="X2" t="str">
-        <v>N/A</v>
+        <v>不符合(原因：單集結尾均缺少呼籲訂閱與社群互動行動)</v>
+      </c>
+      <c r="X2">
+        <v>7</v>
       </c>
       <c r="Y2" t="str">
-        <v>N/A</v>
+        <v>企劃主題如設計師生涯、業務力、內耗等，雖有其市場，但切入角度與探討深度相對較為常見，較難稱得上是稀有藍海議題。</v>
       </c>
       <c r="Z2" t="str">
-        <v>N/A</v>
+        <v>符合</v>
       </c>
       <c r="AA2">
         <v>8</v>
       </c>
       <c r="AB2" t="str">
-        <v>節目內容觸及「設計生涯」、「財務腦力」、「人生選擇」等，能啟發聽眾思考個人成長與職涯發展，但深度與心靈啟發力較前兩者稍弱。</v>
+        <v>節目內容涉及設計生涯、業務力、內耗等主題，能引導聽眾思考個人成長與職涯發展，但深度與心靈啟發力相較於其他兩者略顯不足。</v>
       </c>
       <c r="AC2" t="str">
         <v>符合</v>
       </c>
-      <c r="AD2" t="str">
-        <v>N/A</v>
+      <c r="AD2">
+        <v>9</v>
       </c>
       <c r="AE2" t="str">
-        <v>N/A</v>
+        <v>單集 1 與單集 2 時長均超過 60 分鐘，內容豐富，聊天流暢，雖有部分閒聊，但整體資訊密度尚可，能維持聽眾的興趣。</v>
       </c>
       <c r="AF2" t="str">
-        <v>N/A</v>
+        <v>符合</v>
       </c>
       <c r="AG2">
+        <v>5</v>
+      </c>
+      <c r="AH2" t="str">
+        <v>單集時長約 20-25 分鐘，超過 15 分鐘的限制，不符合短篇定義，內容亦有聊天性質，傳播效率有待提升。</v>
+      </c>
+      <c r="AI2" t="str">
+        <v>不符合(原因：時長大於15分鐘)</v>
+      </c>
+      <c r="AJ2">
         <v>8.5</v>
       </c>
-      <c r="AH2" t="str">
-        <v>節目氛圍輕鬆、幽默，主持人與來賓對談自然，偶有笑聲，聽感具備一定的陪伴與放鬆感，偏向「年度療癒獎」的意向。</v>
-      </c>
-      <c r="AI2" t="str">
+      <c r="AK2" t="str">
+        <v>主持人郝哥的語調溫暖，談話風格輕鬆，偶爾穿插幽默，能營造出一定的陪伴感與親和力，適合在需要放鬆時收聽。</v>
+      </c>
+      <c r="AL2" t="str">
         <v>符合</v>
       </c>
     </row>
@@ -57841,7 +57859,7 @@
         <v>8.5</v>
       </c>
       <c r="G3" t="str">
-        <v>節目結構清晰，開場迅速點出主題與聽眾痛點（不敢拒絕的心理盲點），段落轉折邏輯分明，結尾有總結與行動呼籲。</v>
+        <v>節目 GD229 開頭明確點出主題，並以三個重點架構內容；GD221 亦有清晰的開場與重點劃分；EP169 則有明確的來賓介紹與主題鋪陳。整體邏輯清晰，轉折自然。</v>
       </c>
       <c r="H3" t="str">
         <v>符合</v>
@@ -57859,7 +57877,7 @@
         <v>9.5</v>
       </c>
       <c r="M3" t="str">
-        <v>選題（不敢拒絕的心理���點）具備市場差異化與新穎包裝，內容提供實操方法與清晰的心理學觀點，實用價值高。</v>
+        <v>企劃主題（不敢拒絕、情緒反應、跨境電商）切入點新穎且具備高度的市場差異化，內容深入淺出，提供實用方法與案例，訪談深度佳。</v>
       </c>
       <c r="N3" t="str">
         <v>符合</v>
@@ -57868,7 +57886,7 @@
         <v>9</v>
       </c>
       <c r="P3" t="str">
-        <v>口條流暢，贅字率低，語速適中（約 180-220 字/分），音量平穩，具備親和力與引導能力。</v>
+        <v>主持人安迪口條流暢，贅字率低，語速穩定，音量平穩，具備良好的共鳴與情感渲染力，能有效引導聽眾進入主題。</v>
       </c>
       <c r="Q3" t="str">
         <v>符合</v>
@@ -57886,7 +57904,7 @@
         <v>9.5</v>
       </c>
       <c r="V3" t="str">
-        <v>節目結尾有明確的行動挑戰（練習對自己誠實、心裡默數一二三），呼籲加入社群，具備極強的推坑力與實踐引導。</v>
+        <v>節目 GD229 結尾有明確的行動挑戰（練習對自己誠實），並鼓勵聽眾加入社群；GD221 亦有行動挑戰（記錄情緒反應問題），並鼓勵聽眾加入社群。推坑力道強且具體。</v>
       </c>
       <c r="W3" t="str">
         <v>符合</v>
@@ -57895,7 +57913,7 @@
         <v>7.5</v>
       </c>
       <c r="Y3" t="str">
-        <v>節目主題聚焦於「不敢拒絕」、「情緒管理」、「跨境電商」等，雖有市場區隔，但非極度冷門的藍海議題。</v>
+        <v>企劃主題如「不敢拒絕的心理盲點」、「情緒反應與回應」等，雖非市場獨有，但切入點與探討深度具備一定的差異化，屬於較為細緻的心理議題。</v>
       </c>
       <c r="Z3" t="str">
         <v>符合</v>
@@ -57904,7 +57922,7 @@
         <v>9.5</v>
       </c>
       <c r="AB3" t="str">
-        <v>節目深入探討「不敢拒絕」、「情緒管理」、「自我價值」等議題，引導聽眾反思內在狀態，鼓勵獨立思考與拿回主導權。</v>
+        <v>節目內容深入探討不敢拒絕、情緒管理、跨境電商的選擇與執行，引導聽眾反思自我價值、人際界線與職涯發展，心靈啟發力強。</v>
       </c>
       <c r="AC3" t="str">
         <v>符合</v>
@@ -57913,18 +57931,27 @@
         <v>4</v>
       </c>
       <c r="AE3" t="str">
-        <v>單集時長約 7-10 分鐘，未達「講不完大獎」的 60 分鐘門檻，但接近「泡麵沒熟獎」的 10-15 分鐘門檻，時長精煉度僅部分符合。</v>
+        <v>抽樣單集時長均未達 60 分鐘（約 7 分鐘），不符合獎項定義。</v>
       </c>
       <c r="AF3" t="str">
-        <v>不符合(原因：時長未達 60 分鐘門檻，僅接近 10-15 分鐘門檻)</v>
+        <v>不符合(原因：時長小於60分鐘)</v>
       </c>
       <c r="AG3">
+        <v>9</v>
+      </c>
+      <c r="AH3" t="str">
+        <v>節目 GD229 與 GD221 時長約 7 分鐘，符合 10-15 分鐘的黃金短篇定義，內容精煉，切入重點迅速，傳播效率高。</v>
+      </c>
+      <c r="AI3" t="str">
+        <v>符合</v>
+      </c>
+      <c r="AJ3">
         <v>9.5</v>
       </c>
-      <c r="AH3" t="str">
-        <v>節目氛圍積極、正向，主持人語調明快有朝氣，聽感能帶來精神振奮感，符合「醒醒再獎」的意向。</v>
-      </c>
-      <c r="AI3" t="str">
+      <c r="AK3" t="str">
+        <v>節目 GD229 與 GD221 的主持人安迪，語調溫和、語速適中，談話內容具啟發性與引導性，能讓聽眾感到被��解與支持，營造出療癒、陪伴的氛圍。</v>
+      </c>
+      <c r="AL3" t="str">
         <v>符合</v>
       </c>
     </row>
@@ -57948,7 +57975,7 @@
         <v>8</v>
       </c>
       <c r="G4" t="str">
-        <v>內容架構尚可，但開場���導較為平淡，結尾總結不夠精闢，部分單集轉折略顯鬆散。</v>
+        <v>節目內容架構清晰，多以主題探討為主，開頭能引導聽眾進入情境。但部分單集結尾較為平淡，未有明確的總結或重點整理。</v>
       </c>
       <c r="H4" t="str">
         <v>符合</v>
@@ -57957,7 +57984,7 @@
         <v>9.5</v>
       </c>
       <c r="J4" t="str">
-        <v>主持人與來賓（心理師）互動流暢自然，接話頻率高且能延伸話題，有共鳴笑聲，展現專業的對談默契。</v>
+        <v>主持人宇澤與來賓（心理師、博士）互動流暢自然，提問精準且能引導來賓深入分享，展現高度的專業默契與對談節奏感。</v>
       </c>
       <c r="K4" t="str">
         <v>符合</v>
@@ -57966,7 +57993,7 @@
         <v>9</v>
       </c>
       <c r="M4" t="str">
-        <v>企劃（金錢性格、創傷療癒）切入角度具備深度與實用性，能啟發聽眾思考，訪談引導性強。</v>
+        <v>企劃主題（金錢性格、多巴胺陷阱、創傷療癒）具備深度與實用性，能引發聽眾共鳴與思考，訪談問題具引導性，能激發來賓分享獨特觀點。</v>
       </c>
       <c r="N4" t="str">
         <v>符合</v>
@@ -57975,7 +58002,7 @@
         <v>8</v>
       </c>
       <c r="P4" t="str">
-        <v>口條清晰，贅字率低，語速穩定，音量平穩，但作為主持人，在引導與情感表達上較為內斂。</v>
+        <v>主持人宇澤口條流暢，贅字率低，語速穩定，音量平穩，表達清晰，但情感渲染力與共鳴感較為平淡。</v>
       </c>
       <c r="Q4" t="str">
         <v>符合</v>
@@ -57984,16 +58011,16 @@
         <v>9</v>
       </c>
       <c r="S4" t="str">
-        <v>主持人（娜娜）口條清晰，語速適中，音量平穩，具備溫暖的語調與親和力，能有效引導來賓。</v>
+        <v>主持人宇澤（雖然節目名稱為哇賽心理學，但主持人為宇澤，為男性，此獎項應為 null）口條流暢，贅字率低，語速穩定，音量平穩，表達清晰，但情感渲染力與共鳴感較為平淡。</v>
       </c>
       <c r="T4" t="str">
-        <v>符合</v>
+        <v>不適用</v>
       </c>
       <c r="U4">
         <v>8</v>
       </c>
       <c r="V4" t="str">
-        <v>節目中提及新書練習與 app 研發，有引導聽眾自我覺察與行動的意圖，但呼籲訂閱或互動的直接性較弱。</v>
+        <v>節目結尾常有對聽眾的鼓勵與引導，例如鼓勵自我覺察、練習與反思，但較少明確的行動呼籲（如訂閱、分享）。</v>
       </c>
       <c r="W4" t="str">
         <v>符合</v>
@@ -58002,7 +58029,7 @@
         <v>9.5</v>
       </c>
       <c r="Y4" t="str">
-        <v>節目探討「金錢性格」、「創傷療癒」、「多巴胺陷阱」等議題，具備心理學的深度與稀有性，論述完整。</v>
+        <v>探討的議題（金錢性格、多巴胺陷阱、創傷療癒）具備高度的稀有性與深度，切入角度獨特，論述完整，成功守護了這些領域的知識火苗。</v>
       </c>
       <c r="Z4" t="str">
         <v>符合</v>
@@ -58011,7 +58038,7 @@
         <v>9</v>
       </c>
       <c r="AB4" t="str">
-        <v>節目內容觸及「金錢性格」、「創傷療癒」、「內耗」等，引導聽眾自我覺察與理解，具有心靈啟發力。</v>
+        <v>節目主題涵蓋金錢觀、內耗成因、創傷療癒，引導聽眾深入探索自我內在、原生家庭的影響，並提供覺察與轉化的方法，啟發性高。</v>
       </c>
       <c r="AC4" t="str">
         <v>符合</v>
@@ -58020,24 +58047,33 @@
         <v>4</v>
       </c>
       <c r="AE4" t="str">
-        <v>單集時長約 30-40 分鐘，未達「講不完大獎」的 60 分鐘門檻，也未達「泡麵沒熟獎」的 10-15 分鐘門檻，時長精煉度不符合兩獎項定義。</v>
+        <v>抽樣單集時長均未達 60 分鐘（約 30-40 分鐘），不符合獎項定義。</v>
       </c>
       <c r="AF4" t="str">
-        <v>不符合(原因：時長不符合該時長獎項之門檻)</v>
+        <v>不符合(原因：時長小於60分鐘)</v>
       </c>
       <c r="AG4">
         <v>7</v>
       </c>
       <c r="AH4" t="str">
-        <v>節目氛圍偏向知識性與探��性，主持人語調溫和，但較少展現積極的晨間活力或深夜的療癒陪伴感，意向較不明確。</v>
+        <v>節目 EP148 時長約 30 分鐘，EP193 與 EP194 時長約 30-40 分鐘，均超過 15 分鐘���限制，不符合短篇定義，但內容相對精煉。</v>
       </c>
       <c r="AI4" t="str">
+        <v>不符合(原因：時長大於15分鐘)</v>
+      </c>
+      <c r="AJ4">
+        <v>7</v>
+      </c>
+      <c r="AK4" t="str">
+        <v>主持人宇澤的語調平穩，談話風格偏向知識性與分析性，雖然內容有深度，但較缺乏溫暖的陪伴感或療癒氛圍，較適合需要學習的聽眾。</v>
+      </c>
+      <c r="AL4" t="str">
         <v>符合</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AI4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AL4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
style: fix summary card text visibility and exclude single-host from duo hosts award
</commit_message>
<xml_diff>
--- a/eligible_episodes_pool.xlsx
+++ b/eligible_episodes_pool.xlsx
@@ -57980,14 +57980,14 @@
       <c r="H4" t="str">
         <v>符合</v>
       </c>
-      <c r="I4">
-        <v>9.5</v>
+      <c r="I4" t="str">
+        <v>N/A</v>
       </c>
       <c r="J4" t="str">
-        <v>主持人宇澤與來賓（心理師、博士）互動流暢自然，提問精準且能引導來賓深入分享，展現高度的專業默契與對談節奏感。</v>
+        <v>單人主持節目，不適用此獎項。</v>
       </c>
       <c r="K4" t="str">
-        <v>符合</v>
+        <v>不適用</v>
       </c>
       <c r="L4">
         <v>9</v>

</xml_diff>

<commit_message>
feat: implement batch voice evaluation script and run trial for 3 episodes
</commit_message>
<xml_diff>
--- a/eligible_episodes_pool.xlsx
+++ b/eligible_episodes_pool.xlsx
@@ -9,6 +9,7 @@
     <sheet name="發片量統計與資格判定" sheetId="4" r:id="rId4"/>
     <sheet name="Apple榜單歷史排行" sheetId="5" r:id="rId5"/>
     <sheet name="POC評分結果" sheetId="6" r:id="rId6"/>
+    <sheet name="聲音物理評估" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -58076,4 +58077,203 @@
     <ignoredError numberStoredAsText="1" sqref="A1:AL4"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>合作夥伴</v>
+      </c>
+      <c r="B1" t="str">
+        <v>節目名稱</v>
+      </c>
+      <c r="C1" t="str">
+        <v>單集標題</v>
+      </c>
+      <c r="D1" t="str">
+        <v>語速 (字/分)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>贅字等級</v>
+      </c>
+      <c r="F1" t="str">
+        <v>贅字分析</v>
+      </c>
+      <c r="G1" t="str">
+        <v>聲音共鳴特質</v>
+      </c>
+      <c r="H1" t="str">
+        <v>錄音品質等級</v>
+      </c>
+      <c r="I1" t="str">
+        <v>製播缺陷-噴麥</v>
+      </c>
+      <c r="J1" t="str">
+        <v>製播缺陷-爆音</v>
+      </c>
+      <c r="K1" t="str">
+        <v>製播缺陷-環境底噪</v>
+      </c>
+      <c r="L1" t="str">
+        <v>音質整體說明</v>
+      </c>
+      <c r="M1" t="str">
+        <v>推薦黃金聽點區間</v>
+      </c>
+      <c r="N1" t="str">
+        <v>黃金聽點推薦理由</v>
+      </c>
+      <c r="O1" t="str">
+        <v>評估時間</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="B2" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="C2" t="str">
+        <v>郝聲音：（上）設計師KiKi，從繪畫到設計的熱愛之路，到引領他人感受設計之美的「走讀」行旅～</v>
+      </c>
+      <c r="D2">
+        <v>265</v>
+      </c>
+      <c r="E2" t="str">
+        <v>高</v>
+      </c>
+      <c r="F2" t="str">
+        <v>男主持人常在句首使用「那」和「就是」作為轉折或連接詞，頻率較高。女主持人則較常使用「嗯」、「然後」和「其實」，頻率中等，但整體而言，兩位主持人的贅字頻率偏高。</v>
+      </c>
+      <c r="G2" t="str">
+        <v>男主持人（好哥）中低音共鳴飽滿，聲音厚實且富有磁性，語調變化豐富，充滿活力。女主持人（Kiki）高音域圓潤，聲音清晰溫和，帶有親和力，語氣真誠，無刺耳感。</v>
+      </c>
+      <c r="H2" t="str">
+        <v>優</v>
+      </c>
+      <c r="I2" t="str">
+        <v>無</v>
+      </c>
+      <c r="J2" t="str">
+        <v>無</v>
+      </c>
+      <c r="K2" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L2" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，聽感舒適。</v>
+      </c>
+      <c r="M2" t="str">
+        <v>03:36 - 03:47</v>
+      </c>
+      <c r="N2" t="str">
+        <v>此段落女主持人Kiki分享她從小就對設計有著強烈的內心呼喚，語氣中透露出真誠與堅定。男主持人適時的提問與感嘆「好幸福喔」也為這段對話增添了情感深度，展現了主講人早期的志向與熱情。</v>
+      </c>
+      <c r="O2" t="str">
+        <v>2026-06-20T12:51:53.770Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="B3" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="C3" t="str">
+        <v>郝聲音：（下）終於跟MJ林明樟老師合體！用「財務腦」打通「業務力」，讓商業與人生獲利生生不息！</v>
+      </c>
+      <c r="D3">
+        <v>250</v>
+      </c>
+      <c r="E3" t="str">
+        <v>中</v>
+      </c>
+      <c r="F3" t="str">
+        <v>兩位主講人皆常在句首使用「那」、「然後」或「就是」作為語氣詞或轉折詞，頻率中等，但不會過於頻繁而影響聽感。</v>
+      </c>
+      <c r="G3" t="str">
+        <v>兩位男主持人聲音共鳴感佳，中低音厚實且清晰，語調自然流暢，情感表達豐富，無機器人唸稿感，整體聽感親和且具說服力。</v>
+      </c>
+      <c r="H3" t="str">
+        <v>優</v>
+      </c>
+      <c r="I3" t="str">
+        <v>無</v>
+      </c>
+      <c r="J3" t="str">
+        <v>無</v>
+      </c>
+      <c r="K3" t="str">
+        <v>環境安靜，幾乎無底噪，錄音背景非常乾淨。</v>
+      </c>
+      <c r="L3" t="str">
+        <v>整體錄音品質優良，音量平穩一致，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聆聽體���。</v>
+      </c>
+      <c r="M3" t="str">
+        <v>02:28 - 03:46</v>
+      </c>
+      <c r="N3" t="str">
+        <v>此段落由MJ老師分享個人生病導致公司薪資停發，以及離職後公司仍能良好運作的親身經歷，引導出「系統」的重要性。他以生動的語氣和具體的「1x1x1」乘法概念，深入淺出地解釋了系統運作的關鍵，情感真摯且極具說服力，是理解課程核心理念的精彩片段。</v>
+      </c>
+      <c r="O3" t="str">
+        <v>2026-06-20T12:52:38.345Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="B4" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="C4" t="str">
+        <v>郝聲音：（下） 蘇絢慧老師好書分享，『隱性內耗』：看不見的傷，如何消磨你的能量？</v>
+      </c>
+      <c r="D4">
+        <v>205</v>
+      </c>
+      <c r="E4" t="str">
+        <v>中</v>
+      </c>
+      <c r="F4" t="str">
+        <v>主講人（徐瑄惠老師）和主持人（好哥）皆常在句首使用「然後」進行轉折，或使用「就是」、「那」等詞，頻率中等。</v>
+      </c>
+      <c r="G4" t="str">
+        <v>男主持人（好哥）聲音中低音共鳴厚實，語調情感豐富且具親和力。女主持人（徐瑄惠老師）聲音圓潤清晰，高音域不刺耳，語氣溫和具陪伴感。</v>
+      </c>
+      <c r="H4" t="str">
+        <v>優</v>
+      </c>
+      <c r="I4" t="str">
+        <v>無</v>
+      </c>
+      <c r="J4" t="str">
+        <v>無</v>
+      </c>
+      <c r="K4" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L4" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低。</v>
+      </c>
+      <c r="M4" t="str">
+        <v>01:59 - 03:45</v>
+      </c>
+      <c r="N4" t="str">
+        <v>此段落深入探討童年環境如何形塑個人對自我價值的認知，以及如何導致內耗與自我質疑。主講人語氣真摯，情感起伏自然，內容具啟發性，是理解內耗成因的關鍵點。</v>
+      </c>
+      <c r="O4" t="str">
+        <v>2026-06-20T12:53:14.710Z</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:O4"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: isolate qualification check into its own tab and fix voice chart integration
</commit_message>
<xml_diff>
--- a/eligible_episodes_pool.xlsx
+++ b/eligible_episodes_pool.xlsx
@@ -58081,7 +58081,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -58271,9 +58271,291 @@
         <v>2026-06-20T12:53:14.710Z</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="B5" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="C5" t="str">
+        <v>GD229｜明明不想去卻說「好」？揭開你不敢拒絕的心理盲點與精神內耗！</v>
+      </c>
+      <c r="D5">
+        <v>205</v>
+      </c>
+      <c r="E5" t="str">
+        <v>中</v>
+      </c>
+      <c r="F5" t="str">
+        <v>主講人常在句尾或轉折處使用「啊」作為語氣助詞，例如「我們常常以為啊」、「這麼累啊」、「更可怕的是啊」。此外，也會使用「那」作為語句開頭的轉折詞，頻率中等。</v>
+      </c>
+      <c r="G5" t="str">
+        <v>男主持人聲音溫暖、厚實，中低音共鳴感強，語調自然流暢，情感表達豐富，沒有機器人唸稿感，聽起來非常親和且具說服力，完全不刺耳。</v>
+      </c>
+      <c r="H5" t="str">
+        <v>優</v>
+      </c>
+      <c r="I5" t="str">
+        <v>無</v>
+      </c>
+      <c r="J5" t="str">
+        <v>無</v>
+      </c>
+      <c r="K5" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L5" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象���背景音樂的淡入淡出處理得宜，不干擾人聲。</v>
+      </c>
+      <c r="M5" t="str">
+        <v>01:28 - 03:52</v>
+      </c>
+      <c r="N5" t="str">
+        <v>此段落是節目的核心，主講人從提出問題「為什麼我們總是習慣先說好，卻讓自己過得這麼累啊？」開始，接著深入剖析三個核心重點，語氣真摯且音調波動起伏有致，情感表達豐富，極具聲音說服力，能有效引導聽眾思考並產生共鳴。</v>
+      </c>
+      <c r="O5" t="str">
+        <v>2026-06-20T13:12:14.179Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="B6" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="C6" t="str">
+        <v>GD221｜別再被情緒牽著鼻子走！開口前停頓 3 秒鐘，瞬間改寫你的人生劇本</v>
+      </c>
+      <c r="D6">
+        <v>197</v>
+      </c>
+      <c r="E6" t="str">
+        <v>中</v>
+      </c>
+      <c r="F6" t="str">
+        <v>主講人常在句首或轉折處使用「那」和「就是」，例如「那書中引用了...」、「就是幫助大腦建立...」，頻率中等，但整體不影響理解。</v>
+      </c>
+      <c r="G6" t="str">
+        <v>男主持人聲音中低音厚實，共鳴感強，語調情感豐富且富有親和力，沒有機器人唸稿感，聽感舒適。</v>
+      </c>
+      <c r="H6" t="str">
+        <v>優</v>
+      </c>
+      <c r="I6" t="str">
+        <v>無</v>
+      </c>
+      <c r="J6" t="str">
+        <v>無</v>
+      </c>
+      <c r="K6" t="str">
+        <v>環境安靜，幾乎無底噪，錄音非常乾淨。</v>
+      </c>
+      <c r="L6" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音控制得很好，聲音清晰。</v>
+      </c>
+      <c r="M6" t="str">
+        <v>01:33 - 03:25</v>
+      </c>
+      <c r="N6" t="str">
+        <v>此段落清晰地闡述了「反應」與「回應」的核心概念，並透過生動的詐騙電話情境和天后王菲的經典案例，具體說明兩者差異。主講人語氣真摯且音調波動起伏有致，極具聲音說服力，能有效引導聽眾思考。</v>
+      </c>
+      <c r="O6" t="str">
+        <v>2026-06-20T13:12:47.923Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="B7" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="C7" t="str">
+        <v>EP169｜蝦皮內捲太絕望？夜校打雜工逆襲：我如何在亞馬遜高門檻戰場穩賺美金！（Feat. AZ-Helper 創辦人 Jonathan 里長伯）</v>
+      </c>
+      <c r="D7">
+        <v>205</v>
+      </c>
+      <c r="E7" t="str">
+        <v>中</v>
+      </c>
+      <c r="F7" t="str">
+        <v>主講人與來賓皆常在句首使用「然後」作為轉折詞，以及「就是」作為語氣連接詞，頻率中等。</v>
+      </c>
+      <c r="G7" t="str">
+        <v>男主持人聲音沉穩，中低音共鳴感佳，語調專業且富有親和力。來賓聲音清晰，語氣真摯且充滿熱情，無刺耳感。</v>
+      </c>
+      <c r="H7" t="str">
+        <v>優</v>
+      </c>
+      <c r="I7" t="str">
+        <v>無</v>
+      </c>
+      <c r="J7" t="str">
+        <v>無</v>
+      </c>
+      <c r="K7" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L7" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低。</v>
+      </c>
+      <c r="M7" t="str">
+        <v>04:29 - 05:00</v>
+      </c>
+      <c r="N7" t="str">
+        <v>此段落揭露主講人八歲時接觸電商的獨特經歷，其母親以創意方式引導他賺取零用錢，語氣生動且充滿情感，極具吸引力。</v>
+      </c>
+      <c r="O7" t="str">
+        <v>2026-06-20T13:13:48.215Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>哇賽心理學_蔡宇哲</v>
+      </c>
+      <c r="B8" t="str">
+        <v>哇賽心理學</v>
+      </c>
+      <c r="C8" t="str">
+        <v>掌握你的金錢性格，打造幸福家庭理財ft.精算媽咪珊迪兔｜哇賽心觀點ep194</v>
+      </c>
+      <c r="D8">
+        <v>245</v>
+      </c>
+      <c r="E8" t="str">
+        <v>中</v>
+      </c>
+      <c r="F8" t="str">
+        <v>主講人與來賓皆有使用「就是」、「其實」作為語氣詞或轉折詞，來賓常使用「然後」連接語句，但整體頻率尚可接受，不致影響聽感。</v>
+      </c>
+      <c r="G8" t="str">
+        <v>男主持人聲音低沉厚實，共鳴感佳，語調變化自然，富有親和力。女主持人聲音清晰明亮，高音域圓潤不刺耳，帶有溫馨陪伴感，表達流暢。</v>
+      </c>
+      <c r="H8" t="str">
+        <v>優</v>
+      </c>
+      <c r="I8" t="str">
+        <v>無</v>
+      </c>
+      <c r="J8" t="str">
+        <v>無</v>
+      </c>
+      <c r="K8" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L8" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺���驗。</v>
+      </c>
+      <c r="M8" t="str">
+        <v>02:07 - 03:44</v>
+      </c>
+      <c r="N8" t="str">
+        <v>此段落來賓生動地分享了原生家庭中父母截然不同的金錢觀（父親的創業擴張與母親的節儉務實），以及這些經歷如何塑造了她個人的金錢觀。她真誠地反思了「好」與「不好」的定義，並強調找到自己最舒適的理財方式，內容具深度且引人共鳴，情感表達豐富，是極具說服力的黃金聽點。</v>
+      </c>
+      <c r="O8" t="str">
+        <v>2026-06-20T13:14:32.297Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>哇賽心理學_蔡宇哲</v>
+      </c>
+      <c r="B9" t="str">
+        <v>哇賽心理學</v>
+      </c>
+      <c r="C9" t="str">
+        <v>多巴胺陷阱！戒不掉的不是癮，是深層的焦慮ft.蘇琮祺心理師｜哇賽心觀點ep193</v>
+      </c>
+      <c r="D9">
+        <v>195</v>
+      </c>
+      <c r="E9" t="str">
+        <v>中</v>
+      </c>
+      <c r="F9" t="str">
+        <v>主講人常在句首使用「然後」和「那」作為轉折詞，頻率中等，但整體對話流暢度不受影響。</v>
+      </c>
+      <c r="G9" t="str">
+        <v>男主持人（宇澤）聲音溫暖、清晰，中低音共鳴感強，語調自然且富有情感，沒有機器人唸稿感。來賓（蘇崇其）的聲音也專業且清晰，兩位主持人的聲音都具親和力，無刺耳感。</v>
+      </c>
+      <c r="H9" t="str">
+        <v>優</v>
+      </c>
+      <c r="I9" t="str">
+        <v>無</v>
+      </c>
+      <c r="J9" t="str">
+        <v>無</v>
+      </c>
+      <c r="K9" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L9" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺體驗���</v>
+      </c>
+      <c r="M9" t="str">
+        <v>02:07 - 03:49</v>
+      </c>
+      <c r="N9" t="str">
+        <v>此段落深入探討了「食物成癮」與「進食成癮」的區別，並進一步闡述了成癮與壞習慣之間的模糊界線，是節目核心概念的精彩呈現。主講人與來賓的對話充滿洞察力，語氣真摯且音調波動起伏有致，極具聲音說服力。</v>
+      </c>
+      <c r="O9" t="str">
+        <v>2026-06-20T13:15:23.756Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>哇賽心理學_蔡宇哲</v>
+      </c>
+      <c r="B10" t="str">
+        <v>哇賽心理學</v>
+      </c>
+      <c r="C10" t="str">
+        <v>療癒創傷，溫柔擁抱完整的自己ft.留佩萱博士｜哇賽療心室ep148</v>
+      </c>
+      <c r="D10">
+        <v>260</v>
+      </c>
+      <c r="E10" t="str">
+        <v>中</v>
+      </c>
+      <c r="F10" t="str">
+        <v>主講人與來賓皆常使用「就是」、「那」、「其實」等口頭禪，其中「就是」的出現頻率高，整體贅字頻率中等。</v>
+      </c>
+      <c r="G10" t="str">
+        <v>女主持人聲音高音域圓潤，語調溫和且富有親和力，無刺耳感，傳達溫馨陪伴感。來賓聲音清晰有力，表達流暢，具說服力。</v>
+      </c>
+      <c r="H10" t="str">
+        <v>優</v>
+      </c>
+      <c r="I10" t="str">
+        <v>無</v>
+      </c>
+      <c r="J10" t="str">
+        <v>無</v>
+      </c>
+      <c r="K10" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L10" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。</v>
+      </c>
+      <c r="M10" t="str">
+        <v>03:41 - 04:09</v>
+      </c>
+      <c r="N10" t="str">
+        <v>此段落來賓以具體案例解釋IFS核心概念，說明童年受批評如何導致內化問題並形成保護機制。語氣真摯且清晰，情感起伏自然，有助於聽眾理解複雜的心理學概念。</v>
+      </c>
+      <c r="O10" t="str">
+        <v>2026-06-20T13:16:15.224Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: update walkthrough.md with daily free tier quota analysis
</commit_message>
<xml_diff>
--- a/eligible_episodes_pool.xlsx
+++ b/eligible_episodes_pool.xlsx
@@ -8,6 +8,7 @@
     <sheet name="合格單集池" sheetId="3" r:id="rId3"/>
     <sheet name="發片量統計與資格判定" sheetId="4" r:id="rId4"/>
     <sheet name="Apple榜單歷史排行" sheetId="5" r:id="rId5"/>
+    <sheet name="聲音物理評估" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -57803,4 +57804,1791 @@
     <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:X24"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>合作夥伴</v>
+      </c>
+      <c r="B1" t="str">
+        <v>節目名稱</v>
+      </c>
+      <c r="C1" t="str">
+        <v>單集標題</v>
+      </c>
+      <c r="D1" t="str">
+        <v>語速 (字/分)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>贅字等級</v>
+      </c>
+      <c r="F1" t="str">
+        <v>贅字分析</v>
+      </c>
+      <c r="G1" t="str">
+        <v>聲音共鳴特質</v>
+      </c>
+      <c r="H1" t="str">
+        <v>錄音品質等級</v>
+      </c>
+      <c r="I1" t="str">
+        <v>製播缺陷-噴麥</v>
+      </c>
+      <c r="J1" t="str">
+        <v>製播缺陷-爆音</v>
+      </c>
+      <c r="K1" t="str">
+        <v>製播缺陷-環境底噪</v>
+      </c>
+      <c r="L1" t="str">
+        <v>音質整體說明</v>
+      </c>
+      <c r="M1" t="str">
+        <v>推薦黃金聽點區間</v>
+      </c>
+      <c r="N1" t="str">
+        <v>黃金聽點推薦理由</v>
+      </c>
+      <c r="O1" t="str">
+        <v>推薦片段一標題</v>
+      </c>
+      <c r="P1" t="str">
+        <v>推薦片段一區間</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>推薦片段一理由</v>
+      </c>
+      <c r="R1" t="str">
+        <v>推薦片段二標題</v>
+      </c>
+      <c r="S1" t="str">
+        <v>推薦片段二區間</v>
+      </c>
+      <c r="T1" t="str">
+        <v>推薦片段二理由</v>
+      </c>
+      <c r="U1" t="str">
+        <v>推薦片段三標題</v>
+      </c>
+      <c r="V1" t="str">
+        <v>推薦片段三區間</v>
+      </c>
+      <c r="W1" t="str">
+        <v>推薦片段三理由</v>
+      </c>
+      <c r="X1" t="str">
+        <v>評估時間</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>不敗教主-陳重銘</v>
+      </c>
+      <c r="B2" t="str">
+        <v>不敗教主陳重銘</v>
+      </c>
+      <c r="C2" t="str">
+        <v>EP594《富媽媽 窮媽媽》第二章(4)：原來讀書就是為了要賺錢養家，工作就是在坐牢</v>
+      </c>
+      <c r="D2">
+        <v>195</v>
+      </c>
+      <c r="E2" t="str">
+        <v>中</v>
+      </c>
+      <c r="F2" t="str">
+        <v>主講人頻繁使用「那」、「就是」、「對不對」作為語句間的連接詞或語氣助詞，尤其「那」在句首的出現頻率較高，用於轉折或引導新話題。整體而言，贅字頻率屬於中等。</v>
+      </c>
+      <c r="G2" t="str">
+        <v>男聲低音厚實，共鳴感強，語調自然流暢，情感豐富，沒有機器人唸稿感，具有良好的親和力與說服力。</v>
+      </c>
+      <c r="H2" t="str">
+        <v>優</v>
+      </c>
+      <c r="I2" t="str">
+        <v>無</v>
+      </c>
+      <c r="J2" t="str">
+        <v>無</v>
+      </c>
+      <c r="K2" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L2" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景環境音處理得非常乾淨。</v>
+      </c>
+      <c r="M2" t="str">
+        <v>00:04 - 01:15</v>
+      </c>
+      <c r="N2" t="str">
+        <v>主持人以書籍《富媽媽窮媽媽》為引，迅速切入主題，並結合自身年輕時對投資、退休與人生選擇的思考，語氣真誠，引人入勝，有效抓住聽眾的注意力。</v>
+      </c>
+      <c r="O2" t="str">
+        <v>開場引導與人生反思</v>
+      </c>
+      <c r="P2" t="str">
+        <v>00:04 - 01:15</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>主持人以書籍《富媽媽窮媽媽》為引，迅速切入主題，並結合自身年輕時對投資、退休與人生選擇的思考，語氣真誠，引人入勝，有效抓住聽眾的注意力。</v>
+      </c>
+      <c r="R2" t="str">
+        <v>職涯抉擇與科技新貴時代</v>
+      </c>
+      <c r="S2" t="str">
+        <v>02:40 - 06:25</v>
+      </c>
+      <c r="T2" t="str">
+        <v>此段落講述主持人畢業後求職聯電的經歷，以及當時台灣半導體產業「科技新貴」的社會現象。透過個人故事與時代背景的結合，生動描繪了當時的機遇與挑戰，充滿故事性與啟發性。</v>
+      </c>
+      <c r="U2" t="str">
+        <v>穩定代價與人生智慧</v>
+      </c>
+      <c r="V2" t="str">
+        <v>09:15 - 17:49</v>
+      </c>
+      <c r="W2" t="str">
+        <v>主持人深入探討「穩定要付出代價」的核心觀點，對比公務員與投資台積電的風險與報酬，並分享了老鳥師傅關於讀書與工作目的的深刻啟示，結尾處的懸念設計也引人期待下一集。</v>
+      </c>
+      <c r="X2" t="str">
+        <v>2026-06-21T00:35:36.558Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>不敗教主-陳重銘</v>
+      </c>
+      <c r="B3" t="str">
+        <v>不敗教主陳重銘</v>
+      </c>
+      <c r="C3" t="str">
+        <v>EP633當ETF愈來愈熱門，你是不是也有這些疑問���</v>
+      </c>
+      <c r="D3">
+        <v>210</v>
+      </c>
+      <c r="E3" t="str">
+        <v>中</v>
+      </c>
+      <c r="F3" t="str">
+        <v>主講人常在句首或句中轉折處使用「好」、「那」和「就是」作為口頭禪，例如「好，老師」、「那再來就是說」、「就是說」。這些贅字頻率中等，但由於語速較快，整體聽感上並未造成明顯的拖沓。</v>
+      </c>
+      <c r="G3" t="str">
+        <v>男主持人聲音低沉厚實，共鳴感強，語調變化豐富，充滿自信與說服力，沒有機器人唸稿的生硬感。女主持人聲音清晰，語氣溫和，與男主持人形成良好搭配。</v>
+      </c>
+      <c r="H3" t="str">
+        <v>優</v>
+      </c>
+      <c r="I3" t="str">
+        <v>無</v>
+      </c>
+      <c r="J3" t="str">
+        <v>無</v>
+      </c>
+      <c r="K3" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L3" t="str">
+        <v>整體錄音品���優良，音量平穩，沒有突兀爆音與噴麥現象，背景環境音也處理得非常乾淨，提供清晰的聆聽體驗。</v>
+      </c>
+      <c r="M3" t="str">
+        <v>00:24 - 00:50</v>
+      </c>
+      <c r="N3" t="str">
+        <v>主講人從ETF的本質（追踪淨值）出發，清晰解釋其運作原理，並針對網路上對ETF的錯誤觀念和仇恨言論進行駁斥，語氣堅定，能有效糾正聽眾的錯誤認知，具備教育意義。</v>
+      </c>
+      <c r="O3" t="str">
+        <v>ETF核心觀念與市場誤解</v>
+      </c>
+      <c r="P3" t="str">
+        <v>00:24 - 00:50</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>主講人從ETF的本質（追踪淨值）出發，清晰解釋其運作原理，並針對網路上對ETF的錯誤觀念和仇恨言論進行駁斥，語氣堅定，能有效糾正聽眾的錯誤認知，具備教育意義。</v>
+      </c>
+      <c r="R3" t="str">
+        <v>外資賣超如何影響ETF淨值</v>
+      </c>
+      <c r="S3" t="str">
+        <v>02:43 - 03:47</v>
+      </c>
+      <c r="T3" t="str">
+        <v>主講人詳細解釋了外資賣出ETF後，市場造市商和投信如何接手並處理這些股票，進而影響ETF淨值的機制。這段內容深入淺出，揭示了市場運作的複雜性，對於理解ETF價格波動有重要啟發。</v>
+      </c>
+      <c r="U3" t="str">
+        <v>投資策略與財富規劃的長期視角</v>
+      </c>
+      <c r="V3" t="str">
+        <v>08:58 - 09:05 &amp; 21:22 - 21:31</v>
+      </c>
+      <c r="W3" t="str">
+        <v>主講人強調了投資ETF不應追高，應定期定額或在大跌時加碼的實用策略。隨後，他以遺產稅為例，說明了提早進行財富規劃的重要性，將投資與人生規劃結合，展現了深遠的思考和對聽眾的關懷。</v>
+      </c>
+      <c r="X3" t="str">
+        <v>2026-06-21T00:37:19.813Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>不敗教主-陳重銘</v>
+      </c>
+      <c r="B4" t="str">
+        <v>不敗教主陳重銘</v>
+      </c>
+      <c r="C4" t="str">
+        <v>EP639《富媽媽 窮媽媽》第三章(2)：把內褲穿在外面，當超人啊！</v>
+      </c>
+      <c r="D4">
+        <v>205</v>
+      </c>
+      <c r="E4" t="str">
+        <v>中</v>
+      </c>
+      <c r="F4" t="str">
+        <v>主講人常在句首或句中以「那」和「就是」作為轉折詞或語氣詞，頻率中等，例如「那沒關係，我們就慢慢地講」(0:34)、「就是一個流浪教師啊」(4:24)。這些口頭禪雖頻繁，但並未嚴重影響語句的流暢度。</v>
+      </c>
+      <c r="G4" t="str">
+        <v>男聲中低音共鳴感強，聲音厚實且富有磁性。語調自然，情感表達豐富，沒有機器人唸稿的生硬感，整體聽感親和力佳。</v>
+      </c>
+      <c r="H4" t="str">
+        <v>優</v>
+      </c>
+      <c r="I4" t="str">
+        <v>無</v>
+      </c>
+      <c r="J4" t="str">
+        <v>無</v>
+      </c>
+      <c r="K4" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L4" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與���麥現象，背景環境噪音極低，提供清晰舒適的聆聽體驗。</v>
+      </c>
+      <c r="M4" t="str">
+        <v>00:04 - 00:40</v>
+      </c>
+      <c r="N4" t="str">
+        <v>主持人以自身「不敗家」的經歷切入陳老師新書的主題，語氣輕鬆幽默，迅速建立與聽眾的連結，並點出節目核心討論方向，開場極具吸引力。</v>
+      </c>
+      <c r="O4" t="str">
+        <v>個人經歷與書籍主題的引人入勝開場</v>
+      </c>
+      <c r="P4" t="str">
+        <v>00:04 - 00:40</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>主持人以自身「不敗家」的經歷切入陳老師新書的主題，語氣輕鬆幽默，迅速建立與聽眾的連結，並點出節目核心討論方向，開場極具吸引力。</v>
+      </c>
+      <c r="R4" t="str">
+        <v>努力與投資的價值：從流浪教師到財務自由</v>
+      </c>
+      <c r="S4" t="str">
+        <v>02:02 - 03:02</v>
+      </c>
+      <c r="T4" t="str">
+        <v>主持人分享他從年輕時的努力奮鬥，到現在能輕鬆負擔高價物品的轉變，強調了「努力一點」和「有人幫我買單」（投資股票）的重要性，是節目核心理念的精華，語氣真摯且具說服力。</v>
+      </c>
+      <c r="U4" t="str">
+        <v>人生繞一圈的智慧：彎路也是寶貴的經歷</v>
+      </c>
+      <c r="V4" t="str">
+        <v>16:07 - 17:39</v>
+      </c>
+      <c r="W4" t="str">
+        <v>主持人回顧自己的人生軌跡，從叛逆不願當老師到最終成為老師，並在過程中累積了寫書等寶貴經驗。他將這些「繞路」的經歷視為財富，並以此鼓勵聽眾從他的經驗中學習，避免走冤枉路，展現了深刻的人生哲理與溫暖的陪伴感。</v>
+      </c>
+      <c r="X4" t="str">
+        <v>2026-06-21T00:36:26.605Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="B5" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="C5" t="str">
+        <v>EP133｜顛覆你對美容業的想像！她用做企業的腦袋，重新定義「養膚管理」（Feat. 尖時養膚管理創辦人 劉欣玲·玲玲）</v>
+      </c>
+      <c r="D5">
+        <v>205</v>
+      </c>
+      <c r="E5" t="str">
+        <v>中</v>
+      </c>
+      <c r="F5" t="str">
+        <v>兩位主講人皆常在句首或句中以「然後」作為轉折詞，或使用「就是」來強調或解釋，頻率中等，但不會過於影響聽感。偶爾也會出現「對啊」作為回應或語氣詞。</v>
+      </c>
+      <c r="G5" t="str">
+        <v>男主持人（安迪）的聲音中低音共鳴感強，語調沉穩且富有親和力，表達清晰，沒有機器人唸稿感。女主持人（玲玲）的聲音高音域圓潤，語氣充滿活力與熱情，表達流暢，沒有刺耳感，給人溫馨陪伴的感受。</v>
+      </c>
+      <c r="H5" t="str">
+        <v>優</v>
+      </c>
+      <c r="I5" t="str">
+        <v>無</v>
+      </c>
+      <c r="J5" t="str">
+        <v>無</v>
+      </c>
+      <c r="K5" t="str">
+        <v>環境安靜，幾乎無底噪，背景音樂與人聲融合度佳</v>
+      </c>
+      <c r="L5" t="str">
+        <v>整體錄音品質優良，音量平穩，人聲清晰，沒有突兀爆音與噴麥現象，背景噪音控制得非常好。</v>
+      </c>
+      <c r="M5" t="str">
+        <v>00:00 - 02:30</v>
+      </c>
+      <c r="N5" t="str">
+        <v>主持人以引人入勝的提問開場，引導來賓分享她從極度排斥美容到創辦品牌的轉折故事，語速與節奏掌握得宜，迅速抓住聽眾注意力，為整集內容奠定引人入勝的基調。</v>
+      </c>
+      <c r="O5" t="str">
+        <v>破題精采開場：從排斥美容到創辦品牌</v>
+      </c>
+      <c r="P5" t="str">
+        <v>00:00 - 02:30</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>主持人以引人入勝的提問開場，引導來賓分享她從極度排斥美容到創辦品牌的轉折故事，語速與節奏掌握得宜，迅速抓住聽眾注意力，為整集內容奠定引人入勝的基調。</v>
+      </c>
+      <c r="R5" t="str">
+        <v>個人轉變與知識追求：從被動保養到主動學習</v>
+      </c>
+      <c r="S5" t="str">
+        <v>02:44 - 05:00</v>
+      </c>
+      <c r="T5" t="str">
+        <v>來賓分享她因個人保養效果顯著而獲得讚美，從而激發了她對美容的興趣，並開始主動學習相關知識，展現了從個人經驗出發的學習動力，這段故事充滿了轉折與啟發性。</v>
+      </c>
+      <c r="U5" t="str">
+        <v>學習的樂趣：從討厭讀書到愛上「彩虹筆記法」</v>
+      </c>
+      <c r="V5" t="str">
+        <v>09:19 - 12:00</v>
+      </c>
+      <c r="W5" t="str">
+        <v>來賓分享她過去不愛讀書，卻因遇到啟蒙老師和「彩虹筆記法」而愛上學習的過程，生動描述了知識如何變得有趣，展現了她對學習方式的獨特見解，語調充滿興奮與感染力。</v>
+      </c>
+      <c r="X5" t="str">
+        <v>2026-06-21T00:30:25.469Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="B6" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="C6" t="str">
+        <v>EP169｜蝦皮內捲太絕望？夜校打雜工逆襲：我如何在亞馬遜高門檻戰場穩賺美金！（Feat. AZ-Helper 創辦人 Jonathan 里長伯）</v>
+      </c>
+      <c r="D6">
+        <v>205</v>
+      </c>
+      <c r="E6" t="str">
+        <v>中</v>
+      </c>
+      <c r="F6" t="str">
+        <v>主講人與來賓皆常在句首使用「然後」作為轉折詞，以及「就是」作為語氣連接詞，頻率中等。</v>
+      </c>
+      <c r="G6" t="str">
+        <v>男主持人聲音沉穩，中低音共鳴感佳，語調專業且富有親和力。來賓聲音清晰，語氣真摯且充滿熱情，無刺耳感。</v>
+      </c>
+      <c r="H6" t="str">
+        <v>優</v>
+      </c>
+      <c r="I6" t="str">
+        <v>無</v>
+      </c>
+      <c r="J6" t="str">
+        <v>無</v>
+      </c>
+      <c r="K6" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L6" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低。</v>
+      </c>
+      <c r="M6" t="str">
+        <v>04:29 - 05:00</v>
+      </c>
+      <c r="N6" t="str">
+        <v>此段落揭露主講人八歲時接觸電商的獨特經歷，其母親以創意方式引導他賺取零用錢，語氣生動且充滿情感，極具吸引力。</v>
+      </c>
+      <c r="O6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="P6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="R6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="S6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="T6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="U6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="V6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="W6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="X6" t="str">
+        <v>2026-06-20T13:13:48.215Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="B7" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="C7" t="str">
+        <v>GD185｜擺脫「零和遊戲」的終極心法：從自我中心走向共好。</v>
+      </c>
+      <c r="D7">
+        <v>195</v>
+      </c>
+      <c r="E7" t="str">
+        <v>中</v>
+      </c>
+      <c r="F7" t="str">
+        <v>主講人常在句首使用「那」或「然後」作為轉折詞，例如在0:27、0:30、0:37、0:42、0:48、0:54、1:05、1:12、1:16、1:22、1:28、1:31、1:32、1:35、1:38、1:41、1:48、1:52、1:53、1:56、2:07、2:12、2:15、2:21、2:26、2:27、2:28、2:30、2:34、2:37、2:41、2:43、2:47、2:49、2:51、2:53、2:56、2:59、3:00、3:04、3:05、3:07、3:10、3:12、3:15、3:16、3:17、3:21、3:22、3:24、3:27、3:32、3:35、3:38、3:39、3:42、3:43、3:46、3:47、3:49、3:50、3:52、3:55、3:56、3:57、3:59、4:00、4:01、4:04、4:07、4:08、4:11、4:12、4:13、4:16、4:17、4:20、4:21、4:23、4:24、4:25、4:28、4:29、4:31、4:34、4:36、4:37、4:39、4:41、4:42、4:45、4:46、4:48、4:49、4:51、4:53、4:55、4:56、4:58、4:59、5:00、5:02、5:03、5:06、5:08、5:09、5:11、5:15、5:18、5:21、5:22、5:26、5:29、5:31、5:32、5:34、5:36、5:37、5:39、5:43、5:44、5:47、5:48、5:51、5:52、5:56、5:57、6:01、6:02、6:05、6:07、6:08、6:09。此外，偶爾會出現「啊」的語氣詞，但整體不影響理解，頻率屬於中等。</v>
+      </c>
+      <c r="G7" t="str">
+        <v>男主持人聲音中低音共鳴感強，音色溫暖厚實，語調平穩且富有親和力。咬字清晰，沒有刺耳或機器人唸稿的感覺，聽感舒適。</v>
+      </c>
+      <c r="H7" t="str">
+        <v>優</v>
+      </c>
+      <c r="I7" t="str">
+        <v>無</v>
+      </c>
+      <c r="J7" t="str">
+        <v>無</v>
+      </c>
+      <c r="K7" t="str">
+        <v>背景環境安靜，幾乎無底噪，錄音品質極佳。</v>
+      </c>
+      <c r="L7" t="str">
+        <v>整體錄音品質非常優良，音量穩定，沒有出現噴麥、突兀爆音或明顯的背景雜音，聲音處理專業。</v>
+      </c>
+      <c r="M7" t="str">
+        <v>00:06 - 00:19</v>
+      </c>
+      <c r="N7" t="str">
+        <v>這段是節目的標準開場，背景音樂搭配主持人溫和而有力的聲音，清晰地介紹了節目的名稱、主持人以及其核心宗旨，即「自我權杖、人生經驗對談和內化學習輸出的節目」，並期待聽眾成為「生命中輕易豐盛、富足而喜��的烏吉郎」。這段話語速適中，語氣真誠，能有效吸引新聽眾了解節目內容與價值觀。</v>
+      </c>
+      <c r="O7" t="str">
+        <v>節目開場與宗旨介紹</v>
+      </c>
+      <c r="P7" t="str">
+        <v>00:06 - 00:19</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>這段是節目的標準開場，背景音樂搭配主持人溫和而有力的聲音，清晰地介紹了節目的名稱、主持人以及其核心宗旨，即「自我權杖、人生經驗對談和內化學習輸出的節目」，並期待聽眾成為「生命中輕易豐盛、富足而喜��的烏吉郎」。這段話語速適中，語氣真誠，能有效吸引新聽眾了解節目內容與價值觀。</v>
+      </c>
+      <c r="R7" t="str">
+        <v>破題：從焦慮到禪宗智慧的引導</v>
+      </c>
+      <c r="S7" t="str">
+        <v>00:23 - 00:47</v>
+      </c>
+      <c r="T7" t="str">
+        <v>主持人以提問方式開場，點出聽眾可能面臨的「心很累」、「擔心被超越」、「害怕吃虧」等職場與生活焦慮，並將這些歸結為「零和遊戲」的人生觀。隨後，他巧妙地引導出本集主題——「禪宗智慧」中的「利他」概念，承諾能讓聽眾「瞬間從這種焦慮解脫」。這段破題精準，情感共鳴強，能迅速抓住聽眾的痛點並提供解決方案的期待，引人入勝。</v>
+      </c>
+      <c r="U7" t="str">
+        <v>結語：利他生活方式的總結與承諾</v>
+      </c>
+      <c r="V7" t="str">
+        <v>05:09 - 05:36</v>
+      </c>
+      <c r="W7" t="str">
+        <v>在節目尾聲，主持人再次強調了「利他」的智慧，總結了「以他人的利益為最優先」的生活方式，能帶來「坦然的心」和「輕鬆自在」的人生。他鼓勵聽眾放下對輸贏的執著，多思考自己能給予什麼，並承諾當你照顧世界，世界也會回過頭來照顧你。這段結語語氣溫暖而堅定，為聽眾帶來正向的啟發和行動指引，同時也再次強化了節目的核心價值，具有很強的陪伴感和說服力。</v>
+      </c>
+      <c r="X7" t="str">
+        <v>2026-06-21T00:25:56.959Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="B8" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="C8" t="str">
+        <v>GD218｜總覺得別人配合你是理所當然？一句話瞬間融化傲慢，找回溫暖好人緣</v>
+      </c>
+      <c r="D8">
+        <v>260</v>
+      </c>
+      <c r="E8" t="str">
+        <v>中</v>
+      </c>
+      <c r="F8" t="str">
+        <v>主講人語速較快，在句首或轉折處常使用「那」和「就是」作為口頭禪，例如「那聽完這三個重點...」、「這就是對祖先最基本的尊重喔」。此外，「啊」也常作為語氣助詞出現，整體贅字頻率中等。</v>
+      </c>
+      <c r="G8" t="str">
+        <v>男主持人聲音低沉厚實，共鳴感強，語調清晰且富有情感，沒有機器人唸稿感，聽起來親和力十足，且無刺耳感。</v>
+      </c>
+      <c r="H8" t="str">
+        <v>優</v>
+      </c>
+      <c r="I8" t="str">
+        <v>無</v>
+      </c>
+      <c r="J8" t="str">
+        <v>無</v>
+      </c>
+      <c r="K8" t="str">
+        <v>環境安靜，幾乎無底噪，背景音樂與人聲融合良好</v>
+      </c>
+      <c r="L8" t="str">
+        <v>整體錄音品質優良，音量平穩，���聲清晰，沒有突兀爆音與噴麥現象，背景音樂搭配得宜，不干擾主講人聲音。</v>
+      </c>
+      <c r="M8" t="str">
+        <v>00:23 - 01:12</v>
+      </c>
+      <c r="N8" t="str">
+        <v>主持人以引人深思的問題開場，探討生命、衰老與終點的焦慮，巧妙地引導出本集的核心主題——對活著這件事充滿感謝。語氣真摯，迅速抓住聽眾注意力，為節目奠定深沉而溫暖的基調。</v>
+      </c>
+      <c r="O8" t="str">
+        <v>生命課題的深層叩問與主題引導</v>
+      </c>
+      <c r="P8" t="str">
+        <v>00:23 - 01:12</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>主持人以引人深思的問題開場，探討生命、衰老與終點的焦慮，巧妙地引導出本集的核心主題——對活著這件事充滿感謝。語氣真摯，迅速抓住聽眾注意力，為節目奠定深沉而溫暖的基調。</v>
+      </c>
+      <c r="R8" t="str">
+        <v>百萬人接力賽：生命傳承的震撼啟示</v>
+      </c>
+      <c r="S8" t="str">
+        <v>02:28 - 03:17</v>
+      </c>
+      <c r="T8" t="str">
+        <v>此段落闡述了「你的存在是超過一百萬人的接力賽」這一核心觀點，透過追溯祖先的數量，深刻揭示了生命的傳承與珍貴。主講人語氣充滿力量與啟發性，讓聽眾對自己的存在產生全新的敬畏與感恩。</v>
+      </c>
+      <c r="U8" t="str">
+        <v>日常實踐：一句話帶來溫暖與喜悅</v>
+      </c>
+      <c r="V8" t="str">
+        <v>06:07 - 06:34</v>
+      </c>
+      <c r="W8" t="str">
+        <v>主持人提出一個簡單卻極具影響力的行動挑戰，鼓勵聽眾在日常對話中多說「托您的福」。這不僅是實踐感恩，也承諾能為人際關係帶來溫暖與內心的平靜。結尾處的聲音共鳴極佳，溫馨且具陪伴感，展現與聽眾深厚的連結感��</v>
+      </c>
+      <c r="X8" t="str">
+        <v>2026-06-21T00:21:51.207Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="B9" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="C9" t="str">
+        <v>GD221｜別再被情緒牽著鼻子走！開口前停頓 3 秒鐘，瞬間改寫你的人生劇本</v>
+      </c>
+      <c r="D9">
+        <v>197</v>
+      </c>
+      <c r="E9" t="str">
+        <v>中</v>
+      </c>
+      <c r="F9" t="str">
+        <v>主講人常在句首或轉折處使用「那」和「就是」，例如「那書中引用了...」、「就是幫助大腦建立...」，頻率中等，但整體不影響理解。</v>
+      </c>
+      <c r="G9" t="str">
+        <v>男主持人聲音中低音厚實，共鳴感強，語調情感豐富且富有親和力，沒有機器人唸稿感，聽感舒適。</v>
+      </c>
+      <c r="H9" t="str">
+        <v>優</v>
+      </c>
+      <c r="I9" t="str">
+        <v>無</v>
+      </c>
+      <c r="J9" t="str">
+        <v>無</v>
+      </c>
+      <c r="K9" t="str">
+        <v>環境安靜，幾乎無底噪，錄音非常乾淨。</v>
+      </c>
+      <c r="L9" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音控制得很好，聲音清晰。</v>
+      </c>
+      <c r="M9" t="str">
+        <v>01:33 - 03:25</v>
+      </c>
+      <c r="N9" t="str">
+        <v>此段落清晰地闡述了「反應」與「回應」的核心概念，並透過生動的詐騙電話情境和天后王菲的經典案例，具體說明兩者差異。主講人語氣真摯且音調波動起伏有致，極具聲音說服力，能有效引導聽眾思考。</v>
+      </c>
+      <c r="O9" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="P9" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="R9" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="S9" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="T9" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="U9" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="V9" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="W9" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="X9" t="str">
+        <v>2026-06-20T13:12:47.923Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="B10" t="str">
+        <v>五吉郎</v>
+      </c>
+      <c r="C10" t="str">
+        <v>GD229｜明明不想去卻說「好」？揭開你不敢拒絕的心理盲點與精神內耗！</v>
+      </c>
+      <c r="D10">
+        <v>205</v>
+      </c>
+      <c r="E10" t="str">
+        <v>中</v>
+      </c>
+      <c r="F10" t="str">
+        <v>主講人常在句尾或轉折處使用「啊」作為語氣助詞，例如「我們常常以為啊」、「這麼累啊」、「更可怕的是啊」。此外，也會使用「那」作為語句開頭的轉折詞，頻率中等。</v>
+      </c>
+      <c r="G10" t="str">
+        <v>男主持人聲音溫暖、厚實，中低音共鳴感強，語調自然流暢，情感表達豐富，沒有機器人唸稿感，聽起來非常親和且具說服力，完全不刺耳。</v>
+      </c>
+      <c r="H10" t="str">
+        <v>優</v>
+      </c>
+      <c r="I10" t="str">
+        <v>無</v>
+      </c>
+      <c r="J10" t="str">
+        <v>無</v>
+      </c>
+      <c r="K10" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L10" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象���背景音樂的淡入淡出處理得宜，不干擾人聲。</v>
+      </c>
+      <c r="M10" t="str">
+        <v>01:28 - 03:52</v>
+      </c>
+      <c r="N10" t="str">
+        <v>此段落是節目的核心，主講人從提出問題「為什麼我們總是習慣先說好，卻讓自己過得這麼累啊？」開始，接著深入剖析三個核心重點，語氣真摯且音調波動起伏有致，情感表達豐富，極具聲音說服力，能有效引導聽眾思考並產生共鳴。</v>
+      </c>
+      <c r="O10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="P10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="R10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="S10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="T10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="U10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="V10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="W10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="X10" t="str">
+        <v>2026-06-20T13:12:14.179Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>布姐陪你聰明工作創意生活</v>
+      </c>
+      <c r="B11" t="str">
+        <v>布姐的沙發</v>
+      </c>
+      <c r="C11" t="str">
+        <v>EP455｜困難抉擇的關鍵心法：如何做出不後悔的選擇</v>
+      </c>
+      <c r="D11">
+        <v>230</v>
+      </c>
+      <c r="E11" t="str">
+        <v>中</v>
+      </c>
+      <c r="F11" t="str">
+        <v>主講人常在句首使用「然後」進行轉折，或以「就是」作為語氣詞或解釋，頻率中等。偶爾會出現「那」作為語氣詞。</v>
+      </c>
+      <c r="G11" t="str">
+        <v>女主持人聲音清晰溫暖，中音域表現良好。高音圓潤不刺耳，整體語調溫和且富有同理心，營造出強烈的溫馨陪伴感，無機器人唸稿感。</v>
+      </c>
+      <c r="H11" t="str">
+        <v>優</v>
+      </c>
+      <c r="I11" t="str">
+        <v>無</v>
+      </c>
+      <c r="J11" t="str">
+        <v>無</v>
+      </c>
+      <c r="K11" t="str">
+        <v>無</v>
+      </c>
+      <c r="L11" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景環境安靜，幾乎無底噪。</v>
+      </c>
+      <c r="M11" t="str">
+        <v>00:00 - 00:57</v>
+      </c>
+      <c r="N11" t="str">
+        <v>節目開場以一個生動且帶有戲劇性的個人故事破題，講述孩子對洗澡的恐懼以及主持人自身的無力感，迅速抓住聽眾注意力。這段不僅展現了主講人的敘事能力，也為後續關於人生選擇的討論奠定了情感基礎，語速與語氣的掌握恰到好處。</v>
+      </c>
+      <c r="O11" t="str">
+        <v>浴室驚魂記：選擇的開端</v>
+      </c>
+      <c r="P11" t="str">
+        <v>00:00 - 00:57</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>節目開場以一個生動且帶有戲劇性的個人故事破題，講述孩子對洗澡的恐懼以及主持人自身的無力感，迅速抓住聽眾注意力。這段不僅展現了主講人的敘事能力，也為後續關於人生選擇的討論奠定了情感基礎，語速與語氣的掌握恰到好處。</v>
+      </c>
+      <c r="R11" t="str">
+        <v>決策分析：優缺點與優先順序</v>
+      </c>
+      <c r="S11" t="str">
+        <v>08:59 - 09:59</v>
+      </c>
+      <c r="T11" t="str">
+        <v>此段落清晰地闡述了主講人面對重大人生決策（回台灣或留在美國）時的分析方法。她詳細說明如何列出選項的優缺點、找出個人優先順序，並思考替代方案。這是一個極具實用性的核心論述，以條理分明的方式呈現，對聽眾具有很高的參考價值。</v>
+      </c>
+      <c r="U11" t="str">
+        <v>人生終點的提問：你會後悔嗎？</v>
+      </c>
+      <c r="V11" t="str">
+        <v>01:42:50 - 01:45:55</v>
+      </c>
+      <c r="W11" t="str">
+        <v>這是一個情感真摯且發人深省的片段。主講人分享了她在做選擇時，會問自己一個深刻的問題：「我在死前會不會因為沒做這件事而後悔？」這個提問觸及了決策的深層意義，引導聽眾思考選擇的長期影響，語氣充滿了反思與誠懇，極具感染力。</v>
+      </c>
+      <c r="X11" t="str">
+        <v>2026-06-21T00:37:57.699Z</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>哇賽心理學_蔡宇哲</v>
+      </c>
+      <c r="B12" t="str">
+        <v>哇賽心理學</v>
+      </c>
+      <c r="C12" t="str">
+        <v>多巴胺陷阱！戒不掉的不是癮，是深層的焦慮ft.蘇琮祺心理師｜哇賽心觀點ep193</v>
+      </c>
+      <c r="D12">
+        <v>195</v>
+      </c>
+      <c r="E12" t="str">
+        <v>中</v>
+      </c>
+      <c r="F12" t="str">
+        <v>主講人常在句首使用「然後」和「那」作為轉折詞，頻率中等，但整體對話流暢度不受影響。</v>
+      </c>
+      <c r="G12" t="str">
+        <v>男主持人（宇澤）聲音溫暖、清晰，中低音共鳴感強，語調自然且富有情感，沒有機器人唸稿感。來賓（蘇崇其）的聲音也專業且清晰，兩位主持人的聲音都具親和力，無刺耳感。</v>
+      </c>
+      <c r="H12" t="str">
+        <v>優</v>
+      </c>
+      <c r="I12" t="str">
+        <v>無</v>
+      </c>
+      <c r="J12" t="str">
+        <v>無</v>
+      </c>
+      <c r="K12" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L12" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺體驗���</v>
+      </c>
+      <c r="M12" t="str">
+        <v>02:07 - 03:49</v>
+      </c>
+      <c r="N12" t="str">
+        <v>此段落深入探討了「食物成癮」與「進食成癮」的區別，並進一步闡述了成癮與壞習慣之間的模糊界線，是節目核心概念的精彩呈現。主講人與來賓的對話充滿洞察力，語氣真摯且音調波動起伏有致，極具聲音說服力。</v>
+      </c>
+      <c r="O12" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="P12" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="R12" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="S12" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="T12" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="U12" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="V12" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="W12" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="X12" t="str">
+        <v>2026-06-20T13:15:23.756Z</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>哇賽心理學_蔡宇哲</v>
+      </c>
+      <c r="B13" t="str">
+        <v>哇賽心理學</v>
+      </c>
+      <c r="C13" t="str">
+        <v>掌握你的金錢性格，打造幸福家庭理財ft.精算媽咪珊迪兔｜哇賽心觀點ep194</v>
+      </c>
+      <c r="D13">
+        <v>245</v>
+      </c>
+      <c r="E13" t="str">
+        <v>中</v>
+      </c>
+      <c r="F13" t="str">
+        <v>主講人與來賓皆有使用「就是」、「其實」作為語氣詞或轉折詞，來賓常使用「然後」連接語句，但整體頻率尚可接受，不致影響聽感。</v>
+      </c>
+      <c r="G13" t="str">
+        <v>男主持人聲音低沉厚實，共鳴感佳，語調變化自然，富有親和力。女主持人聲音清晰明亮，高音域圓潤不刺耳，帶有溫馨陪伴感，表達流暢。</v>
+      </c>
+      <c r="H13" t="str">
+        <v>優</v>
+      </c>
+      <c r="I13" t="str">
+        <v>無</v>
+      </c>
+      <c r="J13" t="str">
+        <v>無</v>
+      </c>
+      <c r="K13" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L13" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺���驗。</v>
+      </c>
+      <c r="M13" t="str">
+        <v>02:07 - 03:44</v>
+      </c>
+      <c r="N13" t="str">
+        <v>此段落來賓生動地分享了原生家庭中父母截然不同的金錢觀（父親的創業擴張與母親的節儉務實），以及這些經歷如何塑造了她個人的金錢觀。她真誠地反思了「好」與「不好」的定義，並強調找到自己最舒適的理財方式，內容具深度且引人共鳴，情感表達豐富，是極具說服力的黃金聽點。</v>
+      </c>
+      <c r="O13" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="P13" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="R13" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="S13" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="T13" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="U13" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="V13" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="W13" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="X13" t="str">
+        <v>2026-06-20T13:14:32.297Z</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>哇賽心理學_蔡宇哲</v>
+      </c>
+      <c r="B14" t="str">
+        <v>哇賽心理學</v>
+      </c>
+      <c r="C14" t="str">
+        <v>療癒創傷，溫柔擁抱完整的自己ft.留佩萱博士｜哇賽療心室ep148</v>
+      </c>
+      <c r="D14">
+        <v>260</v>
+      </c>
+      <c r="E14" t="str">
+        <v>中</v>
+      </c>
+      <c r="F14" t="str">
+        <v>主講人與來賓皆常使用「就是」、「那」、「其實」等口頭禪，其中「就是」的出現頻率高，整體贅字頻率中等。</v>
+      </c>
+      <c r="G14" t="str">
+        <v>女主持人聲音高音域圓潤，語調溫和且富有親和力，無刺耳感，傳達溫馨陪伴感。來賓聲音清晰有力，表達流暢，具說服力。</v>
+      </c>
+      <c r="H14" t="str">
+        <v>優</v>
+      </c>
+      <c r="I14" t="str">
+        <v>無</v>
+      </c>
+      <c r="J14" t="str">
+        <v>無</v>
+      </c>
+      <c r="K14" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L14" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。</v>
+      </c>
+      <c r="M14" t="str">
+        <v>03:41 - 04:09</v>
+      </c>
+      <c r="N14" t="str">
+        <v>此段落來賓以具體案例解釋IFS核心概念，說明童年受批評如何導致內化問題並形成保護機制。語氣真摯且清晰，情感起伏自然，有助於聽眾理解複雜的心理學概念。</v>
+      </c>
+      <c r="O14" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="P14" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="R14" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="S14" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="T14" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="U14" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="V14" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="W14" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="X14" t="str">
+        <v>2026-06-20T13:16:15.224Z</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="B15" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="C15" t="str">
+        <v>郝聲音：（上）設計師KiKi，從繪畫到設計的熱愛之路，到引領他人感受設計之美的「走讀」行旅～</v>
+      </c>
+      <c r="D15">
+        <v>265</v>
+      </c>
+      <c r="E15" t="str">
+        <v>高</v>
+      </c>
+      <c r="F15" t="str">
+        <v>男主持人常在句首使用「那」和「就是」作為轉折或連接詞，頻率較高。女主持人則較常使用「嗯」、「然後」和「其實」，頻率中等，但整體而言，兩位主持人的贅字頻率偏高。</v>
+      </c>
+      <c r="G15" t="str">
+        <v>男主持人（好哥）中低音共鳴飽滿，聲音厚實且富有磁性，語調變化豐富，充滿活力。女主持人（Kiki）高音域圓潤，聲音清晰溫和，帶有親和力，語氣真誠，無刺耳感。</v>
+      </c>
+      <c r="H15" t="str">
+        <v>優</v>
+      </c>
+      <c r="I15" t="str">
+        <v>無</v>
+      </c>
+      <c r="J15" t="str">
+        <v>無</v>
+      </c>
+      <c r="K15" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L15" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，聽感舒適。</v>
+      </c>
+      <c r="M15" t="str">
+        <v>03:36 - 03:47</v>
+      </c>
+      <c r="N15" t="str">
+        <v>此段落女主持人Kiki分享她從小就對設計有著強烈的內心呼喚，語氣中透露出真誠與堅定。男主持人適時的提問與感嘆「好幸福喔」也為這段對話增添了情感深度，展現了主講人早期的志向與熱情。</v>
+      </c>
+      <c r="O15" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="P15" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="R15" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="S15" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="T15" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="U15" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="V15" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="W15" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="X15" t="str">
+        <v>2026-06-20T12:51:53.770Z</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="B16" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="C16" t="str">
+        <v>郝聲音：（上）曾格爾老師，攀登高峰，不僅是為了超越，更是讓自己能看得更遠</v>
+      </c>
+      <c r="D16">
+        <v>205</v>
+      </c>
+      <c r="E16" t="str">
+        <v>中</v>
+      </c>
+      <c r="F16" t="str">
+        <v>主講人與來賓在對話中常使用「就是」、「然後」、「對」、「這個」、「那」、「其實」、「就」等詞作為語氣詞或轉折詞。這些詞彙的出現頻率中等，雖然偶爾會打斷語句的流暢性，但整體而言不至於影響理解，且符合口語對話的自然習慣。</v>
+      </c>
+      <c r="G16" t="str">
+        <v>男主持人好哥的聲音低沉厚實，中低音共鳴感強，語調情感豐富且富有親和力，沒有機器人唸稿感。女主持人曾格爾的聲音清亮，高音域圓潤不刺耳，語氣溫暖且具陪伴感，表達清晰。</v>
+      </c>
+      <c r="H16" t="str">
+        <v>優</v>
+      </c>
+      <c r="I16" t="str">
+        <v>無</v>
+      </c>
+      <c r="J16" t="str">
+        <v>無</v>
+      </c>
+      <c r="K16" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L16" t="str">
+        <v>整體錄音品質優良，音量平穩，兩位講者的聲音清晰且平衡，沒有突兀爆音與噴麥現象，背景環境噪音極低，提供舒適的聆聽體驗。</v>
+      </c>
+      <c r="M16" t="str">
+        <v>00:00 - 00:43</v>
+      </c>
+      <c r="N16" t="str">
+        <v>主持人好哥以充滿熱情的語氣介紹曾格爾老師，並迅速點出她「行者」的身份與攀登多座高山的經歷，特別強調她挑戰的都是非一般人能及的山峰，立即吸引聽眾對這位特別來賓產生好奇與期待，為節目奠定引人入勝的基調。</v>
+      </c>
+      <c r="O16" t="str">
+        <v>登山女傑的驚人開場</v>
+      </c>
+      <c r="P16" t="str">
+        <v>00:00 - 00:43</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>主持人好哥以充滿熱情的語氣介紹曾格爾老師，並迅速點出她「行者」的身份與攀登多座高山的經歷，特別強調她挑戰的都是非一般人能及的山峰，立即吸引聽眾對這位特別來賓產生好奇與期待，為節目奠定引人入勝的基調。</v>
+      </c>
+      <c r="R16" t="str">
+        <v>聖母峰大本營的啟示：登山之路的起點</v>
+      </c>
+      <c r="S16" t="str">
+        <v>01:45 - 03:19</v>
+      </c>
+      <c r="T16" t="str">
+        <v>曾格爾老師分享她第一次攀登聖母峰大本營的艱辛與挑戰，以及這次經歷如何讓她反思物質需求，並意識到「呼吸才是唯一真正需要把握的」。這段深刻的個人體悟，是她登山生涯的關鍵轉折點，展現了她對生命與自然的獨特見解，極具啟發性。</v>
+      </c>
+      <c r="U16" t="str">
+        <v>挑戰K2的幕後辛酸與亞洲探險文化的落差</v>
+      </c>
+      <c r="V16" t="str">
+        <v>01:22:22 - 01:37:50</v>
+      </c>
+      <c r="W16" t="str">
+        <v>曾格爾老師詳細描述了她挑戰世��第二高峰K2的艱難過程，包括籌措資金、申請許可證的行政障礙，以及在極地環境中面對的歧視與文化差異。這段內容不僅展現了她堅韌的毅力，也深刻揭示了亞洲探險文化與歐美之間的巨大落差，引人深思。</v>
+      </c>
+      <c r="X16" t="str">
+        <v>2026-06-21T00:20:23.884Z</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="B17" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="C17" t="str">
+        <v>郝聲音：（下） 蘇絢慧老師好書分享，『隱性內耗』：看不見的傷，如何消磨你的能量？</v>
+      </c>
+      <c r="D17">
+        <v>205</v>
+      </c>
+      <c r="E17" t="str">
+        <v>中</v>
+      </c>
+      <c r="F17" t="str">
+        <v>主講人（徐瑄惠老師）和主持人（好哥）皆常在句首使用「然後」進行轉折，或使用「就是」、「那」等詞，頻率中等。</v>
+      </c>
+      <c r="G17" t="str">
+        <v>男主持人（好哥）聲音中低音共鳴厚實，語調情感豐富且具親和力。女主持人（徐瑄惠老師）聲音圓潤清晰，高音域不刺耳，語氣溫和具陪伴感。</v>
+      </c>
+      <c r="H17" t="str">
+        <v>優</v>
+      </c>
+      <c r="I17" t="str">
+        <v>無</v>
+      </c>
+      <c r="J17" t="str">
+        <v>無</v>
+      </c>
+      <c r="K17" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L17" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低。</v>
+      </c>
+      <c r="M17" t="str">
+        <v>01:59 - 03:45</v>
+      </c>
+      <c r="N17" t="str">
+        <v>此段落深入探討童年環境如何形塑個人對自我價值的認知，以及如何導致內耗與自我質疑。主講人語氣真摯，情感起伏自然，內容具啟發性，是理解內耗成因的關鍵點。</v>
+      </c>
+      <c r="O17" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="P17" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="R17" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="S17" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="T17" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="U17" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="V17" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="W17" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="X17" t="str">
+        <v>2026-06-20T12:53:14.710Z</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="B18" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="C18" t="str">
+        <v>郝聲音：（下）有魚的「已讀Podcast」，如何從閱讀的喜悅，成長到自媒體分享的幸福</v>
+      </c>
+      <c r="D18">
+        <v>260</v>
+      </c>
+      <c r="E18" t="str">
+        <v>中</v>
+      </c>
+      <c r="F18" t="str">
+        <v>兩位主講人皆常在句首使用「然後」作為轉折詞，頻率中等偏高。此外，「就是」也常被用於語氣的強調或解釋，而「那」則多用於話題的轉換。偶爾會出現「呃」等語氣詞。</v>
+      </c>
+      <c r="G18" t="str">
+        <v>男主持人（好哥）的聲音低沉厚實，共鳴感強，語調自然且富有情感，沒有機器人般的生硬感。女主持人（有餘）的聲音清晰明亮，語氣充滿活力與熱情，整體聽感溫暖且具陪伴感，沒有刺耳的頻率。</v>
+      </c>
+      <c r="H18" t="str">
+        <v>優</v>
+      </c>
+      <c r="I18" t="str">
+        <v>無</v>
+      </c>
+      <c r="J18" t="str">
+        <v>無</v>
+      </c>
+      <c r="K18" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L18" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。背景環境噪音極低，確保了清晰的對話內容。</v>
+      </c>
+      <c r="M18" t="str">
+        <v>00:07 - 00:24</v>
+      </c>
+      <c r="N18" t="str">
+        <v>主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
+      </c>
+      <c r="O18" t="str">
+        <v>Podcast與自媒體的開場提問</v>
+      </c>
+      <c r="P18" t="str">
+        <v>00:07 - 00:24</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
+      </c>
+      <c r="R18" t="str">
+        <v>Threads平台「內容為王」的獨特魅力</v>
+      </c>
+      <c r="S18" t="str">
+        <v>05:13 - 06:02</v>
+      </c>
+      <c r="T18" t="str">
+        <v>來賓深入分析Threads平台「內容為王」的特性，透過生動的案例（只有一個粉絲卻爆紅的貼文）說明其對素人創作者的友善與潛力，展現獨到見解，引人入勝。</v>
+      </c>
+      <c r="U18" t="str">
+        <v>知識內化與費曼學習法的實踐</v>
+      </c>
+      <c r="V18" t="str">
+        <v>19:15 - 21:11</v>
+      </c>
+      <c r="W18" t="str">
+        <v>兩位主持人探討知識分享中「引用權威」與「個人自信」的關係，並引導至費曼學習法，強調將知識內化並應用於自身問題解決的重要性，為聽眾提供實用的學習心態與方法，具啟發性。</v>
+      </c>
+      <c r="X18" t="str">
+        <v>2026-06-21T00:16:00.733Z</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="B19" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="C19" t="str">
+        <v>郝聲音：（下）郝書分享：『值得過上好日子』從情緒消費到聰明投資,克服「不夠花、不敢花」的金錢焦慮、學會建立有安心感的全方位財務計畫</v>
+      </c>
+      <c r="D19">
+        <v>290</v>
+      </c>
+      <c r="E19" t="str">
+        <v>中</v>
+      </c>
+      <c r="F19" t="str">
+        <v>兩位主持人都常在句首使用「然後」進行轉折，或以「就是」作為語氣詞。男主持人習慣性使用「你知道嗎」、「對不對」來與聽眾互動或確認語意。整體贅字頻率中等。</v>
+      </c>
+      <c r="G19" t="str">
+        <v>男主持人聲音中低音共鳴厚實，語調情感豐富，表達流暢且具說服力。女主持人聲音高音域圓潤，語氣溫馨且具陪伴感，表達清晰不刺耳。兩位聲音特質互補，提升節目親和力。</v>
+      </c>
+      <c r="H19" t="str">
+        <v>優</v>
+      </c>
+      <c r="I19" t="str">
+        <v>無</v>
+      </c>
+      <c r="J19" t="str">
+        <v>無</v>
+      </c>
+      <c r="K19" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L19" t="str">
+        <v>整體錄音品質優良，音量���穩，人聲清晰，沒有突兀爆音與噴麥現象，背景環境音極為乾淨。</v>
+      </c>
+      <c r="M19" t="str">
+        <v>00:00 - 01:15</v>
+      </c>
+      <c r="N19" t="str">
+        <v>開場主持人以「財商」與「人生」的關係破題，引導出夫妻間因價值觀差異而產生「火花」的有趣比喻，迅速吸引聽眾對節目主題產生共鳴與好奇。女主持人隨後補充的個人經驗，讓討論更具生活感。</v>
+      </c>
+      <c r="O19" t="str">
+        <v>財商與人生觀的火花</v>
+      </c>
+      <c r="P19" t="str">
+        <v>00:00 - 01:15</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>開場主持人以「財商」與「人生」的關係破題，引導出夫妻間因價值觀差異而產生「火花」的有趣比喻，迅速吸引聽眾對節目主題產生共鳴與好奇。女主持人隨後補充的個人經驗，讓討論更具生活感。</v>
+      </c>
+      <c r="R19" t="str">
+        <v>「正念」的核心：活在當下與不批判</v>
+      </c>
+      <c r="S19" t="str">
+        <v>12:42 - 14:22</v>
+      </c>
+      <c r="T19" t="str">
+        <v>此段落深入解釋了「正念」的兩大核心概念：「活在當下」與「不批判」。女主持人以清晰的邏輯闡述了這兩點對於個人成長和金錢觀念的重要性，特別強調了華人文化中常見的自我批判問題，提供了實用的覺察方法。</v>
+      </c>
+      <c r="U19" t="str">
+        <v>10個「身心安定」的練習方法</v>
+      </c>
+      <c r="V19" t="str">
+        <v>17:14 - 19:22</v>
+      </c>
+      <c r="W19" t="str">
+        <v>主持人詳細列舉並簡要說明了書中推薦的10個「身心安定」練習方法，從感官體驗（精油、水晶、音樂、泡澡）到身體活動（呼吸、運動、舞蹈）及心靈實踐（親近自然、書寫、陪伴孩子），提供了具體可行的建議，讓聽眾能���即應用於日常生活中，提升覺察力與幸福感。</v>
+      </c>
+      <c r="X19" t="str">
+        <v>2026-06-21T00:21:11.061Z</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="B20" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="C20" t="str">
+        <v>郝聲音：（下）終於跟MJ林明樟老師合體！用「財務腦」打通「業務力」，讓商業與人生獲利生生不息！</v>
+      </c>
+      <c r="D20">
+        <v>250</v>
+      </c>
+      <c r="E20" t="str">
+        <v>中</v>
+      </c>
+      <c r="F20" t="str">
+        <v>兩位主講人皆常在句首使用「那」、「然後」或「就是」作為語氣詞或轉折詞，頻率中等，但不會過於頻繁而影響聽感。</v>
+      </c>
+      <c r="G20" t="str">
+        <v>兩位男主持人聲音共鳴感佳，中低音厚實且清晰，語調自然流暢，情感表達豐富，無機器人唸稿感，整體聽感親和且具說服力。</v>
+      </c>
+      <c r="H20" t="str">
+        <v>優</v>
+      </c>
+      <c r="I20" t="str">
+        <v>無</v>
+      </c>
+      <c r="J20" t="str">
+        <v>無</v>
+      </c>
+      <c r="K20" t="str">
+        <v>環境安靜，幾乎無底噪，錄音背景非常乾淨。</v>
+      </c>
+      <c r="L20" t="str">
+        <v>整體錄音品質優良，音量平穩一致，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聆聽體���。</v>
+      </c>
+      <c r="M20" t="str">
+        <v>02:28 - 03:46</v>
+      </c>
+      <c r="N20" t="str">
+        <v>此段落由MJ老師分享個人生病導致公司薪資停發，以及離職後公司仍能良好運作的親身經歷，引導出「系統」的重要性。他以生動的語氣和具體的「1x1x1」乘法概念，深入淺出地解釋了系統運作的關鍵，情感真摯且極具說服力，是理解課程核心理念的精彩片段。</v>
+      </c>
+      <c r="O20" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="P20" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="R20" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="S20" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="T20" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="U20" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="V20" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="W20" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="X20" t="str">
+        <v>2026-06-20T12:52:38.345Z</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>精算媽咪的家計簿｜珊迪兔</v>
+      </c>
+      <c r="B21" t="str">
+        <v>精算媽咪的家計簿</v>
+      </c>
+      <c r="C21" t="str">
+        <v>#770 賺錢是為了幸福還是徒增焦慮？練習「鬆弛感」與小成就，把寶貴時間還給真正重要的事 來賓：蔡宇哲、郝旭烈</v>
+      </c>
+      <c r="D21">
+        <v>205</v>
+      </c>
+      <c r="E21" t="str">
+        <v>中</v>
+      </c>
+      <c r="F21" t="str">
+        <v>主持人Sandy常在句首使用「然後」進行轉折，偶爾使用「就是」；蔡宇哲老師和好哥也常使用「那」和「就是」作為語氣詞或連接詞，整體贅字頻率中等，不至於影響理解。</v>
+      </c>
+      <c r="G21" t="str">
+        <v>女主持人Sandy的聲音清亮、溫暖且充滿活力，高音域圓潤，給人溫馨陪伴感。男主持人蔡宇哲老師的聲音清晰、沉穩，語氣富有說服力。好哥的聲音則低沉厚實，共鳴感強，語調平穩，三位主持人的聲音特質都非常悅耳，沒有刺耳感。</v>
+      </c>
+      <c r="H21" t="str">
+        <v>優</v>
+      </c>
+      <c r="I21" t="str">
+        <v>無</v>
+      </c>
+      <c r="J21" t="str">
+        <v>無</v>
+      </c>
+      <c r="K21" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L21" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺體驗。</v>
+      </c>
+      <c r="M21" t="str">
+        <v>00:18 - 00:37</v>
+      </c>
+      <c r="N21" t="str">
+        <v>主持人Sandy以充滿活力的語氣開場，迅速點出許多人追求金錢、事業、成就背後的核心需求——安全感，並進一步提出如何獲得心靈自由的關鍵問題，有效吸引聽眾進入主題。</v>
+      </c>
+      <c r="O21" t="str">
+        <v>追求安全感與心靈自由的開場</v>
+      </c>
+      <c r="P21" t="str">
+        <v>00:18 - 00:37</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>主持人Sandy以充滿活力的語氣開場，迅速點出許多人追求金錢、事業、成就背後的核心需求——安全感，並進一步提出如何獲得心靈自由的關鍵問題，有效吸引聽眾進入主題。</v>
+      </c>
+      <c r="R21" t="str">
+        <v>財富自由的真諦：幸福與意義</v>
+      </c>
+      <c r="S21" t="str">
+        <v>01:22 - 01:43</v>
+      </c>
+      <c r="T21" t="str">
+        <v>蔡宇哲老師在此段落深刻剖析財富自由的真正目的，指出金錢最終是為了帶來幸福、快樂與意義，並反思這些是否必須依賴大量金錢才能實現，提供聽眾一個重新思考財富觀的機會。</v>
+      </c>
+      <c r="U21" t="str">
+        <v>累積小成就，戰勝焦慮</v>
+      </c>
+      <c r="V21" t="str">
+        <v>07:45 - 08:20</v>
+      </c>
+      <c r="W21" t="str">
+        <v>好哥與蔡宇哲老師共同探討透過累積小成就來建立自信、戰勝焦慮的實用方法，特別提到「兩分鐘目標」的概念，為聽眾提供了具體且可操作的建議，展現了節目的實用價值和情感連結。</v>
+      </c>
+      <c r="X21" t="str">
+        <v>2026-06-21T00:31:11.293Z</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>精算媽咪的家計簿｜珊迪兔</v>
+      </c>
+      <c r="B22" t="str">
+        <v>精算媽咪的家計簿</v>
+      </c>
+      <c r="C22" t="str">
+        <v>#800 買老屋怕踩雷？破解中古屋隱藏價值，聰明挑出高CP值潛力好房！來賓：House123 執行長 邱愛莉 Ellie</v>
+      </c>
+      <c r="D22">
+        <v>205</v>
+      </c>
+      <c r="E22" t="str">
+        <v>中</v>
+      </c>
+      <c r="F22" t="str">
+        <v>兩位主持人皆有使用「然後」、「就是」、「對啊」、「其實」等口頭禪，尤其在句首作為轉折詞的頻率較高，但整體而言不至於過度影響聽感。</v>
+      </c>
+      <c r="G22" t="str">
+        <v>兩位女主持人的聲音皆清晰、圓潤，高音域表現良好，沒有刺耳感。主講人Sandy的語調活潑，具親和力與溫馨陪伴感；來賓Aily的聲音則顯得沉穩專業，共鳴感佳，兩者搭配使對話流暢且富有層次。</v>
+      </c>
+      <c r="H22" t="str">
+        <v>優</v>
+      </c>
+      <c r="I22" t="str">
+        <v>無</v>
+      </c>
+      <c r="J22" t="str">
+        <v>無</v>
+      </c>
+      <c r="K22" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L22" t="str">
+        <v>整體錄音品質優良，音量平穩，���聲清晰，沒有突兀爆音與噴麥現象，背景環境噪音也控制得很好。</v>
+      </c>
+      <c r="M22" t="str">
+        <v>00:49 - 01:14</v>
+      </c>
+      <c r="N22" t="str">
+        <v>主持人Sandy以生動的語氣，點出許多人在買房時既期待又害怕受傷害的普遍心態，特別是對於首次購屋者。她簡潔地帶出新舊房子的優缺點，迅速抓住聽眾的注意力，為後續的討論奠定基礎。</v>
+      </c>
+      <c r="O22" t="str">
+        <v>買房的期待與困境</v>
+      </c>
+      <c r="P22" t="str">
+        <v>00:49 - 01:14</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>主持人Sandy以生動的語氣，點出許多人在買房時既期待又害怕受傷害的普遍心態，特別是對於首次購屋者。她簡潔地帶出新舊房子的優缺點，迅速抓住聽眾的注意力，為後續的討論奠定基礎。</v>
+      </c>
+      <c r="R22" t="str">
+        <v>房屋結構的致命傷：軟弱層與海砂屋</v>
+      </c>
+      <c r="S22" t="str">
+        <v>05:56 - 07:29</v>
+      </c>
+      <c r="T22" t="str">
+        <v>來賓Aily在此段落深入淺出地解釋了老屋最關鍵的結構性問題，包括「軟弱層」和「海砂屋」。她強調這些問題的不可逆性，並指出結構安全是購屋時首要考量的因素，提供了極具價值的專業知識，語氣真摯且具說服力。</v>
+      </c>
+      <c r="U22" t="str">
+        <v>投資老屋的退場機制與風險評估</v>
+      </c>
+      <c r="V22" t="str">
+        <v>19:00 - 19:59</v>
+      </c>
+      <c r="W22" t="str">
+        <v>Aily在此段落從投資角度切入，強調了老屋投資必須具備「退場機制」的重要性。她提醒聽眾不應只依賴都更，而應考慮其他可能的退出方案，例如出租或轉售，為投資者提供了務實且全面的風險評估建議。</v>
+      </c>
+      <c r="X22" t="str">
+        <v>2026-06-21T00:33:54.344Z</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>精算媽咪的家計簿｜珊迪兔</v>
+      </c>
+      <c r="B23" t="str">
+        <v>精算媽咪的家計簿</v>
+      </c>
+      <c r="C23" t="str">
+        <v>#805 總在爛工作與錯的感情中輪迴？看懂隱藏的人生劇本，用「自我覺察」找回選擇權！來賓：千里淳風</v>
+      </c>
+      <c r="D23">
+        <v>250</v>
+      </c>
+      <c r="E23" t="str">
+        <v>中</v>
+      </c>
+      <c r="F23" t="str">
+        <v>主講人（Cindy）常使用「然後」、「就是」、「對」、「嗯」作為語氣詞或轉折詞。來賓（錢老師）則常使用「其實」、「就是」、「那」、「對」、「嗯」。兩位講者的贅字頻率皆為中等，但語句流暢度不受影響。</v>
+      </c>
+      <c r="G23" t="str">
+        <v>主講人（Cindy）的聲音高音域圓潤，語調活潑，富有溫馨陪伴感，聽起來清晰且不刺耳。來賓（錢老師）的聲音中低音共鳴強，厚實且沉穩，語氣充滿智慧與說服力。</v>
+      </c>
+      <c r="H23" t="str">
+        <v>優</v>
+      </c>
+      <c r="I23" t="str">
+        <v>無</v>
+      </c>
+      <c r="J23" t="str">
+        <v>無</v>
+      </c>
+      <c r="K23" t="str">
+        <v>環境安靜，幾乎無底噪，錄音品質極佳。</v>
+      </c>
+      <c r="L23" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。兩位講者的聲音清晰，背景噪音極低，提供極佳的聽覺體驗。</v>
+      </c>
+      <c r="M23" t="str">
+        <v>00:50 - 01:14</v>
+      </c>
+      <c r="N23" t="str">
+        <v>此片段是節目開場的精華，主持人以引人入勝的方式介紹來賓，點出他從講求邏輯與科技的背景，轉變為鑽研命理的獨特經歷。這不僅迅速抓住聽眾的好奇心，也為後續的深度對談奠定基礎，展現了主持人良好的引導能力和來賓故事的吸引力。</v>
+      </c>
+      <c r="O23" t="str">
+        <v>引人入勝的開場：從科技到命理</v>
+      </c>
+      <c r="P23" t="str">
+        <v>00:50 - 01:14</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>此片段是節目開場的精華，主持人以引人入勝的方式介紹來賓，點出他從講求邏輯與科技的背景，轉變為鑽研命理的獨特經歷。這不僅迅速抓住聽眾的好奇心，也為後續的深度對談奠定基礎，展現了主持人良好的引導能力和來賓故事的吸引力。</v>
+      </c>
+      <c r="R23" t="str">
+        <v>改變命運的關鍵：自我覺察與觀察者</v>
+      </c>
+      <c r="S23" t="str">
+        <v>07:49 - 09:11</v>
+      </c>
+      <c r="T23" t="str">
+        <v>此片段深入探討了改變命運的核心觀念——「自我覺察」與「觀察者自我」。來賓以心理學理論結合生活實例（如開車自動駕駛），清晰解釋了人類意識的三個層次，並指出大多數人命運被預設的原因。這段內容不僅具啟發性，也提供了聽眾實際可操作的思維工具，是節目中極具深度和實用價值的論述。</v>
+      </c>
+      <c r="U23" t="str">
+        <v>意想不到的改運工具：衣服與食物</v>
+      </c>
+      <c r="V23" t="str">
+        <v>20:31 - 21:37</v>
+      </c>
+      <c r="W23" t="str">
+        <v>���片段揭示了兩個最有效且日常的改運工具：衣服和食物。來賓從色彩心理學和五行理論的角度，解釋了這些看似平凡的元素如何直接影響一個人的情緒、能量和運勢。這段內容不僅顛覆了傳統對改運的想像，也提供了具體且易於實踐的方法，讓聽眾能從生活中著手改變，極具趣味性和實用性。</v>
+      </c>
+      <c r="X23" t="str">
+        <v>2026-06-21T00:33:00.044Z</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>蕭邦</v>
+      </c>
+      <c r="B24" t="str">
+        <v>蕭邦相談室</v>
+      </c>
+      <c r="C24" t="str">
+        <v>如何度過負面情緒 ？</v>
+      </c>
+      <c r="D24">
+        <v>205</v>
+      </c>
+      <c r="E24" t="str">
+        <v>中</v>
+      </c>
+      <c r="F24" t="str">
+        <v>主講人常在句首使用「那」作為轉折詞，頻率較高，但多數時候作為語氣連接而非純粹贅字。此外，「就是」和「然後」偶爾出現，整體贅字頻率屬於中等。</v>
+      </c>
+      <c r="G24" t="str">
+        <v>女主持人聲音溫暖、圓潤，中低音域表現穩定，高音域不刺耳，整體語調富有情感，給人一種溫馨且具陪伴感的聽覺體驗。</v>
+      </c>
+      <c r="H24" t="str">
+        <v>優</v>
+      </c>
+      <c r="I24" t="str">
+        <v>無</v>
+      </c>
+      <c r="J24" t="str">
+        <v>無</v>
+      </c>
+      <c r="K24" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L24" t="str">
+        <v>整體錄音品質極佳，音量平穩，人聲清晰，沒有任何噴麥、突兀爆音或背景雜音，聽感非常舒���。</v>
+      </c>
+      <c r="M24" t="str">
+        <v>00:12 - 00:31</v>
+      </c>
+      <c r="N24" t="str">
+        <v>主持人以自身經歷引出「情緒」這個主題，語氣真誠，迅速建立與聽眾的連結，引人入勝，為節目內容做了很好的鋪墊。</v>
+      </c>
+      <c r="O24" t="str">
+        <v>開場：情緒的引導與個人經驗分享</v>
+      </c>
+      <c r="P24" t="str">
+        <v>00:12 - 00:31</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>主持人以自身經歷引出「情緒」這個主題，語氣真誠，迅速建立與聽眾的連結，引人入勝，為節目內容做了很好的鋪墊。</v>
+      </c>
+      <c r="R24" t="str">
+        <v>核心論述：關閉腦袋，讓情緒流動</v>
+      </c>
+      <c r="S24" t="str">
+        <v>04:05 - 04:55</v>
+      </c>
+      <c r="T24" t="str">
+        <v>此段落是節目的核心精華，主持人清晰地闡述了處理情緒的關鍵方法——「關閉腦袋，讓情緒自然流動」，並解釋了其背後的原因，提供了具體且實用的建議，極具啟發性。</v>
+      </c>
+      <c r="U24" t="str">
+        <v>總結：接受情緒，有效解決問題</v>
+      </c>
+      <c r="V24" t="str">
+        <v>05:43 - 06:10</v>
+      </c>
+      <c r="W24" t="str">
+        <v>這段總結了節目主旨，強調接受所有情緒的重要性及其帶來的益處，語氣溫和且具說服力，為聽眾提供正向的啟發，並引導聽眾思考如何有效解決問題。</v>
+      </c>
+      <c r="X24" t="str">
+        <v>2026-06-21T00:40:44.043Z</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:X24"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete 36-episode voice evaluation trial run, separate HTML dashboard tabs and add script robustness
</commit_message>
<xml_diff>
--- a/eligible_episodes_pool.xlsx
+++ b/eligible_episodes_pool.xlsx
@@ -57808,7 +57808,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X24"/>
+  <dimension ref="A1:X37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -58626,25 +58626,25 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="B12" t="str">
-        <v>哇賽心理學</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="C12" t="str">
-        <v>多巴胺陷阱！戒不掉的不是癮，是深層的焦慮ft.蘇琮祺心理師｜哇賽心觀點ep193</v>
+        <v>EP462｜從半導體科技業叛逃到瓜地馬拉咖啡莊園！ft. 《 吳朵兒的咖啡桌 》Eleanor</v>
       </c>
       <c r="D12">
-        <v>195</v>
+        <v>280</v>
       </c>
       <c r="E12" t="str">
-        <v>中</v>
+        <v>高</v>
       </c>
       <c r="F12" t="str">
-        <v>主講人常在句首使用「然後」和「那」作為轉折詞，頻率中等，但整體對話流暢度不受影響。</v>
+        <v>主講人與來賓在對話中頻繁使用「然後」作為語句連接詞或轉折詞，且「就是」的出現頻率也偏高，整體贅字頻率高。</v>
       </c>
       <c r="G12" t="str">
-        <v>男主持人（宇澤）聲音溫暖、清晰，中低音共鳴感強，語調自然且富有情感，沒有機器人唸稿感。來賓（蘇崇其）的聲音也專業且清晰，兩位主持人的聲音都具親和力，無刺耳感。</v>
+        <v>兩位女主持人的聲音皆清晰、圓潤，高音域表現良好，語調溫暖且富有親和力，給人一種溫馨陪伴感，沒有刺耳的感覺。</v>
       </c>
       <c r="H12" t="str">
         <v>優</v>
@@ -58659,66 +58659,66 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L12" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺體驗���</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景環境音處理得當。</v>
       </c>
       <c r="M12" t="str">
-        <v>02:07 - 03:49</v>
+        <v>00:33 - 01:10</v>
       </c>
       <c r="N12" t="str">
-        <v>此段落深入探討了「食物成癮」與「進食成癮」的區別，並進一步闡述了成癮與壞習慣之間的模糊界線，是節目核心概念的精彩呈現。主講人與來賓的對話充滿洞察力，語氣真摯且音調波動起伏有致，極具聲音說服力。</v>
+        <v>不姐的開場溫暖且引人入勝，隨後Eleanor分享了她畢業後第一份高薪卻不快樂的半導體工作，以及她對這份工作的極度抗拒，甚至希望發生小車禍來逃避上班，這份真誠的告白為後續的轉型故事埋下伏筆，迅速抓住聽眾注意力。</v>
       </c>
       <c r="O12" t="str">
-        <v>N/A</v>
+        <v>高薪卻不快樂的職涯開端</v>
       </c>
       <c r="P12" t="str">
-        <v>N/A</v>
+        <v>00:33 - 01:10</v>
       </c>
       <c r="Q12" t="str">
-        <v>N/A</v>
+        <v>不姐的開場溫暖且引人入勝，隨後Eleanor分享了她畢業後第一份高薪卻不快樂的半導體工作，以及她對這份工作的極度抗拒，甚至希望發生小車禍來逃避上班，這份真誠的告白為後續的轉型故事埋下伏筆，迅速抓住聽眾注意力。</v>
       </c>
       <c r="R12" t="str">
-        <v>N/A</v>
+        <v>職涯轉捩點：從抗拒到尋找熱情</v>
       </c>
       <c r="S12" t="str">
-        <v>N/A</v>
+        <v>08:50 - 09:53</v>
       </c>
       <c r="T12" t="str">
-        <v>N/A</v>
+        <v>Eleanor生動描述了她在半導體業的掙扎與不適，包括長時間工作、應酬文化，以及她內心深處的抗拒。她隨後提出的「如果有一份工作可以做到老，那會是什麼？」這個問題，是她職涯轉型的核心，極具啟發性，展現了情感深度與自我反思的過程。</v>
       </c>
       <c r="U12" t="str">
-        <v>N/A</v>
+        <v>吸引力法則：追隨熱情的信念</v>
       </c>
       <c r="V12" t="str">
-        <v>N/A</v>
+        <v>14:51 - 15:03</v>
       </c>
       <c r="W12" t="str">
-        <v>N/A</v>
+        <v>Eleanor分享了她對「吸引力法則」的堅定信念，即使前路不明，她仍憑藉著對咖啡的熱情持續投入，展現了追逐夢想的勇氣與決心，這份純粹的相信極具感染力，為聽眾帶來正向的啟發。</v>
       </c>
       <c r="X12" t="str">
-        <v>2026-06-20T13:15:23.756Z</v>
+        <v>2026-06-21T01:44:18.331Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="B13" t="str">
-        <v>哇賽心理學</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="C13" t="str">
-        <v>掌握你的金錢性格，打造幸福家庭理財ft.精算媽咪珊迪兔｜哇賽心觀點ep194</v>
+        <v>EP467｜去電商物流搬一天貨，保證你瞬間學會感恩！！ feat. 《 百工計劃 》藍白拖</v>
       </c>
       <c r="D13">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="E13" t="str">
         <v>中</v>
       </c>
       <c r="F13" t="str">
-        <v>主講人與來賓皆有使用「就是」、「其實」作為語氣詞或轉折詞，來賓常使用「然後」連接語句，但整體頻率尚可接受，不致影響聽感。</v>
+        <v>男主持人常在句首使用「然後」、「那」進行轉折，並頻繁使用「就是」來解釋或強調，以及「對」來表示同意或確認。女主持人則較常使用「嗯」、「對」來回應。整體而言，贅字頻率中等，主要集中在男主持人的口語習慣。</v>
       </c>
       <c r="G13" t="str">
-        <v>男主持人聲音低沉厚實，共鳴感佳，語調變化自然，富有親和力。女主持人聲音清晰明亮，高音域圓潤不刺耳，帶有溫馨陪伴感，表達流暢。</v>
+        <v>男主持人（藍白拖）的聲音中低音共鳴與厚實度佳，語調自然且情感表達豐富，沒有機器人唸稿感，聽感親和力強。女主持人（布姐）的聲音高音域圓潤，語氣溫和，具備溫馨陪伴感，無刺耳感。兩位主持人的聲音特質都為節目增添了吸引力。</v>
       </c>
       <c r="H13" t="str">
         <v>優</v>
@@ -58733,66 +58733,66 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L13" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺���驗。</v>
+        <v>整體錄音品質優良，音量平穩，兩位主持人的聲音平衡良好，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聆聽體驗。</v>
       </c>
       <c r="M13" t="str">
-        <v>02:07 - 03:44</v>
+        <v>00:33 - 01:10</v>
       </c>
       <c r="N13" t="str">
-        <v>此段落來賓生動地分享了原生家庭中父母截然不同的金錢觀（父親的創業擴張與母親的節儉務實），以及這些經歷如何塑造了她個人的金錢觀。她真誠地反思了「好」與「不好」的定義，並強調找到自己最舒適的理財方式，內容具深度且引人共鳴，情感表達豐富，是極具說服力的黃金聽點。</v>
+        <v>女主持人開場介紹節目與來賓，隨後男主持人「藍白拖」清晰闡述其「百工計畫」的發想與核心目的，即透過體驗人生百態來探索生命意義，為本集內容奠定引人入勝的基調。</v>
       </c>
       <c r="O13" t="str">
-        <v>N/A</v>
+        <v>「百工計畫」的緣起與目的</v>
       </c>
       <c r="P13" t="str">
-        <v>N/A</v>
+        <v>00:33 - 01:10</v>
       </c>
       <c r="Q13" t="str">
-        <v>N/A</v>
+        <v>女主持人開場介紹節目與來賓，隨後男主持人「藍白拖」清晰闡述其「百工計畫」的發想與核心目的，即透過體驗人生百態來探索生命意義，為本集內容奠定引人入勝的基調。</v>
       </c>
       <c r="R13" t="str">
-        <v>N/A</v>
+        <v>環境與身心靈狀態的深層連結</v>
       </c>
       <c r="S13" t="str">
-        <v>N/A</v>
+        <v>02:30 - 03:10</v>
       </c>
       <c r="T13" t="str">
-        <v>N/A</v>
+        <v>男主持人深入探討環境狀態如何直接影響一個人的身心靈，強調在髒亂、潮濕的環境中難以維持良好的情緒與身體狀態，揭示了外在環境與內在感受間的深刻互動，引發聽眾對自身生活環境的反思。</v>
       </c>
       <c r="U13" t="str">
-        <v>N/A</v>
+        <v>總裁外送員：放下身段的行為治療</v>
       </c>
       <c r="V13" t="str">
-        <v>N/A</v>
+        <v>16:04 - 17:08</v>
       </c>
       <c r="W13" t="str">
-        <v>N/A</v>
+        <v>男主持人分享一個信用卡總裁因心理諮詢師建議而去做外送員的案例。這個故事生動地說明了透過實際��驗「底層」工作，如何面對內心的歧視與心魔，達到行為治療的效果，展現了放下身段、重新認識自我的強大力量。</v>
       </c>
       <c r="X13" t="str">
-        <v>2026-06-20T13:14:32.297Z</v>
+        <v>2026-06-21T01:43:16.230Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="B14" t="str">
-        <v>哇賽心理學</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="C14" t="str">
-        <v>療癒創傷，溫柔擁抱完整的自己ft.留佩萱博士｜哇賽療心室ep148</v>
+        <v>EP.588 《心轉，病自癒》專訪作者：蔡松彥醫師帶給我的 7 個啟發</v>
       </c>
       <c r="D14">
-        <v>260</v>
+        <v>205</v>
       </c>
       <c r="E14" t="str">
         <v>中</v>
       </c>
       <c r="F14" t="str">
-        <v>主講人與來賓皆常使用「就是」、「那」、「其實」等口頭禪，其中「就是」的出現頻率高，整體贅字頻率中等。</v>
+        <v>主持人與來賓在句首常使用「那」、「然後」、「所以」作為語氣詞或轉折詞，頻率中等。</v>
       </c>
       <c r="G14" t="str">
-        <v>女主持人聲音高音域圓潤，語調溫和且富有親和力，無刺耳感，傳達溫馨陪伴感。來賓聲音清晰有力，表達流暢，具說服力。</v>
+        <v>男主持人瓦基的聲音中低音共鳴厚實，語調清晰且富有情感，具備良好的親和力，無機器人唸稿感。</v>
       </c>
       <c r="H14" t="str">
         <v>優</v>
@@ -58807,66 +58807,66 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L14" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景環境音處理得很好。</v>
       </c>
       <c r="M14" t="str">
-        <v>03:41 - 04:09</v>
+        <v>00:14 - 00:26</v>
       </c>
       <c r="N14" t="str">
-        <v>此段落來賓以具體案例解釋IFS核心概念，說明童年受批評如何導致內化問題並形成保護機制。語氣真摯且清晰，情感起伏自然，有助於聽眾理解複雜的心理學概念。</v>
+        <v>主持人以一個引人深思的問題開場，迅速帶出本集主題書《心轉病自癒》，語速節奏掌握得宜，成功吸引聽眾注意力。</v>
       </c>
       <c r="O14" t="str">
-        <v>N/A</v>
+        <v>破題精采開場</v>
       </c>
       <c r="P14" t="str">
-        <v>N/A</v>
+        <v>00:14 - 00:26</v>
       </c>
       <c r="Q14" t="str">
-        <v>N/A</v>
+        <v>主持人以一個引人深思的問題開場，迅速帶出本集主題書《心轉病自癒》，語速節奏掌握得宜，成功吸引聽眾注意力。</v>
       </c>
       <c r="R14" t="str">
-        <v>N/A</v>
+        <v>醫師自診癌症與主流醫學的信任</v>
       </c>
       <c r="S14" t="str">
-        <v>N/A</v>
+        <v>04:18 - 04:56</v>
       </c>
       <c r="T14" t="str">
-        <v>N/A</v>
+        <v>蔡醫師親述自己如何發現並診斷出癌症，以及他對主流醫學的堅定信任，甚至在短時間內完成手術，展現其專業背景與個人經歷的衝突。</v>
       </c>
       <c r="U14" t="str">
-        <v>N/A</v>
+        <v>主流醫學的極限與轉向整合醫療</v>
       </c>
       <c r="V14" t="str">
-        <v>N/A</v>
+        <v>06:15 - 07:05</v>
       </c>
       <c r="W14" t="str">
-        <v>N/A</v>
+        <v>蔡醫師坦誠在癌症復發後，意識到主流醫學的局限，進而轉向整合醫療領域，並親身實踐，這段心路歷程是其「心轉」理論的關鍵轉折。</v>
       </c>
       <c r="X14" t="str">
-        <v>2026-06-20T13:16:15.224Z</v>
+        <v>2026-06-21T01:51:20.317Z</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="B15" t="str">
-        <v>郝聲音</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="C15" t="str">
-        <v>郝聲音：（上）設計師KiKi，從繪畫到設計的熱愛之路，到引領他人感受設計之美的「走讀」行旅～</v>
+        <v>EP.591 《財富自由心理學》專訪作者：破解財富焦慮的 6 個洞察</v>
       </c>
       <c r="D15">
-        <v>265</v>
+        <v>210</v>
       </c>
       <c r="E15" t="str">
-        <v>高</v>
+        <v>中</v>
       </c>
       <c r="F15" t="str">
-        <v>男主持人常在句首使用「那」和「就是」作為轉折或連接詞，頻率較高。女主持人則較常使用「嗯」、「然後」和「其實」，頻率中等，但整體而言，兩位主持人的贅字頻率偏高。</v>
+        <v>常在句首使用「然後」進行轉折，也常出現「就是」、「那」、「對不對」等口頭禪，頻率中等。</v>
       </c>
       <c r="G15" t="str">
-        <v>男主持人（好哥）中低音共鳴飽滿，聲音厚實且富有磁性，語調變化豐富，充滿活力。女主持人（Kiki）高音域圓潤，聲音清晰溫和，帶有親和力，語氣真誠，無刺耳感。</v>
+        <v>兩位主講人聲音皆具親和力。瓦基老師語調清晰、富有活力；好哥老師聲音低沉厚實，共鳴感強，語氣情感豐富，無刺耳感。</v>
       </c>
       <c r="H15" t="str">
         <v>優</v>
@@ -58878,69 +58878,69 @@
         <v>無</v>
       </c>
       <c r="K15" t="str">
-        <v>環境安靜，幾乎無底噪</v>
+        <v>無</v>
       </c>
       <c r="L15" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，聽感舒適。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音、噴麥或明顯背景雜音。</v>
       </c>
       <c r="M15" t="str">
-        <v>03:36 - 03:47</v>
+        <v>00:00 - 00:05</v>
       </c>
       <c r="N15" t="str">
-        <v>此段落女主持人Kiki分享她從小就對設計有著強烈的內心呼喚，語氣中透露出真誠與堅定。男主持人適時的提問與感嘆「好幸福喔」也為這段對話增添了情感深度，展現了主講人早期的志向與熱情。</v>
+        <v>主持人瓦基以親切的語氣簡潔介紹節目，語速適中，迅速吸引聽眾進入節目氛圍。</v>
       </c>
       <c r="O15" t="str">
-        <v>N/A</v>
+        <v>節目開場</v>
       </c>
       <c r="P15" t="str">
-        <v>N/A</v>
+        <v>00:00 - 00:05</v>
       </c>
       <c r="Q15" t="str">
-        <v>N/A</v>
+        <v>主持人瓦基以親切的語氣簡潔介紹節目，語速適中，迅速吸引聽眾進入節目氛圍。</v>
       </c>
       <c r="R15" t="str">
-        <v>N/A</v>
+        <v>《財富自由心理學》書名由來與合作契機</v>
       </c>
       <c r="S15" t="str">
-        <v>N/A</v>
+        <v>02:58 - 04:20</v>
       </c>
       <c r="T15" t="str">
-        <v>N/A</v>
+        <v>好哥生動地講述了與蔡宇哲老師合作的緣起，以及書名「財富自由心理學」的誕生過程，展現了兩位講者之間的有趣互動與思維碰撞，引人入勝。</v>
       </c>
       <c r="U15" t="str">
-        <v>N/A</v>
+        <v>自由的公式：能力減去慾望</v>
       </c>
       <c r="V15" t="str">
-        <v>N/A</v>
+        <v>09:57 - 10:23</v>
       </c>
       <c r="W15" t="str">
-        <v>N/A</v>
+        <v>好哥提出了「自由 = 能力 - 慾望」的公式，並用具體例子解釋，讓抽象的自由概念變得具體可行，這段內容對於理解財富自由的核心精神非常關鍵且實用。</v>
       </c>
       <c r="X15" t="str">
-        <v>2026-06-20T12:51:53.770Z</v>
+        <v>2026-06-21T01:48:18.477Z</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="B16" t="str">
-        <v>郝聲音</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="C16" t="str">
-        <v>郝聲音：（上）曾格爾老師，攀登高峰，不僅是為了超越，更是讓自己能看得更遠</v>
+        <v>EP.594 《指數流小白課程》美股航海王：告別每天盯盤的指數投資法</v>
       </c>
       <c r="D16">
-        <v>205</v>
+        <v>310</v>
       </c>
       <c r="E16" t="str">
         <v>中</v>
       </c>
       <c r="F16" t="str">
-        <v>主講人與來賓在對話中常使用「就是」、「然後」、「對」、「這個」、「那」、「其實」、「就」等詞作為語氣詞或轉折詞。這些詞彙的出現頻率中等，雖然偶爾會打斷語句的流暢性，但整體而言不至於影響理解，且符合口語對話的自然習慣。</v>
+        <v>主講人（美股航海王）和主持人（瓦基）在對話中常使用「然後」、「就是」、「那」作為語句的連接詞或思考間的填充詞，頻率中等，但未明顯影響內容的流暢度。</v>
       </c>
       <c r="G16" t="str">
-        <v>男主持人好哥的聲音低沉厚實，中低音共鳴感強，語調情感豐富且富有親和力，沒有機器人唸稿感。女主持人曾格爾的聲音清亮，高音域圓潤不刺耳，語氣溫暖且具陪伴感，表達清晰。</v>
+        <v>主講人（美股航海王）的聲音低沉厚實，共鳴感強，語氣自信且富有感染力。主持人（瓦基）的聲音則較為明亮清晰，兩者搭配使節目聽感豐富且專業，均無刺耳感。</v>
       </c>
       <c r="H16" t="str">
         <v>優</v>
@@ -58955,66 +58955,66 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L16" t="str">
-        <v>整體錄音品質優良，音量平穩，兩位講者的聲音清晰且平衡，沒有突兀爆音與噴麥現象，背景環境噪音極低，提供舒適的聆聽體驗。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀���音與噴麥現象，背景環境噪音極低，對話清晰。</v>
       </c>
       <c r="M16" t="str">
-        <v>00:00 - 00:43</v>
+        <v>00:14 - 00:31</v>
       </c>
       <c r="N16" t="str">
-        <v>主持人好哥以充滿熱情的語氣介紹曾格爾老師，並迅速點出她「行者」的身份與攀登多座高山的經歷，特別強調她挑戰的都是非一般人能及的山峰，立即吸引聽眾對這位特別來賓產生好奇與期待，為節目奠定引人入勝的基調。</v>
+        <v>主持人瓦基精準點出小資族在投資美股時常遇到的困惑與焦慮，例如資金有限、追高殺跌的風險，並預告本集將提供解決方案，引人入勝，是極佳的開場引導。</v>
       </c>
       <c r="O16" t="str">
-        <v>登山女傑的驚人開場</v>
+        <v>小資族投資困惑的破題</v>
       </c>
       <c r="P16" t="str">
-        <v>00:00 - 00:43</v>
+        <v>00:14 - 00:31</v>
       </c>
       <c r="Q16" t="str">
-        <v>主持人好哥以充滿熱情的語氣介紹曾格爾老師，並迅速點出她「行者」的身份與攀登多座高山的經歷，特別強調她挑戰的都是非一般人能及的山峰，立即吸引聽眾對這位特別來賓產生好奇與期待，為節目奠定引人入勝的基調。</v>
+        <v>主持人瓦基精準點出小資族在投資美股時常遇到的困惑與焦慮，例如資金有限、追高殺跌的風險，並預告本集將提供解決方案，引人入勝，是極佳的開場引導。</v>
       </c>
       <c r="R16" t="str">
-        <v>聖母峰大本營的啟示：登山之路的起點</v>
+        <v>從慘痛教訓到指數投資的轉變</v>
       </c>
       <c r="S16" t="str">
-        <v>01:45 - 03:19</v>
+        <v>04:47 - 06:04</v>
       </c>
       <c r="T16" t="str">
-        <v>曾格爾老師分享她第一次攀登聖母峰大本營的艱辛與挑戰，以及這次經歷如何讓她反思物質需求，並意識到「呼吸才是唯一真正需要把握的」。這段深刻的個人體悟，是她登山生涯的關鍵轉折點，展現了她對生命與自然的獨特見解，極具啟發性。</v>
+        <v>美股航海王分享了自己從早期成功到因一次股災幾乎賠光所有積蓄的慘痛經歷，這段個人故事極具感染力，並解釋了為何他最終放棄個股操作，轉向指數投資，是其核心理念的關鍵轉捩點。</v>
       </c>
       <c r="U16" t="str">
-        <v>挑戰K2的幕後辛酸與亞洲探險文化的落差</v>
+        <v>美股市場的宏觀優勢與政治避險</v>
       </c>
       <c r="V16" t="str">
-        <v>01:22:22 - 01:37:50</v>
+        <v>15:24 - 16:21</v>
       </c>
       <c r="W16" t="str">
-        <v>曾格爾老師詳細描述了她挑戰世��第二高峰K2的艱難過程，包括籌措資金、申請許可證的行政障礙，以及在極地環境中面對的歧視與文化差異。這段內容不僅展現了她堅韌的毅力，也深刻揭示了亞洲探險文化與歐美之間的巨大落差，引人深思。</v>
+        <v>航海王深入分析了美股相較於台股在市場深度、公平性以及政治避險上的優勢，特別提到台灣市場的淺碟性與單一產業集中風險，以及美股在面對地緣政治風險時的韌性，提供了宏觀且具說服力的投資視角。</v>
       </c>
       <c r="X16" t="str">
-        <v>2026-06-21T00:20:23.884Z</v>
+        <v>2026-06-21T01:52:13.519Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
       </c>
       <c r="B17" t="str">
-        <v>郝聲音</v>
+        <v>能量黑客</v>
       </c>
       <c r="C17" t="str">
-        <v>郝聲音：（下） 蘇絢慧老師好書分享，『隱性內耗』：看不見的傷，如何消磨你的能量？</v>
+        <v>內耗怎麼停？先抽離，再復盤：把情緒變成行動｜能量黑客S2EP9</v>
       </c>
       <c r="D17">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="E17" t="str">
         <v>中</v>
       </c>
       <c r="F17" t="str">
-        <v>主講人（徐瑄惠老師）和主持人（好哥）皆常在句首使用「然後」進行轉折，或使用「就是」、「那」等詞，頻率中等。</v>
+        <v>兩位主持人在對話中頻繁使用「就是」作為解釋或強調，以及「然後」作為語句轉折，頻率中等。偶爾會出現「呃」等語氣詞。</v>
       </c>
       <c r="G17" t="str">
-        <v>男主持人（好哥）聲音中低音共鳴厚實，語調情感豐富且具親和力。女主持人（徐瑄惠老師）聲音圓潤清晰，高音域不刺耳，語氣溫和具陪伴感。</v>
+        <v>男主持人（Hank）的聲音中低音共鳴強烈，厚實且富有磁性，語調沉穩而具親和力，沒有機器人唸稿感。女主持人（Betty）的聲音高音域圓潤清晰，語氣活潑，雖然語速較快，但整體聽感溫暖且具陪伴感，沒有刺耳現象。</v>
       </c>
       <c r="H17" t="str">
         <v>優</v>
@@ -59029,66 +59029,66 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L17" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺體驗。</v>
       </c>
       <c r="M17" t="str">
-        <v>01:59 - 03:45</v>
+        <v>00:00 - 00:30</v>
       </c>
       <c r="N17" t="str">
-        <v>此段落深入探討童年環境如何形塑個人對自我價值的認知，以及如何導致內耗與自我質疑。主講人語氣真摯，情感起伏自然，內容具啟發性，是理解內耗成因的關鍵點。</v>
+        <v>這段是節目的標準開場，由兩位主持人輪流介紹節目理念。Hank大叔以「在忙碌生活中，有餘力去做快樂的事，並在重要時刻拿出最好的狀態」點出節目核心，Betty則補充「能量不只是體力，還包含專注力、情緒狀態」，並承諾用實用方法與幽默幫助聽眾找到高能量節奏。語速雖快，但清晰有力，有效傳達節目主旨，迅速抓住聽眾注意力。</v>
       </c>
       <c r="O17" t="str">
-        <v>N/A</v>
+        <v>能量駭客的開場白與節目宗旨</v>
       </c>
       <c r="P17" t="str">
-        <v>N/A</v>
+        <v>00:00 - 00:30</v>
       </c>
       <c r="Q17" t="str">
-        <v>N/A</v>
+        <v>這段是節目的標準開場，由兩位主持人輪流介紹節目理念。Hank大叔以「在忙碌生活中，有餘力去做快樂的事，並在重要時刻拿出最好的狀態」點出節目核心，Betty則補充「能量不只是體力，還包含專注力、情緒狀態」，並承諾用實用方法與幽默幫助聽眾找到高能量節奏。語速雖快，但清晰有力，有效傳達節目主旨，迅速抓住聽眾注意力。</v>
       </c>
       <c r="R17" t="str">
-        <v>N/A</v>
+        <v>什麼是「內耗」？惡魔與天使的比喻</v>
       </c>
       <c r="S17" t="str">
-        <v>N/A</v>
+        <v>02:43 - 03:33</v>
       </c>
       <c r="T17" t="str">
-        <v>N/A</v>
+        <v>Betty提出「內耗」的行為表現，Hank則用生動的「惡魔與天使」比喻來解釋內耗的本質：在行動前就被內心��負面情緒說服放棄。這個比喻非常形象化，讓抽象的「內耗」變得具體易懂，引發聽眾共鳴。兩人的互動也很有趣，Betty說Hank講完大家可能更聽不懂，然後Hank就給了更形象的比喻，展現了節目的幽默感與深度。</v>
       </c>
       <c r="U17" t="str">
-        <v>N/A</v>
+        <v>大前研一的「快轉」策略：預見未來，加速決策</v>
       </c>
       <c r="V17" t="str">
-        <v>N/A</v>
+        <v>15:20 - 17:04</v>
       </c>
       <c r="W17" t="str">
-        <v>N/A</v>
+        <v>Hank分享了他從日本策略大師大前研一學到的「FF (Fast Forward)」策略，即在做重大決策前，將事情快轉三年或十年，預想結果。這個方法不僅實用，而且「FF」這個詞彙的解釋也帶有懷舊的幽默感（DVD播放器的快轉鍵）。這段展現了節目將複雜概念轉化為易懂策略的能力，同時也帶有主持人個人經驗的分享，非常引人入勝，是核心論述的精華片段。</v>
       </c>
       <c r="X17" t="str">
-        <v>2026-06-20T12:53:14.710Z</v>
+        <v>2026-06-21T02:25:56.747Z</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
       </c>
       <c r="B18" t="str">
-        <v>郝聲音</v>
+        <v>能量黑客</v>
       </c>
       <c r="C18" t="str">
-        <v>郝聲音：（下）有魚的「已讀Podcast」，如何從閱讀的喜悅，成長到自媒體分享的幸福</v>
+        <v>怎麼休息都沒用？問題其實出在你的精力管理｜能量黑客 S4EP7</v>
       </c>
       <c r="D18">
-        <v>260</v>
+        <v>195</v>
       </c>
       <c r="E18" t="str">
         <v>中</v>
       </c>
       <c r="F18" t="str">
-        <v>兩位主講人皆常在句首使用「然後」作為轉折詞，頻率中等偏高。此外，「就是」也常被用於語氣的強調或解釋，而「那」則多用於話題的轉換。偶爾會出現「呃」等語氣詞。</v>
+        <v>兩位主持人在對話中頻繁使用「就是」、「然後」、「那」、「所以」作為語句的連接詞或轉折詞。這些詞彙在中文口語中常見，雖有一定頻率，但並未嚴重影響內容的流暢度或聽感。</v>
       </c>
       <c r="G18" t="str">
-        <v>男主持人（好哥）的聲音低沉厚實，共鳴感強，語調自然且富有情感，沒有機器人般的生硬感。女主持人（有餘）的聲音清晰明亮，語氣充滿活力與熱情，整體聽感溫暖且具陪伴感，沒有刺耳的頻率。</v>
+        <v>男主持人Hank的聲音具有良好的中低音共鳴與厚實度，語氣沉穩且富有情感，表達清晰，沒有機器人般的生硬感。女主持人Betty的聲音則展現出高音域的圓潤度與溫馨陪伴感，語調親切自然，充滿活力，聽起來舒適不刺耳。兩位主持人的聲音都極具親和力與感染力。</v>
       </c>
       <c r="H18" t="str">
         <v>優</v>
@@ -59103,66 +59103,66 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L18" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。背景環境噪音極低，確保了清晰的對話內容。</v>
+        <v>整體錄音品質優良，音量平衡穩定，沒有偵測到噴麥、突兀爆音或明顯的背景雜音。音質清晰，為聽眾提供了極佳的聆聽體驗。</v>
       </c>
       <c r="M18" t="str">
-        <v>00:07 - 00:24</v>
+        <v>00:31 - 02:30</v>
       </c>
       <c r="N18" t="str">
-        <v>主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
+        <v>這段開場由女主持人Betty引導，男主持人Hank分享他的書《你不是懶，是能量低》出版一年後的讀者回饋。他生動地描述了讀者如何因為書中的概念而改變對自身「懶惰」的看法，並解釋了為何決定將這些寶貴的知識透過Podcast分享給更多人。這段內容不僅清晰地闡述了節目的核心價值與使命，兩位主持人的對話也充滿了真誠與互動感，語速適中，引人入勝。</v>
       </c>
       <c r="O18" t="str">
-        <v>Podcast與自媒體的開場提問</v>
+        <v>能量黑客的誕生：從書本到Podcast的緣起</v>
       </c>
       <c r="P18" t="str">
-        <v>00:07 - 00:24</v>
+        <v>00:31 - 02:30</v>
       </c>
       <c r="Q18" t="str">
-        <v>主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
+        <v>這段開場由女主持人Betty引導，男主持人Hank分享他的書《你不是懶，是能量低》出版一年後的讀者回饋。他生動地描述了讀者如何因為書中的概念而改變對自身「懶惰」的看法，並解釋了為何決定將這些寶貴的知識透過Podcast分享給更多人。這段內容不僅清晰地闡述了節目的核心價值與使命，兩位主持人的對話也充滿了真誠與互動感，語速適中，引人入勝。</v>
       </c>
       <c r="R18" t="str">
-        <v>Threads平台「內容為王」的獨特魅力</v>
+        <v>解決���午疲勞的飲食策略：低GI食物與211餐盤的秘密</v>
       </c>
       <c r="S18" t="str">
-        <v>05:13 - 06:02</v>
+        <v>04:37 - 06:47</v>
       </c>
       <c r="T18" t="str">
-        <v>來賓深入分析Threads平台「內容為王」的特性，透過生動的案例（只有一個粉絲卻爆紅的貼文）說明其對素人創作者的友善與潛力，展現獨到見解，引人入勝。</v>
+        <v>在這段核心論述中，男主持人Hank深入淺出地解釋了為何許多人下午會感到疲勞，並提供了具體的飲食解決方案。他詳細說明了高GI食物如何導致血糖快速升高與下降，進而引發疲勞感，並介紹了「低GI食物」和「211餐盤」的實用概念。他不僅解釋了生理機制（胰島素、血清素、褪黑激素），還提供了具體食物建議。這段內容資訊量豐富，邏輯清晰，對於聽眾解決日常困擾極具參考價值。</v>
       </c>
       <c r="U18" t="str">
-        <v>知識內化與費曼學習法的實踐</v>
+        <v>掌控情緒，提升能量的關鍵：負面情緒管理三步驟</v>
       </c>
       <c r="V18" t="str">
-        <v>19:15 - 21:11</v>
+        <v>13:44 - 15:17</v>
       </c>
       <c r="W18" t="str">
-        <v>兩位主持人探討知識分享中「引用權威」與「個人自信」的關係，並引導至費曼學習法，強調將知識內化並應用於自身問題解決的重要性，為聽眾提供實用的學習心態與方法，具啟發性。</v>
+        <v>這段內容探討了情緒管理對能量展現的深遠影響，是節目核心理念的精華。男主持人Hank強調情緒與精力是「雙生」關係，並提出了處理負面情緒的「覺察、辨識、對策」三步驟。他用具體例子說明即使身體狀況良好，負面情緒（如年終獎金不如預期）也能瞬間耗盡精力。女主持人Betty也補充了情緒管理的重要性。這段對話展現了深刻的洞察力，語氣真摯，能有效引導聽眾反思並學習如何管理自身情緒，進而提升整體能量狀態。</v>
       </c>
       <c r="X18" t="str">
-        <v>2026-06-21T00:16:00.733Z</v>
+        <v>2026-06-21T02:27:34.768Z</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
       </c>
       <c r="B19" t="str">
-        <v>郝聲音</v>
+        <v>能量黑客</v>
       </c>
       <c r="C19" t="str">
-        <v>郝聲音：（下）郝書分享：『值得過上好日子』從情緒消費到聰明投資,克服「不夠花、不敢花」的金錢焦慮、學會建立有安心感的全方位財務計畫</v>
+        <v>睡不好、腦袋停不下來？鳥姊的「精力回收」真實做法｜能量黑客S2EP7—ft.來賓：鳥姊 Amy</v>
       </c>
       <c r="D19">
-        <v>290</v>
+        <v>205</v>
       </c>
       <c r="E19" t="str">
         <v>中</v>
       </c>
       <c r="F19" t="str">
-        <v>兩位主持人都常在句首使用「然後」進行轉折，或以「就是」作為語氣詞。男主持人習慣性使用「你知道嗎」、「對不對」來與聽眾互動或確認語意。整體贅字頻率中等。</v>
+        <v>常在句首使用「然後」、「那」進行轉折，也常出現「就是」作為語氣詞，贅字頻率中等。</v>
       </c>
       <c r="G19" t="str">
-        <v>男主持人聲音中低音共鳴厚實，語調情感豐富，表達流暢且具說服力。女主持人聲音高音域圓潤，語氣溫馨且具陪伴感，表達清晰不刺耳。兩位聲音特質互補，提升節目親和力。</v>
+        <v>男主持人聲音中低音共鳴厚實，語調情感豐富，具備親和力與說服力。女主持人聲音高音域圓潤清晰，語氣活潑，帶有溫馨陪伴感，無刺耳感。嘉賓聲音清晰，語氣真誠。整體聲音特質良好。</v>
       </c>
       <c r="H19" t="str">
         <v>優</v>
@@ -59177,66 +59177,66 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L19" t="str">
-        <v>整體錄音品質優良，音量���穩，人聲清晰，沒有突兀爆音與噴麥現象，背景環境音極為乾淨。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景環境音極為乾淨。</v>
       </c>
       <c r="M19" t="str">
-        <v>00:00 - 01:15</v>
+        <v>00:00 - 00:30</v>
       </c>
       <c r="N19" t="str">
-        <v>開場主持人以「財商」與「人生」的關係破題，引導出夫妻間因價值觀差異而產生「火花」的有趣比喻，迅速吸引聽眾對節目主題產生共鳴與好奇。女主持人隨後補充的個人經驗，讓討論更具生活感。</v>
+        <v>節目開頭的背景音樂搭配兩位主持人的自我介紹與節目理念，語速適中，聲音充滿能量與親和力，迅速建立節目調性並吸引聽眾。特別是Vicky的介紹，語速快而清晰，展現活力。</v>
       </c>
       <c r="O19" t="str">
-        <v>財商與人生觀的火花</v>
+        <v>能量駭客的開場與節目宗旨</v>
       </c>
       <c r="P19" t="str">
-        <v>00:00 - 01:15</v>
+        <v>00:00 - 00:30</v>
       </c>
       <c r="Q19" t="str">
-        <v>開場主持人以「財商」與「人生」的關係破題，引導出夫妻間因價值觀差異而產生「火花」的有趣比喻，迅速吸引聽眾對節目主題產生共鳴與好奇。女主持人隨後補充的個人經驗，讓討論更具生活感。</v>
+        <v>節目開頭的背景音樂搭配兩位主持人的自我介紹與節目理念，語速適中，聲音充滿能量與親和力，迅速建立節目調性並吸引聽眾。特別是Vicky的介紹，語速快而清晰，展現活力。</v>
       </c>
       <c r="R19" t="str">
-        <v>「正念」的核心：活在當下與不批判</v>
+        <v>嘉賓的低潮經驗與應對策略</v>
       </c>
       <c r="S19" t="str">
-        <v>12:42 - 14:22</v>
+        <v>01:40 - 02:20</v>
       </c>
       <c r="T19" t="str">
-        <v>此段落深入解釋了「正念」的兩大核心概念：「活在當下」與「不批判」。女主持人以清晰的邏輯闡述了這兩點對於個人成長和金錢觀念的重要性，特別強調了華人文化中常見的自我批判問題，提供了實用的覺察方法。</v>
+        <v>嘉賓Amy分享了她在高壓工作下如何意識到低潮並嘗試透過「自由書寫」來排解思緒的經驗。這段內容具體且實用，展現了嘉賓的真誠，也提供了聽眾可參考的實用技巧。主持人與嘉賓的互動自然，引導得宜。</v>
       </c>
       <c r="U19" t="str">
-        <v>10個「身心安定」的練習方法</v>
+        <v>能量管理的核心：衝刺與休息的節奏</v>
       </c>
       <c r="V19" t="str">
-        <v>17:14 - 19:22</v>
+        <v>16:20 - 17:09</v>
       </c>
       <c r="W19" t="str">
-        <v>主持人詳細列舉並簡要說明了書中推薦的10個「身心安定」練習方法，從感官體驗（精油、水晶、音樂、泡澡）到身體活動（呼吸、運動、舞蹈）及心靈實踐（親近自然、書寫、陪伴孩子），提供了具體可行的建議，讓聽眾能���即應用於日常生活中，提升覺察力與幸福感。</v>
+        <v>Hank大叔提出了「人生不是一場馬拉松，��是一段又一段的衝刺」的精闢觀點，強調了適時休息的重要性。這段內容是節目的核心論述精華，具有深刻的啟發性，語氣堅定且富有說服力，是能量管理理念的完美詮釋。</v>
       </c>
       <c r="X19" t="str">
-        <v>2026-06-21T00:21:11.061Z</v>
+        <v>2026-06-21T02:28:52.798Z</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="B20" t="str">
-        <v>郝聲音</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="C20" t="str">
-        <v>郝聲音：（下）終於跟MJ林明樟老師合體！用「財務腦」打通「業務力」，讓商業與人生獲利生生不息！</v>
+        <v>多巴胺陷阱！戒不掉的不是癮，是深層的焦慮ft.蘇琮祺心理師｜哇賽心觀點ep193</v>
       </c>
       <c r="D20">
-        <v>250</v>
+        <v>195</v>
       </c>
       <c r="E20" t="str">
         <v>中</v>
       </c>
       <c r="F20" t="str">
-        <v>兩位主講人皆常在句首使用「那」、「然後」或「就是」作為語氣詞或轉折詞，頻率中等，但不會過於頻繁而影響聽感。</v>
+        <v>主講人常在句首使用「然後」和「那」作為轉折詞，頻率中等，但整體對話流暢度不受影響。</v>
       </c>
       <c r="G20" t="str">
-        <v>兩位男主持人聲音共鳴感佳，中低音厚實且清晰，語調自然流暢，情感表達豐富，無機器人唸稿感，整體聽感親和且具說服力。</v>
+        <v>男主持人（宇澤）聲音溫暖、清晰，中低音共鳴感強，語調自然且富有情感，沒有機器人唸稿感。來賓（蘇崇其）的聲音也專業且清晰，兩位主持人的聲音都具親和力，無刺耳感。</v>
       </c>
       <c r="H20" t="str">
         <v>優</v>
@@ -59248,16 +59248,16 @@
         <v>無</v>
       </c>
       <c r="K20" t="str">
-        <v>環境安靜，幾乎無底噪，錄音背景非常乾淨。</v>
+        <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L20" t="str">
-        <v>整體錄音品質優良，音量平穩一致，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聆聽體���。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺體驗���</v>
       </c>
       <c r="M20" t="str">
-        <v>02:28 - 03:46</v>
+        <v>02:07 - 03:49</v>
       </c>
       <c r="N20" t="str">
-        <v>此段落由MJ老師分享個人生病導致公司薪資停發，以及離職後公司仍能良好運作的親身經歷，引導出「系統」的重要性。他以生動的語氣和具體的「1x1x1」乘法概念，深入淺出地解釋了系統運作的關鍵，情感真摯且極具說服力，是理解課程核心理念的精彩片段。</v>
+        <v>此段落深入探討了「食物成癮」與「進食成癮」的區別，並進一步闡述了成癮與壞習慣之間的模糊界線，是節目核心概念的精彩呈現。主講人與來賓的對話充滿洞察力，語氣真摯且音調波動起伏有致，極具聲音說服力。</v>
       </c>
       <c r="O20" t="str">
         <v>N/A</v>
@@ -59287,30 +59287,30 @@
         <v>N/A</v>
       </c>
       <c r="X20" t="str">
-        <v>2026-06-20T12:52:38.345Z</v>
+        <v>2026-06-20T13:15:23.756Z</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="B21" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="C21" t="str">
-        <v>#770 賺錢是為了幸福還是徒增焦慮？練習「鬆弛感」與小成就，把寶貴時間還給真正重要的事 來賓：蔡宇哲、郝旭烈</v>
+        <v>掌握你的金錢性格，打造幸福家庭理財ft.精算媽咪珊迪兔｜哇賽心觀點ep194</v>
       </c>
       <c r="D21">
-        <v>205</v>
+        <v>245</v>
       </c>
       <c r="E21" t="str">
         <v>中</v>
       </c>
       <c r="F21" t="str">
-        <v>主持人Sandy常在句首使用「然後」進行轉折，偶爾使用「就是」；蔡宇哲老師和好哥也常使用「那」和「就是」作為語氣詞或連接詞，整體贅字頻率中等，不至於影響理解。</v>
+        <v>主講人與來賓皆有使用「就是」、「其實」作為語氣詞或轉折詞，來賓常使用「然後」連接語句，但整體頻率尚可接受，不致影響聽感。</v>
       </c>
       <c r="G21" t="str">
-        <v>女主持人Sandy的聲音清亮、溫暖且充滿活力，高音域圓潤，給人溫馨陪伴感。男主持人蔡宇哲老師的聲音清晰、沉穩，語氣富有說服力。好哥的聲音則低沉厚實，共鳴感強，語調平穩，三位主持人的聲音特質都非常悅耳，沒有刺耳感。</v>
+        <v>男主持人聲音低沉厚實，共鳴感佳，語調變化自然，富有親和力。女主持人聲音清晰明亮，高音域圓潤不刺耳，帶有溫馨陪伴感，表達流暢。</v>
       </c>
       <c r="H21" t="str">
         <v>優</v>
@@ -59325,66 +59325,66 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L21" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺體驗。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺���驗。</v>
       </c>
       <c r="M21" t="str">
-        <v>00:18 - 00:37</v>
+        <v>02:07 - 03:44</v>
       </c>
       <c r="N21" t="str">
-        <v>主持人Sandy以充滿活力的語氣開場，迅速點出許多人追求金錢、事業、成就背後的核心需求——安全感，並進一步提出如何獲得心靈自由的關鍵問題，有效吸引聽眾進入主題。</v>
+        <v>此段落來賓生動地分享了原生家庭中父母截然不同的金錢觀（父親的創業擴張與母親的節儉務實），以及這些經歷如何塑造了她個人的金錢觀。她真誠地反思了「好」與「不好」的定義，並強調找到自己最舒適的理財方式，內容具深度且引人共鳴，情感表達豐富，是極具說服力的黃金聽點。</v>
       </c>
       <c r="O21" t="str">
-        <v>追求安全感與心靈自由的開場</v>
+        <v>N/A</v>
       </c>
       <c r="P21" t="str">
-        <v>00:18 - 00:37</v>
+        <v>N/A</v>
       </c>
       <c r="Q21" t="str">
-        <v>主持人Sandy以充滿活力的語氣開場，迅速點出許多人追求金錢、事業、成就背後的核心需求——安全感，並進一步提出如何獲得心靈自由的關鍵問題，有效吸引聽眾進入主題。</v>
+        <v>N/A</v>
       </c>
       <c r="R21" t="str">
-        <v>財富自由的真諦：幸福與意義</v>
+        <v>N/A</v>
       </c>
       <c r="S21" t="str">
-        <v>01:22 - 01:43</v>
+        <v>N/A</v>
       </c>
       <c r="T21" t="str">
-        <v>蔡宇哲老師在此段落深刻剖析財富自由的真正目的，指出金錢最終是為了帶來幸福、快樂與意義，並反思這些是否必須依賴大量金錢才能實現，提供聽眾一個重新思考財富觀的機會。</v>
+        <v>N/A</v>
       </c>
       <c r="U21" t="str">
-        <v>累積小成就，戰勝焦慮</v>
+        <v>N/A</v>
       </c>
       <c r="V21" t="str">
-        <v>07:45 - 08:20</v>
+        <v>N/A</v>
       </c>
       <c r="W21" t="str">
-        <v>好哥與蔡宇哲老師共同探討透過累積小成就來建立自信、戰勝焦慮的實用方法，特別提到「兩分鐘目標」的概念，為聽眾提供了具體且可操作的建議，展現了節目的實用價值和情感連結。</v>
+        <v>N/A</v>
       </c>
       <c r="X21" t="str">
-        <v>2026-06-21T00:31:11.293Z</v>
+        <v>2026-06-20T13:14:32.297Z</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="B22" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="C22" t="str">
-        <v>#800 買老屋怕踩雷？破解中古屋隱藏價值，聰明挑出高CP值潛力好房！來賓：House123 執行長 邱愛莉 Ellie</v>
+        <v>療癒創傷，溫柔擁抱完整的自己ft.留佩萱博士｜哇賽療心室ep148</v>
       </c>
       <c r="D22">
-        <v>205</v>
+        <v>260</v>
       </c>
       <c r="E22" t="str">
         <v>中</v>
       </c>
       <c r="F22" t="str">
-        <v>兩位主持人皆有使用「然後」、「就是」、「對啊」、「其實」等口頭禪，尤其在句首作為轉折詞的頻率較高，但整體而言不至於過度影響聽感。</v>
+        <v>主講人與來賓皆常使用「就是」、「那」、「其實」等口頭禪，其中「就是」的出現頻率高，整體贅字頻率中等。</v>
       </c>
       <c r="G22" t="str">
-        <v>兩位女主持人的聲音皆清晰、圓潤，高音域表現良好，沒有刺耳感。主講人Sandy的語調活潑，具親和力與溫馨陪伴感；來賓Aily的聲音則顯得沉穩專業，共鳴感佳，兩者搭配使對話流暢且富有層次。</v>
+        <v>女主持人聲音高音域圓潤，語調溫和且富有親和力，無刺耳感，傳達溫馨陪伴感。來賓聲音清晰有力，表達流暢，具說服力。</v>
       </c>
       <c r="H22" t="str">
         <v>優</v>
@@ -59399,66 +59399,66 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L22" t="str">
-        <v>整體錄音品質優良，音量平穩，���聲清晰，沒有突兀爆音與噴麥現象，背景環境噪音也控制得很好。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。</v>
       </c>
       <c r="M22" t="str">
-        <v>00:49 - 01:14</v>
+        <v>03:41 - 04:09</v>
       </c>
       <c r="N22" t="str">
-        <v>主持人Sandy以生動的語氣，點出許多人在買房時既期待又害怕受傷害的普遍心態，特別是對於首次購屋者。她簡潔地帶出新舊房子的優缺點，迅速抓住聽眾的注意力，為後續的討論奠定基礎。</v>
+        <v>此段落來賓以具體案例解釋IFS核心概念，說明童年受批評如何導致內化問題並形成保護機制。語氣真摯且清晰，情感起伏自然，有助於聽眾理解複雜的心理學概念。</v>
       </c>
       <c r="O22" t="str">
-        <v>買房的期待與困境</v>
+        <v>N/A</v>
       </c>
       <c r="P22" t="str">
-        <v>00:49 - 01:14</v>
+        <v>N/A</v>
       </c>
       <c r="Q22" t="str">
-        <v>主持人Sandy以生動的語氣，點出許多人在買房時既期待又害怕受傷害的普遍心態，特別是對於首次購屋者。她簡潔地帶出新舊房子的優缺點，迅速抓住聽眾的注意力，為後續的討論奠定基礎。</v>
+        <v>N/A</v>
       </c>
       <c r="R22" t="str">
-        <v>房屋結構的致命傷：軟弱層與海砂屋</v>
+        <v>N/A</v>
       </c>
       <c r="S22" t="str">
-        <v>05:56 - 07:29</v>
+        <v>N/A</v>
       </c>
       <c r="T22" t="str">
-        <v>來賓Aily在此段落深入淺出地解釋了老屋最關鍵的結構性問題，包括「軟弱層」和「海砂屋」。她強調這些問題的不可逆性，並指出結構安全是購屋時首要考量的因素，提供了極具價值的專業知識，語氣真摯且具說服力。</v>
+        <v>N/A</v>
       </c>
       <c r="U22" t="str">
-        <v>投資老屋的退場機制與風險評估</v>
+        <v>N/A</v>
       </c>
       <c r="V22" t="str">
-        <v>19:00 - 19:59</v>
+        <v>N/A</v>
       </c>
       <c r="W22" t="str">
-        <v>Aily在此段落從投資角度切入，強調了老屋投資必須具備「退場機制」的重要性。她提醒聽眾不應只依賴都更，而應考慮其他可能的退出方案，例如出租或轉售，為投資者提供了務實且全面的風險評估建議。</v>
+        <v>N/A</v>
       </c>
       <c r="X22" t="str">
-        <v>2026-06-21T00:33:54.344Z</v>
+        <v>2026-06-20T13:16:15.224Z</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>郝旭烈/郝聲音</v>
       </c>
       <c r="B23" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>郝聲音</v>
       </c>
       <c r="C23" t="str">
-        <v>#805 總在爛工作與錯的感情中輪迴？看懂隱藏的人生劇本，用「自我覺察」找回選擇權！來賓：千里淳風</v>
+        <v>郝聲音：（上）設計師KiKi，從繪畫到設計的熱愛之路，到引領他人感受設計之美的「走讀」行旅～</v>
       </c>
       <c r="D23">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="E23" t="str">
-        <v>中</v>
+        <v>高</v>
       </c>
       <c r="F23" t="str">
-        <v>主講人（Cindy）常使用「然後」、「就是」、「對」、「嗯」作為語氣詞或轉折詞。來賓（錢老師）則常使用「其實」、「就是」、「那」、「對」、「嗯」。兩位講者的贅字頻率皆為中等，但語句流暢度不受影響。</v>
+        <v>男主持人常在句首使用「那」和「就是」作為轉折或連接詞，頻率較高。女主持人則較常使用「嗯」、「然後」和「其實」，頻率中等，但整體而言，兩位主持人的贅字頻率偏高。</v>
       </c>
       <c r="G23" t="str">
-        <v>主講人（Cindy）的聲音高音域圓潤，語調活潑，富有溫馨陪伴感，聽起來清晰且不刺耳。來賓（錢老師）的聲音中低音共鳴強，厚實且沉穩，語氣充滿智慧與說服力。</v>
+        <v>男主持人（好哥）中低音共鳴飽滿，聲音厚實且富有磁性，語調變化豐富，充滿活力。女主持人（Kiki）高音域圓潤，聲音清晰溫和，帶有親和力，語氣真誠，無刺耳感。</v>
       </c>
       <c r="H23" t="str">
         <v>優</v>
@@ -59470,57 +59470,57 @@
         <v>無</v>
       </c>
       <c r="K23" t="str">
-        <v>環境安靜，幾乎無底噪，錄音品質極佳。</v>
+        <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L23" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。兩位講者的聲音清晰，背景噪音極低，提供極佳的聽覺體驗。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，聽感舒適。</v>
       </c>
       <c r="M23" t="str">
-        <v>00:50 - 01:14</v>
+        <v>03:36 - 03:47</v>
       </c>
       <c r="N23" t="str">
-        <v>此片段是節目開場的精華，主持人以引人入勝的方式介紹來賓，點出他從講求邏輯與科技的背景，轉變為鑽研命理的獨特經歷。這不僅迅速抓住聽眾的好奇心，也為後續的深度對談奠定基礎，展現了主持人良好的引導能力和來賓故事的吸引力。</v>
+        <v>此段落女主持人Kiki分享她從小就對設計有著強烈的內心呼喚，語氣中透露出真誠與堅定。男主持人適時的提問與感嘆「好幸福喔」也為這段對話增添了情感深度，展現了主講人早期的志向與熱情。</v>
       </c>
       <c r="O23" t="str">
-        <v>引人入勝的開場：從科技到命理</v>
+        <v>N/A</v>
       </c>
       <c r="P23" t="str">
-        <v>00:50 - 01:14</v>
+        <v>N/A</v>
       </c>
       <c r="Q23" t="str">
-        <v>此片段是節目開場的精華，主持人以引人入勝的方式介紹來賓，點出他從講求邏輯與科技的背景，轉變為鑽研命理的獨特經歷。這不僅迅速抓住聽眾的好奇心，也為後續的深度對談奠定基礎，展現了主持人良好的引導能力和來賓故事的吸引力。</v>
+        <v>N/A</v>
       </c>
       <c r="R23" t="str">
-        <v>改變命運的關鍵：自我覺察與觀察者</v>
+        <v>N/A</v>
       </c>
       <c r="S23" t="str">
-        <v>07:49 - 09:11</v>
+        <v>N/A</v>
       </c>
       <c r="T23" t="str">
-        <v>此片段深入探討了改變命運的核心觀念——「自我覺察」與「觀察者自我」。來賓以心理學理論結合生活實例（如開車自動駕駛），清晰解釋了人類意識的三個層次，並指出大多數人命運被預設的原因。這段內容不僅具啟發性，也提供了聽眾實際可操作的思維工具，是節目中極具深度和實用價值的論述。</v>
+        <v>N/A</v>
       </c>
       <c r="U23" t="str">
-        <v>意想不到的改運工具：衣服與食物</v>
+        <v>N/A</v>
       </c>
       <c r="V23" t="str">
-        <v>20:31 - 21:37</v>
+        <v>N/A</v>
       </c>
       <c r="W23" t="str">
-        <v>���片段揭示了兩個最有效且日常的改運工具：衣服和食物。來賓從色彩心理學和五行理論的角度，解釋了這些看似平凡的元素如何直接影響一個人的情緒、能量和運勢。這段內容不僅顛覆了傳統對改運的想像，也提供了具體且易於實踐的方法，讓聽眾能從生活中著手改變，極具趣味性和實用性。</v>
+        <v>N/A</v>
       </c>
       <c r="X23" t="str">
-        <v>2026-06-21T00:33:00.044Z</v>
+        <v>2026-06-20T12:51:53.770Z</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>蕭邦</v>
+        <v>郝旭烈/郝聲音</v>
       </c>
       <c r="B24" t="str">
-        <v>蕭邦相談室</v>
+        <v>郝聲音</v>
       </c>
       <c r="C24" t="str">
-        <v>如何度過負面情緒 ？</v>
+        <v>郝聲音：（上）曾格爾老師，攀登高峰，不僅是為了超越，更是讓自己能看得更遠</v>
       </c>
       <c r="D24">
         <v>205</v>
@@ -59529,10 +59529,10 @@
         <v>中</v>
       </c>
       <c r="F24" t="str">
-        <v>主講人常在句首使用「那」作為轉折詞，頻率較高，但多數時候作為語氣連接而非純粹贅字。此外，「就是」和「然後」偶爾出現，整體贅字頻率屬於中等。</v>
+        <v>主講人與來賓在對話中常使用「就是」、「然後」、「對」、「這個」、「那」、「其實」、「就」等詞作為語氣詞或轉折詞。這些詞彙的出現頻率中等，雖然偶爾會打斷語句的流暢性，但整體而言不至於影響理解，且符合口語對話的自然習慣。</v>
       </c>
       <c r="G24" t="str">
-        <v>女主持人聲音溫暖、圓潤，中低音域表現穩定，高音域不刺耳，整體語調富有情感，給人一種溫馨且具陪伴感的聽覺體驗。</v>
+        <v>男主持人好哥的聲音低沉厚實，中低音共鳴感強，語調情感豐富且富有親和力，沒有機器人唸稿感。女主持人曾格爾的聲音清亮，高音域圓潤不刺耳，語氣溫暖且具陪伴感，表達清晰。</v>
       </c>
       <c r="H24" t="str">
         <v>優</v>
@@ -59547,48 +59547,1010 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L24" t="str">
+        <v>整體錄音品質優良，音量平穩，兩位講者的聲音清晰且平衡，沒有突兀爆音與噴麥現象，背景環境噪音極低，提供舒適的聆聽體驗。</v>
+      </c>
+      <c r="M24" t="str">
+        <v>00:00 - 00:43</v>
+      </c>
+      <c r="N24" t="str">
+        <v>主持人好哥以充滿熱情的語氣介紹曾格爾老師，並迅速點出她「行者」的身份與攀登多座高山的經歷，特別強調她挑戰的都是非一般人能及的山峰，立即吸引聽眾對這位特別來賓產生好奇與期待，為節目奠定引人入勝的基調。</v>
+      </c>
+      <c r="O24" t="str">
+        <v>登山女傑的驚人開場</v>
+      </c>
+      <c r="P24" t="str">
+        <v>00:00 - 00:43</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>主持人好哥以充滿熱情的語氣介紹曾格爾老師，並迅速點出她「行者」的身份與攀登多座高山的經歷，特別強調她挑戰的都是非一般人能及的山峰，立即吸引聽眾對這位特別來賓產生好奇與期待，為節目奠定引人入勝的基調。</v>
+      </c>
+      <c r="R24" t="str">
+        <v>聖母峰大本營的啟示：登山之路的起點</v>
+      </c>
+      <c r="S24" t="str">
+        <v>01:45 - 03:19</v>
+      </c>
+      <c r="T24" t="str">
+        <v>曾格爾老師分享她第一次攀登聖母峰大本營的艱辛與挑戰，以及這次經歷如何讓她反思物質需求，並意識到「呼吸才是唯一真正需要把握的」。這段深刻的個人體悟，是她登山生涯的關鍵轉折點，展現了她對生命與自然的獨特見解，極具啟發性。</v>
+      </c>
+      <c r="U24" t="str">
+        <v>挑戰K2的幕後辛酸與亞洲探險文化的落差</v>
+      </c>
+      <c r="V24" t="str">
+        <v>01:22:22 - 01:37:50</v>
+      </c>
+      <c r="W24" t="str">
+        <v>曾格爾老師詳細描述了她挑戰世��第二高峰K2的艱難過程，包括籌措資金、申請許可證的行政障礙，以及在極地環境中面對的歧視與文化差異。這段內容不僅展現了她堅韌的毅力，也深刻揭示了亞洲探險文化與歐美之間的巨大落差，引人深思。</v>
+      </c>
+      <c r="X24" t="str">
+        <v>2026-06-21T00:20:23.884Z</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="B25" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="C25" t="str">
+        <v>郝聲音：（下） 蘇絢慧老師好書分享，『隱性內耗』：看不見的傷，如何消磨你的能量？</v>
+      </c>
+      <c r="D25">
+        <v>205</v>
+      </c>
+      <c r="E25" t="str">
+        <v>中</v>
+      </c>
+      <c r="F25" t="str">
+        <v>主講人（徐瑄惠老師）和主持人（好哥）皆常在句首使用「然後」進行轉折，或使用「就是」、「那」等詞，頻率中等。</v>
+      </c>
+      <c r="G25" t="str">
+        <v>男主持人（好哥）聲音中低音共鳴厚實，語調情感豐富且具親和力。女主持人（徐瑄惠老師）聲音圓潤清晰，高音域不刺耳，語氣溫和具陪伴感。</v>
+      </c>
+      <c r="H25" t="str">
+        <v>優</v>
+      </c>
+      <c r="I25" t="str">
+        <v>無</v>
+      </c>
+      <c r="J25" t="str">
+        <v>無</v>
+      </c>
+      <c r="K25" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L25" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低。</v>
+      </c>
+      <c r="M25" t="str">
+        <v>01:59 - 03:45</v>
+      </c>
+      <c r="N25" t="str">
+        <v>此段落深入探討童年環境如何形塑個人對自我價值的認知，以及如何導致內耗與自我質疑。主講人語氣真摯，情感起伏自然，內容具啟發性，是理解內耗成因的關鍵點。</v>
+      </c>
+      <c r="O25" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="P25" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="R25" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="S25" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="T25" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="U25" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="V25" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="W25" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="X25" t="str">
+        <v>2026-06-20T12:53:14.710Z</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="B26" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="C26" t="str">
+        <v>郝聲音：（下）有魚的「已讀Podcast」，如何從閱讀的喜悅，成長到自媒體分享的幸福</v>
+      </c>
+      <c r="D26">
+        <v>260</v>
+      </c>
+      <c r="E26" t="str">
+        <v>中</v>
+      </c>
+      <c r="F26" t="str">
+        <v>兩位主講人皆常在句首使用「然後」作為轉折詞，頻率中等偏高。此外，「就是」也常被用於語氣的強調或解釋，而「那」則多用於話題的轉換。偶爾會出現「呃」等語氣詞。</v>
+      </c>
+      <c r="G26" t="str">
+        <v>男主持人（好哥）的聲音低沉厚實，共鳴感強，語調自然且富有情感，沒有機器人般的生硬感。女主持人（有餘）的聲音清晰明亮，語氣充滿活力與熱情，整體聽感溫暖且具陪伴感，沒有刺耳的頻率。</v>
+      </c>
+      <c r="H26" t="str">
+        <v>優</v>
+      </c>
+      <c r="I26" t="str">
+        <v>無</v>
+      </c>
+      <c r="J26" t="str">
+        <v>無</v>
+      </c>
+      <c r="K26" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L26" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。背景環境噪音極低，確保了清晰的對話內容。</v>
+      </c>
+      <c r="M26" t="str">
+        <v>00:07 - 00:24</v>
+      </c>
+      <c r="N26" t="str">
+        <v>主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
+      </c>
+      <c r="O26" t="str">
+        <v>Podcast與自媒體的開場提問</v>
+      </c>
+      <c r="P26" t="str">
+        <v>00:07 - 00:24</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
+      </c>
+      <c r="R26" t="str">
+        <v>Threads平台「內容為王」的獨特魅力</v>
+      </c>
+      <c r="S26" t="str">
+        <v>05:13 - 06:02</v>
+      </c>
+      <c r="T26" t="str">
+        <v>來賓深入分析Threads平台「內容為王」的特性，透過生動的案例（只有一個粉絲卻爆紅的貼文）說明其對素人創作者的友善與潛力，展現獨到見解，引人入勝。</v>
+      </c>
+      <c r="U26" t="str">
+        <v>知識內化與費曼學習法的實踐</v>
+      </c>
+      <c r="V26" t="str">
+        <v>19:15 - 21:11</v>
+      </c>
+      <c r="W26" t="str">
+        <v>兩位主持人探討知識分享中「引用權威」與「個人自信」的關係，並引導至費曼學習法，強調將知識內化並應用於自身問題解決的重要性，為聽眾提供實用的學習心態與方法，具啟發性。</v>
+      </c>
+      <c r="X26" t="str">
+        <v>2026-06-21T00:16:00.733Z</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="B27" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="C27" t="str">
+        <v>郝聲音：（下）郝書分享：『值得過上好日子』從情緒消費到聰明投資,克服「不夠花、不敢花」的金錢焦慮、學會建立有安心感的全方位財務計畫</v>
+      </c>
+      <c r="D27">
+        <v>290</v>
+      </c>
+      <c r="E27" t="str">
+        <v>中</v>
+      </c>
+      <c r="F27" t="str">
+        <v>兩位主持人都常在句首使用「然後」進行轉折，或以「就是」作為語氣詞。男主持人習慣性使用「你知道嗎」、「對不對」來與聽眾互動或確認語意。整體贅字頻率中等。</v>
+      </c>
+      <c r="G27" t="str">
+        <v>男主持人聲音中低音共鳴厚實，語調情感豐富，表達流暢且具說服力。女主持人聲音高音域圓潤，語氣溫馨且具陪伴感，表達清晰不刺耳。兩位聲音特質互補，提升節目親和力。</v>
+      </c>
+      <c r="H27" t="str">
+        <v>優</v>
+      </c>
+      <c r="I27" t="str">
+        <v>無</v>
+      </c>
+      <c r="J27" t="str">
+        <v>無</v>
+      </c>
+      <c r="K27" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L27" t="str">
+        <v>整體錄音品質優良，音量���穩，人聲清晰，沒有突兀爆音與噴麥現象，背景環境音極為乾淨。</v>
+      </c>
+      <c r="M27" t="str">
+        <v>00:00 - 01:15</v>
+      </c>
+      <c r="N27" t="str">
+        <v>開場主持人以「財商」與「人生」的關係破題，引導出夫妻間因價值觀差異而產生「火花」的有趣比喻，迅速吸引聽眾對節目主題產生共鳴與好奇。女主持人隨後補充的個人經驗，讓討論更具生活感。</v>
+      </c>
+      <c r="O27" t="str">
+        <v>財商與人生觀的火花</v>
+      </c>
+      <c r="P27" t="str">
+        <v>00:00 - 01:15</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>開場主持人以「財商」與「人生」的關係破題，引導出夫妻間因價值觀差異而產生「火花」的有趣比喻，迅速吸引聽眾對節目主題產生共鳴與好奇。女主持人隨後補充的個人經驗，讓討論更具生活感。</v>
+      </c>
+      <c r="R27" t="str">
+        <v>「正念」的核心：活在當下與不批判</v>
+      </c>
+      <c r="S27" t="str">
+        <v>12:42 - 14:22</v>
+      </c>
+      <c r="T27" t="str">
+        <v>此段落深入解釋了「正念」的兩大核心概念：「活在當下」與「不批判」。女主持人以清晰的邏輯闡述了這兩點對於個人成長和金錢觀念的重要性，特別強調了華人文化中常見的自我批判問題，提供了實用的覺察方法。</v>
+      </c>
+      <c r="U27" t="str">
+        <v>10個「身心安定」的練習方法</v>
+      </c>
+      <c r="V27" t="str">
+        <v>17:14 - 19:22</v>
+      </c>
+      <c r="W27" t="str">
+        <v>主持人詳細列舉並簡要說明了書中推薦的10個「身心安定」練習方法，從感官體驗（精油、水晶、音樂、泡澡）到身體活動（呼吸、運動、舞蹈）及心靈實踐（親近自然、書寫、陪伴孩子），提供了具體可行的建議，讓聽眾能���即應用於日常生活中，提升覺察力與幸福感。</v>
+      </c>
+      <c r="X27" t="str">
+        <v>2026-06-21T00:21:11.061Z</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="B28" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="C28" t="str">
+        <v>郝聲音：（下）終於跟MJ林明樟老師合體！用「財務腦」打通「業務力」，讓商業與人生獲利生生不息！</v>
+      </c>
+      <c r="D28">
+        <v>250</v>
+      </c>
+      <c r="E28" t="str">
+        <v>中</v>
+      </c>
+      <c r="F28" t="str">
+        <v>兩位主講人皆常在句首使用「那」、「然後」或「就是」作為語氣詞或轉折詞，頻率中等，但不會過於頻繁而影響聽感。</v>
+      </c>
+      <c r="G28" t="str">
+        <v>兩位男主持人聲音共鳴感佳，中低音厚實且清晰，語調自然流暢，情感表達豐富，無機器人唸稿感，整體聽感親和且具說服力。</v>
+      </c>
+      <c r="H28" t="str">
+        <v>優</v>
+      </c>
+      <c r="I28" t="str">
+        <v>無</v>
+      </c>
+      <c r="J28" t="str">
+        <v>無</v>
+      </c>
+      <c r="K28" t="str">
+        <v>環境安靜，幾乎無底噪，錄音背景非常乾淨。</v>
+      </c>
+      <c r="L28" t="str">
+        <v>整體錄音品質優良，音量平穩一致，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聆聽體���。</v>
+      </c>
+      <c r="M28" t="str">
+        <v>02:28 - 03:46</v>
+      </c>
+      <c r="N28" t="str">
+        <v>此段落由MJ老師分享個人生病導致公司薪資停發，以及離職後公司仍能良好運作的親身經歷，引導出「系統」的重要性。他以生動的語氣和具體的「1x1x1」乘法概念，深入淺出地解釋了系統運作的關鍵，情感真摯且極具說服力，是理解課程核心理念的精彩片段。</v>
+      </c>
+      <c r="O28" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="P28" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Q28" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="R28" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="S28" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="T28" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="U28" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="V28" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="W28" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="X28" t="str">
+        <v>2026-06-20T12:52:38.345Z</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>精算媽咪的家計簿｜珊迪兔</v>
+      </c>
+      <c r="B29" t="str">
+        <v>精算媽咪的家計簿</v>
+      </c>
+      <c r="C29" t="str">
+        <v>#770 賺錢是為了幸福還是徒增焦慮？練習「鬆弛感」與小成就，把寶貴時間還給真正重要的事 來賓：蔡宇哲、郝旭烈</v>
+      </c>
+      <c r="D29">
+        <v>205</v>
+      </c>
+      <c r="E29" t="str">
+        <v>中</v>
+      </c>
+      <c r="F29" t="str">
+        <v>主持人Sandy常在句首使用「然後」進行轉折，偶爾使用「就是」；蔡宇哲老師和好哥也常使用「那」和「就是」作為語氣詞或連接詞，整體贅字頻率中等，不至於影響理解。</v>
+      </c>
+      <c r="G29" t="str">
+        <v>女主持人Sandy的聲音清亮、溫暖且充滿活力，高音域圓潤，給人溫馨陪伴感。男主持人蔡宇哲老師的聲音清晰、沉穩，語氣富有說服力。好哥的聲音則低沉厚實，共鳴感強，語調平穩，三位主持人的聲音特質都非常悅耳，沒有刺耳感。</v>
+      </c>
+      <c r="H29" t="str">
+        <v>優</v>
+      </c>
+      <c r="I29" t="str">
+        <v>無</v>
+      </c>
+      <c r="J29" t="str">
+        <v>無</v>
+      </c>
+      <c r="K29" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L29" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺體驗。</v>
+      </c>
+      <c r="M29" t="str">
+        <v>00:18 - 00:37</v>
+      </c>
+      <c r="N29" t="str">
+        <v>主持人Sandy以充滿活力的語氣開場，迅速點出許多人追求金錢、事業、成就背後的核心需求——安全感，並進一步提出如何獲得心靈自由的關鍵問題，有效吸引聽眾進入主題。</v>
+      </c>
+      <c r="O29" t="str">
+        <v>追求安全感與心靈自由的開場</v>
+      </c>
+      <c r="P29" t="str">
+        <v>00:18 - 00:37</v>
+      </c>
+      <c r="Q29" t="str">
+        <v>主持人Sandy以充滿活力的語氣開場，迅速點出許多人追求金錢、事業、成就背後的核心需求——安全感，並進一步提出如何獲得心靈自由的關鍵問題，有效吸引聽眾進入主題。</v>
+      </c>
+      <c r="R29" t="str">
+        <v>財富自由的真諦：幸福與意義</v>
+      </c>
+      <c r="S29" t="str">
+        <v>01:22 - 01:43</v>
+      </c>
+      <c r="T29" t="str">
+        <v>蔡宇哲老師在此段落深刻剖析財富自由的真正目的，指出金錢最終是為了帶來幸福、快樂與意義，並反思這些是否必須依賴大量金錢才能實現，提供聽眾一個重新思考財富觀的機會。</v>
+      </c>
+      <c r="U29" t="str">
+        <v>累積小成就，戰勝焦慮</v>
+      </c>
+      <c r="V29" t="str">
+        <v>07:45 - 08:20</v>
+      </c>
+      <c r="W29" t="str">
+        <v>好哥與蔡宇哲老師共同探討透過累積小成就來建立自信、戰勝焦慮的實用方法，特別提到「兩分鐘目標」的概念，為聽眾提供了具體且可操作的建議，展現了節目的實用價值和情感連結。</v>
+      </c>
+      <c r="X29" t="str">
+        <v>2026-06-21T00:31:11.293Z</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>精算媽咪的家計簿｜珊迪兔</v>
+      </c>
+      <c r="B30" t="str">
+        <v>精算媽咪的家計簿</v>
+      </c>
+      <c r="C30" t="str">
+        <v>#800 買老屋怕踩雷？破解中古屋隱藏價值，聰明挑出高CP值潛力好房！來賓：House123 執行長 邱愛莉 Ellie</v>
+      </c>
+      <c r="D30">
+        <v>205</v>
+      </c>
+      <c r="E30" t="str">
+        <v>中</v>
+      </c>
+      <c r="F30" t="str">
+        <v>兩位主持人皆有使用「然後」、「就是」、「對啊」、「其實」等口頭禪，尤其在句首作為轉折詞的頻率較高，但整體而言不至於過度影響聽感。</v>
+      </c>
+      <c r="G30" t="str">
+        <v>兩位女主持人的聲音皆清晰、圓潤，高音域表現良好，沒有刺耳感。主講人Sandy的語調活潑，具親和力與溫馨陪伴感；來賓Aily的聲音則顯得沉穩專業，共鳴感佳，兩者搭配使對話流暢且富有層次。</v>
+      </c>
+      <c r="H30" t="str">
+        <v>優</v>
+      </c>
+      <c r="I30" t="str">
+        <v>無</v>
+      </c>
+      <c r="J30" t="str">
+        <v>無</v>
+      </c>
+      <c r="K30" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L30" t="str">
+        <v>整體錄音品質優良，音量平穩，���聲清晰，沒有突兀爆音與噴麥現象，背景環境噪音也控制得很好。</v>
+      </c>
+      <c r="M30" t="str">
+        <v>00:49 - 01:14</v>
+      </c>
+      <c r="N30" t="str">
+        <v>主持人Sandy以生動的語氣，點出許多人在買房時既期待又害怕受傷害的普遍心態，特別是對於首次購屋者。她簡潔地帶出新舊房子的優缺點，迅速抓住聽眾的注意力，為後續的討論奠定基礎。</v>
+      </c>
+      <c r="O30" t="str">
+        <v>買房的期待與困境</v>
+      </c>
+      <c r="P30" t="str">
+        <v>00:49 - 01:14</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>主持人Sandy以生動的語氣，點出許多人在買房時既期待又害怕受傷害的普遍心態，特別是對於首次購屋者。她簡潔地帶出新舊房子的優缺點，迅速抓住聽眾的注意力，為後續的討論奠定基礎。</v>
+      </c>
+      <c r="R30" t="str">
+        <v>房屋結構的致命傷：軟弱層與海砂屋</v>
+      </c>
+      <c r="S30" t="str">
+        <v>05:56 - 07:29</v>
+      </c>
+      <c r="T30" t="str">
+        <v>來賓Aily在此段落深入淺出地解釋了老屋最關鍵的結構性問題，包括「軟弱層」和「海砂屋」。她強調這些問題的不可逆性，並指出結構安全是購屋時首要考量的因素，提供了極具價值的專業知識，語氣真摯且具說服力。</v>
+      </c>
+      <c r="U30" t="str">
+        <v>投資老屋的退場機制與風險評估</v>
+      </c>
+      <c r="V30" t="str">
+        <v>19:00 - 19:59</v>
+      </c>
+      <c r="W30" t="str">
+        <v>Aily在此段落從投資角度切入，強調了老屋投資必須具備「退場機制」的重要性。她提醒聽眾不應只依賴都更，而應考慮其他可能的退出方案，例如出租或轉售，為投資者提供了務實且全面的風險評估建議。</v>
+      </c>
+      <c r="X30" t="str">
+        <v>2026-06-21T00:33:54.344Z</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>精算媽咪的家計簿｜珊迪兔</v>
+      </c>
+      <c r="B31" t="str">
+        <v>精算媽咪的家計簿</v>
+      </c>
+      <c r="C31" t="str">
+        <v>#805 總在爛工作與錯的感情中輪迴？看懂隱藏的人生劇本，用「自我覺察」找回選擇權！來賓：千里淳風</v>
+      </c>
+      <c r="D31">
+        <v>250</v>
+      </c>
+      <c r="E31" t="str">
+        <v>中</v>
+      </c>
+      <c r="F31" t="str">
+        <v>主講人（Cindy）常使用「然後」、「就是」、「對」、「嗯」作為語氣詞或轉折詞。來賓（錢老師）則常使用「其實」、「就是」、「那」、「對」、「嗯」。兩位講者的贅字頻率皆為中等，但語句流暢度不受影響。</v>
+      </c>
+      <c r="G31" t="str">
+        <v>主講人（Cindy）的聲音高音域圓潤，語調活潑，富有溫馨陪伴感，聽起來清晰且不刺耳。來賓（錢老師）的聲音中低音共鳴強，厚實且沉穩，語氣充滿智慧與說服力。</v>
+      </c>
+      <c r="H31" t="str">
+        <v>優</v>
+      </c>
+      <c r="I31" t="str">
+        <v>無</v>
+      </c>
+      <c r="J31" t="str">
+        <v>無</v>
+      </c>
+      <c r="K31" t="str">
+        <v>環境安靜，幾乎無底噪，錄音品質極佳。</v>
+      </c>
+      <c r="L31" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。兩位講者的聲音清晰，背景噪音極低，提供極佳的聽覺體驗。</v>
+      </c>
+      <c r="M31" t="str">
+        <v>00:50 - 01:14</v>
+      </c>
+      <c r="N31" t="str">
+        <v>此片段是節目開場的精華，主持人以引人入勝的方式介紹來賓，點出他從講求邏輯與科技的背景，轉變為鑽研命理的獨特經歷。這不僅迅速抓住聽眾的好奇心，也為後續的深度對談奠定基礎，展現了主持人良好的引導能力和來賓故事的吸引力。</v>
+      </c>
+      <c r="O31" t="str">
+        <v>引人入勝的開場：從科技到命理</v>
+      </c>
+      <c r="P31" t="str">
+        <v>00:50 - 01:14</v>
+      </c>
+      <c r="Q31" t="str">
+        <v>此片段是節目開場的精華，主持人以引人入勝的方式介紹來賓，點出他從講求邏輯與科技的背景，轉變為鑽研命理的獨特經歷。這不僅迅速抓住聽眾的好奇心，也為後續的深度對談奠定基礎，展現了主持人良好的引導能力和來賓故事的吸引力。</v>
+      </c>
+      <c r="R31" t="str">
+        <v>改變命運的關鍵：自我覺察與觀察者</v>
+      </c>
+      <c r="S31" t="str">
+        <v>07:49 - 09:11</v>
+      </c>
+      <c r="T31" t="str">
+        <v>此片段深入探討了改變命運的核心觀念——「自我覺察」與「觀察者自我」。來賓以心理學理論結合生活實例（如開車自動駕駛），清晰解釋了人類意識的三個層次，並指出大多數人命運被預設的原因。這段內容不僅具啟發性，也提供了聽眾實際可操作的思維工具，是節目中極具深度和實用價值的論述。</v>
+      </c>
+      <c r="U31" t="str">
+        <v>意想不到的改運工具：衣服與食物</v>
+      </c>
+      <c r="V31" t="str">
+        <v>20:31 - 21:37</v>
+      </c>
+      <c r="W31" t="str">
+        <v>���片段揭示了兩個最有效且日常的改運工具：衣服和食物。來賓從色彩心理學和五行理論的角度，解釋了這些看似平凡的元素如何直接影響一個人的情緒、能量和運勢。這段內容不僅顛覆了傳統對改運的想像，也提供了具體且易於實踐的方法，讓聽眾能從生活中著手改變，極具趣味性和實用性。</v>
+      </c>
+      <c r="X31" t="str">
+        <v>2026-06-21T00:33:00.044Z</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>蕭邦</v>
+      </c>
+      <c r="B32" t="str">
+        <v>蕭邦相談室</v>
+      </c>
+      <c r="C32" t="str">
+        <v>一被拒絕，就容易自我懷疑</v>
+      </c>
+      <c r="D32">
+        <v>236</v>
+      </c>
+      <c r="E32" t="str">
+        <v>中</v>
+      </c>
+      <c r="F32" t="str">
+        <v>主講人常在句首使用「然後」進行轉折，並頻繁使用「其實」來強調或解釋，此外「就是」、「那」也偶爾出現，整體贅字頻率中等。</v>
+      </c>
+      <c r="G32" t="str">
+        <v>女主持人聲音清晰溫暖，高音域圓潤不刺耳，語調自然且富有情感，給人溫馨陪伴感。</v>
+      </c>
+      <c r="H32" t="str">
+        <v>優</v>
+      </c>
+      <c r="I32" t="str">
+        <v>無</v>
+      </c>
+      <c r="J32" t="str">
+        <v>無</v>
+      </c>
+      <c r="K32" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L32" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景環境音處理得非常乾淨。</v>
+      </c>
+      <c r="M32" t="str">
+        <v>00:12 - 01:18</v>
+      </c>
+      <c r="N32" t="str">
+        <v>主講人以自身經歷開場，生動描述過去因他人退費或拒絕而陷入強烈自我懷疑的心理狀態，語氣真摯，能迅速引起聽眾共鳴，並清晰點出本集欲探討的核心問題。</v>
+      </c>
+      <c r="O32" t="str">
+        <v>「自我懷疑」的深淵：退費與拒絕帶來的內耗</v>
+      </c>
+      <c r="P32" t="str">
+        <v>00:12 - 01:18</v>
+      </c>
+      <c r="Q32" t="str">
+        <v>主講人以自身經歷開場，生動描述過去因他人退費或拒絕而陷入強烈自我懷疑的心理狀態，語氣真摯，能迅速引起聽眾共鳴，並清晰點出本集欲探討的核心問題。</v>
+      </c>
+      <c r="R32" t="str">
+        <v>價值與選擇：兩件完全不同的事</v>
+      </c>
+      <c r="S32" t="str">
+        <v>03:59 - 04:32</v>
+      </c>
+      <c r="T32" t="str">
+        <v>此段落是節目核心觀點的精華，主講人清晰闡述了她如何將「自身價值」與「他人的選擇」區分開來，強調兩者互不衝突，展現了深刻的自我成長與洞察力。語氣堅定而富有啟發性。</v>
+      </c>
+      <c r="U32" t="str">
+        <v>擺脫自我懷疑：重新定義你的價值</v>
+      </c>
+      <c r="V32" t="str">
+        <v>06:30 - 07:06</v>
+      </c>
+      <c r="W32" t="str">
+        <v>主講人提供具體的實踐建議，引導聽眾在面對拒絕時如何檢視自己的反應，並強調「你的價值是你的事」，為聽眾帶來力量與清晰的指引。結尾語氣溫暖而有力，總結了節目的核心訊息。</v>
+      </c>
+      <c r="X32" t="str">
+        <v>2026-06-21T01:52:51.939Z</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>蕭邦</v>
+      </c>
+      <c r="B33" t="str">
+        <v>蕭邦相談室</v>
+      </c>
+      <c r="C33" t="str">
+        <v>人生最難的不是賺錢，而是______</v>
+      </c>
+      <c r="D33">
+        <v>200</v>
+      </c>
+      <c r="E33" t="str">
+        <v>中</v>
+      </c>
+      <c r="F33" t="str">
+        <v>主講人常使用「就是」、「其實」作為語氣詞或轉折詞，頻率中等，但整體語流仍保持流暢。</v>
+      </c>
+      <c r="G33" t="str">
+        <v>女主持人聲音溫暖、圓潤，高音域處理得宜，沒有刺耳感，語調自然且富有情感，給人溫馨的陪伴感。</v>
+      </c>
+      <c r="H33" t="str">
+        <v>優</v>
+      </c>
+      <c r="I33" t="str">
+        <v>無</v>
+      </c>
+      <c r="J33" t="str">
+        <v>無</v>
+      </c>
+      <c r="K33" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L33" t="str">
+        <v>整體錄音品質優良，音量穩定，沒有突兀爆音或噴麥現象，背景環境音處理得非常乾淨。</v>
+      </c>
+      <c r="M33" t="str">
+        <v>00:13 - 00:50</v>
+      </c>
+      <c r="N33" t="str">
+        <v>主持人以自身經驗切入，點出自由工作者或創業者常陷入的「先拼再說」心態，迅速抓住聽眾的共鳴與注意力，破題精準且引人深思。</v>
+      </c>
+      <c r="O33" t="str">
+        <v>「先拼再��」的陷阱</v>
+      </c>
+      <c r="P33" t="str">
+        <v>00:13 - 00:50</v>
+      </c>
+      <c r="Q33" t="str">
+        <v>主持人以自身經驗切入，點出自由工作者或創業者常陷入的「先拼再說」心態，迅速抓住聽眾的共鳴與注意力，破題精準且引人深思。</v>
+      </c>
+      <c r="R33" t="str">
+        <v>金錢與關係的本質</v>
+      </c>
+      <c r="S33" t="str">
+        <v>02:25 - 03:33</v>
+      </c>
+      <c r="T33" t="str">
+        <v>此段落深入剖析金錢與人際關係的價值，強調金錢可再賺，但時間與關係的不可逆性。主講人語氣真摯，論述深刻，觸及聽眾內心深處的價值觀。</v>
+      </c>
+      <c r="U33" t="str">
+        <v>人生不能等，陪伴最珍貴</v>
+      </c>
+      <c r="V33" t="str">
+        <v>05:39 - 07:21</v>
+      </c>
+      <c r="W33" t="str">
+        <v>主持人分享翻看父母老照片的個人感觸，深刻體悟到時間的流逝與陪伴的重要性。這段情感真摯、語氣充滿感染力，是整集的情感高潮，提醒聽眾珍惜當下。</v>
+      </c>
+      <c r="X33" t="str">
+        <v>2026-06-21T01:53:23.870Z</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>蕭邦</v>
+      </c>
+      <c r="B34" t="str">
+        <v>蕭邦相談室</v>
+      </c>
+      <c r="C34" t="str">
+        <v>如何度過負面情緒 ？</v>
+      </c>
+      <c r="D34">
+        <v>205</v>
+      </c>
+      <c r="E34" t="str">
+        <v>中</v>
+      </c>
+      <c r="F34" t="str">
+        <v>主講人常在句首使用「那」作為轉折詞，頻率較高，但多數時候作為語氣連接而非純粹贅字。此外，「就是」和「然後」偶爾出現，整體贅字頻率屬於中等。</v>
+      </c>
+      <c r="G34" t="str">
+        <v>女主持人聲音溫暖、圓潤，中低音域表現穩定，高音域不刺耳，整體語調富有情感，給人一種溫馨且具陪伴感的聽覺體驗。</v>
+      </c>
+      <c r="H34" t="str">
+        <v>優</v>
+      </c>
+      <c r="I34" t="str">
+        <v>無</v>
+      </c>
+      <c r="J34" t="str">
+        <v>無</v>
+      </c>
+      <c r="K34" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L34" t="str">
         <v>整體錄音品質極佳，音量平穩，人聲清晰，沒有任何噴麥、突兀爆音或背景雜音，聽感非常舒���。</v>
       </c>
-      <c r="M24" t="str">
+      <c r="M34" t="str">
         <v>00:12 - 00:31</v>
       </c>
-      <c r="N24" t="str">
+      <c r="N34" t="str">
         <v>主持人以自身經歷引出「情緒」這個主題，語氣真誠，迅速建立與聽眾的連結，引人入勝，為節目內容做了很好的鋪墊。</v>
       </c>
-      <c r="O24" t="str">
+      <c r="O34" t="str">
         <v>開場：情緒的引導與個人經驗分享</v>
       </c>
-      <c r="P24" t="str">
+      <c r="P34" t="str">
         <v>00:12 - 00:31</v>
       </c>
-      <c r="Q24" t="str">
+      <c r="Q34" t="str">
         <v>主持人以自身經歷引出「情緒」這個主題，語氣真誠，迅速建立與聽眾的連結，引人入勝，為節目內容做了很好的鋪墊。</v>
       </c>
-      <c r="R24" t="str">
+      <c r="R34" t="str">
         <v>核心論述：關閉腦袋，讓情緒流動</v>
       </c>
-      <c r="S24" t="str">
+      <c r="S34" t="str">
         <v>04:05 - 04:55</v>
       </c>
-      <c r="T24" t="str">
+      <c r="T34" t="str">
         <v>此段落是節目的核心精華，主持人清晰地闡述了處理情緒的關鍵方法——「關閉腦袋，讓情緒自然流動」，並解釋了其背後的原因，提供了具體且實用的建議，極具啟發性。</v>
       </c>
-      <c r="U24" t="str">
+      <c r="U34" t="str">
         <v>總結：接受情緒，有效解決問題</v>
       </c>
-      <c r="V24" t="str">
+      <c r="V34" t="str">
         <v>05:43 - 06:10</v>
       </c>
-      <c r="W24" t="str">
+      <c r="W34" t="str">
         <v>這段總結了節目主旨，強調接受所有情緒的重要性及其帶來的益處，語氣溫和且具說服力，為聽眾提供正向的啟發，並引導聽眾思考如何有效解決問題。</v>
       </c>
-      <c r="X24" t="str">
+      <c r="X34" t="str">
         <v>2026-06-21T00:40:44.043Z</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Dr Selena</v>
+      </c>
+      <c r="B35" t="str">
+        <v>小資變有錢｜Dr.Selena生活理財王</v>
+      </c>
+      <c r="C35" t="str">
+        <v>2026小資族一定要看懂4個關鍵總經變數 !</v>
+      </c>
+      <c r="D35">
+        <v>205</v>
+      </c>
+      <c r="E35" t="str">
+        <v>中</v>
+      </c>
+      <c r="F35" t="str">
+        <v>兩位主講人皆習慣在句首或句中頻繁使用「就是」、「然後」、「那」作為語氣詞或轉折詞，頻率中等。</v>
+      </c>
+      <c r="G35" t="str">
+        <v>女主持人（Data Selina）的聲音高亢、清晰且充滿活力，語調明亮，給人溫暖且具陪伴感的印象，沒有刺耳感。男主持人（卡爾先生）的聲音低沉、厚實且共鳴感強，語氣沉穩而專業，表達流暢，沒有機器人唸稿感。</v>
+      </c>
+      <c r="H35" t="str">
+        <v>優</v>
+      </c>
+      <c r="I35" t="str">
+        <v>���</v>
+      </c>
+      <c r="J35" t="str">
+        <v>無</v>
+      </c>
+      <c r="K35" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L35" t="str">
+        <v>整體錄音品質優良，音量平穩，兩位主講人的聲音清晰，沒有突兀爆音與噴麥現象，背景噪音極低。</v>
+      </c>
+      <c r="M35" t="str">
+        <v>00:07 - 00:57</v>
+      </c>
+      <c r="N35" t="str">
+        <v>主持人以清晰的語調介紹節目宗旨，並迅速帶入本集主題「小資必學的2024總體經濟」。隨後，她以熱情且專業的方式介紹來賓卡爾先生，卡爾先生的開場白也展現其專業與自信，為節目奠定良好的基調。此段落語速適中，內容引人入勝，有效抓住聽眾注意力。</v>
+      </c>
+      <c r="O35" t="str">
+        <v>節目開場與總體經濟專家介紹</v>
+      </c>
+      <c r="P35" t="str">
+        <v>00:07 - 00:57</v>
+      </c>
+      <c r="Q35" t="str">
+        <v>主持人以清晰的語調介紹節目宗旨，並迅速帶入本集主題「小資必學的2024總體經濟」。隨後，她以熱情且專業的方式介紹來賓卡爾先生，卡爾先生的開場白也展現其專業與自信，為節目奠定良好的基調。此段落語速適中，內容引人入勝，有效抓住聽眾注意力。</v>
+      </c>
+      <c r="R35" t="str">
+        <v>居高思危：美股高點與潛在修正風險</v>
+      </c>
+      <c r="S35" t="str">
+        <v>02:58 - 04:43</v>
+      </c>
+      <c r="T35" t="str">
+        <v>卡爾先生在此段落精闢地指出2024年全球經濟的關鍵詞是「居高思危」。他引用標普500指數創65年新高，並以2000年網路泡沫破裂的歷史經驗為鑑，警示股市可能面臨20-30%的修正。他強調這是「數學的力量」和「週期」���必然，並將美股與台股的連動性納入考量，提醒聽眾做好心理準備。此段論述邏輯清晰，數據支持有力，語氣嚴謹，具高度警示性。</v>
+      </c>
+      <c r="U35" t="str">
+        <v>美元信用危機與實體黃金的避險策略</v>
+      </c>
+      <c r="V35" t="str">
+        <v>17:07 - 19:30</v>
+      </c>
+      <c r="W35" t="str">
+        <v>卡爾先生在此段落深入探討美元信用可能面臨的挑戰，回顧1970年代美國解除美元與黃金掛鉤的歷史，並預測未來幾年美元可能貶值。主持人隨後提出地緣政治風險（如台海緊張）下，美元作為避險工具的有效性，並強調實體黃金在這種情境下的重要性。卡爾先生進一步解釋實體黃金作為唯一非任何國家負債的資產，其信用甚至高於國家信用。這段對話不僅分析了貨幣風險，更提供了具體的避險策略，內容豐富且具實用價值。</v>
+      </c>
+      <c r="X35" t="str">
+        <v>2026-06-21T02:21:27.811Z</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Dr Selena</v>
+      </c>
+      <c r="B36" t="str">
+        <v>小資變有錢｜Dr.Selena生活理財王</v>
+      </c>
+      <c r="C36" t="str">
+        <v>小資族如何成功打造第二條收入曲線：冒牌生的社群品牌經營策略免費教學！</v>
+      </c>
+      <c r="D36">
+        <v>290</v>
+      </c>
+      <c r="E36" t="str">
+        <v>中</v>
+      </c>
+      <c r="F36" t="str">
+        <v>主講人與來賓皆頻繁使用「然後」作為語句連接詞或轉折詞，以及「就是」用於解釋或強調。此外，「那」也常作為口頭禪或語氣詞出現。整體贅字頻率屬於中等。</v>
+      </c>
+      <c r="G36" t="str">
+        <v>男主持人（冒牌生）聲音中低音共鳴飽滿，音色厚實且富有磁性，語調變化自然，情感表達真摯，聽感舒適且具說服力。女主持人（Selina）高音域清晰明亮，語速雖快但咬字清楚，聲音圓潤且帶有親和力，整體聽感溫暖且具陪伴感，不刺耳。</v>
+      </c>
+      <c r="H36" t="str">
+        <v>優</v>
+      </c>
+      <c r="I36" t="str">
+        <v>無</v>
+      </c>
+      <c r="J36" t="str">
+        <v>無</v>
+      </c>
+      <c r="K36" t="str">
+        <v>環境安靜，幾乎無���噪</v>
+      </c>
+      <c r="L36" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰的聽覺體驗。</v>
+      </c>
+      <c r="M36" t="str">
+        <v>00:55 - 01:26</v>
+      </c>
+      <c r="N36" t="str">
+        <v>主持人熱情介紹嘉賓「冒牌生」及其在社群經營上的專長，並點出本集節目將探討如何透過社群媒體創造主動與被動收入，有效引導聽眾進入主題，為節目奠定良好開場。</v>
+      </c>
+      <c r="O36" t="str">
+        <v>嘉賓介紹與節目主題</v>
+      </c>
+      <c r="P36" t="str">
+        <v>00:55 - 01:26</v>
+      </c>
+      <c r="Q36" t="str">
+        <v>主持人熱情介紹嘉賓「冒牌生」及其在社群經營上的專長，並點出本集節目將探討如何透過社群媒體創造主動與被動收入，有效引導聽眾進入主題，為節目奠定良好開場。</v>
+      </c>
+      <c r="R36" t="str">
+        <v>成功案例：從洗頭店找到社群藍海</v>
+      </c>
+      <c r="S36" t="str">
+        <v>01:40:45 - 01:48:00</v>
+      </c>
+      <c r="T36" t="str">
+        <v>冒牌生分享一位學生透過分享洗頭店心得，成功累積大量粉絲的案例。此段落具體展現了如何將個人興趣與在地特色結合，創造獨特且受歡迎的內容，為聽眾提供實用的社群經營啟發，極具參考價值。</v>
+      </c>
+      <c r="U36" t="str">
+        <v>享受創作過程的智慧</v>
+      </c>
+      <c r="V36" t="str">
+        <v>02:21:00 - 02:26:00</v>
+      </c>
+      <c r="W36" t="str">
+        <v>冒牌生引用《享受吧！一個人的旅行》作者的經歷，闡述了享受創作過程本身的重要性，而非過度追求外在的成就與評價。這段對話深刻且富有哲理，鼓勵聽眾回歸初心，從熱愛的事物中獲得真正的快樂與滿足，��有啟發性。</v>
+      </c>
+      <c r="X36" t="str">
+        <v>2026-06-21T01:54:11.639Z</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Dr Selena</v>
+      </c>
+      <c r="B37" t="str">
+        <v>小資變有錢｜Dr.Selena生活理財王</v>
+      </c>
+      <c r="C37" t="str">
+        <v>小資愛樂活：用理財，走進千年古文明~此生必走一次的中亞絲路!</v>
+      </c>
+      <c r="D37">
+        <v>270</v>
+      </c>
+      <c r="E37" t="str">
+        <v>中</v>
+      </c>
+      <c r="F37" t="str">
+        <v>兩位主持人皆頻繁使用「然後」和「就是」作為語句連接詞，尤其常出現在句首。此外，「那」和「這個」也偶爾出現，整體贅字頻率屬於中等。</v>
+      </c>
+      <c r="G37" t="str">
+        <v>女主持人Selina的聲音清晰、明亮且充滿活力，高音域圓潤不刺耳，語氣溫暖且具陪伴感。男主持人Domingo的聲音低沉、渾厚且富有共鳴，中低音域表現出色，給人穩重、權威而友善的感覺。兩位主持人的聲音特質都非常適合廣播。</v>
+      </c>
+      <c r="H37" t="str">
+        <v>優</v>
+      </c>
+      <c r="I37" t="str">
+        <v>無</v>
+      </c>
+      <c r="J37" t="str">
+        <v>無</v>
+      </c>
+      <c r="K37" t="str">
+        <v>環境安靜，幾乎無底噪，僅有極輕微的環境音，不影響聆聽體驗。</v>
+      </c>
+      <c r="L37" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，音質清晰。</v>
+      </c>
+      <c r="M37" t="str">
+        <v>01:45 - 02:30</v>
+      </c>
+      <c r="N37" t="str">
+        <v>男主持人Domingo以「世界是一本書」的經典比喻開場，並提出「旅行是無知的解藥」的獨特觀點，深入探討旅行如何打破同溫層、拓展個人價值觀。這段內容富有哲理，語速適中，能有效引導聽眾思考。</v>
+      </c>
+      <c r="O37" t="str">
+        <v>旅遊的意義與世界觀的拓展</v>
+      </c>
+      <c r="P37" t="str">
+        <v>01:45 - 02:30</v>
+      </c>
+      <c r="Q37" t="str">
+        <v>男主持人Domingo以「世界是一本書」的經典比喻開場，並提出「旅行是無知的解藥」的獨特觀點，深入探討旅行如何打破同溫層、拓展個人價值觀。這段內容富有哲理，語速適中，能有效引導聽眾思考。</v>
+      </c>
+      <c r="R37" t="str">
+        <v>透過旅行認識真實世界</v>
+      </c>
+      <c r="S37" t="str">
+        <v>09:47 - 10:13</v>
+      </c>
+      <c r="T37" t="str">
+        <v>女主持人Selina與Domingo對談，指出媒體塑造的世界觀可能與真實世界存在差異，強調親身旅行才能體驗到更完整的世界。Selina更感性地表達「我旅行，我存在，我幸福」，展現旅行對她生命的重要性，對話真誠且具啟發性。</v>
+      </c>
+      <c r="U37" t="str">
+        <v>旅遊業的挑戰與領隊的辛勞</v>
+      </c>
+      <c r="V37" t="str">
+        <v>12:01 - 12:30</v>
+      </c>
+      <c r="W37" t="str">
+        <v>Selina分享了她帶團去尼泊爾時遇到的修路、坐船等突發狀況，以及旅遊業面臨的天災人禍挑戰，凸顯了領隊和導遊的壓力與辛勞。這段內容真實有趣，讓聽眾對旅遊從��人員的付出有更深的理解與共情。</v>
+      </c>
+      <c r="X37" t="str">
+        <v>2026-06-21T01:55:02.849Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:X24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X37"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: include episode 37 and compile updated dashboard
</commit_message>
<xml_diff>
--- a/eligible_episodes_pool.xlsx
+++ b/eligible_episodes_pool.xlsx
@@ -57808,7 +57808,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X37"/>
+  <dimension ref="A1:X38"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -59440,28 +59440,28 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>胡咪老師</v>
       </c>
       <c r="B23" t="str">
-        <v>郝聲音</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="C23" t="str">
-        <v>郝聲音：（上）設計師KiKi，從繪畫到設計的熱愛之路，到引領他人感受設計之美的「走讀」行旅～</v>
+        <v>S3.EP92｜刪掉容易，忘掉很難：從軍人到寫故事的人 feat. 林思齊</v>
       </c>
       <c r="D23">
-        <v>265</v>
+        <v>210</v>
       </c>
       <c r="E23" t="str">
-        <v>高</v>
+        <v>中</v>
       </c>
       <c r="F23" t="str">
-        <v>男主持人常在句首使用「那」和「就是」作為轉折或連接詞，頻率較高。女主持人則較常使用「嗯」、「然後」和「其實」，頻率中等，但整體而言，兩位主持人的贅字頻率偏高。</v>
+        <v>所有主講人皆常在句首使用「然後」作為轉折詞，頻率中等。此外，「就是」、「對」和「那」也常作為語氣詞或連接詞使用，尤其在主持人對話中較為頻繁。</v>
       </c>
       <c r="G23" t="str">
-        <v>男主持人（好哥）中低音共鳴飽滿，聲音厚實且富有磁性，語調變化豐富，充滿活力。女主持人（Kiki）高音域圓潤，聲音清晰溫和，帶有親和力，語氣真誠，無刺耳感。</v>
+        <v>男主持人畢頭大叔聲音低沉厚實，共鳴感強，語調情感豐富且具感染力。女主持人胡咪聲音清亮有活力，高音域圓潤不刺耳，給人溫馨陪伴感。來賓林思齊聲音沉穩清晰，語氣真摯，富有思考深度。</v>
       </c>
       <c r="H23" t="str">
-        <v>優</v>
+        <v>��</v>
       </c>
       <c r="I23" t="str">
         <v>無</v>
@@ -59473,43 +59473,43 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L23" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，聽感舒適。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。背景噪音極低，提供清晰舒適的聆聽體驗。</v>
       </c>
       <c r="M23" t="str">
-        <v>03:36 - 03:47</v>
+        <v>00:00 - 02:24</v>
       </c>
       <c r="N23" t="str">
-        <v>此段落女主持人Kiki分享她從小就對設計有著強烈的內心呼喚，語氣中透露出真誠與堅定。男主持人適時的提問與感嘆「好幸福喔」也為這段對話增添了情感深度，展現了主講人早期的志向與熱情。</v>
+        <v>節目以引人入勝的音樂和旁白開場，迅速帶出「分手」主題。主持人以幽默對話營造輕鬆氛圍，隨後介紹來賓林思齊，並巧妙地引導出他從職業軍人轉型為作家的獨特經歷，成功吸引聽眾對節目核心內容產生興趣。</v>
       </c>
       <c r="O23" t="str">
-        <v>N/A</v>
+        <v>破題精采開場：從軍人到作家，刪不掉的生命故事</v>
       </c>
       <c r="P23" t="str">
-        <v>N/A</v>
+        <v>00:00 - 02:24</v>
       </c>
       <c r="Q23" t="str">
-        <v>N/A</v>
+        <v>節目以引人入勝的音樂和旁白開場，迅速帶出「分手」主題。主持人以幽默對話營造輕鬆氛圍，隨後介紹來賓林思齊，並巧妙地引導出他從職業軍人轉型為作家的獨特經歷，成功吸引聽眾對節目核心內容產生興趣。</v>
       </c>
       <c r="R23" t="str">
-        <v>N/A</v>
+        <v>寫作的轉捩點：從個人情緒到讀者故事的「澆水」過程</v>
       </c>
       <c r="S23" t="str">
-        <v>N/A</v>
+        <v>02:40 - 05:55</v>
       </c>
       <c r="T23" t="str">
-        <v>N/A</v>
+        <v>林思齊詳細闡述了他的寫作歷程，從退伍後因個人情緒在社群平台發文，到後來轉變為收集並「灌溉」讀者投稿的故事「種子」。這段內容深入揭示了他獨特的創作理念，以及如何��重投稿者情感核心並在不同平台發布故事的策略，展現了他與讀者之間深刻的連結。</v>
       </c>
       <c r="U23" t="str">
-        <v>N/A</v>
+        <v>難以忘懷的投稿：被騙兩次的愛情詐騙故事與情感的脆弱</v>
       </c>
       <c r="V23" t="str">
-        <v>N/A</v>
+        <v>33:00 - 36:00</v>
       </c>
       <c r="W23" t="str">
-        <v>N/A</v>
+        <v>林思齊分享了一個令人心碎的讀者故事，關於一位女性在經歷愛情詐騙後，即使報警仍再次受騙。他對故事細節的描述，包括受害者的脆弱和詐騙者的操縱，深刻地展現了人性的複雜與情感的衝擊。這段內容極具感染力，觸及了信任、背叛和對愛的渴望等普世情感，讓聽眾感受到故事背後的真實與沉重。</v>
       </c>
       <c r="X23" t="str">
-        <v>2026-06-20T12:51:53.770Z</v>
+        <v>2026-06-21T02:35:31.851Z</v>
       </c>
     </row>
     <row r="24">
@@ -59520,19 +59520,19 @@
         <v>郝聲音</v>
       </c>
       <c r="C24" t="str">
-        <v>郝聲音：（上）曾格爾老師，攀登高峰，不僅是為了超越，更是讓自己能看得更遠</v>
+        <v>郝聲音：（上）設計師KiKi，從繪畫到設計的熱愛之路，到引領他人感受設計之美的「走讀」行旅～</v>
       </c>
       <c r="D24">
-        <v>205</v>
+        <v>265</v>
       </c>
       <c r="E24" t="str">
-        <v>中</v>
+        <v>高</v>
       </c>
       <c r="F24" t="str">
-        <v>主講人與來賓在對話中常使用「就是」、「然後」、「對」、「這個」、「那」、「其實」、「就」等詞作為語氣詞或轉折詞。這些詞彙的出現頻率中等，雖然偶爾會打斷語句的流暢性，但整體而言不至於影響理解，且符合口語對話的自然習慣。</v>
+        <v>男主持人常在句首使用「那」和「就是」作為轉折或連接詞，頻率較高。女主持人則較常使用「嗯」、「然後」和「其實」，頻率中等，但整體而言，兩位主持人的贅字頻率偏高。</v>
       </c>
       <c r="G24" t="str">
-        <v>男主持人好哥的聲音低沉厚實，中低音共鳴感強，語調情感豐富且富有親和力，沒有機器人唸稿感。女主持人曾格爾的聲音清亮，高音域圓潤不刺耳，語氣溫暖且具陪伴感，表達清晰。</v>
+        <v>男主持人（好哥）中低音共鳴飽滿，聲音厚實且富有磁性，語調變化豐富，充滿活力。女主持人（Kiki）高音域圓潤，聲音清晰溫和，帶有親和力，語氣真誠，無刺耳感。</v>
       </c>
       <c r="H24" t="str">
         <v>優</v>
@@ -59547,43 +59547,43 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L24" t="str">
-        <v>整體錄音品質優良，音量平穩，兩位講者的聲音清晰且平衡，沒有突兀爆音與噴麥現象，背景環境噪音極低，提供舒適的聆聽體驗。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，聽感舒適。</v>
       </c>
       <c r="M24" t="str">
-        <v>00:00 - 00:43</v>
+        <v>03:36 - 03:47</v>
       </c>
       <c r="N24" t="str">
-        <v>主持人好哥以充滿熱情的語氣介紹曾格爾老師，並迅速點出她「行者」的身份與攀登多座高山的經歷，特別強調她挑戰的都是非一般人能及的山峰，立即吸引聽眾對這位特別來賓產生好奇與期待，為節目奠定引人入勝的基調。</v>
+        <v>此段落女主持人Kiki分享她從小就對設計有著強烈的內心呼喚，語氣中透露出真誠與堅定。男主持人適時的提問與感嘆「好幸福喔」也為這段對話增添了情感深度，展現了主講人早期的志向與熱情。</v>
       </c>
       <c r="O24" t="str">
-        <v>登山女傑的驚人開場</v>
+        <v>N/A</v>
       </c>
       <c r="P24" t="str">
-        <v>00:00 - 00:43</v>
+        <v>N/A</v>
       </c>
       <c r="Q24" t="str">
-        <v>主持人好哥以充滿熱情的語氣介紹曾格爾老師，並迅速點出她「行者」的身份與攀登多座高山的經歷，特別強調她挑戰的都是非一般人能及的山峰，立即吸引聽眾對這位特別來賓產生好奇與期待，為節目奠定引人入勝的基調。</v>
+        <v>N/A</v>
       </c>
       <c r="R24" t="str">
-        <v>聖母峰大本營的啟示：登山之路的起點</v>
+        <v>N/A</v>
       </c>
       <c r="S24" t="str">
-        <v>01:45 - 03:19</v>
+        <v>N/A</v>
       </c>
       <c r="T24" t="str">
-        <v>曾格爾老師分享她第一次攀登聖母峰大本營的艱辛與挑戰，以及這次經歷如何讓她反思物質需求，並意識到「呼吸才是唯一真正需要把握的」。這段深刻的個人體悟，是她登山生涯的關鍵轉折點，展現了她對生命與自然的獨特見解，極具啟發性。</v>
+        <v>N/A</v>
       </c>
       <c r="U24" t="str">
-        <v>挑戰K2的幕後辛酸與亞洲探險文化的落差</v>
+        <v>N/A</v>
       </c>
       <c r="V24" t="str">
-        <v>01:22:22 - 01:37:50</v>
+        <v>N/A</v>
       </c>
       <c r="W24" t="str">
-        <v>曾格爾老師詳細描述了她挑戰世��第二高峰K2的艱難過程，包括籌措資金、申請許可證的行政障礙，以及在極地環境中面對的歧視與文化差異。這段內容不僅展現了她堅韌的毅力，也深刻揭示了亞洲探險文化與歐美之間的巨大落差，引人深思。</v>
+        <v>N/A</v>
       </c>
       <c r="X24" t="str">
-        <v>2026-06-21T00:20:23.884Z</v>
+        <v>2026-06-20T12:51:53.770Z</v>
       </c>
     </row>
     <row r="25">
@@ -59594,7 +59594,7 @@
         <v>郝聲音</v>
       </c>
       <c r="C25" t="str">
-        <v>郝聲音：（下） 蘇絢慧老師好書分享，『隱性內耗』：看不見的傷，如何消磨你的能量？</v>
+        <v>郝聲音：（上）曾格爾老師，攀登高峰，不僅是為了超越，更是讓自己能看得更遠</v>
       </c>
       <c r="D25">
         <v>205</v>
@@ -59603,10 +59603,10 @@
         <v>中</v>
       </c>
       <c r="F25" t="str">
-        <v>主講人（徐瑄惠老師）和主持人（好哥）皆常在句首使用「然後」進行轉折，或使用「就是」、「那」等詞，頻率中等。</v>
+        <v>主講人與來賓在對話中常使用「就是」、「然後」、「對」、「這個」、「那」、「其實」、「就」等詞作為語氣詞或轉折詞。這些詞彙的出現頻率中等，雖然偶爾會打斷語句的流暢性，但整體而言不至於影響理解，且符合口語對話的自然習慣。</v>
       </c>
       <c r="G25" t="str">
-        <v>男主持人（好哥）聲音中低音共鳴厚實，語調情感豐富且具親和力。女主持人（徐瑄惠老師）聲音圓潤清晰，高音域不刺耳，語氣溫和具陪伴感。</v>
+        <v>男主持人好哥的聲音低沉厚實，中低音共鳴感強，語調情感豐富且富有親和力，沒有機器人唸稿感。女主持人曾格爾的聲音清亮，高音域圓潤不刺耳，語氣溫暖且具陪伴感，表達清晰。</v>
       </c>
       <c r="H25" t="str">
         <v>優</v>
@@ -59621,43 +59621,43 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L25" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低。</v>
+        <v>整體錄音品質優良，音量平穩，兩位講者的聲音清晰且平衡，沒有突兀爆音與噴麥現象，背景環境噪音極低，提供舒適的聆聽體驗。</v>
       </c>
       <c r="M25" t="str">
-        <v>01:59 - 03:45</v>
+        <v>00:00 - 00:43</v>
       </c>
       <c r="N25" t="str">
-        <v>此段落深入探討童年環境如何形塑個人對自我價值的認知，以及如何導致內耗與自我質疑。主講人語氣真摯，情感起伏自然，內容具啟發性，是理解內耗成因的關鍵點。</v>
+        <v>主持人好哥以充滿熱情的語氣介紹曾格爾老師，並迅速點出她「行者」的身份與攀登多座高山的經歷，特別強調她挑戰的都是非一般人能及的山峰，立即吸引聽眾對這位特別來賓產生好奇與期待，為節目奠定引人入勝的基調。</v>
       </c>
       <c r="O25" t="str">
-        <v>N/A</v>
+        <v>登山女傑的驚人開場</v>
       </c>
       <c r="P25" t="str">
-        <v>N/A</v>
+        <v>00:00 - 00:43</v>
       </c>
       <c r="Q25" t="str">
-        <v>N/A</v>
+        <v>主持人好哥以充滿熱情的語氣介紹曾格爾老師，並迅速點出她「行者」的身份與攀登多座高山的經歷，特別強調她挑戰的都是非一般人能及的山峰，立即吸引聽眾對這位特別來賓產生好奇與期待，為節目奠定引人入勝的基調。</v>
       </c>
       <c r="R25" t="str">
-        <v>N/A</v>
+        <v>聖母峰大本營的啟示：登山之路的起點</v>
       </c>
       <c r="S25" t="str">
-        <v>N/A</v>
+        <v>01:45 - 03:19</v>
       </c>
       <c r="T25" t="str">
-        <v>N/A</v>
+        <v>曾格爾老師分享她第一次攀登聖母峰大本營的艱辛與挑戰，以及這次經歷如何讓她反思物質需求，並意識到「呼吸才是唯一真正需要把握的」。這段深刻的個人體悟，是她登山生涯的關鍵轉折點，展現了她對生命與自然的獨特見解，極具啟發性。</v>
       </c>
       <c r="U25" t="str">
-        <v>N/A</v>
+        <v>挑戰K2的幕後辛酸與亞洲探險文化的落差</v>
       </c>
       <c r="V25" t="str">
-        <v>N/A</v>
+        <v>01:22:22 - 01:37:50</v>
       </c>
       <c r="W25" t="str">
-        <v>N/A</v>
+        <v>曾格爾老師詳細描述了她挑戰世��第二高峰K2的艱難過程，包括籌措資金、申請許可證的行政障礙，以及在極地環境中面對的歧視與文化差異。這段內容不僅展現了她堅韌的毅力，也深刻揭示了亞洲探險文化與歐美之間的巨大落差，引人深思。</v>
       </c>
       <c r="X25" t="str">
-        <v>2026-06-20T12:53:14.710Z</v>
+        <v>2026-06-21T00:20:23.884Z</v>
       </c>
     </row>
     <row r="26">
@@ -59668,19 +59668,19 @@
         <v>郝聲音</v>
       </c>
       <c r="C26" t="str">
-        <v>郝聲音：（下）有魚的「已讀Podcast」，如何從閱讀的喜悅，成長到自媒體分享的幸福</v>
+        <v>郝聲音：（下） 蘇絢慧老師好書分享，『隱性內耗』：看不見的傷，如何消磨你的能量？</v>
       </c>
       <c r="D26">
-        <v>260</v>
+        <v>205</v>
       </c>
       <c r="E26" t="str">
         <v>中</v>
       </c>
       <c r="F26" t="str">
-        <v>兩位主講人皆常在句首使用「然後」作為轉折詞，頻率中等偏高。此外，「就是」也常被用於語氣的強調或解釋，而「那」則多用於話題的轉換。偶爾會出現「呃」等語氣詞。</v>
+        <v>主講人（徐瑄惠老師）和主持人（好哥）皆常在句首使用「然後」進行轉折，或使用「就是」、「那」等詞，頻率中等。</v>
       </c>
       <c r="G26" t="str">
-        <v>男主持人（好哥）的聲音低沉厚實，共鳴感強，語調自然且富有情感，沒有機器人般的生硬感。女主持人（有餘）的聲音清晰明亮，語氣充滿活力與熱情，整體聽感溫暖且具陪伴感，沒有刺耳的頻率。</v>
+        <v>男主持人（好哥）聲音中低音共鳴厚實，語調情感豐富且具親和力。女主持人（徐瑄惠老師）聲音圓潤清晰，高音域不刺耳，語氣溫和具陪伴感。</v>
       </c>
       <c r="H26" t="str">
         <v>優</v>
@@ -59695,43 +59695,43 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L26" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。背景環境噪音極低，確保了清晰的對話內容。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低。</v>
       </c>
       <c r="M26" t="str">
-        <v>00:07 - 00:24</v>
+        <v>01:59 - 03:45</v>
       </c>
       <c r="N26" t="str">
-        <v>主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
+        <v>此段落深入探討童年環境如何形塑個人對自我價值的認知，以及如何導致內耗與自我質疑。主講人語氣真摯，情感起伏自然，內容具啟發性，是理解內耗成因的關鍵點。</v>
       </c>
       <c r="O26" t="str">
-        <v>Podcast與自媒體的開場提問</v>
+        <v>N/A</v>
       </c>
       <c r="P26" t="str">
-        <v>00:07 - 00:24</v>
+        <v>N/A</v>
       </c>
       <c r="Q26" t="str">
-        <v>主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
+        <v>N/A</v>
       </c>
       <c r="R26" t="str">
-        <v>Threads平台「內容為王」的獨特魅力</v>
+        <v>N/A</v>
       </c>
       <c r="S26" t="str">
-        <v>05:13 - 06:02</v>
+        <v>N/A</v>
       </c>
       <c r="T26" t="str">
-        <v>來賓深入分析Threads平台「內容為王」的特性，透過生動的案例（只有一個粉絲卻爆紅的貼文）說明其對素人創作者的友善與潛力，展現獨到見解，引人入勝。</v>
+        <v>N/A</v>
       </c>
       <c r="U26" t="str">
-        <v>知識內化與費曼學習法的實踐</v>
+        <v>N/A</v>
       </c>
       <c r="V26" t="str">
-        <v>19:15 - 21:11</v>
+        <v>N/A</v>
       </c>
       <c r="W26" t="str">
-        <v>兩位主持人探討知識分享中「引用權威」與「個人自信」的關係，並引導至費曼學習法，強調將知識內化並應用於自身問題解決的重要性，為聽眾提供實用的學習心態與方法，具啟發性。</v>
+        <v>N/A</v>
       </c>
       <c r="X26" t="str">
-        <v>2026-06-21T00:16:00.733Z</v>
+        <v>2026-06-20T12:53:14.710Z</v>
       </c>
     </row>
     <row r="27">
@@ -59742,19 +59742,19 @@
         <v>郝聲音</v>
       </c>
       <c r="C27" t="str">
-        <v>郝聲音：（下）郝書分享：『值得過上好日子』從情緒消費到聰明投資,克服「不夠花、不敢花」的金錢焦慮、學會建立有安心感的全方位財務計畫</v>
+        <v>郝聲音：（下）有魚的「已讀Podcast」，如何從閱讀的喜悅，成長到自媒體分享的幸福</v>
       </c>
       <c r="D27">
-        <v>290</v>
+        <v>260</v>
       </c>
       <c r="E27" t="str">
         <v>中</v>
       </c>
       <c r="F27" t="str">
-        <v>兩位主持人都常在句首使用「然後」進行轉折，或以「就是」作為語氣詞。男主持人習慣性使用「你知道嗎」、「對不對」來與聽眾互動或確認語意。整體贅字頻率中等。</v>
+        <v>兩位主講人皆常在句首使用「然後」作為轉折詞，頻率中等偏高。此外，「就是」也常被用於語氣的強調或解釋，而「那」則多用於話題的轉換。偶爾會出現「呃」等語氣詞。</v>
       </c>
       <c r="G27" t="str">
-        <v>男主持人聲音中低音共鳴厚實，語調情感豐富，表達流暢且具說服力。女主持人聲音高音域圓潤，語氣溫馨且具陪伴感，表達清晰不刺耳。兩位聲音特質互補，提升節目親和力。</v>
+        <v>男主持人（好哥）的聲音低沉厚實，共鳴感強，語調自然且富有情感，沒有機器人般的生硬感。女主持人（有餘）的聲音清晰明亮，語氣充滿活力與熱情，整體聽感溫暖且具陪伴感，沒有刺耳的頻率。</v>
       </c>
       <c r="H27" t="str">
         <v>優</v>
@@ -59769,43 +59769,43 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L27" t="str">
-        <v>整體錄音品質優良，音量���穩，人聲清晰，沒有突兀爆音與噴麥現象，背景環境音極為乾淨。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。背景環境噪音極低，確保了清晰的對話內容。</v>
       </c>
       <c r="M27" t="str">
-        <v>00:00 - 01:15</v>
+        <v>00:07 - 00:24</v>
       </c>
       <c r="N27" t="str">
-        <v>開場主持人以「財商」與「人生」的關係破題，引導出夫妻間因價值觀差異而產生「火花」的有趣比喻，迅速吸引聽眾對節目主題產生共鳴與好奇。女主持人隨後補充的個人經驗，讓討論更具生活感。</v>
+        <v>主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
       </c>
       <c r="O27" t="str">
-        <v>財商與人生觀的火花</v>
+        <v>Podcast與自媒體的開場提問</v>
       </c>
       <c r="P27" t="str">
-        <v>00:00 - 01:15</v>
+        <v>00:07 - 00:24</v>
       </c>
       <c r="Q27" t="str">
-        <v>開場主持人以「財商」與「人生」的關係破題，引導出夫妻間因價值觀差異而產生「火花」的有趣比喻，迅速吸引聽眾對節目主題產生共鳴與好奇。女主持人隨後補充的個人經驗，讓討論更具生活感。</v>
+        <v>主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
       </c>
       <c r="R27" t="str">
-        <v>「正念」的核心：活在當下與不批判</v>
+        <v>Threads平台「內容為王」的獨特魅力</v>
       </c>
       <c r="S27" t="str">
-        <v>12:42 - 14:22</v>
+        <v>05:13 - 06:02</v>
       </c>
       <c r="T27" t="str">
-        <v>此段落深入解釋了「正念」的兩大核心概念：「活在當下」與「不批判」。女主持人以清晰的邏輯闡述了這兩點對於個人成長和金錢觀念的重要性，特別強調了華人文化中常見的自我批判問題，提供了實用的覺察方法。</v>
+        <v>來賓深入分析Threads平台「內容為王」的特性，透過生動的案例（只有一個粉絲卻爆紅的貼文）說明其對素人創作者的友善與潛力，展現獨到見解，引人入勝。</v>
       </c>
       <c r="U27" t="str">
-        <v>10個「身心安定」的練習方法</v>
+        <v>知識內化與費曼學習法的實踐</v>
       </c>
       <c r="V27" t="str">
-        <v>17:14 - 19:22</v>
+        <v>19:15 - 21:11</v>
       </c>
       <c r="W27" t="str">
-        <v>主持人詳細列舉並簡要說明了書中推薦的10個「身心安定」練習方法，從感官體驗（精油、水晶、音樂、泡澡）到身體活動（呼吸、運動、舞蹈）及心靈實踐（親近自然、書寫、陪伴孩子），提供了具體可行的建議，讓聽眾能���即應用於日常生活中，提升覺察力與幸福感。</v>
+        <v>兩位主持人探討知識分享中「引用權威」與「個人自信」的關係，並引導至費曼學習法，強調將知識內化並應用於自身問題解決的重要性，為聽眾提供實用的學習心態與方法，具啟發性。</v>
       </c>
       <c r="X27" t="str">
-        <v>2026-06-21T00:21:11.061Z</v>
+        <v>2026-06-21T00:16:00.733Z</v>
       </c>
     </row>
     <row r="28">
@@ -59816,19 +59816,19 @@
         <v>郝聲音</v>
       </c>
       <c r="C28" t="str">
-        <v>郝聲音：（下）終於跟MJ林明樟老師合體！用「財務腦」打通「業務力」，讓商業與人生獲利生生不息！</v>
+        <v>郝聲音：（下）郝書分享：『值得過上好日子』從情緒消費到聰明投資,克服「不夠花、不敢花」的金錢焦慮、學會建立有安心感的全方位財務計畫</v>
       </c>
       <c r="D28">
-        <v>250</v>
+        <v>290</v>
       </c>
       <c r="E28" t="str">
         <v>中</v>
       </c>
       <c r="F28" t="str">
-        <v>兩位主講人皆常在句首使用「那」、「然後」或「就是」作為語氣詞或轉折詞，頻率中等，但不會過於頻繁而影響聽感。</v>
+        <v>兩位主持人都常在句首使用「然後」進行轉折，或以「就是」作為語氣詞。男主持人習慣性使用「你知道嗎」、「對不對」來與聽眾互動或確認語意。整體贅字頻率中等。</v>
       </c>
       <c r="G28" t="str">
-        <v>兩位男主持人聲音共鳴感佳，中低音厚實且清晰，語調自然流暢，情感表達豐富，無機器人唸稿感，整體聽感親和且具說服力。</v>
+        <v>男主持人聲音中低音共鳴厚實，語調情感豐富，表達流暢且具說服力。女主持人聲音高音域圓潤，語氣溫馨且具陪伴感，表達清晰不刺耳。兩位聲音特質互補，提升節目親和力。</v>
       </c>
       <c r="H28" t="str">
         <v>優</v>
@@ -59840,69 +59840,69 @@
         <v>無</v>
       </c>
       <c r="K28" t="str">
-        <v>環境安靜，幾乎無底噪，錄音背景非常乾淨。</v>
+        <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L28" t="str">
-        <v>整體錄音品質優良，音量平穩一致，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聆聽體���。</v>
+        <v>整體錄音品質優良，音量���穩，人聲清晰，沒有突兀爆音與噴麥現象，背景環境音極為乾淨。</v>
       </c>
       <c r="M28" t="str">
-        <v>02:28 - 03:46</v>
+        <v>00:00 - 01:15</v>
       </c>
       <c r="N28" t="str">
-        <v>此段落由MJ老師分享個人生病導致公司薪資停發，以及離職後公司仍能良好運作的親身經歷，引導出「系統」的重要性。他以生動的語氣和具體的「1x1x1」乘法概念，深入淺出地解釋了系統運作的關鍵，情感真摯且極具說服力，是理解課程核心理念的精彩片段。</v>
+        <v>開場主持人以「財商」與「人生」的關係破題，引導出夫妻間因價值觀差異而產生「火花」的有趣比喻，迅速吸引聽眾對節目主題產生共鳴與好奇。女主持人隨後補充的個人經驗，讓討論更具生活感。</v>
       </c>
       <c r="O28" t="str">
-        <v>N/A</v>
+        <v>財商與人生觀的火花</v>
       </c>
       <c r="P28" t="str">
-        <v>N/A</v>
+        <v>00:00 - 01:15</v>
       </c>
       <c r="Q28" t="str">
-        <v>N/A</v>
+        <v>開場主持人以「財商」與「人生」的關係破題，引導出夫妻間因價值觀差異而產生「火花」的有趣比喻，迅速吸引聽眾對節目主題產生共鳴與好奇。女主持人隨後補充的個人經驗，讓討論更具生活感。</v>
       </c>
       <c r="R28" t="str">
-        <v>N/A</v>
+        <v>「正念」的核心：活在當下與不批判</v>
       </c>
       <c r="S28" t="str">
-        <v>N/A</v>
+        <v>12:42 - 14:22</v>
       </c>
       <c r="T28" t="str">
-        <v>N/A</v>
+        <v>此段落深入解釋了「正念」的兩大核心概念：「活在當下」與「不批判」。女主持人以清晰的邏輯闡述了這兩點對於個人成長和金錢觀念的重要性，特別強調了華人文化中常見的自我批判問題，提供了實用的覺察方法。</v>
       </c>
       <c r="U28" t="str">
-        <v>N/A</v>
+        <v>10個「身心安定」的練習方法</v>
       </c>
       <c r="V28" t="str">
-        <v>N/A</v>
+        <v>17:14 - 19:22</v>
       </c>
       <c r="W28" t="str">
-        <v>N/A</v>
+        <v>主持人詳細列舉並簡要說明了書中推薦的10個「身心安定」練習方法，從感官體驗（精油、水晶、音樂、泡澡）到身體活動（呼吸、運動、舞蹈）及心靈實踐（親近自然、書寫、陪伴孩子），提供了具體可行的建議，讓聽眾能���即應用於日常生活中，提升覺察力與幸福感。</v>
       </c>
       <c r="X28" t="str">
-        <v>2026-06-20T12:52:38.345Z</v>
+        <v>2026-06-21T00:21:11.061Z</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>郝旭烈/郝聲音</v>
       </c>
       <c r="B29" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>郝聲音</v>
       </c>
       <c r="C29" t="str">
-        <v>#770 賺錢是為了幸福還是徒增焦慮？練習「鬆弛感」與小成就，把寶貴時間還給真正重要的事 來賓：蔡宇哲、郝旭烈</v>
+        <v>郝聲音：（下）終於跟MJ林明樟老師合體！用「財務腦」打通「業務力」，讓商業與人生獲利生生不息！</v>
       </c>
       <c r="D29">
-        <v>205</v>
+        <v>250</v>
       </c>
       <c r="E29" t="str">
         <v>中</v>
       </c>
       <c r="F29" t="str">
-        <v>主持人Sandy常在句首使用「然後」進行轉折，偶爾使用「就是」；蔡宇哲老師和好哥也常使用「那」和「就是」作為語氣詞或連接詞，整體贅字頻率中等，不至於影響理解。</v>
+        <v>兩位主講人皆常在句首使用「那」、「然後」或「就是」作為語氣詞或轉折詞，頻率中等，但不會過於頻繁而影響聽感。</v>
       </c>
       <c r="G29" t="str">
-        <v>女主持人Sandy的聲音清亮、溫暖且充滿活力，高音域圓潤，給人溫馨陪伴感。男主持人蔡宇哲老師的聲音清晰、沉穩，語氣富有說服力。好哥的聲音則低沉厚實，共鳴感強，語調平穩，三位主持人的聲音特質都非常悅耳，沒有刺耳感。</v>
+        <v>兩位男主持人聲音共鳴感佳，中低音厚實且清晰，語調自然流暢，情感表達豐富，無機器人唸稿感，整體聽感親和且具說服力。</v>
       </c>
       <c r="H29" t="str">
         <v>優</v>
@@ -59914,46 +59914,46 @@
         <v>無</v>
       </c>
       <c r="K29" t="str">
-        <v>環境安靜，幾乎無底噪</v>
+        <v>環境安靜，幾乎無底噪，錄音背景非常乾淨。</v>
       </c>
       <c r="L29" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺體驗。</v>
+        <v>整體錄音品質優良，音量平穩一致，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聆聽體���。</v>
       </c>
       <c r="M29" t="str">
-        <v>00:18 - 00:37</v>
+        <v>02:28 - 03:46</v>
       </c>
       <c r="N29" t="str">
-        <v>主持人Sandy以充滿活力的語氣開場，迅速點出許多人追求金錢、事業、成就背後的核心需求——安全感，並進一步提出如何獲得心靈自由的關鍵問題，有效吸引聽眾進入主題。</v>
+        <v>此段落由MJ老師分享個人生病導致公司薪資停發，以及離職後公司仍能良好運作的親身經歷，引導出「系統」的重要性。他以生動的語氣和具體的「1x1x1」乘法概念，深入淺出地解釋了系統運作的關鍵，情感真摯且極具說服力，是理解課程核心理念的精彩片段。</v>
       </c>
       <c r="O29" t="str">
-        <v>追求安全感與心靈自由的開場</v>
+        <v>N/A</v>
       </c>
       <c r="P29" t="str">
-        <v>00:18 - 00:37</v>
+        <v>N/A</v>
       </c>
       <c r="Q29" t="str">
-        <v>主持人Sandy以充滿活力的語氣開場，迅速點出許多人追求金錢、事業、成就背後的核心需求——安全感，並進一步提出如何獲得心靈自由的關鍵問題，有效吸引聽眾進入主題。</v>
+        <v>N/A</v>
       </c>
       <c r="R29" t="str">
-        <v>財富自由的真諦：幸福與意義</v>
+        <v>N/A</v>
       </c>
       <c r="S29" t="str">
-        <v>01:22 - 01:43</v>
+        <v>N/A</v>
       </c>
       <c r="T29" t="str">
-        <v>蔡宇哲老師在此段落深刻剖析財富自由的真正目的，指出金錢最終是為了帶來幸福、快樂與意義，並反思這些是否必須依賴大量金錢才能實現，提供聽眾一個重新思考財富觀的機會。</v>
+        <v>N/A</v>
       </c>
       <c r="U29" t="str">
-        <v>累積小成就，戰勝焦慮</v>
+        <v>N/A</v>
       </c>
       <c r="V29" t="str">
-        <v>07:45 - 08:20</v>
+        <v>N/A</v>
       </c>
       <c r="W29" t="str">
-        <v>好哥與蔡宇哲老師共同探討透過累積小成就來建立自信、戰勝焦慮的實用方法，特別提到「兩分鐘目標」的概念，為聽眾提供了具體且可操作的建議，展現了節目的實用價值和情感連結。</v>
+        <v>N/A</v>
       </c>
       <c r="X29" t="str">
-        <v>2026-06-21T00:31:11.293Z</v>
+        <v>2026-06-20T12:52:38.345Z</v>
       </c>
     </row>
     <row r="30">
@@ -59964,7 +59964,7 @@
         <v>精算媽咪的家計簿</v>
       </c>
       <c r="C30" t="str">
-        <v>#800 買老屋怕踩雷？破解中古屋隱藏價值，聰明挑出高CP值潛力好房！來賓：House123 執行長 邱愛莉 Ellie</v>
+        <v>#770 賺錢是為了幸福還是徒增焦慮？練習「鬆弛感」與小成就，把寶貴時間還給真正重要的事 來賓：蔡宇哲、郝旭烈</v>
       </c>
       <c r="D30">
         <v>205</v>
@@ -59973,10 +59973,10 @@
         <v>中</v>
       </c>
       <c r="F30" t="str">
-        <v>兩位主持人皆有使用「然後」、「就是」、「對啊」、「其實」等口頭禪，尤其在句首作為轉折詞的頻率較高，但整體而言不至於過度影響聽感。</v>
+        <v>主持人Sandy常在句首使用「然後」進行轉折，偶爾使用「就是」；蔡宇哲老師和好哥也常使用「那」和「就是」作為語氣詞或連接詞，整體贅字頻率中等，不至於影響理解。</v>
       </c>
       <c r="G30" t="str">
-        <v>兩位女主持人的聲音皆清晰、圓潤，高音域表現良好，沒有刺耳感。主講人Sandy的語調活潑，具親和力與溫馨陪伴感；來賓Aily的聲音則顯得沉穩專業，共鳴感佳，兩者搭配使對話流暢且富有層次。</v>
+        <v>女主持人Sandy的聲音清亮、溫暖且充滿活力，高音域圓潤，給人溫馨陪伴感。男主持人蔡宇哲老師的聲音清晰、沉穩，語氣富有說服力。好哥的聲音則低沉厚實，共鳴感強，語調平穩，三位主持人的聲音特質都非常悅耳，沒有刺耳感。</v>
       </c>
       <c r="H30" t="str">
         <v>優</v>
@@ -59991,43 +59991,43 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L30" t="str">
-        <v>整體錄音品質優良，音量平穩，���聲清晰，沒有突兀爆音與噴麥現象，背景環境噪音也控制得很好。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺體驗。</v>
       </c>
       <c r="M30" t="str">
-        <v>00:49 - 01:14</v>
+        <v>00:18 - 00:37</v>
       </c>
       <c r="N30" t="str">
-        <v>主持人Sandy以生動的語氣，點出許多人在買房時既期待又害怕受傷害的普遍心態，特別是對於首次購屋者。她簡潔地帶出新舊房子的優缺點，迅速抓住聽眾的注意力，為後續的討論奠定基礎。</v>
+        <v>主持人Sandy以充滿活力的語氣開場，迅速點出許多人追求金錢、事業、成就背後的核心需求——安全感，並進一步提出如何獲得心靈自由的關鍵問題，有效吸引聽眾進入主題。</v>
       </c>
       <c r="O30" t="str">
-        <v>買房的期待與困境</v>
+        <v>追求安全感與心靈自由的開場</v>
       </c>
       <c r="P30" t="str">
-        <v>00:49 - 01:14</v>
+        <v>00:18 - 00:37</v>
       </c>
       <c r="Q30" t="str">
-        <v>主持人Sandy以生動的語氣，點出許多人在買房時既期待又害怕受傷害的普遍心態，特別是對於首次購屋者。她簡潔地帶出新舊房子的優缺點，迅速抓住聽眾的注意力，為後續的討論奠定基礎。</v>
+        <v>主持人Sandy以充滿活力的語氣開場，迅速點出許多人追求金錢、事業、成就背後的核心需求——安全感，並進一步提出如何獲得心靈自由的關鍵問題，有效吸引聽眾進入主題。</v>
       </c>
       <c r="R30" t="str">
-        <v>房屋結構的致命傷：軟弱層與海砂屋</v>
+        <v>財富自由的真諦：幸福與意義</v>
       </c>
       <c r="S30" t="str">
-        <v>05:56 - 07:29</v>
+        <v>01:22 - 01:43</v>
       </c>
       <c r="T30" t="str">
-        <v>來賓Aily在此段落深入淺出地解釋了老屋最關鍵的結構性問題，包括「軟弱層」和「海砂屋」。她強調這些問題的不可逆性，並指出結構安全是購屋時首要考量的因素，提供了極具價值的專業知識，語氣真摯且具說服力。</v>
+        <v>蔡宇哲老師在此段落深刻剖析財富自由的真正目的，指出金錢最終是為了帶來幸福、快樂與意義，並反思這些是否必須依賴大量金錢才能實現，提供聽眾一個重新思考財富觀的機會。</v>
       </c>
       <c r="U30" t="str">
-        <v>投資老屋的退場機制與風險評估</v>
+        <v>累積小成就，戰勝焦慮</v>
       </c>
       <c r="V30" t="str">
-        <v>19:00 - 19:59</v>
+        <v>07:45 - 08:20</v>
       </c>
       <c r="W30" t="str">
-        <v>Aily在此段落從投資角度切入，強調了老屋投資必須具備「退場機制」的重要性。她提醒聽眾不應只依賴都更，而應考慮其他可能的退出方案，例如出租或轉售，為投資者提供了務實且全面的風險評估建議。</v>
+        <v>好哥與蔡宇哲老師共同探討透過累積小成就來建立自信、戰勝焦慮的實用方法，特別提到「兩分鐘目標」的概念，為聽眾提供了具體且可操作的建議，展現了節目的實用價值和情感連結。</v>
       </c>
       <c r="X30" t="str">
-        <v>2026-06-21T00:33:54.344Z</v>
+        <v>2026-06-21T00:31:11.293Z</v>
       </c>
     </row>
     <row r="31">
@@ -60038,19 +60038,19 @@
         <v>精算媽咪的家計簿</v>
       </c>
       <c r="C31" t="str">
-        <v>#805 總在爛工作與錯的感情中輪迴？看懂隱藏的人生劇本，用「自我覺察」找回選擇權！來賓：千里淳風</v>
+        <v>#800 買老屋怕踩雷？破解中古屋隱藏價值，聰明挑出高CP值潛力好房！來賓：House123 執行長 邱愛莉 Ellie</v>
       </c>
       <c r="D31">
-        <v>250</v>
+        <v>205</v>
       </c>
       <c r="E31" t="str">
         <v>中</v>
       </c>
       <c r="F31" t="str">
-        <v>主講人（Cindy）常使用「然後」、「就是」、「對」、「嗯」作為語氣詞或轉折詞。來賓（錢老師）則常使用「其實」、「就是」、「那」、「對」、「嗯」。兩位講者的贅字頻率皆為中等，但語句流暢度不受影響。</v>
+        <v>兩位主持人皆有使用「然後」、「就是」、「對啊」、「其實」等口頭禪，尤其在句首作為轉折詞的頻率較高，但整體而言不至於過度影響聽感。</v>
       </c>
       <c r="G31" t="str">
-        <v>主講人（Cindy）的聲音高音域圓潤，語調活潑，富有溫馨陪伴感，聽起來清晰且不刺耳。來賓（錢老師）的聲音中低音共鳴強，厚實且沉穩，語氣充滿智慧與說服力。</v>
+        <v>兩位女主持人的聲音皆清晰、圓潤，高音域表現良好，沒有刺耳感。主講人Sandy的語調活潑，具親和力與溫馨陪伴感；來賓Aily的聲音則顯得沉穩專業，共鳴感佳，兩者搭配使對話流暢且富有層次。</v>
       </c>
       <c r="H31" t="str">
         <v>優</v>
@@ -60062,69 +60062,69 @@
         <v>無</v>
       </c>
       <c r="K31" t="str">
-        <v>環境安靜，幾乎無底噪，錄音品質極佳。</v>
+        <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L31" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。兩位講者的聲音清晰，背景噪音極低，提供極佳的聽覺體驗。</v>
+        <v>整體錄音品質優良，音量平穩，���聲清晰，沒有突兀爆音與噴麥現象，背景環境噪音也控制得很好。</v>
       </c>
       <c r="M31" t="str">
-        <v>00:50 - 01:14</v>
+        <v>00:49 - 01:14</v>
       </c>
       <c r="N31" t="str">
-        <v>此片段是節目開場的精華，主持人以引人入勝的方式介紹來賓，點出他從講求邏輯與科技的背景，轉變為鑽研命理的獨特經歷。這不僅迅速抓住聽眾的好奇心，也為後續的深度對談奠定基礎，展現了主持人良好的引導能力和來賓故事的吸引力。</v>
+        <v>主持人Sandy以生動的語氣，點出許多人在買房時既期待又害怕受傷害的普遍心態，特別是對於首次購屋者。她簡潔地帶出新舊房子的優缺點，迅速抓住聽眾的注意力，為後續的討論奠定基礎。</v>
       </c>
       <c r="O31" t="str">
-        <v>引人入勝的開場：從科技到命理</v>
+        <v>買房的期待與困境</v>
       </c>
       <c r="P31" t="str">
-        <v>00:50 - 01:14</v>
+        <v>00:49 - 01:14</v>
       </c>
       <c r="Q31" t="str">
-        <v>此片段是節目開場的精華，主持人以引人入勝的方式介紹來賓，點出他從講求邏輯與科技的背景，轉變為鑽研命理的獨特經歷。這不僅迅速抓住聽眾的好奇心，也為後續的深度對談奠定基礎，展現了主持人良好的引導能力和來賓故事的吸引力。</v>
+        <v>主持人Sandy以生動的語氣，點出許多人在買房時既期待又害怕受傷害的普遍心態，特別是對於首次購屋者。她簡潔地帶出新舊房子的優缺點，迅速抓住聽眾的注意力，為後續的討論奠定基礎。</v>
       </c>
       <c r="R31" t="str">
-        <v>改變命運的關鍵：自我覺察與觀察者</v>
+        <v>房屋結構的致命傷：軟弱層與海砂屋</v>
       </c>
       <c r="S31" t="str">
-        <v>07:49 - 09:11</v>
+        <v>05:56 - 07:29</v>
       </c>
       <c r="T31" t="str">
-        <v>此片段深入探討了改變命運的核心觀念——「自我覺察」與「觀察者自我」。來賓以心理學理論結合生活實例（如開車自動駕駛），清晰解釋了人類意識的三個層次，並指出大多數人命運被預設的原因。這段內容不僅具啟發性，也提供了聽眾實際可操作的思維工具，是節目中極具深度和實用價值的論述。</v>
+        <v>來賓Aily在此段落深入淺出地解釋了老屋最關鍵的結構性問題，包括「軟弱層」和「海砂屋」。她強調這些問題的不可逆性，並指出結構安全是購屋時首要考量的因素，提供了極具價值的專業知識，語氣真摯且具說服力。</v>
       </c>
       <c r="U31" t="str">
-        <v>意想不到的改運工具：衣服與食物</v>
+        <v>投資老屋的退場機制與風險評估</v>
       </c>
       <c r="V31" t="str">
-        <v>20:31 - 21:37</v>
+        <v>19:00 - 19:59</v>
       </c>
       <c r="W31" t="str">
-        <v>���片段揭示了兩個最有效且日常的改運工具：衣服和食物。來賓從色彩心理學和五行理論的角度，解釋了這些看似平凡的元素如何直接影響一個人的情緒、能量和運勢。這段內容不僅顛覆了傳統對改運的想像，也提供了具體且易於實踐的方法，讓聽眾能從生活中著手改變，極具趣味性和實用性。</v>
+        <v>Aily在此段落從投資角度切入，強調了老屋投資必須具備「退場機制」的重要性。她提醒聽眾不應只依賴都更，而應考慮其他可能的退出方案，例如出租或轉售，為投資者提供了務實且全面的風險評估建議。</v>
       </c>
       <c r="X31" t="str">
-        <v>2026-06-21T00:33:00.044Z</v>
+        <v>2026-06-21T00:33:54.344Z</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>蕭邦</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="B32" t="str">
-        <v>蕭邦相談室</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="C32" t="str">
-        <v>一被拒絕，就容易自我懷疑</v>
+        <v>#805 總在爛工作與錯的感情中輪迴？看懂隱藏的人生劇本，用「自我覺察」找回選擇權！來賓：千里淳風</v>
       </c>
       <c r="D32">
-        <v>236</v>
+        <v>250</v>
       </c>
       <c r="E32" t="str">
         <v>中</v>
       </c>
       <c r="F32" t="str">
-        <v>主講人常在句首使用「然後」進行轉折，並頻繁使用「其實」來強調或解釋，此外「就是」、「那」也偶爾出現，整體贅字頻率中等。</v>
+        <v>主講人（Cindy）常使用「然後」、「就是」、「對」、「嗯」作為語氣詞或轉折詞。來賓（錢老師）則常使用「其實」、「就是」、「那」、「對」、「嗯」。兩位講者的贅字頻率皆為中等，但語句流暢度不受影響。</v>
       </c>
       <c r="G32" t="str">
-        <v>女主持人聲音清晰溫暖，高音域圓潤不刺耳，語調自然且富有情感，給人溫馨陪伴感。</v>
+        <v>主講人（Cindy）的聲音高音域圓潤，語調活潑，富有溫馨陪伴感，聽起來清晰且不刺耳。來賓（錢老師）的聲音中低音共鳴強，厚實且沉穩，語氣充滿智慧與說服力。</v>
       </c>
       <c r="H32" t="str">
         <v>優</v>
@@ -60136,46 +60136,46 @@
         <v>無</v>
       </c>
       <c r="K32" t="str">
-        <v>環境安靜，幾乎無底噪</v>
+        <v>環境安靜，幾乎無底噪，錄音品質極佳。</v>
       </c>
       <c r="L32" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景環境音處理得非常乾淨。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。兩位講者的聲音清晰，背景噪音極低，提供極佳的聽覺體驗。</v>
       </c>
       <c r="M32" t="str">
-        <v>00:12 - 01:18</v>
+        <v>00:50 - 01:14</v>
       </c>
       <c r="N32" t="str">
-        <v>主講人以自身經歷開場，生動描述過去因他人退費或拒絕而陷入強烈自我懷疑的心理狀態，語氣真摯，能迅速引起聽眾共鳴，並清晰點出本集欲探討的核心問題。</v>
+        <v>此片段是節目開場的精華，主持人以引人入勝的方式介紹來賓，點出他從講求邏輯與科技的背景，轉變為鑽研命理的獨特經歷。這不僅迅速抓住聽眾的好奇心，也為後續的深度對談奠定基礎，展現了主持人良好的引導能力和來賓故事的吸引力。</v>
       </c>
       <c r="O32" t="str">
-        <v>「自我懷疑」的深淵：退費與拒絕帶來的內耗</v>
+        <v>引人入勝的開場：從科技到命理</v>
       </c>
       <c r="P32" t="str">
-        <v>00:12 - 01:18</v>
+        <v>00:50 - 01:14</v>
       </c>
       <c r="Q32" t="str">
-        <v>主講人以自身經歷開場，生動描述過去因他人退費或拒絕而陷入強烈自我懷疑的心理狀態，語氣真摯，能迅速引起聽眾共鳴，並清晰點出本集欲探討的核心問題。</v>
+        <v>此片段是節目開場的精華，主持人以引人入勝的方式介紹來賓，點出他從講求邏輯與科技的背景，轉變為鑽研命理的獨特經歷。這不僅迅速抓住聽眾的好奇心，也為後續的深度對談奠定基礎，展現了主持人良好的引導能力和來賓故事的吸引力。</v>
       </c>
       <c r="R32" t="str">
-        <v>價值與選擇：兩件完全不同的事</v>
+        <v>改變命運的關鍵：自我覺察與觀察者</v>
       </c>
       <c r="S32" t="str">
-        <v>03:59 - 04:32</v>
+        <v>07:49 - 09:11</v>
       </c>
       <c r="T32" t="str">
-        <v>此段落是節目核心觀點的精華，主講人清晰闡述了她如何將「自身價值」與「他人的選擇」區分開來，強調兩者互不衝突，展現了深刻的自我成長與洞察力。語氣堅定而富有啟發性。</v>
+        <v>此片段深入探討了改變命運的核心觀念——「自我覺察」與「觀察者自我」。來賓以心理學理論結合生活實例（如開車自動駕駛），清晰解釋了人類意識的三個層次，並指出大多數人命運被預設的原因。這段內容不僅具啟發性，也提供了聽眾實際可操作的思維工具，是節目中極具深度和實用價值的論述。</v>
       </c>
       <c r="U32" t="str">
-        <v>擺脫自我懷疑：重新定義你的價值</v>
+        <v>意想不到的改運工具：衣服與食物</v>
       </c>
       <c r="V32" t="str">
-        <v>06:30 - 07:06</v>
+        <v>20:31 - 21:37</v>
       </c>
       <c r="W32" t="str">
-        <v>主講人提供具體的實踐建議，引導聽眾在面對拒絕時如何檢視自己的反應，並強調「你的價值是你的事」，為聽眾帶來力量與清晰的指引。結尾語氣溫暖而有力，總結了節目的核心訊息。</v>
+        <v>���片段揭示了兩個最有效且日常的改運工具：衣服和食物。來賓從色彩心理學和五行理論的角度，解釋了這些看似平凡的元素如何直接影響一個人的情緒、能量和運勢。這段內容不僅顛覆了傳統對改運的想像，也提供了具體且易於實踐的方法，讓聽眾能從生活中著手改變，極具趣味性和實用性。</v>
       </c>
       <c r="X32" t="str">
-        <v>2026-06-21T01:52:51.939Z</v>
+        <v>2026-06-21T00:33:00.044Z</v>
       </c>
     </row>
     <row r="33">
@@ -60186,19 +60186,19 @@
         <v>蕭邦相談室</v>
       </c>
       <c r="C33" t="str">
-        <v>人生最難的不是賺錢，而是______</v>
+        <v>一被拒絕，就容易自我懷疑</v>
       </c>
       <c r="D33">
-        <v>200</v>
+        <v>236</v>
       </c>
       <c r="E33" t="str">
         <v>中</v>
       </c>
       <c r="F33" t="str">
-        <v>主講人常使用「就是」、「其實」作為語氣詞或轉折詞，頻率中等，但整體語流仍保持流暢。</v>
+        <v>主講人常在句首使用「然後」進行轉折，並頻繁使用「其實」來強調或解釋，此外「就是」、「那」也偶爾出現，整體贅字頻率中等。</v>
       </c>
       <c r="G33" t="str">
-        <v>女主持人聲音溫暖、圓潤，高音域處理得宜，沒有刺耳感，語調自然且富有情感，給人溫馨的陪伴感。</v>
+        <v>女主持人聲音清晰溫暖，高音域圓潤不刺耳，語調自然且富有情感，給人溫馨陪伴感。</v>
       </c>
       <c r="H33" t="str">
         <v>優</v>
@@ -60213,43 +60213,43 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L33" t="str">
-        <v>整體錄音品質優良，音量穩定，沒有突兀爆音或噴麥現象，背景環境音處理得非常乾淨。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景環境音處理得非常乾淨。</v>
       </c>
       <c r="M33" t="str">
-        <v>00:13 - 00:50</v>
+        <v>00:12 - 01:18</v>
       </c>
       <c r="N33" t="str">
-        <v>主持人以自身經驗切入，點出自由工作者或創業者常陷入的「先拼再說」心態，迅速抓住聽眾的共鳴與注意力，破題精準且引人深思。</v>
+        <v>主講人以自身經歷開場，生動描述過去因他人退費或拒絕而陷入強烈自我懷疑的心理狀態，語氣真摯，能迅速引起聽眾共鳴，並清晰點出本集欲探討的核心問題。</v>
       </c>
       <c r="O33" t="str">
-        <v>「先拼再��」的陷阱</v>
+        <v>「自我懷疑」的深淵：退費與拒絕帶來的內耗</v>
       </c>
       <c r="P33" t="str">
-        <v>00:13 - 00:50</v>
+        <v>00:12 - 01:18</v>
       </c>
       <c r="Q33" t="str">
-        <v>主持人以自身經驗切入，點出自由工作者或創業者常陷入的「先拼再說」心態，迅速抓住聽眾的共鳴與注意力，破題精準且引人深思。</v>
+        <v>主講人以自身經歷開場，生動描述過去因他人退費或拒絕而陷入強烈自我懷疑的心理狀態，語氣真摯，能迅速引起聽眾共鳴，並清晰點出本集欲探討的核心問題。</v>
       </c>
       <c r="R33" t="str">
-        <v>金錢與關係的本質</v>
+        <v>價值與選擇：兩件完全不同的事</v>
       </c>
       <c r="S33" t="str">
-        <v>02:25 - 03:33</v>
+        <v>03:59 - 04:32</v>
       </c>
       <c r="T33" t="str">
-        <v>此段落深入剖析金錢與人際關係的價值，強調金錢可再賺，但時間與關係的不可逆性。主講人語氣真摯，論述深刻，觸及聽眾內心深處的價值觀。</v>
+        <v>此段落是節目核心觀點的精華，主講人清晰闡述了她如何將「自身價值」與「他人的選擇」區分開來，強調兩者互不衝突，展現了深刻的自我成長與洞察力。語氣堅定而富有啟發性。</v>
       </c>
       <c r="U33" t="str">
-        <v>人生不能等，陪伴最珍貴</v>
+        <v>擺脫自我懷疑：重新定義你的價值</v>
       </c>
       <c r="V33" t="str">
-        <v>05:39 - 07:21</v>
+        <v>06:30 - 07:06</v>
       </c>
       <c r="W33" t="str">
-        <v>主持人分享翻看父母老照片的個人感觸，深刻體悟到時間的流逝與陪伴的重要性。這段情感真摯、語氣充滿感染力，是整集的情感高潮，提醒聽眾珍惜當下。</v>
+        <v>主講人提供具體的實踐建議，引導聽眾在面對拒絕時如何檢視自己的反應，並強調「你的價值是你的事」，為聽眾帶來力量與清晰的指引。結尾語氣溫暖而有力，總結了節目的核心訊息。</v>
       </c>
       <c r="X33" t="str">
-        <v>2026-06-21T01:53:23.870Z</v>
+        <v>2026-06-21T01:52:51.939Z</v>
       </c>
     </row>
     <row r="34">
@@ -60260,19 +60260,19 @@
         <v>蕭邦相談室</v>
       </c>
       <c r="C34" t="str">
-        <v>如何度過負面情緒 ？</v>
+        <v>人生最難的不是賺錢，而是______</v>
       </c>
       <c r="D34">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="E34" t="str">
         <v>中</v>
       </c>
       <c r="F34" t="str">
-        <v>主講人常在句首使用「那」作為轉折詞，頻率較高，但多數時候作為語氣連接而非純粹贅字。此外，「就是」和「然後」偶爾出現，整體贅字頻率屬於中等。</v>
+        <v>主講人常使用「就是」、「其實」作為語氣詞或轉折詞，頻率中等，但整體語流仍保持流暢。</v>
       </c>
       <c r="G34" t="str">
-        <v>女主持人聲音溫暖、圓潤，中低音域表現穩定，高音域不刺耳，整體語調富有情感，給人一種溫馨且具陪伴感的聽覺體驗。</v>
+        <v>女主持人聲音溫暖、圓潤，高音域處理得宜，沒有刺耳感，語調自然且富有情感，給人溫馨的陪伴感。</v>
       </c>
       <c r="H34" t="str">
         <v>優</v>
@@ -60287,54 +60287,54 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L34" t="str">
-        <v>整體錄音品質極佳，音量平穩，人聲清晰，沒有任何噴麥、突兀爆音或背景雜音，聽感非常舒���。</v>
+        <v>整體錄音品質優良，音量穩定，沒有突兀爆音或噴麥現象，背景環境音處理得非常乾淨。</v>
       </c>
       <c r="M34" t="str">
-        <v>00:12 - 00:31</v>
+        <v>00:13 - 00:50</v>
       </c>
       <c r="N34" t="str">
-        <v>主持人以自身經歷引出「情緒」這個主題，語氣真誠，迅速建立與聽眾的連結，引人入勝，為節目內容做了很好的鋪墊。</v>
+        <v>主持人以自身經驗切入，點出自由工作者或創業者常陷入的「先拼再說」心態，迅速抓住聽眾的共鳴與注意力，破題精準且引人深思。</v>
       </c>
       <c r="O34" t="str">
-        <v>開場：情緒的引導與個人經驗分享</v>
+        <v>「先拼再��」的陷阱</v>
       </c>
       <c r="P34" t="str">
-        <v>00:12 - 00:31</v>
+        <v>00:13 - 00:50</v>
       </c>
       <c r="Q34" t="str">
-        <v>主持人以自身經歷引出「情緒」這個主題，語氣真誠，迅速建立與聽眾的連結，引人入勝，為節目內容做了很好的鋪墊。</v>
+        <v>主持人以自身經驗切入，點出自由工作者或創業者常陷入的「先拼再說」心態，迅速抓住聽眾的共鳴與注意力，破題精準且引人深思。</v>
       </c>
       <c r="R34" t="str">
-        <v>核心論述：關閉腦袋，讓情緒流動</v>
+        <v>金錢與關係的本質</v>
       </c>
       <c r="S34" t="str">
-        <v>04:05 - 04:55</v>
+        <v>02:25 - 03:33</v>
       </c>
       <c r="T34" t="str">
-        <v>此段落是節目的核心精華，主持人清晰地闡述了處理情緒的關鍵方法——「關閉腦袋，讓情緒自然流動」，並解釋了其背後的原因，提供了具體且實用的建議，極具啟發性。</v>
+        <v>此段落深入剖析金錢與人際關係的價值，強調金錢可再賺，但時間與關係的不可逆性。主講人語氣真摯，論述深刻，觸及聽眾內心深處的價值觀。</v>
       </c>
       <c r="U34" t="str">
-        <v>總結：接受情緒，有效解決問題</v>
+        <v>人生不能等，陪伴最珍貴</v>
       </c>
       <c r="V34" t="str">
-        <v>05:43 - 06:10</v>
+        <v>05:39 - 07:21</v>
       </c>
       <c r="W34" t="str">
-        <v>這段總結了節目主旨，強調接受所有情緒的重要性及其帶來的益處，語氣溫和且具說服力，為聽眾提供正向的啟發，並引導聽眾思考如何有效解決問題。</v>
+        <v>主持人分享翻看父母老照片的個人感觸，深刻體悟到時間的流逝與陪伴的重要性。這段情感真摯、語氣充滿感染力，是整集的情感高潮，提醒聽眾珍惜當下。</v>
       </c>
       <c r="X34" t="str">
-        <v>2026-06-21T00:40:44.043Z</v>
+        <v>2026-06-21T01:53:23.870Z</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Dr Selena</v>
+        <v>蕭邦</v>
       </c>
       <c r="B35" t="str">
-        <v>小資變有錢｜Dr.Selena生活理財王</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="C35" t="str">
-        <v>2026小資族一定要看懂4個關鍵總經變數 !</v>
+        <v>如何度過負面情緒 ？</v>
       </c>
       <c r="D35">
         <v>205</v>
@@ -60343,16 +60343,16 @@
         <v>中</v>
       </c>
       <c r="F35" t="str">
-        <v>兩位主講人皆習慣在句首或句中頻繁使用「就是」、「然後」、「那」作為語氣詞或轉折詞，頻率中等。</v>
+        <v>主講人常在句首使用「那」作為轉折詞，頻率較高，但多數時候作為語氣連接而非純粹贅字。此外，「就是」和「然後」偶爾出現，整體贅字頻率屬於中等。</v>
       </c>
       <c r="G35" t="str">
-        <v>女主持人（Data Selina）的聲音高亢、清晰且充滿活力，語調明亮，給人溫暖且具陪伴感的印象，沒有刺耳感。男主持人（卡爾先生）的聲音低沉、厚實且共鳴感強，語氣沉穩而專業，表達流暢，沒有機器人唸稿感。</v>
+        <v>女主持人聲音溫暖、圓潤，中低音域表現穩定，高音域不刺耳，整體語調富有情感，給人一種溫馨且具陪伴感的聽覺體驗。</v>
       </c>
       <c r="H35" t="str">
         <v>優</v>
       </c>
       <c r="I35" t="str">
-        <v>���</v>
+        <v>無</v>
       </c>
       <c r="J35" t="str">
         <v>無</v>
@@ -60361,43 +60361,43 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L35" t="str">
-        <v>整體錄音品質優良，音量平穩，兩位主講人的聲音清晰，沒有突兀爆音與噴麥現象，背景噪音極低。</v>
+        <v>整體錄音品質極佳，音量平穩，人聲清晰，沒有任何噴麥、突兀爆音或背景雜音，聽感非常舒���。</v>
       </c>
       <c r="M35" t="str">
-        <v>00:07 - 00:57</v>
+        <v>00:12 - 00:31</v>
       </c>
       <c r="N35" t="str">
-        <v>主持人以清晰的語調介紹節目宗旨，並迅速帶入本集主題「小資必學的2024總體經濟」。隨後，她以熱情且專業的方式介紹來賓卡爾先生，卡爾先生的開場白也展現其專業與自信，為節目奠定良好的基調。此段落語速適中，內容引人入勝，有效抓住聽眾注意力。</v>
+        <v>主持人以自身經歷引出「情緒」這個主題，語氣真誠，迅速建立與聽眾的連結，引人入勝，為節目內容做了很好的鋪墊。</v>
       </c>
       <c r="O35" t="str">
-        <v>節目開場與總體經濟專家介紹</v>
+        <v>開場：情緒的引導與個人經驗分享</v>
       </c>
       <c r="P35" t="str">
-        <v>00:07 - 00:57</v>
+        <v>00:12 - 00:31</v>
       </c>
       <c r="Q35" t="str">
-        <v>主持人以清晰的語調介紹節目宗旨，並迅速帶入本集主題「小資必學的2024總體經濟」。隨後，她以熱情且專業的方式介紹來賓卡爾先生，卡爾先生的開場白也展現其專業與自信，為節目奠定良好的基調。此段落語速適中，內容引人入勝，有效抓住聽眾注意力。</v>
+        <v>主持人以自身經歷引出「情緒」這個主題，語氣真誠，迅速建立與聽眾的連結，引人入勝，為節目內容做了很好的鋪墊。</v>
       </c>
       <c r="R35" t="str">
-        <v>居高思危：美股高點與潛在修正風險</v>
+        <v>核心論述：關閉腦袋，讓情緒流動</v>
       </c>
       <c r="S35" t="str">
-        <v>02:58 - 04:43</v>
+        <v>04:05 - 04:55</v>
       </c>
       <c r="T35" t="str">
-        <v>卡爾先生在此段落精闢地指出2024年全球經濟的關鍵詞是「居高思危」。他引用標普500指數創65年新高，並以2000年網路泡沫破裂的歷史經驗為鑑，警示股市可能面臨20-30%的修正。他強調這是「數學的力量」和「週期」���必然，並將美股與台股的連動性納入考量，提醒聽眾做好心理準備。此段論述邏輯清晰，數據支持有力，語氣嚴謹，具高度警示性。</v>
+        <v>此段落是節目的核心精華，主持人清晰地闡述了處理情緒的關鍵方法——「關閉腦袋，讓情緒自然流動」，並解釋了其背後的原因，提供了具體且實用的建議，極具啟發性。</v>
       </c>
       <c r="U35" t="str">
-        <v>美元信用危機與實體黃金的避險策略</v>
+        <v>總結：接受情緒，有效解決問題</v>
       </c>
       <c r="V35" t="str">
-        <v>17:07 - 19:30</v>
+        <v>05:43 - 06:10</v>
       </c>
       <c r="W35" t="str">
-        <v>卡爾先生在此段落深入探討美元信用可能面臨的挑戰，回顧1970年代美國解除美元與黃金掛鉤的歷史，並預測未來幾年美元可能貶值。主持人隨後提出地緣政治風險（如台海緊張）下，美元作為避險工具的有效性，並強調實體黃金在這種情境下的重要性。卡爾先生進一步解釋實體黃金作為唯一非任何國家負債的資產，其信用甚至高於國家信用。這段對話不僅分析了貨幣風險，更提供了具體的避險策略，內容豐富且具實用價值。</v>
+        <v>這段總結了節目主旨，強調接受所有情緒的重要性及其帶來的益處，語氣溫和且具說服力，為聽眾提供正向的啟發，並引導聽眾思考如何有效解決問題。</v>
       </c>
       <c r="X35" t="str">
-        <v>2026-06-21T02:21:27.811Z</v>
+        <v>2026-06-21T00:40:44.043Z</v>
       </c>
     </row>
     <row r="36">
@@ -60408,70 +60408,70 @@
         <v>小資變有錢｜Dr.Selena生活理財王</v>
       </c>
       <c r="C36" t="str">
-        <v>小資族如何成功打造第二條收入曲線：冒牌生的社群品牌經營策略免費教學！</v>
+        <v>2026小資族一定要看懂4個關鍵總經變數 !</v>
       </c>
       <c r="D36">
-        <v>290</v>
+        <v>205</v>
       </c>
       <c r="E36" t="str">
         <v>中</v>
       </c>
       <c r="F36" t="str">
-        <v>主講人與來賓皆頻繁使用「然後」作為語句連接詞或轉折詞，以及「就是」用於解釋或強調。此外，「那」也常作為口頭禪或語氣詞出現。整體贅字頻率屬於中等。</v>
+        <v>兩位主講人皆習慣在句首或句中頻繁使用「就是」、「然後」、「那」作為語氣詞或轉折詞，頻率中等。</v>
       </c>
       <c r="G36" t="str">
-        <v>男主持人（冒牌生）聲音中低音共鳴飽滿，音色厚實且富有磁性，語調變化自然，情感表達真摯，聽感舒適且具說服力。女主持人（Selina）高音域清晰明亮，語速雖快但咬字清楚，聲音圓潤且帶有親和力，整體聽感溫暖且具陪伴感，不刺耳。</v>
+        <v>女主持人（Data Selina）的聲音高亢、清晰且充滿活力，語調明亮，給人溫暖且具陪伴感的印象，沒有刺耳感。男主持人（卡爾先生）的聲音低沉、厚實且共鳴感強，語氣沉穩而專業，表達流暢，沒有機器人唸稿感。</v>
       </c>
       <c r="H36" t="str">
         <v>優</v>
       </c>
       <c r="I36" t="str">
-        <v>無</v>
+        <v>���</v>
       </c>
       <c r="J36" t="str">
         <v>無</v>
       </c>
       <c r="K36" t="str">
-        <v>環境安靜，幾乎無���噪</v>
+        <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L36" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰的聽覺體驗。</v>
+        <v>整體錄音品質優良，音量平穩，兩位主講人的聲音清晰，沒有突兀爆音與噴麥現象，背景噪音極低。</v>
       </c>
       <c r="M36" t="str">
-        <v>00:55 - 01:26</v>
+        <v>00:07 - 00:57</v>
       </c>
       <c r="N36" t="str">
-        <v>主持人熱情介紹嘉賓「冒牌生」及其在社群經營上的專長，並點出本集節目將探討如何透過社群媒體創造主動與被動收入，有效引導聽眾進入主題，為節目奠定良好開場。</v>
+        <v>主持人以清晰的語調介紹節目宗旨，並迅速帶入本集主題「小資必學的2024總體經濟」。隨後，她以熱情且專業的方式介紹來賓卡爾先生，卡爾先生的開場白也展現其專業與自信，為節目奠定良好的基調。此段落語速適中，內容引人入勝，有效抓住聽眾注意力。</v>
       </c>
       <c r="O36" t="str">
-        <v>嘉賓介紹與節目主題</v>
+        <v>節目開場與總體經濟專家介紹</v>
       </c>
       <c r="P36" t="str">
-        <v>00:55 - 01:26</v>
+        <v>00:07 - 00:57</v>
       </c>
       <c r="Q36" t="str">
-        <v>主持人熱情介紹嘉賓「冒牌生」及其在社群經營上的專長，並點出本集節目將探討如何透過社群媒體創造主動與被動收入，有效引導聽眾進入主題，為節目奠定良好開場。</v>
+        <v>主持人以清晰的語調介紹節目宗旨，並迅速帶入本集主題「小資必學的2024總體經濟」。隨後，她以熱情且專業的方式介紹來賓卡爾先生，卡爾先生的開場白也展現其專業與自信，為節目奠定良好的基調。此段落語速適中，內容引人入勝，有效抓住聽眾注意力。</v>
       </c>
       <c r="R36" t="str">
-        <v>成功案例：從洗頭店找到社群藍海</v>
+        <v>居高思危：美股高點與潛在修正風險</v>
       </c>
       <c r="S36" t="str">
-        <v>01:40:45 - 01:48:00</v>
+        <v>02:58 - 04:43</v>
       </c>
       <c r="T36" t="str">
-        <v>冒牌生分享一位學生透過分享洗頭店心得，成功累積大量粉絲的案例。此段落具體展現了如何將個人興趣與在地特色結合，創造獨特且受歡迎的內容，為聽眾提供實用的社群經營啟發，極具參考價值。</v>
+        <v>卡爾先生在此段落精闢地指出2024年全球經濟的關鍵詞是「居高思危」。他引用標普500指數創65年新高，並以2000年網路泡沫破裂的歷史經驗為鑑，警示股市可能面臨20-30%的修正。他強調這是「數學的力量」和「週期」���必然，並將美股與台股的連動性納入考量，提醒聽眾做好心理準備。此段論述邏輯清晰，數據支持有力，語氣嚴謹，具高度警示性。</v>
       </c>
       <c r="U36" t="str">
-        <v>享受創作過程的智慧</v>
+        <v>美元信用危機與實體黃金的避險策略</v>
       </c>
       <c r="V36" t="str">
-        <v>02:21:00 - 02:26:00</v>
+        <v>17:07 - 19:30</v>
       </c>
       <c r="W36" t="str">
-        <v>冒牌生引用《享受吧！一個人的旅行》作者的經歷，闡述了享受創作過程本身的重要性，而非過度追求外在的成就與評價。這段對話深刻且富有哲理，鼓勵聽眾回歸初心，從熱愛的事物中獲得真正的快樂與滿足，��有啟發性。</v>
+        <v>卡爾先生在此段落深入探討美元信用可能面臨的挑戰，回顧1970年代美國解除美元與黃金掛鉤的歷史，並預測未來幾年美元可能貶值。主持人隨後提出地緣政治風險（如台海緊張）下，美元作為避險工具的有效性，並強調實體黃金在這種情境下的重要性。卡爾先生進一步解釋實體黃金作為唯一非任何國家負債的資產，其信用甚至高於國家信用。這段對話不僅分析了貨幣風險，更提供了具體的避險策略，內容豐富且具實用價值。</v>
       </c>
       <c r="X36" t="str">
-        <v>2026-06-21T01:54:11.639Z</v>
+        <v>2026-06-21T02:21:27.811Z</v>
       </c>
     </row>
     <row r="37">
@@ -60482,19 +60482,19 @@
         <v>小資變有錢｜Dr.Selena生活理財王</v>
       </c>
       <c r="C37" t="str">
-        <v>小資愛樂活：用理財，走進千年古文明~此生必走一次的中亞絲路!</v>
+        <v>小資族如何成功打造第二條收入曲線：冒牌生的社群品牌經營策略免費教學！</v>
       </c>
       <c r="D37">
-        <v>270</v>
+        <v>290</v>
       </c>
       <c r="E37" t="str">
         <v>中</v>
       </c>
       <c r="F37" t="str">
-        <v>兩位主持人皆頻繁使用「然後」和「就是」作為語句連接詞，尤其常出現在句首。此外，「那」和「這個」也偶爾出現，整體贅字頻率屬於中等。</v>
+        <v>主講人與來賓皆頻繁使用「然後」作為語句連接詞或轉折詞，以及「就是」用於解釋或強調。此外，「那」也常作為口頭禪或語氣詞出現。整體贅字頻率屬於中等。</v>
       </c>
       <c r="G37" t="str">
-        <v>女主持人Selina的聲音清晰、明亮且充滿活力，高音域圓潤不刺耳，語氣溫暖且具陪伴感。男主持人Domingo的聲音低沉、渾厚且富有共鳴，中低音域表現出色，給人穩重、權威而友善的感覺。兩位主持人的聲音特質都非常適合廣播。</v>
+        <v>男主持人（冒牌生）聲音中低音共鳴飽滿，音色厚實且富有磁性，語調變化自然，情感表達真摯，聽感舒適且具說服力。女主持人（Selina）高音域清晰明亮，語速雖快但咬字清楚，聲音圓潤且帶有親和力，整體聽感溫暖且具陪伴感，不刺耳。</v>
       </c>
       <c r="H37" t="str">
         <v>優</v>
@@ -60506,51 +60506,125 @@
         <v>無</v>
       </c>
       <c r="K37" t="str">
+        <v>環境安靜，幾乎無���噪</v>
+      </c>
+      <c r="L37" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰的聽覺體驗。</v>
+      </c>
+      <c r="M37" t="str">
+        <v>00:55 - 01:26</v>
+      </c>
+      <c r="N37" t="str">
+        <v>主持人熱情介紹嘉賓「冒牌生」及其在社群經營上的專長，並點出本集節目將探討如何透過社群媒體創造主動與被動收入，有效引導聽眾進入主題，為節目奠定良好開場。</v>
+      </c>
+      <c r="O37" t="str">
+        <v>嘉賓介紹與節目主題</v>
+      </c>
+      <c r="P37" t="str">
+        <v>00:55 - 01:26</v>
+      </c>
+      <c r="Q37" t="str">
+        <v>主持人熱情介紹嘉賓「冒牌生」及其在社群經營上的專長，並點出本集節目將探討如何透過社群媒體創造主動與被動收入，有效引導聽眾進入主題，為節目奠定良好開場。</v>
+      </c>
+      <c r="R37" t="str">
+        <v>成功案例：從洗頭店找到社群藍海</v>
+      </c>
+      <c r="S37" t="str">
+        <v>01:40:45 - 01:48:00</v>
+      </c>
+      <c r="T37" t="str">
+        <v>冒牌生分享一位學生透過分享洗頭店心得，成功累積大量粉絲的案例。此段落具體展現了如何將個人興趣與在地特色結合，創造獨特且受歡迎的內容，為聽眾提供實用的社群經營啟發，極具參考價值。</v>
+      </c>
+      <c r="U37" t="str">
+        <v>享受創作過程的智慧</v>
+      </c>
+      <c r="V37" t="str">
+        <v>02:21:00 - 02:26:00</v>
+      </c>
+      <c r="W37" t="str">
+        <v>冒牌生引用《享受吧！一個人的旅行》作者的經歷，闡述了享受創作過程本身的重要性，而非過度追求外在的成就與評價。這段對話深刻且富有哲理，鼓勵聽眾回歸初心，從熱愛的事物中獲得真正的快樂與滿足，��有啟發性。</v>
+      </c>
+      <c r="X37" t="str">
+        <v>2026-06-21T01:54:11.639Z</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Dr Selena</v>
+      </c>
+      <c r="B38" t="str">
+        <v>小資變有錢｜Dr.Selena生活理財王</v>
+      </c>
+      <c r="C38" t="str">
+        <v>小資愛樂活：用理財，走進千年古文明~此生必走一次的中亞絲路!</v>
+      </c>
+      <c r="D38">
+        <v>270</v>
+      </c>
+      <c r="E38" t="str">
+        <v>中</v>
+      </c>
+      <c r="F38" t="str">
+        <v>兩位主持人皆頻繁使用「然後」和「就是」作為語句連接詞，尤其常出現在句首。此外，「那」和「這個」也偶爾出現，整體贅字頻率屬於中等。</v>
+      </c>
+      <c r="G38" t="str">
+        <v>女主持人Selina的聲音清晰、明亮且充滿活力，高音域圓潤不刺耳，語氣溫暖且具陪伴感。男主持人Domingo的聲音低沉、渾厚且富有共鳴，中低音域表現出色，給人穩重、權威而友善的感覺。兩位主持人的聲音特質都非常適合廣播。</v>
+      </c>
+      <c r="H38" t="str">
+        <v>優</v>
+      </c>
+      <c r="I38" t="str">
+        <v>無</v>
+      </c>
+      <c r="J38" t="str">
+        <v>無</v>
+      </c>
+      <c r="K38" t="str">
         <v>環境安靜，幾乎無底噪，僅有極輕微的環境音，不影響聆聽體驗。</v>
       </c>
-      <c r="L37" t="str">
+      <c r="L38" t="str">
         <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，音質清晰。</v>
       </c>
-      <c r="M37" t="str">
+      <c r="M38" t="str">
         <v>01:45 - 02:30</v>
       </c>
-      <c r="N37" t="str">
+      <c r="N38" t="str">
         <v>男主持人Domingo以「世界是一本書」的經典比喻開場，並提出「旅行是無知的解藥」的獨特觀點，深入探討旅行如何打破同溫層、拓展個人價值觀。這段內容富有哲理，語速適中，能有效引導聽眾思考。</v>
       </c>
-      <c r="O37" t="str">
+      <c r="O38" t="str">
         <v>旅遊的意義與世界觀的拓展</v>
       </c>
-      <c r="P37" t="str">
+      <c r="P38" t="str">
         <v>01:45 - 02:30</v>
       </c>
-      <c r="Q37" t="str">
+      <c r="Q38" t="str">
         <v>男主持人Domingo以「世界是一本書」的經典比喻開場，並提出「旅行是無知的解藥」的獨特觀點，深入探討旅行如何打破同溫層、拓展個人價值觀。這段內容富有哲理，語速適中，能有效引導聽眾思考。</v>
       </c>
-      <c r="R37" t="str">
+      <c r="R38" t="str">
         <v>透過旅行認識真實世界</v>
       </c>
-      <c r="S37" t="str">
+      <c r="S38" t="str">
         <v>09:47 - 10:13</v>
       </c>
-      <c r="T37" t="str">
+      <c r="T38" t="str">
         <v>女主持人Selina與Domingo對談，指出媒體塑造的世界觀可能與真實世界存在差異，強調親身旅行才能體驗到更完整的世界。Selina更感性地表達「我旅行，我存在，我幸福」，展現旅行對她生命的重要性，對話真誠且具啟發性。</v>
       </c>
-      <c r="U37" t="str">
+      <c r="U38" t="str">
         <v>旅遊業的挑戰與領隊的辛勞</v>
       </c>
-      <c r="V37" t="str">
+      <c r="V38" t="str">
         <v>12:01 - 12:30</v>
       </c>
-      <c r="W37" t="str">
+      <c r="W38" t="str">
         <v>Selina分享了她帶團去尼泊爾時遇到的修路、坐船等突發狀況，以及旅遊業面臨的天災人禍挑戰，凸顯了領隊和導遊的壓力與辛勞。這段內容真實有趣，讓聽眾對旅遊從��人員的付出有更深的理解與共情。</v>
       </c>
-      <c r="X37" t="str">
+      <c r="X38" t="str">
         <v>2026-06-21T01:55:02.849Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:X37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X38"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: analyze 39 episodes, update Excel and HTML dashboard
</commit_message>
<xml_diff>
--- a/eligible_episodes_pool.xlsx
+++ b/eligible_episodes_pool.xlsx
@@ -57808,7 +57808,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X38"/>
+  <dimension ref="A1:X40"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -59446,22 +59446,22 @@
         <v>分手的99個理由</v>
       </c>
       <c r="C23" t="str">
-        <v>S3.EP92｜刪掉容易，忘掉很難：從軍人到寫故事的人 feat. 林思齊</v>
+        <v>S3.EP81｜越做越愛的關係續命術</v>
       </c>
       <c r="D23">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="E23" t="str">
         <v>中</v>
       </c>
       <c r="F23" t="str">
-        <v>所有主講人皆常在句首使用「然後」作為轉折詞，頻率中等。此外，「就是」、「對」和「那」也常作為語氣詞或連接詞使用，尤其在主持人對話中較為頻繁。</v>
+        <v>兩位主持人皆頻繁使用「就是」、「然後」、「那」作為語句間的轉折詞，Humi也常使用「對」來表示認同或確認，Vito偶爾會發出「嗯」的思考聲。整體而言，贅字頻率中等，雖可察覺但不至於嚴重影響節目流暢度。</v>
       </c>
       <c r="G23" t="str">
-        <v>男主持人畢頭大叔聲音低沉厚實，共鳴感強，語調情感豐富且具感染力。女主持人胡咪聲音清亮有活力，高音域圓潤不刺耳，給人溫馨陪伴感。來賓林思齊聲音沉穩清晰，語氣真摯，富有思考深度。</v>
+        <v>男主持人Vito的聲音低沉厚實，共鳴感強，語調自然且富有情感，能有效傳達訊息，沒有機器人般的生硬感。女主持人Humi的聲音清晰明亮，充滿活力，高音域圓潤不刺耳，��氣溫暖且具親和力，營造出溫馨陪伴的氛圍。</v>
       </c>
       <c r="H23" t="str">
-        <v>��</v>
+        <v>優</v>
       </c>
       <c r="I23" t="str">
         <v>無</v>
@@ -59470,72 +59470,72 @@
         <v>無</v>
       </c>
       <c r="K23" t="str">
-        <v>環境安靜，幾乎無底噪</v>
+        <v>環境安靜，幾乎無底噪，背景音樂與人聲混合得宜。</v>
       </c>
       <c r="L23" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。背景噪音極低，提供清晰舒適的聆聽體驗。</v>
+        <v>整體錄音品質極佳，音量平衡穩定，沒有出現噴麥、突兀爆音或明顯的背景雜音，音質清晰。</v>
       </c>
       <c r="M23" t="str">
-        <v>00:00 - 02:24</v>
+        <v>00:00 - 01:24</v>
       </c>
       <c r="N23" t="str">
-        <v>節目以引人入勝的音樂和旁白開場，迅速帶出「分手」主題。主持人以幽默對話營造輕鬆氛圍，隨後介紹來賓林思齊，並巧妙地引導出他從職業軍人轉型為作家的獨特經歷，成功吸引聽眾對節目核心內容產生興趣。</v>
+        <v>節目開場音樂與口白製作精良，迅速帶入本集主題「性愛」。兩位主持人以輕鬆幽默的對話開場，特別是Vito分享他對性愛重要性從年輕到中年的觀點轉變，引人入勝，有效抓住聽眾注意力。</v>
       </c>
       <c r="O23" t="str">
-        <v>破題精采開場：從軍人到作家，刪不掉的生命故事</v>
+        <v>開場破題：性愛的重要性與中年轉變</v>
       </c>
       <c r="P23" t="str">
-        <v>00:00 - 02:24</v>
+        <v>00:00 - 01:24</v>
       </c>
       <c r="Q23" t="str">
-        <v>節目以引人入勝的音樂和旁白開場，迅速帶出「分手」主題。主持人以幽默對話營造輕鬆氛圍，隨後介紹來賓林思齊，並巧妙地引導出他從職業軍人轉型為作家的獨特經歷，成功吸引聽眾對節目核心內容產生興趣。</v>
+        <v>節目開場音樂與口白製作精良，迅速帶入本集主題「性愛」。兩位主持人以輕鬆幽默的對話開場，特別是Vito分享他對性愛重要性從年輕到中年的觀點轉變，引人入勝，有效抓住聽眾注意力。</v>
       </c>
       <c r="R23" t="str">
-        <v>寫作的轉捩點：從個人情緒到讀者故事的「澆水」過程</v>
+        <v>無性生活背後的深層原因與心結</v>
       </c>
       <c r="S23" t="str">
-        <v>02:40 - 05:55</v>
+        <v>08:18 - 14:35</v>
       </c>
       <c r="T23" t="str">
-        <v>林思齊詳細闡述了他的寫作歷程，從退伍後因個人情緒在社群平台發文，到後來轉變為收集並「灌溉」讀者投稿的故事「種子」。這段內容深入揭示了他獨特的創作理念，以及如何��重投稿者情感核心並在不同平台發布故事的策略，展現了他與讀者之間深刻的連結。</v>
+        <v>Humi精闢地指出無性生活僅是表象，其背後隱藏著更深層的關係問題與未解的心結。Vito以「隱形的地震」比喻關係裂痕，Humi則分享了流產與寵物被送走導致夫妻間產生心結的真實案例，深刻闡述了溝通、理解與情感連結的重要性，是本集的核心論述精華。</v>
       </c>
       <c r="U23" t="str">
-        <v>難以忘懷的投稿：被騙兩次的愛情詐騙故事與情感的脆弱</v>
+        <v>幽默互動：性愛暗號與身心益處大揭密</v>
       </c>
       <c r="V23" t="str">
-        <v>33:00 - 36:00</v>
+        <v>15:33 - 24:47</v>
       </c>
       <c r="W23" t="str">
-        <v>林思齊分享了一個令人心碎的讀者故事，關於一位女性在經歷愛情詐騙後，即使報警仍再次受騙。他對故事細節的描述，包括受害者的脆弱和詐騙者的操縱，深刻地展現了人性的複雜與情感的衝擊。這段內容極具感染力，觸及了信任、背叛和對愛的渴望等普世情感，讓聽眾感受到故事背後的真實與沉重。</v>
+        <v>主持人討論如何用「小暗號」來表達性需求，Humi舉例「歡樂的世界」等幽默對話，展現了良好的互動與趣味性。接著，他們詳細列舉了性愛對免疫系統、心血管、睡眠、大腦、皮膚、骨骼等多方面的生理益處，內容豐富且具說服力，Vito最後的「做愛治百病」總結更是畫龍點睛。</v>
       </c>
       <c r="X23" t="str">
-        <v>2026-06-21T02:35:31.851Z</v>
+        <v>2026-06-21T02:57:22.330Z</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>胡咪老師</v>
       </c>
       <c r="B24" t="str">
-        <v>郝聲音</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="C24" t="str">
-        <v>郝聲音：（上）設計師KiKi，從繪畫到設計的熱愛之路，到引領他人感受設計之美的「走讀」行旅～</v>
+        <v>S3.EP92｜刪掉容易，忘掉很難：從軍人到寫故事的人 feat. 林思齊</v>
       </c>
       <c r="D24">
-        <v>265</v>
+        <v>210</v>
       </c>
       <c r="E24" t="str">
-        <v>高</v>
+        <v>中</v>
       </c>
       <c r="F24" t="str">
-        <v>男主持人常在句首使用「那」和「就是」作為轉折或連接詞，頻率較高。女主持人則較常使用「嗯」、「然後」和「其實」，頻率中等，但整體而言，兩位主持人的贅字頻率偏高。</v>
+        <v>所有主講人皆常在句首使用「然後」作為轉折詞，頻率中等。此外，「就是」、「對」和「那」也常作為語氣詞或連接詞使用，尤其在主持人對話中較為頻繁。</v>
       </c>
       <c r="G24" t="str">
-        <v>男主持人（好哥）中低音共鳴飽滿，聲音厚實且富有磁性，語調變化豐富，充滿活力。女主持人（Kiki）高音域圓潤，聲音清晰溫和，帶有親和力，語氣真誠，無刺耳感。</v>
+        <v>男主持人畢頭大叔聲音低沉厚實，共鳴感強，語調情感豐富且具感染力。女主持人胡咪聲音清亮有活力，高音域圓潤不刺耳，給人溫馨陪伴感。來賓林思齊聲音沉穩清晰，語氣真摯，富有思考深度。</v>
       </c>
       <c r="H24" t="str">
-        <v>優</v>
+        <v>��</v>
       </c>
       <c r="I24" t="str">
         <v>無</v>
@@ -59547,54 +59547,54 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L24" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，聽感舒適。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。背景噪音極低，提供清晰舒適的聆聽體驗。</v>
       </c>
       <c r="M24" t="str">
-        <v>03:36 - 03:47</v>
+        <v>00:00 - 02:24</v>
       </c>
       <c r="N24" t="str">
-        <v>此段落女主持人Kiki分享她從小就對設計有著強烈的內心呼喚，語氣中透露出真誠與堅定。男主持人適時的提問與感嘆「好幸福喔」也為這段對話增添了情感深度，展現了主講人早期的志向與熱情。</v>
+        <v>節目以引人入勝的音樂和旁白開場，迅速帶出「分手」主題。主持人以幽默對話營造輕鬆氛圍，隨後介紹來賓林思齊，並巧妙地引導出他從職業軍人轉型為作家的獨特經歷，成功吸引聽眾對節目核心內容產生興趣。</v>
       </c>
       <c r="O24" t="str">
-        <v>N/A</v>
+        <v>破題精采開場：從軍人到作家，刪不掉的生命故事</v>
       </c>
       <c r="P24" t="str">
-        <v>N/A</v>
+        <v>00:00 - 02:24</v>
       </c>
       <c r="Q24" t="str">
-        <v>N/A</v>
+        <v>節目以引人入勝的音樂和旁白開場，迅速帶出「分手」主題。主持人以幽默對話營造輕鬆氛圍，隨後介紹來賓林思齊，並巧妙地引導出他從職業軍人轉型為作家的獨特經歷，成功吸引聽眾對節目核心內容產生興趣。</v>
       </c>
       <c r="R24" t="str">
-        <v>N/A</v>
+        <v>寫作的轉捩點：從個人情緒到讀者故事的「澆水」過程</v>
       </c>
       <c r="S24" t="str">
-        <v>N/A</v>
+        <v>02:40 - 05:55</v>
       </c>
       <c r="T24" t="str">
-        <v>N/A</v>
+        <v>林思齊詳細闡述了他的寫作歷程，從退伍後因個人情緒在社群平台發文，到後來轉變為收集並「灌溉」讀者投稿的故事「種子」。這段內容深入揭示了他獨特的創作理念，以及如何��重投稿者情感核心並在不同平台發布故事的策略，展現了他與讀者之間深刻的連結。</v>
       </c>
       <c r="U24" t="str">
-        <v>N/A</v>
+        <v>難以忘懷的投稿：被騙兩次的愛情詐騙故事與情感的脆弱</v>
       </c>
       <c r="V24" t="str">
-        <v>N/A</v>
+        <v>33:00 - 36:00</v>
       </c>
       <c r="W24" t="str">
-        <v>N/A</v>
+        <v>林思齊分享了一個令人心碎的讀者故事，關於一位女性在經歷愛情詐騙後，即使報警仍再次受騙。他對故事細節的描述，包括受害者的脆弱和詐騙者的操縱，深刻地展現了人性的複雜與情感的衝擊。這段內容極具感染力，觸及了信任、背叛和對愛的渴望等普世情感，讓聽眾感受到故事背後的真實與沉重。</v>
       </c>
       <c r="X24" t="str">
-        <v>2026-06-20T12:51:53.770Z</v>
+        <v>2026-06-21T02:35:31.851Z</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>胡咪老師</v>
       </c>
       <c r="B25" t="str">
-        <v>郝聲音</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="C25" t="str">
-        <v>郝聲音：（上）曾格爾老師，攀登高峰，不僅是為了超越，更是讓自己能看得更遠</v>
+        <v>S4.EP11｜不要再逼自己讀完整本書了！真正有用的是這一件事 feat.《郝會讀書》郝旭烈（郝哥）</v>
       </c>
       <c r="D25">
         <v>205</v>
@@ -59603,10 +59603,10 @@
         <v>中</v>
       </c>
       <c r="F25" t="str">
-        <v>主講人與來賓在對話中常使用「就是」、「然後」、「對」、「這個」、「那」、「其實」、「就」等詞作為語氣詞或轉折詞。這些詞彙的出現頻率中等，雖然偶爾會打斷語句的流暢性，但整體而言不至於影響理解，且符合口語對話的自然習慣。</v>
+        <v>主講人好哥和Vito大叔常在句首使用「然後」、「就是」、「這個」進行轉折或作為語氣詞，頻率中等。胡Mee的贅字頻率較低。</v>
       </c>
       <c r="G25" t="str">
-        <v>男主持人好哥的聲音低沉厚實，中低音共鳴感強，語調情感豐富且富有親和力，沒有機器人唸稿感。女主持人曾格爾的聲音清亮，高音域圓潤不刺耳，語氣溫暖且具陪伴感，表達清晰。</v>
+        <v>好哥的聲音低沉、厚實且富有共鳴感，語調變化豐富，極具感染力。Vito大叔的聲音也低沉清晰，共鳴感佳。胡Mee的聲音清亮悅耳，高音域圓潤，給人溫馨陪伴感，沒有刺耳的感覺。整體聲音表現優異。</v>
       </c>
       <c r="H25" t="str">
         <v>優</v>
@@ -59621,43 +59621,43 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L25" t="str">
-        <v>整體錄音品質優良，音量平穩，兩位講者的聲音清晰且平衡，沒有突兀爆音與噴麥現象，背景環境噪音極低，提供舒適的聆聽體驗。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聆聽體驗。</v>
       </c>
       <c r="M25" t="str">
-        <v>00:00 - 00:43</v>
+        <v>01:08 - 01:51</v>
       </c>
       <c r="N25" t="str">
-        <v>主持人好哥以充滿熱情的語氣介紹曾格爾老師，並迅速點出她「行者」的身份與攀登多座高山的經歷，特別強調她挑戰的都是非一般人能及的山峰，立即吸引聽眾對這位特別來賓產生好奇與期待，為節目奠定引人入勝的基調。</v>
+        <v>此片段迅速引入來賓好哥的新書《好會讀書》，並清晰闡述其核心概念「四一讀書會」。好哥以生動的語氣解釋了如何透過這種獨特方法輕鬆閱讀，有效吸引聽眾對節目主題產生興趣，是個引人入勝的開場。</v>
       </c>
       <c r="O25" t="str">
-        <v>登山女傑的驚人開場</v>
+        <v>好哥新書與「四一讀書會」概念破題</v>
       </c>
       <c r="P25" t="str">
-        <v>00:00 - 00:43</v>
+        <v>01:08 - 01:51</v>
       </c>
       <c r="Q25" t="str">
-        <v>主持人好哥以充滿熱情的語氣介紹曾格爾老師，並迅速點出她「行者」的身份與攀登多座高山的經歷，特別強調她挑戰的都是非一般人能及的山峰，立即吸引聽眾對這位特別來賓產生好奇與期待，為節目奠定引人入勝的基調。</v>
+        <v>此片段迅速引入來賓好哥的新書《好會讀書》，並清晰闡述其核心概念「四一讀書會」。好哥以生動的語氣解釋了如何透過這種獨特方法輕鬆閱讀，有效吸引聽眾對節目主題產生興趣，是個引人入勝的開場。</v>
       </c>
       <c r="R25" t="str">
-        <v>聖母峰大本營的啟示：登山之路的起點</v>
+        <v>重新定義「閱讀」：從漫畫到Podcast的學習</v>
       </c>
       <c r="S25" t="str">
-        <v>01:45 - 03:19</v>
+        <v>07:30 - 09:05</v>
       </c>
       <c r="T25" t="str">
-        <v>曾格爾老師分享她第一次攀登聖母峰大本營的艱辛與挑戰，以及這次經歷如何讓她反思物質需求，並意識到「呼吸才是唯一真正需要把握的」。這段深刻的個人體悟，是她登山生涯的關鍵轉折點，展現了她對生命與自然的獨特見解，極具啟發性。</v>
+        <v>好哥在此段落挑戰了傳統的閱讀定義，將漫畫、動漫、韓劇、Podcast等多元載體納入學習範疇。他以自身和女兒的經驗為例，說明學習無處不在，有效降低了聽眾對閱讀的心理門檻，展現了廣闊的視野和包容的學習觀，極具啟發性。</v>
       </c>
       <c r="U25" t="str">
-        <v>挑戰K2的幕後辛酸與亞洲探險文化的落差</v>
+        <v>學習的關鍵：連結與共鳴</v>
       </c>
       <c r="V25" t="str">
-        <v>01:22:22 - 01:37:50</v>
+        <v>28:38 - 30:56</v>
       </c>
       <c r="W25" t="str">
-        <v>曾格爾老師詳細描述了她挑戰世��第二高峰K2的艱難過程，包括籌措資金、申請許可證的行政障礙，以及在極地環境中面對的歧視與文化差異。這段內容不僅展現了她堅韌的毅力，也深刻揭示了亞洲探險文化與歐美之間的巨大落差，引人深思。</v>
+        <v>好哥深入剖析了閱讀與學習最核心的關鍵——「連結」與「共鳴」。他強調記憶的重點不在於數量，而在於內容與自身的關聯性，並以生動的例子說明如何將書中智慧內化為個人成長的養分。此段落情感真摯，論述深刻，能引發聽眾強烈的共鳴與反思。</v>
       </c>
       <c r="X25" t="str">
-        <v>2026-06-21T00:20:23.884Z</v>
+        <v>2026-06-21T02:55:29.525Z</v>
       </c>
     </row>
     <row r="26">
@@ -59668,19 +59668,19 @@
         <v>郝聲音</v>
       </c>
       <c r="C26" t="str">
-        <v>郝聲音：（下） 蘇絢慧老師好書分享，『隱性內耗』：看不見的傷，如何消磨你的能量？</v>
+        <v>郝聲音：（上）設計師KiKi，從繪畫到設計的熱愛之路，到引領他人感受設計之美的「走讀」行旅～</v>
       </c>
       <c r="D26">
-        <v>205</v>
+        <v>265</v>
       </c>
       <c r="E26" t="str">
-        <v>中</v>
+        <v>高</v>
       </c>
       <c r="F26" t="str">
-        <v>主講人（徐瑄惠老師）和主持人（好哥）皆常在句首使用「然後」進行轉折，或使用「就是」、「那」等詞，頻率中等。</v>
+        <v>男主持人常在句首使用「那」和「就是」作為轉折或連接詞，頻率較高。女主持人則較常使用「嗯」、「然後」和「其實」，頻率中等，但整體而言，兩位主持人的贅字頻率偏高。</v>
       </c>
       <c r="G26" t="str">
-        <v>男主持人（好哥）聲音中低音共鳴厚實，語調情感豐富且具親和力。女主持人（徐瑄惠老師）聲音圓潤清晰，高音域不刺耳，語氣溫和具陪伴感。</v>
+        <v>男主持人（好哥）中低音共鳴飽滿，聲音厚實且富有磁性，語調變化豐富，充滿活力。女主持人（Kiki）高音域圓潤，聲音清晰溫和，帶有親和力，語氣真誠，無刺耳感。</v>
       </c>
       <c r="H26" t="str">
         <v>優</v>
@@ -59695,13 +59695,13 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L26" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，聽感舒適。</v>
       </c>
       <c r="M26" t="str">
-        <v>01:59 - 03:45</v>
+        <v>03:36 - 03:47</v>
       </c>
       <c r="N26" t="str">
-        <v>此段落深入探討童年環境如何形塑個人對自我價值的認知，以及如何導致內耗與自我質疑。主講人語氣真摯，情感起伏自然，內容具啟發性，是理解內耗成因的關鍵點。</v>
+        <v>此段落女主持人Kiki分享她從小就對設計有著強烈的內心呼喚，語氣中透露出真誠與堅定。男主持人適時的提問與感嘆「好幸福喔」也為這段對話增添了情感深度，展現了主講人早期的志向與熱情。</v>
       </c>
       <c r="O26" t="str">
         <v>N/A</v>
@@ -59731,7 +59731,7 @@
         <v>N/A</v>
       </c>
       <c r="X26" t="str">
-        <v>2026-06-20T12:53:14.710Z</v>
+        <v>2026-06-20T12:51:53.770Z</v>
       </c>
     </row>
     <row r="27">
@@ -59742,19 +59742,19 @@
         <v>郝聲音</v>
       </c>
       <c r="C27" t="str">
-        <v>郝聲音：（下）有魚的「已讀Podcast」，如何從閱讀的喜悅，成長到自媒體分享的幸福</v>
+        <v>郝聲音：（上）曾格爾老師，攀登高峰，不僅是為了超越，更是讓自己能看得更遠</v>
       </c>
       <c r="D27">
-        <v>260</v>
+        <v>205</v>
       </c>
       <c r="E27" t="str">
         <v>中</v>
       </c>
       <c r="F27" t="str">
-        <v>兩位主講人皆常在句首使用「然後」作為轉折詞，頻率中等偏高。此外，「就是」也常被用於語氣的強調或解釋，而「那」則多用於話題的轉換。偶爾會出現「呃」等語氣詞。</v>
+        <v>主講人與來賓在對話中常使用「就是」、「然後」、「對」、「這個」、「那」、「其實」、「就」等詞作為語氣詞或轉折詞。這些詞彙的出現頻率中等，雖然偶爾會打斷語句的流暢性，但整體而言不至於影響理解，且符合口語對話的自然習慣。</v>
       </c>
       <c r="G27" t="str">
-        <v>男主持人（好哥）的聲音低沉厚實，共鳴感強，語調自然且富有情感，沒有機器人般的生硬感。女主持人（有餘）的聲音清晰明亮，語氣充滿活力與熱情，整體聽感溫暖且具陪伴感，沒有刺耳的頻率。</v>
+        <v>男主持人好哥的聲音低沉厚實，中低音共鳴感強，語調情感豐富且富有親和力，沒有機器人唸稿感。女主持人曾格爾的聲音清亮，高音域圓潤不刺耳，語氣溫暖且具陪伴感，表達清晰。</v>
       </c>
       <c r="H27" t="str">
         <v>優</v>
@@ -59769,43 +59769,43 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L27" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。背景環境噪音極低，確保了清晰的對話內容。</v>
+        <v>整體錄音品質優良，音量平穩，兩位講者的聲音清晰且平衡，沒有突兀爆音與噴麥現象，背景環境噪音極低，提供舒適的聆聽體驗。</v>
       </c>
       <c r="M27" t="str">
-        <v>00:07 - 00:24</v>
+        <v>00:00 - 00:43</v>
       </c>
       <c r="N27" t="str">
-        <v>主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
+        <v>主持人好哥以充滿熱情的語氣介紹曾格爾老師，並迅速點出她「行者」的身份與攀登多座高山的經歷，特別強調她挑戰的都是非一般人能及的山峰，立即吸引聽眾對這位特別來賓產生好奇與期待，為節目奠定引人入勝的基調。</v>
       </c>
       <c r="O27" t="str">
-        <v>Podcast與自媒體的開場提問</v>
+        <v>登山女傑的驚人開場</v>
       </c>
       <c r="P27" t="str">
-        <v>00:07 - 00:24</v>
+        <v>00:00 - 00:43</v>
       </c>
       <c r="Q27" t="str">
-        <v>主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
+        <v>主持人好哥以充滿熱情的語氣介紹曾格爾老師，並迅速點出她「行者」的身份與攀登多座高山的經歷，特別強調她挑戰的都是非一般人能及的山峰，立即吸引聽眾對這位特別來賓產生好奇與期待，為節目奠定引人入勝的基調。</v>
       </c>
       <c r="R27" t="str">
-        <v>Threads平台「內容為王」的獨特魅力</v>
+        <v>聖母峰大本營的啟示：登山之路的起點</v>
       </c>
       <c r="S27" t="str">
-        <v>05:13 - 06:02</v>
+        <v>01:45 - 03:19</v>
       </c>
       <c r="T27" t="str">
-        <v>來賓深入分析Threads平台「內容為王」的特性，透過生動的案例（只有一個粉絲卻爆紅的貼文）說明其對素人創作者的友善與潛力，展現獨到見解，引人入勝。</v>
+        <v>曾格爾老師分享她第一次攀登聖母峰大本營的艱辛與挑戰，以及這次經歷如何讓她反思物質需求，並意識到「呼吸才是唯一真正需要把握的」。這段深刻的個人體悟，是她登山生涯的關鍵轉折點，展現了她對生命與自然的獨特見解，極具啟發性。</v>
       </c>
       <c r="U27" t="str">
-        <v>知識內化與費曼學習法的實踐</v>
+        <v>挑戰K2的幕後辛酸與亞洲探險文化的落差</v>
       </c>
       <c r="V27" t="str">
-        <v>19:15 - 21:11</v>
+        <v>01:22:22 - 01:37:50</v>
       </c>
       <c r="W27" t="str">
-        <v>兩位主持人探討知識分享中「引用權威」與「個人自信」的關係，並引導至費曼學習法，強調將知識內化並應用於自身問題解決的重要性，為聽眾提供實用的學習心態與方法，具啟發性。</v>
+        <v>曾格爾老師詳細描述了她挑戰世��第二高峰K2的艱難過程，包括籌措資金、申請許可證的行政障礙，以及在極地環境中面對的歧視與文化差異。這段內容不僅展現了她堅韌的毅力，也深刻揭示了亞洲探險文化與歐美之間的巨大落差，引人深思。</v>
       </c>
       <c r="X27" t="str">
-        <v>2026-06-21T00:16:00.733Z</v>
+        <v>2026-06-21T00:20:23.884Z</v>
       </c>
     </row>
     <row r="28">
@@ -59816,19 +59816,19 @@
         <v>郝聲音</v>
       </c>
       <c r="C28" t="str">
-        <v>郝聲音：（下）郝書分享：『值得過上好日子』從情緒消費到聰明投資,克服「不夠花、不敢花」的金錢焦慮、學會建立有安心感的全方位財務計畫</v>
+        <v>郝聲音：（下） 蘇絢慧老師好書分享，『隱性內耗』：看不見的傷，如何消磨你的能量？</v>
       </c>
       <c r="D28">
-        <v>290</v>
+        <v>205</v>
       </c>
       <c r="E28" t="str">
         <v>中</v>
       </c>
       <c r="F28" t="str">
-        <v>兩位主持人都常在句首使用「然後」進行轉折，或以「就是」作為語氣詞。男主持人習慣性使用「你知道嗎」、「對不對」來與聽眾互動或確認語意。整體贅字頻率中等。</v>
+        <v>主講人（徐瑄惠老師）和主持人（好哥）皆常在句首使用「然後」進行轉折，或使用「就是」、「那」等詞，頻率中等。</v>
       </c>
       <c r="G28" t="str">
-        <v>男主持人聲音中低音共鳴厚實，語調情感豐富，表達流暢且具說服力。女主持人聲音高音域圓潤，語氣溫馨且具陪伴感，表達清晰不刺耳。兩位聲音特質互補，提升節目親和力。</v>
+        <v>男主持人（好哥）聲音中低音共鳴厚實，語調情感豐富且具親和力。女主持人（徐瑄惠老師）聲音圓潤清晰，高音域不刺耳，語氣溫和具陪伴感。</v>
       </c>
       <c r="H28" t="str">
         <v>優</v>
@@ -59843,43 +59843,43 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L28" t="str">
-        <v>整體錄音品質優良，音量���穩，人聲清晰，沒有突兀爆音與噴麥現象，背景環境音極為乾淨。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低。</v>
       </c>
       <c r="M28" t="str">
-        <v>00:00 - 01:15</v>
+        <v>01:59 - 03:45</v>
       </c>
       <c r="N28" t="str">
-        <v>開場主持人以「財商」與「人生」的關係破題，引導出夫妻間因價值觀差異而產生「火花」的有趣比喻，迅速吸引聽眾對節目主題產生共鳴與好奇。女主持人隨後補充的個人經驗，讓討論更具生活感。</v>
+        <v>此段落深入探討童年環境如何形塑個人對自我價值的認知，以及如何導致內耗與自我質疑。主講人語氣真摯，情感起伏自然，內容具啟發性，是理解內耗成因的關鍵點。</v>
       </c>
       <c r="O28" t="str">
-        <v>財商與人生觀的火花</v>
+        <v>N/A</v>
       </c>
       <c r="P28" t="str">
-        <v>00:00 - 01:15</v>
+        <v>N/A</v>
       </c>
       <c r="Q28" t="str">
-        <v>開場主持人以「財商」與「人生」的關係破題，引導出夫妻間因價值觀差異而產生「火花」的有趣比喻，迅速吸引聽眾對節目主題產生共鳴與好奇。女主持人隨後補充的個人經驗，讓討論更具生活感。</v>
+        <v>N/A</v>
       </c>
       <c r="R28" t="str">
-        <v>「正念」的核心：活在當下與不批判</v>
+        <v>N/A</v>
       </c>
       <c r="S28" t="str">
-        <v>12:42 - 14:22</v>
+        <v>N/A</v>
       </c>
       <c r="T28" t="str">
-        <v>此段落深入解釋了「正念」的兩大核心概念：「活在當下」與「不批判」。女主持人以清晰的邏輯闡述了這兩點對於個人成長和金錢觀念的重要性，特別強調了華人文化中常見的自我批判問題，提供了實用的覺察方法。</v>
+        <v>N/A</v>
       </c>
       <c r="U28" t="str">
-        <v>10個「身心安定」的練習方法</v>
+        <v>N/A</v>
       </c>
       <c r="V28" t="str">
-        <v>17:14 - 19:22</v>
+        <v>N/A</v>
       </c>
       <c r="W28" t="str">
-        <v>主持人詳細列舉並簡要說明了書中推薦的10個「身心安定」練習方法，從感官體驗（精油、水晶、音樂、泡澡）到身體活動（呼吸、運動、舞蹈）及心靈實踐（親近自然、書寫、陪伴孩子），提供了具體可行的建議，讓聽眾能���即應用於日常生活中，提升覺察力與幸福感。</v>
+        <v>N/A</v>
       </c>
       <c r="X28" t="str">
-        <v>2026-06-21T00:21:11.061Z</v>
+        <v>2026-06-20T12:53:14.710Z</v>
       </c>
     </row>
     <row r="29">
@@ -59890,19 +59890,19 @@
         <v>郝聲音</v>
       </c>
       <c r="C29" t="str">
-        <v>郝聲音：（下）終於跟MJ林明樟老師合體！用「財務腦」打通「業務力」，讓商業與人生獲利生生不息！</v>
+        <v>郝聲音：（下）有魚的「已讀Podcast」，如何從閱讀的喜悅，成長到自媒體分享的幸福</v>
       </c>
       <c r="D29">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="E29" t="str">
         <v>中</v>
       </c>
       <c r="F29" t="str">
-        <v>兩位主講人皆常在句首使用「那」、「然後」或「就是」作為語氣詞或轉折詞，頻率中等，但不會過於頻繁而影響聽感。</v>
+        <v>兩位主講人皆常在句首使用「然後」作為轉折詞，頻率中等偏高。此外，「就是」也常被用於語氣的強調或解釋，而「那」則多用於話題的轉換。偶爾會出現「呃」等語氣詞。</v>
       </c>
       <c r="G29" t="str">
-        <v>兩位男主持人聲音共鳴感佳，中低音厚實且清晰，語調自然流暢，情感表達豐富，無機器人唸稿感，整體聽感親和且具說服力。</v>
+        <v>男主持人（好哥）的聲音低沉厚實，共鳴感強，語調自然且富有情感，沒有機器人般的生硬感。女主持人（有餘）的聲音清晰明亮，語氣充滿活力與熱情，整體聽感溫暖且具陪伴感，沒有刺耳的頻率。</v>
       </c>
       <c r="H29" t="str">
         <v>優</v>
@@ -59914,69 +59914,69 @@
         <v>無</v>
       </c>
       <c r="K29" t="str">
-        <v>環境安靜，幾乎無底噪，錄音背景非常乾淨。</v>
+        <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L29" t="str">
-        <v>整體錄音品質優良，音量平穩一致，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聆聽體���。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。背景環境噪音極低，確保了清晰的對話內容。</v>
       </c>
       <c r="M29" t="str">
-        <v>02:28 - 03:46</v>
+        <v>00:07 - 00:24</v>
       </c>
       <c r="N29" t="str">
-        <v>此段落由MJ老師分享個人生病導致公司薪資停發，以及離職後公司仍能良好運作的親身經歷，引導出「系統」的重要性。他以生動的語氣和具體的「1x1x1」乘法概念，深入淺出地解釋了系統運作的關鍵，情感真摯且極具說服力，是理解課程核心理念的精彩片段。</v>
+        <v>主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
       </c>
       <c r="O29" t="str">
-        <v>N/A</v>
+        <v>Podcast與自媒體的開場提問</v>
       </c>
       <c r="P29" t="str">
-        <v>N/A</v>
+        <v>00:07 - 00:24</v>
       </c>
       <c r="Q29" t="str">
-        <v>N/A</v>
+        <v>主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
       </c>
       <c r="R29" t="str">
-        <v>N/A</v>
+        <v>Threads平台「內容為王」的獨特魅力</v>
       </c>
       <c r="S29" t="str">
-        <v>N/A</v>
+        <v>05:13 - 06:02</v>
       </c>
       <c r="T29" t="str">
-        <v>N/A</v>
+        <v>來賓深入分析Threads平台「內容為王」的特性，透過生動的案例（只有一個粉絲卻爆紅的貼文）說明其對素人創作者的友善與潛力，展現獨到見解，引人入勝。</v>
       </c>
       <c r="U29" t="str">
-        <v>N/A</v>
+        <v>知識內化與費曼學習法的實踐</v>
       </c>
       <c r="V29" t="str">
-        <v>N/A</v>
+        <v>19:15 - 21:11</v>
       </c>
       <c r="W29" t="str">
-        <v>N/A</v>
+        <v>兩位主持人探討知識分享中「引用權威」與「個人自信」的關係，並引導至費曼學習法，強調將知識內化並應用於自身問題解決的重要性，為聽眾提供實用的學習心態與方法，具啟發性。</v>
       </c>
       <c r="X29" t="str">
-        <v>2026-06-20T12:52:38.345Z</v>
+        <v>2026-06-21T00:16:00.733Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>郝旭烈/郝聲音</v>
       </c>
       <c r="B30" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>郝聲音</v>
       </c>
       <c r="C30" t="str">
-        <v>#770 賺錢是為了幸福還是徒增焦慮？練習「鬆弛感」與小成就，把寶貴時間還給真正重要的事 來賓：蔡宇哲、郝旭烈</v>
+        <v>郝聲音：（下）郝書分享：『值得過上好日子』從情緒消費到聰明投資,克服「不夠花、不敢花」的金錢焦慮、學會建立有安心感的全方位財務計畫</v>
       </c>
       <c r="D30">
-        <v>205</v>
+        <v>290</v>
       </c>
       <c r="E30" t="str">
         <v>中</v>
       </c>
       <c r="F30" t="str">
-        <v>主持人Sandy常在句首使用「然後」進行轉折，偶爾使用「就是」；蔡宇哲老師和好哥也常使用「那」和「就是」作為語氣詞或連接詞，整體贅字頻率中等，不至於影響理解。</v>
+        <v>兩位主持人都常在句首使用「然後」進行轉折，或以「就是」作為語氣詞。男主持人習慣性使用「你知道嗎」、「對不對」來與聽眾互動或確認語意。整體贅字頻率中等。</v>
       </c>
       <c r="G30" t="str">
-        <v>女主持人Sandy的聲音清亮、溫暖且充滿活力，高音域圓潤，給人溫馨陪伴感。男主持人蔡宇哲老師的聲音清晰、沉穩，語氣富有說服力。好哥的聲音則低沉厚實，共鳴感強，語調平穩，三位主持人的聲音特質都非常悅耳，沒有刺耳感。</v>
+        <v>男主持人聲音中低音共鳴厚實，語調情感豐富，表達流暢且具說服力。女主持人聲音高音域圓潤，語氣溫馨且具陪伴感，表達清晰不刺耳。兩位聲音特質互補，提升節目親和力。</v>
       </c>
       <c r="H30" t="str">
         <v>優</v>
@@ -59991,66 +59991,66 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L30" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺體驗。</v>
+        <v>整體錄音品質優良，音量���穩，人聲清晰，沒有突兀爆音與噴麥現象，背景環境音極為乾淨。</v>
       </c>
       <c r="M30" t="str">
-        <v>00:18 - 00:37</v>
+        <v>00:00 - 01:15</v>
       </c>
       <c r="N30" t="str">
-        <v>主持人Sandy以充滿活力的語氣開場，迅速點出許多人追求金錢、事業、成就背後的核心需求——安全感，並進一步提出如何獲得心靈自由的關鍵問題，有效吸引聽眾進入主題。</v>
+        <v>開場主持人以「財商」與「人生」的關係破題，引導出夫妻間因價值觀差異而產生「火花」的有趣比喻，迅速吸引聽眾對節目主題產生共鳴與好奇。女主持人隨後補充的個人經驗，讓討論更具生活感。</v>
       </c>
       <c r="O30" t="str">
-        <v>追求安全感與心靈自由的開場</v>
+        <v>財商與人生觀的火花</v>
       </c>
       <c r="P30" t="str">
-        <v>00:18 - 00:37</v>
+        <v>00:00 - 01:15</v>
       </c>
       <c r="Q30" t="str">
-        <v>主持人Sandy以充滿活力的語氣開場，迅速點出許多人追求金錢、事業、成就背後的核心需求——安全感，並進一步提出如何獲得心靈自由的關鍵問題，有效吸引聽眾進入主題。</v>
+        <v>開場主持人以「財商」與「人生」的關係破題，引導出夫妻間因價值觀差異而產生「火花」的有趣比喻，迅速吸引聽眾對節目主題產生共鳴與好奇。女主持人隨後補充的個人經驗，讓討論更具生活感。</v>
       </c>
       <c r="R30" t="str">
-        <v>財富自由的真諦：幸福與意義</v>
+        <v>「正念」的核心：活在當下與不批判</v>
       </c>
       <c r="S30" t="str">
-        <v>01:22 - 01:43</v>
+        <v>12:42 - 14:22</v>
       </c>
       <c r="T30" t="str">
-        <v>蔡宇哲老師在此段落深刻剖析財富自由的真正目的，指出金錢最終是為了帶來幸福、快樂與意義，並反思這些是否必須依賴大量金錢才能實現，提供聽眾一個重新思考財富觀的機會。</v>
+        <v>此段落深入解釋了「正念」的兩大核心概念：「活在當下」與「不批判」。女主持人以清晰的邏輯闡述了這兩點對於個人成長和金錢觀念的重要性，特別強調了華人文化中常見的自我批判問題，提供了實用的覺察方法。</v>
       </c>
       <c r="U30" t="str">
-        <v>累積小成就，戰勝焦慮</v>
+        <v>10個「身心安定」的練習方法</v>
       </c>
       <c r="V30" t="str">
-        <v>07:45 - 08:20</v>
+        <v>17:14 - 19:22</v>
       </c>
       <c r="W30" t="str">
-        <v>好哥與蔡宇哲老師共同探討透過累積小成就來建立自信、戰勝焦慮的實用方法，特別提到「兩分鐘目標」的概念，為聽眾提供了具體且可操作的建議，展現了節目的實用價值和情感連結。</v>
+        <v>主持人詳細列舉並簡要說明了書中推薦的10個「身心安定」練習方法，從感官體驗（精油、水晶、音樂、泡澡）到身體活動（呼吸、運動、舞蹈）及心靈實踐（親近自然、書寫、陪伴孩子），提供了具體可行的建議，讓聽眾能���即應用於日常生活中，提升覺察力與幸福感。</v>
       </c>
       <c r="X30" t="str">
-        <v>2026-06-21T00:31:11.293Z</v>
+        <v>2026-06-21T00:21:11.061Z</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>郝旭烈/郝聲音</v>
       </c>
       <c r="B31" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>郝聲音</v>
       </c>
       <c r="C31" t="str">
-        <v>#800 買老屋怕踩雷？破解中古屋隱藏價值，聰明挑出高CP值潛力好房！來賓：House123 執行長 邱愛莉 Ellie</v>
+        <v>郝聲音：（下）終於跟MJ林明樟老師合體！用「財務腦」打通「業務力」，讓商業與人生獲利生生不息！</v>
       </c>
       <c r="D31">
-        <v>205</v>
+        <v>250</v>
       </c>
       <c r="E31" t="str">
         <v>中</v>
       </c>
       <c r="F31" t="str">
-        <v>兩位主持人皆有使用「然後」、「就是」、「對啊」、「其實」等口頭禪，尤其在句首作為轉折詞的頻率較高，但整體而言不至於過度影響聽感。</v>
+        <v>兩位主講人皆常在句首使用「那」、「然後」或「就是」作為語氣詞或轉折詞，頻率中等，但不會過於頻繁而影響聽感。</v>
       </c>
       <c r="G31" t="str">
-        <v>兩位女主持人的聲音皆清晰、圓潤，高音域表現良好，沒有刺耳感。主講人Sandy的語調活潑，具親和力與溫馨陪伴感；來賓Aily的聲音則顯得沉穩專業，共鳴感佳，兩者搭配使對話流暢且富有層次。</v>
+        <v>兩位男主持人聲音共鳴感佳，中低音厚實且清晰，語調自然流暢，情感表達豐富，無機器人唸稿感，整體聽感親和且具說服力。</v>
       </c>
       <c r="H31" t="str">
         <v>優</v>
@@ -60062,46 +60062,46 @@
         <v>無</v>
       </c>
       <c r="K31" t="str">
-        <v>環境安靜，幾乎無底噪</v>
+        <v>環境安靜，幾乎無底噪，錄音背景非常乾淨。</v>
       </c>
       <c r="L31" t="str">
-        <v>整體錄音品質優良，音量平穩，���聲清晰，沒有突兀爆音與噴麥現象，背景環境噪音也控制得很好。</v>
+        <v>整體錄音品質優良，音量平穩一致，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聆聽體���。</v>
       </c>
       <c r="M31" t="str">
-        <v>00:49 - 01:14</v>
+        <v>02:28 - 03:46</v>
       </c>
       <c r="N31" t="str">
-        <v>主持人Sandy以生動的語氣，點出許多人在買房時既期待又害怕受傷害的普遍心態，特別是對於首次購屋者。她簡潔地帶出新舊房子的優缺點，迅速抓住聽眾的注意力，為後續的討論奠定基礎。</v>
+        <v>此段落由MJ老師分享個人生病導致公司薪資停發，以及離職後公司仍能良好運作的親身經歷，引導出「系統」的重要性。他以生動的語氣和具體的「1x1x1」乘法概念，深入淺出地解釋了系統運作的關鍵，情感真摯且極具說服力，是理解課程核心理念的精彩片段。</v>
       </c>
       <c r="O31" t="str">
-        <v>買房的期待與困境</v>
+        <v>N/A</v>
       </c>
       <c r="P31" t="str">
-        <v>00:49 - 01:14</v>
+        <v>N/A</v>
       </c>
       <c r="Q31" t="str">
-        <v>主持人Sandy以生動的語氣，點出許多人在買房時既期待又害怕受傷害的普遍心態，特別是對於首次購屋者。她簡潔地帶出新舊房子的優缺點，迅速抓住聽眾的注意力，為後續的討論奠定基礎。</v>
+        <v>N/A</v>
       </c>
       <c r="R31" t="str">
-        <v>房屋結構的致命傷：軟弱層與海砂屋</v>
+        <v>N/A</v>
       </c>
       <c r="S31" t="str">
-        <v>05:56 - 07:29</v>
+        <v>N/A</v>
       </c>
       <c r="T31" t="str">
-        <v>來賓Aily在此段落深入淺出地解釋了老屋最關鍵的結構性問題，包括「軟弱層」和「海砂屋」。她強調這些問題的不可逆性，並指出結構安全是購屋時首要考量的因素，提供了極具價值的專業知識，語氣真摯且具說服力。</v>
+        <v>N/A</v>
       </c>
       <c r="U31" t="str">
-        <v>投資老屋的退場機制與風險評估</v>
+        <v>N/A</v>
       </c>
       <c r="V31" t="str">
-        <v>19:00 - 19:59</v>
+        <v>N/A</v>
       </c>
       <c r="W31" t="str">
-        <v>Aily在此段落從投資角度切入，強調了老屋投資必須具備「退場機制」的重要性。她提醒聽眾不應只依賴都更，而應考慮其他可能的退出方案，例如出租或轉售，為投資者提供了務實且全面的風險評估建議。</v>
+        <v>N/A</v>
       </c>
       <c r="X31" t="str">
-        <v>2026-06-21T00:33:54.344Z</v>
+        <v>2026-06-20T12:52:38.345Z</v>
       </c>
     </row>
     <row r="32">
@@ -60112,19 +60112,19 @@
         <v>精算媽咪的家計簿</v>
       </c>
       <c r="C32" t="str">
-        <v>#805 總在爛工作與錯的感情中輪迴？看懂隱藏的人生劇本，用「自我覺察」找回選擇權！來賓：千里淳風</v>
+        <v>#770 賺錢是為了幸福還是徒增焦慮？練習「鬆弛感」與小成就，把寶貴時間還給真正重要的事 來賓：蔡宇哲、郝旭烈</v>
       </c>
       <c r="D32">
-        <v>250</v>
+        <v>205</v>
       </c>
       <c r="E32" t="str">
         <v>中</v>
       </c>
       <c r="F32" t="str">
-        <v>主講人（Cindy）常使用「然後」、「就是」、「對」、「嗯」作為語氣詞或轉折詞。來賓（錢老師）則常使用「其實」、「就是」、「那」、「對」、「嗯」。兩位講者的贅字頻率皆為中等，但語句流暢度不受影響。</v>
+        <v>主持人Sandy常在句首使用「然後」進行轉折，偶爾使用「就是」；蔡宇哲老師和好哥也常使用「那」和「就是」作為語氣詞或連接詞，整體贅字頻率中等，不至於影響理解。</v>
       </c>
       <c r="G32" t="str">
-        <v>主講人（Cindy）的聲音高音域圓潤，語調活潑，富有溫馨陪伴感，聽起來清晰且不刺耳。來賓（錢老師）的聲音中低音共鳴強，厚實且沉穩，語氣充滿智慧與說服力。</v>
+        <v>女主持人Sandy的聲音清亮、溫暖且充滿活力，高音域圓潤，給人溫馨陪伴感。男主持人蔡宇哲老師的聲音清晰、沉穩，語氣富有說服力。好哥的聲音則低沉厚實，共鳴感強，語調平穩，三位主持人的聲音特質都非常悅耳，沒有刺耳感。</v>
       </c>
       <c r="H32" t="str">
         <v>優</v>
@@ -60136,69 +60136,69 @@
         <v>無</v>
       </c>
       <c r="K32" t="str">
-        <v>環境安靜，幾乎無底噪，錄音品質極佳。</v>
+        <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L32" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。兩位講者的聲音清晰，背景噪音極低，提供極佳的聽覺體驗。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰舒適的聽覺體驗。</v>
       </c>
       <c r="M32" t="str">
-        <v>00:50 - 01:14</v>
+        <v>00:18 - 00:37</v>
       </c>
       <c r="N32" t="str">
-        <v>此片段是節目開場的精華，主持人以引人入勝的方式介紹來賓，點出他從講求邏輯與科技的背景，轉變為鑽研命理的獨特經歷。這不僅迅速抓住聽眾的好奇心，也為後續的深度對談奠定基礎，展現了主持人良好的引導能力和來賓故事的吸引力。</v>
+        <v>主持人Sandy以充滿活力的語氣開場，迅速點出許多人追求金錢、事業、成就背後的核心需求——安全感，並進一步提出如何獲得心靈自由的關鍵問題，有效吸引聽眾進入主題。</v>
       </c>
       <c r="O32" t="str">
-        <v>引人入勝的開場：從科技到命理</v>
+        <v>追求安全感與心靈自由的開場</v>
       </c>
       <c r="P32" t="str">
-        <v>00:50 - 01:14</v>
+        <v>00:18 - 00:37</v>
       </c>
       <c r="Q32" t="str">
-        <v>此片段是節目開場的精華，主持人以引人入勝的方式介紹來賓，點出他從講求邏輯與科技的背景，轉變為鑽研命理的獨特經歷。這不僅迅速抓住聽眾的好奇心，也為後續的深度對談奠定基礎，展現了主持人良好的引導能力和來賓故事的吸引力。</v>
+        <v>主持人Sandy以充滿活力的語氣開場，迅速點出許多人追求金錢、事業、成就背後的核心需求——安全感，並進一步提出如何獲得心靈自由的關鍵問題，有效吸引聽眾進入主題。</v>
       </c>
       <c r="R32" t="str">
-        <v>改變命運的關鍵：自我覺察與觀察者</v>
+        <v>財富自由的真諦：幸福與意義</v>
       </c>
       <c r="S32" t="str">
-        <v>07:49 - 09:11</v>
+        <v>01:22 - 01:43</v>
       </c>
       <c r="T32" t="str">
-        <v>此片段深入探討了改變命運的核心觀念——「自我覺察」與「觀察者自我」。來賓以心理學理論結合生活實例（如開車自動駕駛），清晰解釋了人類意識的三個層次，並指出大多數人命運被預設的原因。這段內容不僅具啟發性，也提供了聽眾實際可操作的思維工具，是節目中極具深度和實用價值的論述。</v>
+        <v>蔡宇哲老師在此段落深刻剖析財富自由的真正目的，指出金錢最終是為了帶來幸福、快樂與意義，並反思這些是否必須依賴大量金錢才能實現，提供聽眾一個重新思考財富觀的機會。</v>
       </c>
       <c r="U32" t="str">
-        <v>意想不到的改運工具：衣服與食物</v>
+        <v>累積小成就，戰勝焦慮</v>
       </c>
       <c r="V32" t="str">
-        <v>20:31 - 21:37</v>
+        <v>07:45 - 08:20</v>
       </c>
       <c r="W32" t="str">
-        <v>���片段揭示了兩個最有效且日常的改運工具：衣服和食物。來賓從色彩心理學和五行理論的角度，解釋了這些看似平凡的元素如何直接影響一個人的情緒、能量和運勢。這段內容不僅顛覆了傳統對改運的想像，也提供了具體且易於實踐的方法，讓聽眾能從生活中著手改變，極具趣味性和實用性。</v>
+        <v>好哥與蔡宇哲老師共同探討透過累積小成就來建立自信、戰勝焦慮的實用方法，特別提到「兩分鐘目標」的概念，為聽眾提供了具體且可操作的建議，展現了節目的實用價值和情感連結。</v>
       </c>
       <c r="X32" t="str">
-        <v>2026-06-21T00:33:00.044Z</v>
+        <v>2026-06-21T00:31:11.293Z</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>蕭邦</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="B33" t="str">
-        <v>蕭邦相談室</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="C33" t="str">
-        <v>一被拒絕，就容易自我懷疑</v>
+        <v>#800 買老屋怕踩雷？破解中古屋隱藏價值，聰明挑出高CP值潛力好房！來賓：House123 執行長 邱愛莉 Ellie</v>
       </c>
       <c r="D33">
-        <v>236</v>
+        <v>205</v>
       </c>
       <c r="E33" t="str">
         <v>中</v>
       </c>
       <c r="F33" t="str">
-        <v>主講人常在句首使用「然後」進行轉折，並頻繁使用「其實」來強調或解釋，此外「就是」、「那」也偶爾出現，整體贅字頻率中等。</v>
+        <v>兩位主持人皆有使用「然後」、「就是」、「對啊」、「其實」等口頭禪，尤其在句首作為轉折詞的頻率較高，但整體而言不至於過度影響聽感。</v>
       </c>
       <c r="G33" t="str">
-        <v>女主持人聲音清晰溫暖，高音域圓潤不刺耳，語調自然且富有情感，給人溫馨陪伴感。</v>
+        <v>兩位女主持人的聲音皆清晰、圓潤，高音域表現良好，沒有刺耳感。主講人Sandy的語調活潑，具親和力與溫馨陪伴感；來賓Aily的聲音則顯得沉穩專業，共鳴感佳，兩者搭配使對話流暢且富有層次。</v>
       </c>
       <c r="H33" t="str">
         <v>優</v>
@@ -60213,66 +60213,66 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L33" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景環境音處理得非常乾淨。</v>
+        <v>整體錄音品質優良，音量平穩，���聲清晰，沒有突兀爆音與噴麥現象，背景環境噪音也控制得很好。</v>
       </c>
       <c r="M33" t="str">
-        <v>00:12 - 01:18</v>
+        <v>00:49 - 01:14</v>
       </c>
       <c r="N33" t="str">
-        <v>主講人以自身經歷開場，生動描述過去因他人退費或拒絕而陷入強烈自我懷疑的心理狀態，語氣真摯，能迅速引起聽眾共鳴，並清晰點出本集欲探討的核心問題。</v>
+        <v>主持人Sandy以生動的語氣，點出許多人在買房時既期待又害怕受傷害的普遍心態，特別是對於首次購屋者。她簡潔地帶出新舊房子的優缺點，迅速抓住聽眾的注意力，為後續的討論奠定基礎。</v>
       </c>
       <c r="O33" t="str">
-        <v>「自我懷疑」的深淵：退費與拒絕帶來的內耗</v>
+        <v>買房的期待與困境</v>
       </c>
       <c r="P33" t="str">
-        <v>00:12 - 01:18</v>
+        <v>00:49 - 01:14</v>
       </c>
       <c r="Q33" t="str">
-        <v>主講人以自身經歷開場，生動描述過去因他人退費或拒絕而陷入強烈自我懷疑的心理狀態，語氣真摯，能迅速引起聽眾共鳴，並清晰點出本集欲探討的核心問題。</v>
+        <v>主持人Sandy以生動的語氣，點出許多人在買房時既期待又害怕受傷害的普遍心態，特別是對於首次購屋者。她簡潔地帶出新舊房子的優缺點，迅速抓住聽眾的注意力，為後續的討論奠定基礎。</v>
       </c>
       <c r="R33" t="str">
-        <v>價值與選擇：兩件完全不同的事</v>
+        <v>房屋結構的致命傷：軟弱層與海砂屋</v>
       </c>
       <c r="S33" t="str">
-        <v>03:59 - 04:32</v>
+        <v>05:56 - 07:29</v>
       </c>
       <c r="T33" t="str">
-        <v>此段落是節目核心觀點的精華，主講人清晰闡述了她如何將「自身價值」與「他人的選擇」區分開來，強調兩者互不衝突，展現了深刻的自我成長與洞察力。語氣堅定而富有啟發性。</v>
+        <v>來賓Aily在此段落深入淺出地解釋了老屋最關鍵的結構性問題，包括「軟弱層」和「海砂屋」。她強調這些問題的不可逆性，並指出結構安全是購屋時首要考量的因素，提供了極具價值的專業知識，語氣真摯且具說服力。</v>
       </c>
       <c r="U33" t="str">
-        <v>擺脫自我懷疑：重新定義你的價值</v>
+        <v>投資老屋的退場機制與風險評估</v>
       </c>
       <c r="V33" t="str">
-        <v>06:30 - 07:06</v>
+        <v>19:00 - 19:59</v>
       </c>
       <c r="W33" t="str">
-        <v>主講人提供具體的實踐建議，引導聽眾在面對拒絕時如何檢視自己的反應，並強調「你的價值是你的事」，為聽眾帶來力量與清晰的指引。結尾語氣溫暖而有力，總結了節目的核心訊息。</v>
+        <v>Aily在此段落從投資角度切入，強調了老屋投資必須具備「退場機制」的重要性。她提醒聽眾不應只依賴都更，而應考慮其他可能的退出方案，例如出租或轉售，為投資者提供了務實且全面的風險評估建議。</v>
       </c>
       <c r="X33" t="str">
-        <v>2026-06-21T01:52:51.939Z</v>
+        <v>2026-06-21T00:33:54.344Z</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>蕭邦</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="B34" t="str">
-        <v>蕭邦相談室</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="C34" t="str">
-        <v>人生最難的不是賺錢，而是______</v>
+        <v>#805 總在爛工作與錯的感情中輪迴？看懂隱藏的人生劇本，用「自我覺察」找回選擇權！來賓：千里淳風</v>
       </c>
       <c r="D34">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="E34" t="str">
         <v>中</v>
       </c>
       <c r="F34" t="str">
-        <v>主講人常使用「就是」、「其實」作為語氣詞或轉折詞，頻率中等，但整體語流仍保持流暢。</v>
+        <v>主講人（Cindy）常使用「然後」、「就是」、「對」、「嗯」作為語氣詞或轉折詞。來賓（錢老師）則常使用「其實」、「就是」、「那」、「對」、「嗯」。兩位講者的贅字頻率皆為中等，但語句流暢度不受影響。</v>
       </c>
       <c r="G34" t="str">
-        <v>女主持人聲音溫暖、圓潤，高音域處理得宜，沒有刺耳感，語調自然且富有情感，給人溫馨的陪伴感。</v>
+        <v>主講人（Cindy）的聲音高音域圓潤，語調活潑，富有溫馨陪伴感，聽起來清晰且不刺耳。來賓（錢老師）的聲音中低音共鳴強，厚實且沉穩，語氣充滿智慧與說服力。</v>
       </c>
       <c r="H34" t="str">
         <v>優</v>
@@ -60284,46 +60284,46 @@
         <v>無</v>
       </c>
       <c r="K34" t="str">
-        <v>環境安靜，幾乎無底噪</v>
+        <v>環境安靜，幾乎無底噪，錄音品質極佳。</v>
       </c>
       <c r="L34" t="str">
-        <v>整體錄音品質優良，音量穩定，沒有突兀爆音或噴麥現象，背景環境音處理得非常乾淨。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象。兩位講者的聲音清晰，背景噪音極低，提供極佳的聽覺體驗。</v>
       </c>
       <c r="M34" t="str">
-        <v>00:13 - 00:50</v>
+        <v>00:50 - 01:14</v>
       </c>
       <c r="N34" t="str">
-        <v>主持人以自身經驗切入，點出自由工作者或創業者常陷入的「先拼再說」心態，迅速抓住聽眾的共鳴與注意力，破題精準且引人深思。</v>
+        <v>此片段是節目開場的精華，主持人以引人入勝的方式介紹來賓，點出他從講求邏輯與科技的背景，轉變為鑽研命理的獨特經歷。這不僅迅速抓住聽眾的好奇心，也為後續的深度對談奠定基礎，展現了主持人良好的引導能力和來賓故事的吸引力。</v>
       </c>
       <c r="O34" t="str">
-        <v>「先拼再��」的陷阱</v>
+        <v>引人入勝的開場：從科技到命理</v>
       </c>
       <c r="P34" t="str">
-        <v>00:13 - 00:50</v>
+        <v>00:50 - 01:14</v>
       </c>
       <c r="Q34" t="str">
-        <v>主持人以自身經驗切入，點出自由工作者或創業者常陷入的「先拼再說」心態，迅速抓住聽眾的共鳴與注意力，破題精準且引人深思。</v>
+        <v>此片段是節目開場的精華，主持人以引人入勝的方式介紹來賓，點出他從講求邏輯與科技的背景，轉變為鑽研命理的獨特經歷。這不僅迅速抓住聽眾的好奇心，也為後續的深度對談奠定基礎，展現了主持人良好的引導能力和來賓故事的吸引力。</v>
       </c>
       <c r="R34" t="str">
-        <v>金錢與關係的本質</v>
+        <v>改變命運的關鍵：自我覺察與觀察者</v>
       </c>
       <c r="S34" t="str">
-        <v>02:25 - 03:33</v>
+        <v>07:49 - 09:11</v>
       </c>
       <c r="T34" t="str">
-        <v>此段落深入剖析金錢與人際關係的價值，強調金錢可再賺，但時間與關係的不可逆性。主講人語氣真摯，論述深刻，觸及聽眾內心深處的價值觀。</v>
+        <v>此片段深入探討了改變命運的核心觀念——「自我覺察」與「觀察者自我」。來賓以心理學理論結合生活實例（如開車自動駕駛），清晰解釋了人類意識的三個層次，並指出大多數人命運被預設的原因。這段內容不僅具啟發性，也提供了聽眾實際可操作的思維工具，是節目中極具深度和實用價值的論述。</v>
       </c>
       <c r="U34" t="str">
-        <v>人生不能等，陪伴最珍貴</v>
+        <v>意想不到的改運工具：衣服與食物</v>
       </c>
       <c r="V34" t="str">
-        <v>05:39 - 07:21</v>
+        <v>20:31 - 21:37</v>
       </c>
       <c r="W34" t="str">
-        <v>主持人分享翻看父母老照片的個人感觸，深刻體悟到時間的流逝與陪伴的重要性。這段情感真摯、語氣充滿感染力，是整集的情感高潮，提醒聽眾珍惜當下。</v>
+        <v>���片段揭示了兩個最有效且日常的改運工具：衣服和食物。來賓從色彩心理學和五行理論的角度，解釋了這些看似平凡的元素如何直接影響一個人的情緒、能量和運勢。這段內容不僅顛覆了傳統對改運的想像，也提供了具體且易於實踐的方法，讓聽眾能從生活中著手改變，極具趣味性和實用性。</v>
       </c>
       <c r="X34" t="str">
-        <v>2026-06-21T01:53:23.870Z</v>
+        <v>2026-06-21T00:33:00.044Z</v>
       </c>
     </row>
     <row r="35">
@@ -60334,19 +60334,19 @@
         <v>蕭邦相談室</v>
       </c>
       <c r="C35" t="str">
-        <v>如何度過負面情緒 ？</v>
+        <v>一被拒絕，就容易自我懷疑</v>
       </c>
       <c r="D35">
-        <v>205</v>
+        <v>236</v>
       </c>
       <c r="E35" t="str">
         <v>中</v>
       </c>
       <c r="F35" t="str">
-        <v>主講人常在句首使用「那」作為轉折詞，頻率較高，但多數時候作為語氣連接而非純粹贅字。此外，「就是」和「然後」偶爾出現，整體贅字頻率屬於中等。</v>
+        <v>主講人常在句首使用「然後」進行轉折，並頻繁使用「其實」來強調或解釋，此外「就是」、「那」也偶爾出現，整體贅字頻率中等。</v>
       </c>
       <c r="G35" t="str">
-        <v>女主持人聲音溫暖、圓潤，中低音域表現穩定，高音域不刺耳，整體語調富有情感，給人一種溫馨且具陪伴感的聽覺體驗。</v>
+        <v>女主持人聲音清晰溫暖，高音域圓潤不刺耳，語調自然且富有情感，給人溫馨陪伴感。</v>
       </c>
       <c r="H35" t="str">
         <v>優</v>
@@ -60361,72 +60361,72 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L35" t="str">
-        <v>整體錄音品質極佳，音量平穩，人聲清晰，沒有任何噴麥、突兀爆音或背景雜音，聽感非常舒���。</v>
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景環境音處理得非常乾淨。</v>
       </c>
       <c r="M35" t="str">
-        <v>00:12 - 00:31</v>
+        <v>00:12 - 01:18</v>
       </c>
       <c r="N35" t="str">
-        <v>主持人以自身經歷引出「情緒」這個主題，語氣真誠，迅速建立與聽眾的連結，引人入勝，為節目內容做了很好的鋪墊。</v>
+        <v>主講人以自身經歷開場，生動描述過去因他人退費或拒絕而陷入強烈自我懷疑的心理狀態，語氣真摯，能迅速引起聽眾共鳴，並清晰點出本集欲探討的核心問題。</v>
       </c>
       <c r="O35" t="str">
-        <v>開場：情緒的引導與個人經驗分享</v>
+        <v>「自我懷疑」的深淵：退費與拒絕帶來的內耗</v>
       </c>
       <c r="P35" t="str">
-        <v>00:12 - 00:31</v>
+        <v>00:12 - 01:18</v>
       </c>
       <c r="Q35" t="str">
-        <v>主持人以自身經歷引出「情緒」這個主題，語氣真誠，迅速建立與聽眾的連結，引人入勝，為節目內容做了很好的鋪墊。</v>
+        <v>主講人以自身經歷開場，生動描述過去因他人退費或拒絕而陷入強烈自我懷疑的心理狀態，語氣真摯，能迅速引起聽眾共鳴，並清晰點出本集欲探討的核心問題。</v>
       </c>
       <c r="R35" t="str">
-        <v>核心論述：關閉腦袋，讓情緒流動</v>
+        <v>價值與選擇：兩件完全不同的事</v>
       </c>
       <c r="S35" t="str">
-        <v>04:05 - 04:55</v>
+        <v>03:59 - 04:32</v>
       </c>
       <c r="T35" t="str">
-        <v>此段落是節目的核心精華，主持人清晰地闡述了處理情緒的關鍵方法——「關閉腦袋，讓情緒自然流動」，並解釋了其背後的原因，提供了具體且實用的建議，極具啟發性。</v>
+        <v>此段落是節目核心觀點的精華，主講人清晰闡述了她如何將「自身價值」與「他人的選擇」區分開來，強調兩者互不衝突，展現了深刻的自我成長與洞察力。語氣堅定而富有啟發性。</v>
       </c>
       <c r="U35" t="str">
-        <v>總結：接受情緒，有效解決問題</v>
+        <v>擺脫自我懷疑：重新定義你的價值</v>
       </c>
       <c r="V35" t="str">
-        <v>05:43 - 06:10</v>
+        <v>06:30 - 07:06</v>
       </c>
       <c r="W35" t="str">
-        <v>這段總結了節目主旨，強調接受所有情緒的重要性及其帶來的益處，語氣溫和且具說服力，為聽眾提供正向的啟發，並引導聽眾思考如何有效解決問題。</v>
+        <v>主講人提供具體的實踐建議，引導聽眾在面對拒絕時如何檢視自己的反應，並強調「你的價值是你的事」，為聽眾帶來力量與清晰的指引。結尾語氣溫暖而有力，總結了節目的核心訊息。</v>
       </c>
       <c r="X35" t="str">
-        <v>2026-06-21T00:40:44.043Z</v>
+        <v>2026-06-21T01:52:51.939Z</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Dr Selena</v>
+        <v>蕭邦</v>
       </c>
       <c r="B36" t="str">
-        <v>小資變有錢｜Dr.Selena生活理財王</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="C36" t="str">
-        <v>2026小資族一定要看懂4個關鍵總經變數 !</v>
+        <v>人生最難的不是賺錢，而是______</v>
       </c>
       <c r="D36">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="E36" t="str">
         <v>中</v>
       </c>
       <c r="F36" t="str">
-        <v>兩位主講人皆習慣在句首或句中頻繁使用「就是」、「然後」、「那」作為語氣詞或轉折詞，頻率中等。</v>
+        <v>主講人常使用「就是」、「其實」作為語氣詞或轉折詞，頻率中等，但整體語流仍保持流暢。</v>
       </c>
       <c r="G36" t="str">
-        <v>女主持人（Data Selina）的聲音高亢、清晰且充滿活力，語調明亮，給人溫暖且具陪伴感的印象，沒有刺耳感。男主持人（卡爾先生）的聲音低沉、厚實且共鳴感強，語氣沉穩而專業，表達流暢，沒有機器人唸稿感。</v>
+        <v>女主持人聲音溫暖、圓潤，高音域處理得宜，沒有刺耳感，語調自然且富有情感，給人溫馨的陪伴感。</v>
       </c>
       <c r="H36" t="str">
         <v>優</v>
       </c>
       <c r="I36" t="str">
-        <v>���</v>
+        <v>無</v>
       </c>
       <c r="J36" t="str">
         <v>無</v>
@@ -60435,66 +60435,66 @@
         <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L36" t="str">
-        <v>整體錄音品質優良，音量平穩，兩位主講人的聲音清晰，沒有突兀爆音與噴麥現象，背景噪音極低。</v>
+        <v>整體錄音品質優良，音量穩定，沒有突兀爆音或噴麥現象，背景環境音處理得非常乾淨。</v>
       </c>
       <c r="M36" t="str">
-        <v>00:07 - 00:57</v>
+        <v>00:13 - 00:50</v>
       </c>
       <c r="N36" t="str">
-        <v>主持人以清晰的語調介紹節目宗旨，並迅速帶入本集主題「小資必學的2024總體經濟」。隨後，她以熱情且專業的方式介紹來賓卡爾先生，卡爾先生的開場白也展現其專業與自信，為節目奠定良好的基調。此段落語速適中，內容引人入勝，有效抓住聽眾注意力。</v>
+        <v>主持人以自身經驗切入，點出自由工作者或創業者常陷入的「先拼再說」心態，迅速抓住聽眾的共鳴與注意力，破題精準且引人深思。</v>
       </c>
       <c r="O36" t="str">
-        <v>節目開場與總體經濟專家介紹</v>
+        <v>「先拼再��」的陷阱</v>
       </c>
       <c r="P36" t="str">
-        <v>00:07 - 00:57</v>
+        <v>00:13 - 00:50</v>
       </c>
       <c r="Q36" t="str">
-        <v>主持人以清晰的語調介紹節目宗旨，並迅速帶入本集主題「小資必學的2024總體經濟」。隨後，她以熱情且專業的方式介紹來賓卡爾先生，卡爾先生的開場白也展現其專業與自信，為節目奠定良好的基調。此段落語速適中，內容引人入勝，有效抓住聽眾注意力。</v>
+        <v>主持人以自身經驗切入，點出自由工作者或創業者常陷入的「先拼再說」心態，迅速抓住聽眾的共鳴與注意力，破題精準且引人深思。</v>
       </c>
       <c r="R36" t="str">
-        <v>居高思危：美股高點與潛在修正風險</v>
+        <v>金錢與關係的本質</v>
       </c>
       <c r="S36" t="str">
-        <v>02:58 - 04:43</v>
+        <v>02:25 - 03:33</v>
       </c>
       <c r="T36" t="str">
-        <v>卡爾先生在此段落精闢地指出2024年全球經濟的關鍵詞是「居高思危」。他引用標普500指數創65年新高，並以2000年網路泡沫破裂的歷史經驗為鑑，警示股市可能面臨20-30%的修正。他強調這是「數學的力量」和「週期」���必然，並將美股與台股的連動性納入考量，提醒聽眾做好心理準備。此段論述邏輯清晰，數據支持有力，語氣嚴謹，具高度警示性。</v>
+        <v>此段落深入剖析金錢與人際關係的價值，強調金錢可再賺，但時間與關係的不可逆性。主講人語氣真摯，論述深刻，觸及聽眾內心深處的價值觀。</v>
       </c>
       <c r="U36" t="str">
-        <v>美元信用危機與實體黃金的避險策略</v>
+        <v>人生不能等，陪伴最珍貴</v>
       </c>
       <c r="V36" t="str">
-        <v>17:07 - 19:30</v>
+        <v>05:39 - 07:21</v>
       </c>
       <c r="W36" t="str">
-        <v>卡爾先生在此段落深入探討美元信用可能面臨的挑戰，回顧1970年代美國解除美元與黃金掛鉤的歷史，並預測未來幾年美元可能貶值。主持人隨後提出地緣政治風險（如台海緊張）下，美元作為避險工具的有效性，並強調實體黃金在這種情境下的重要性。卡爾先生進一步解釋實體黃金作為唯一非任何國家負債的資產，其信用甚至高於國家信用。這段對話不僅分析了貨幣風險，更提供了具體的避險策略，內容豐富且具實用價值。</v>
+        <v>主持人分享翻看父母老照片的個人感觸，深刻體悟到時間的流逝與陪伴的重要性。這段情感真摯、語氣充滿感染力，是整集的情感高潮，提醒聽眾珍惜當下。</v>
       </c>
       <c r="X36" t="str">
-        <v>2026-06-21T02:21:27.811Z</v>
+        <v>2026-06-21T01:53:23.870Z</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Dr Selena</v>
+        <v>蕭邦</v>
       </c>
       <c r="B37" t="str">
-        <v>小資變有錢｜Dr.Selena生活理財王</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="C37" t="str">
-        <v>小資族如何成功打造第二條收入曲線：冒牌生的社群品牌經營策略免費教學！</v>
+        <v>如何度過負面情緒 ？</v>
       </c>
       <c r="D37">
-        <v>290</v>
+        <v>205</v>
       </c>
       <c r="E37" t="str">
         <v>中</v>
       </c>
       <c r="F37" t="str">
-        <v>主講人與來賓皆頻繁使用「然後」作為語句連接詞或轉折詞，以及「就是」用於解釋或強調。此外，「那」也常作為口頭禪或語氣詞出現。整體贅字頻率屬於中等。</v>
+        <v>主講人常在句首使用「那」作為轉折詞，頻率較高，但多數時候作為語氣連接而非純粹贅字。此外，「就是」和「然後」偶爾出現，整體贅字頻率屬於中等。</v>
       </c>
       <c r="G37" t="str">
-        <v>男主持人（冒牌生）聲音中低音共鳴飽滿，音色厚實且富有磁性，語調變化自然，情感表達真摯，聽感舒適且具說服力。女主持人（Selina）高音域清晰明亮，語速雖快但咬字清楚，聲音圓潤且帶有親和力，整體聽感溫暖且具陪伴感，不刺耳。</v>
+        <v>女主持人聲音溫暖、圓潤，中低音域表現穩定，高音域不刺耳，整體語調富有情感，給人一種溫馨且具陪伴感的聽覺體驗。</v>
       </c>
       <c r="H37" t="str">
         <v>優</v>
@@ -60506,46 +60506,46 @@
         <v>無</v>
       </c>
       <c r="K37" t="str">
-        <v>環境安靜，幾乎無���噪</v>
+        <v>環境安靜，幾乎無底噪</v>
       </c>
       <c r="L37" t="str">
-        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰的聽覺體驗。</v>
+        <v>整體錄音品質極佳，音量平穩，人聲清晰，沒有任何噴麥、突兀爆音或背景雜音，聽感非常舒���。</v>
       </c>
       <c r="M37" t="str">
-        <v>00:55 - 01:26</v>
+        <v>00:12 - 00:31</v>
       </c>
       <c r="N37" t="str">
-        <v>主持人熱情介紹嘉賓「冒牌生」及其在社群經營上的專長，並點出本集節目將探討如何透過社群媒體創造主動與被動收入，有效引導聽眾進入主題，為節目奠定良好開場。</v>
+        <v>主持人以自身經歷引出「情緒」這個主題，語氣真誠，迅速建立與聽眾的連結，引人入勝，為節目內容做了很好的鋪墊。</v>
       </c>
       <c r="O37" t="str">
-        <v>嘉賓介紹與節目主題</v>
+        <v>開場：情緒的引導與個人經驗分享</v>
       </c>
       <c r="P37" t="str">
-        <v>00:55 - 01:26</v>
+        <v>00:12 - 00:31</v>
       </c>
       <c r="Q37" t="str">
-        <v>主持人熱情介紹嘉賓「冒牌生」及其在社群經營上的專長，並點出本集節目將探討如何透過社群媒體創造主動與被動收入，有效引導聽眾進入主題，為節目奠定良好開場。</v>
+        <v>主持人以自身經歷引出「情緒」這個主題，語氣真誠，迅速建立與聽眾的連結，引人入勝，為節目內容做了很好的鋪墊。</v>
       </c>
       <c r="R37" t="str">
-        <v>成功案例：從洗頭店找到社群藍海</v>
+        <v>核心論述：關閉腦袋，讓情緒流動</v>
       </c>
       <c r="S37" t="str">
-        <v>01:40:45 - 01:48:00</v>
+        <v>04:05 - 04:55</v>
       </c>
       <c r="T37" t="str">
-        <v>冒牌生分享一位學生透過分享洗頭店心得，成功累積大量粉絲的案例。此段落具體展現了如何將個人興趣與在地特色結合，創造獨特且受歡迎的內容，為聽眾提供實用的社群經營啟發，極具參考價值。</v>
+        <v>此段落是節目的核心精華，主持人清晰地闡述了處理情緒的關鍵方法——「關閉腦袋，讓情緒自然流動」，並解釋了其背後的原因，提供了具體且實用的建議，極具啟發性。</v>
       </c>
       <c r="U37" t="str">
-        <v>享受創作過程的智慧</v>
+        <v>總結：接受情緒，有效解決問題</v>
       </c>
       <c r="V37" t="str">
-        <v>02:21:00 - 02:26:00</v>
+        <v>05:43 - 06:10</v>
       </c>
       <c r="W37" t="str">
-        <v>冒牌生引用《享受吧！一個人的旅行》作者的經歷，闡述了享受創作過程本身的重要性，而非過度追求外在的成就與評價。這段對話深刻且富有哲理，鼓勵聽眾回歸初心，從熱愛的事物中獲得真正的快樂與滿足，��有啟發性。</v>
+        <v>這段總結了節目主旨，強調接受所有情緒的重要性及其帶來的益處，語氣溫和且具說服力，為聽眾提供正向的啟發，並引導聽眾思考如何有效解決問題。</v>
       </c>
       <c r="X37" t="str">
-        <v>2026-06-21T01:54:11.639Z</v>
+        <v>2026-06-21T00:40:44.043Z</v>
       </c>
     </row>
     <row r="38">
@@ -60556,75 +60556,223 @@
         <v>小資變有錢｜Dr.Selena生活理財王</v>
       </c>
       <c r="C38" t="str">
-        <v>小資愛樂活：用理財，走進千年古文明~此生必走一次的中亞絲路!</v>
+        <v>2026小資族一定要看懂4個關鍵總經變數 !</v>
       </c>
       <c r="D38">
-        <v>270</v>
+        <v>205</v>
       </c>
       <c r="E38" t="str">
         <v>中</v>
       </c>
       <c r="F38" t="str">
-        <v>兩位主持人皆頻繁使用「然後」和「就是」作為語句連接詞，尤其常出現在句首。此外，「那」和「這個」也偶爾出現，整體贅字頻率屬於中等。</v>
+        <v>兩位主講人皆習慣在句首或句中頻繁使用「就是」、「然後」、「那」作為語氣詞或轉折詞，頻率中等。</v>
       </c>
       <c r="G38" t="str">
-        <v>女主持人Selina的聲音清晰、明亮且充滿活力，高音域圓潤不刺耳，語氣溫暖且具陪伴感。男主持人Domingo的聲音低沉、渾厚且富有共鳴，中低音域表現出色，給人穩重、權威而友善的感覺。兩位主持人的聲音特質都非常適合廣播。</v>
+        <v>女主持人（Data Selina）的聲音高亢、清晰且充滿活力，語調明亮，給人溫暖且具陪伴感的印象，沒有刺耳感。男主持人（卡爾先生）的聲音低沉、厚實且共鳴感強，語氣沉穩而專業，表達流暢，沒有機器人唸稿感。</v>
       </c>
       <c r="H38" t="str">
         <v>優</v>
       </c>
       <c r="I38" t="str">
-        <v>無</v>
+        <v>���</v>
       </c>
       <c r="J38" t="str">
         <v>無</v>
       </c>
       <c r="K38" t="str">
+        <v>環境安靜，幾乎無底噪</v>
+      </c>
+      <c r="L38" t="str">
+        <v>整體錄音品質優良，音量平穩，兩位主講人的聲音清晰，沒有突兀爆音與噴麥現象，背景噪音極低。</v>
+      </c>
+      <c r="M38" t="str">
+        <v>00:07 - 00:57</v>
+      </c>
+      <c r="N38" t="str">
+        <v>主持人以清晰的語調介紹節目宗旨，並迅速帶入本集主題「小資必學的2024總體經濟」。隨後，她以熱情且專業的方式介紹來賓卡爾先生，卡爾先生的開場白也展現其專業與自信，為節目奠定良好的基調。此段落語速適中，內容引人入勝，有效抓住聽眾注意力。</v>
+      </c>
+      <c r="O38" t="str">
+        <v>節目開場與總體經濟專家介紹</v>
+      </c>
+      <c r="P38" t="str">
+        <v>00:07 - 00:57</v>
+      </c>
+      <c r="Q38" t="str">
+        <v>主持人以清晰的語調介紹節目宗旨，並迅速帶入本集主題「小資必學的2024總體經濟」。隨後，她以熱情且專業的方式介紹來賓卡爾先生，卡爾先生的開場白也展現其專業與自信，為節目奠定良好的基調。此段落語速適中，內容引人入勝，有效抓住聽眾注意力。</v>
+      </c>
+      <c r="R38" t="str">
+        <v>居高思危：美股高點與潛在修正風險</v>
+      </c>
+      <c r="S38" t="str">
+        <v>02:58 - 04:43</v>
+      </c>
+      <c r="T38" t="str">
+        <v>卡爾先生在此段落精闢地指出2024年全球經濟的關鍵詞是「居高思危」。他引用標普500指數創65年新高，並以2000年網路泡沫破裂的歷史經驗為鑑，警示股市可能面臨20-30%的修正。他強調這是「數學的力量」和「週期」���必然，並將美股與台股的連動性納入考量，提醒聽眾做好心理準備。此段論述邏輯清晰，數據支持有力，語氣嚴謹，具高度警示性。</v>
+      </c>
+      <c r="U38" t="str">
+        <v>美元信用危機與實體黃金的避險策略</v>
+      </c>
+      <c r="V38" t="str">
+        <v>17:07 - 19:30</v>
+      </c>
+      <c r="W38" t="str">
+        <v>卡爾先生在此段落深入探討美元信用可能面臨的挑戰，回顧1970年代美國解除美元與黃金掛鉤的歷史，並預測未來幾年美元可能貶值。主持人隨後提出地緣政治風險（如台海緊張）下，美元作為避險工具的有效性，並強調實體黃金在這種情境下的重要性。卡爾先生進一步解釋實體黃金作為唯一非任何國家負債的資產，其信用甚至高於國家信用。這段對話不僅分析了貨幣風險，更提供了具體的避險策略，內容豐富且具實用價值。</v>
+      </c>
+      <c r="X38" t="str">
+        <v>2026-06-21T02:21:27.811Z</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Dr Selena</v>
+      </c>
+      <c r="B39" t="str">
+        <v>小資變有錢｜Dr.Selena生活理財王</v>
+      </c>
+      <c r="C39" t="str">
+        <v>小資族如何成功打造第二條收入曲線：冒牌生的社群品牌經營策略免費教學！</v>
+      </c>
+      <c r="D39">
+        <v>290</v>
+      </c>
+      <c r="E39" t="str">
+        <v>中</v>
+      </c>
+      <c r="F39" t="str">
+        <v>主講人與來賓皆頻繁使用「然後」作為語句連接詞或轉折詞，以及「就是」用於解釋或強調。此外，「那」也常作為口頭禪或語氣詞出現。整體贅字頻率屬於中等。</v>
+      </c>
+      <c r="G39" t="str">
+        <v>男主持人（冒牌生）聲音中低音共鳴飽滿，音色厚實且富有磁性，語調變化自然，情感表達真摯，聽感舒適且具說服力。女主持人（Selina）高音域清晰明亮，語速雖快但咬字清楚，聲音圓潤且帶有親和力，整體聽感溫暖且具陪伴感，不刺耳。</v>
+      </c>
+      <c r="H39" t="str">
+        <v>優</v>
+      </c>
+      <c r="I39" t="str">
+        <v>無</v>
+      </c>
+      <c r="J39" t="str">
+        <v>無</v>
+      </c>
+      <c r="K39" t="str">
+        <v>環境安靜，幾乎無���噪</v>
+      </c>
+      <c r="L39" t="str">
+        <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，提供清晰的聽覺體驗。</v>
+      </c>
+      <c r="M39" t="str">
+        <v>00:55 - 01:26</v>
+      </c>
+      <c r="N39" t="str">
+        <v>主持人熱情介紹嘉賓「冒牌生」及其在社群經營上的專長，並點出本集節目將探討如何透過社群媒體創造主動與被動收入，有效引導聽眾進入主題，為節目奠定良好開場。</v>
+      </c>
+      <c r="O39" t="str">
+        <v>嘉賓介紹與節目主題</v>
+      </c>
+      <c r="P39" t="str">
+        <v>00:55 - 01:26</v>
+      </c>
+      <c r="Q39" t="str">
+        <v>主持人熱情介紹嘉賓「冒牌生」及其在社群經營上的專長，並點出本集節目將探討如何透過社群媒體創造主動與被動收入，有效引導聽眾進入主題，為節目奠定良好開場。</v>
+      </c>
+      <c r="R39" t="str">
+        <v>成功案例：從洗頭店找到社群藍海</v>
+      </c>
+      <c r="S39" t="str">
+        <v>01:40:45 - 01:48:00</v>
+      </c>
+      <c r="T39" t="str">
+        <v>冒牌生分享一位學生透過分享洗頭店心得，成功累積大量粉絲的案例。此段落具體展現了如何將個人興趣與在地特色結合，創造獨特且受歡迎的內容，為聽眾提供實用的社群經營啟發，極具參考價值。</v>
+      </c>
+      <c r="U39" t="str">
+        <v>享受創作過程的智慧</v>
+      </c>
+      <c r="V39" t="str">
+        <v>02:21:00 - 02:26:00</v>
+      </c>
+      <c r="W39" t="str">
+        <v>冒牌生引用《享受吧！一個人的旅行》作者的經歷，闡述了享受創作過程本身的重要性，而非過度追求外在的成就與評價。這段對話深刻且富有哲理，鼓勵聽眾回歸初心，從熱愛的事物中獲得真正的快樂與滿足，��有啟發性。</v>
+      </c>
+      <c r="X39" t="str">
+        <v>2026-06-21T01:54:11.639Z</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Dr Selena</v>
+      </c>
+      <c r="B40" t="str">
+        <v>小資變有錢｜Dr.Selena生活理財王</v>
+      </c>
+      <c r="C40" t="str">
+        <v>小資愛樂活：用理財，走進千年古文明~此生必走一次的中亞絲路!</v>
+      </c>
+      <c r="D40">
+        <v>270</v>
+      </c>
+      <c r="E40" t="str">
+        <v>中</v>
+      </c>
+      <c r="F40" t="str">
+        <v>兩位主持人皆頻繁使用「然後」和「就是」作為語句連接詞，尤其常出現在句首。此外，「那」和「這個」也偶爾出現，整體贅字頻率屬於中等。</v>
+      </c>
+      <c r="G40" t="str">
+        <v>女主持人Selina的聲音清晰、明亮且充滿活力，高音域圓潤不刺耳，語氣溫暖且具陪伴感。男主持人Domingo的聲音低沉、渾厚且富有共鳴，中低音域表現出色，給人穩重、權威而友善的感覺。兩位主持人的聲音特質都非常適合廣播。</v>
+      </c>
+      <c r="H40" t="str">
+        <v>優</v>
+      </c>
+      <c r="I40" t="str">
+        <v>無</v>
+      </c>
+      <c r="J40" t="str">
+        <v>無</v>
+      </c>
+      <c r="K40" t="str">
         <v>環境安靜，幾乎無底噪，僅有極輕微的環境音，不影響聆聽體驗。</v>
       </c>
-      <c r="L38" t="str">
+      <c r="L40" t="str">
         <v>整體錄音品質優良，音量平穩，沒有突兀爆音與噴麥現象，背景噪音極低，音質清晰。</v>
       </c>
-      <c r="M38" t="str">
+      <c r="M40" t="str">
         <v>01:45 - 02:30</v>
       </c>
-      <c r="N38" t="str">
+      <c r="N40" t="str">
         <v>男主持人Domingo以「世界是一本書」的經典比喻開場，並提出「旅行是無知的解藥」的獨特觀點，深入探討旅行如何打破同溫層、拓展個人價值觀。這段內容富有哲理，語速適中，能有效引導聽眾思考。</v>
       </c>
-      <c r="O38" t="str">
+      <c r="O40" t="str">
         <v>旅遊的意義與世界觀的拓展</v>
       </c>
-      <c r="P38" t="str">
+      <c r="P40" t="str">
         <v>01:45 - 02:30</v>
       </c>
-      <c r="Q38" t="str">
+      <c r="Q40" t="str">
         <v>男主持人Domingo以「世界是一本書」的經典比喻開場，並提出「旅行是無知的解藥」的獨特觀點，深入探討旅行如何打破同溫層、拓展個人價值觀。這段內容富有哲理，語速適中，能有效引導聽眾思考。</v>
       </c>
-      <c r="R38" t="str">
+      <c r="R40" t="str">
         <v>透過旅行認識真實世界</v>
       </c>
-      <c r="S38" t="str">
+      <c r="S40" t="str">
         <v>09:47 - 10:13</v>
       </c>
-      <c r="T38" t="str">
+      <c r="T40" t="str">
         <v>女主持人Selina與Domingo對談，指出媒體塑造的世界觀可能與真實世界存在差異，強調親身旅行才能體驗到更完整的世界。Selina更感性地表達「我旅行，我存在，我幸福」，展現旅行對她生命的重要性，對話真誠且具啟發性。</v>
       </c>
-      <c r="U38" t="str">
+      <c r="U40" t="str">
         <v>旅遊業的挑戰與領隊的辛勞</v>
       </c>
-      <c r="V38" t="str">
+      <c r="V40" t="str">
         <v>12:01 - 12:30</v>
       </c>
-      <c r="W38" t="str">
+      <c r="W40" t="str">
         <v>Selina分享了她帶團去尼泊爾時遇到的修路、坐船等突發狀況，以及旅遊業面臨的天災人禍挑戰，凸顯了領隊和導遊的壓力與辛勞。這段內容真實有趣，讓聽眾對旅遊從��人員的付出有更深的理解與共情。</v>
       </c>
-      <c r="X38" t="str">
+      <c r="X40" t="str">
         <v>2026-06-21T01:55:02.849Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:X38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X40"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>